<commit_message>
Clean Dribl team names in parser; show fixtures as 'Home v Away' with league below
</commit_message>
<xml_diff>
--- a/Manningham_fixtures_and_overlaps.xlsx
+++ b/Manningham_fixtures_and_overlaps.xlsx
@@ -827,7 +827,7 @@
       </c>
       <c r="L2" s="10" t="inlineStr">
         <is>
-          <t>Caboolture Sports FC Caboolture Sports FC Senior Men</t>
+          <t>Caboolture Sports FC Senior Men</t>
         </is>
       </c>
       <c r="M2" s="10" t="inlineStr">
@@ -6286,7 +6286,7 @@
       </c>
       <c r="K74" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC Seniors MUFC - State League Women's</t>
+          <t>Manningham United Blues FC Seniors</t>
         </is>
       </c>
       <c r="L74" s="10" t="inlineStr">
@@ -6362,12 +6362,12 @@
       </c>
       <c r="K75" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U8J (Slater's)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed (Slater's)</t>
         </is>
       </c>
       <c r="L75" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U8J (Duke's)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed (Duke's)</t>
         </is>
       </c>
       <c r="M75" s="12" t="inlineStr">
@@ -6438,12 +6438,12 @@
       </c>
       <c r="K76" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U7J (White)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (White)</t>
         </is>
       </c>
       <c r="L76" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U7J (Purple)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Purple)</t>
         </is>
       </c>
       <c r="M76" s="10" t="inlineStr">
@@ -6514,7 +6514,7 @@
       </c>
       <c r="K77" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - B Mixed MUFC - Junior Boys U12B (Andre)</t>
+          <t>Manningham United Blues FC U12 Juniors - B Mixed (Andre)</t>
         </is>
       </c>
       <c r="L77" s="12" t="inlineStr">
@@ -6666,7 +6666,7 @@
       </c>
       <c r="K79" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U10 MiniRoos - Kangaroos Mixed MUFC - Miniroos Boys U10 Kangas</t>
+          <t>Manningham United Blues FC U10 MiniRoos - Kangaroos Mixed</t>
         </is>
       </c>
       <c r="L79" s="12" t="inlineStr">
@@ -6742,7 +6742,7 @@
       </c>
       <c r="K80" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U9W (Souttar's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Souttar's)</t>
         </is>
       </c>
       <c r="L80" s="10" t="inlineStr">
@@ -7578,7 +7578,7 @@
       </c>
       <c r="K91" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC Seniors MUFC - State League Women's</t>
+          <t>Manningham United Blues FC Seniors</t>
         </is>
       </c>
       <c r="L91" s="12" t="inlineStr">
@@ -7654,7 +7654,7 @@
       </c>
       <c r="K92" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC Seniors MUFC - Women's Metro League</t>
+          <t>Manningham United Blues FC Seniors</t>
         </is>
       </c>
       <c r="L92" s="10" t="inlineStr">
@@ -7730,7 +7730,7 @@
       </c>
       <c r="K93" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U8J (Slater's)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed (Slater's)</t>
         </is>
       </c>
       <c r="L93" s="12" t="inlineStr">
@@ -8034,7 +8034,7 @@
       </c>
       <c r="K97" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U8J (Duke's)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed (Duke's)</t>
         </is>
       </c>
       <c r="L97" s="12" t="inlineStr">
@@ -8110,7 +8110,7 @@
       </c>
       <c r="K98" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U7J (White)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (White)</t>
         </is>
       </c>
       <c r="L98" s="10" t="inlineStr">
@@ -8186,7 +8186,7 @@
       </c>
       <c r="K99" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U7J (Purple)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Purple)</t>
         </is>
       </c>
       <c r="L99" s="12" t="inlineStr">
@@ -8262,7 +8262,7 @@
       </c>
       <c r="K100" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U9W (Corica's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Corica's)</t>
         </is>
       </c>
       <c r="L100" s="10" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="K106" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - A Female MUFC - Junior Girls U12A (Sienna)</t>
+          <t>Manningham United Blues FC U12 Juniors - A Female (Sienna)</t>
         </is>
       </c>
       <c r="L106" s="10" t="inlineStr">
@@ -8794,7 +8794,7 @@
       </c>
       <c r="K107" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - C Female MUFC - Junior Girls U12C (Tahlia)</t>
+          <t>Manningham United Blues FC U12 Juniors - C Female (Tahlia)</t>
         </is>
       </c>
       <c r="L107" s="12" t="inlineStr">
@@ -8870,7 +8870,7 @@
       </c>
       <c r="K108" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U17/18 Juniors - B Female MUFC - Junior Girls 17/18 (Marilyn)</t>
+          <t>Manningham United Blues FC U17/18 Juniors - B Female (Marilyn)</t>
         </is>
       </c>
       <c r="L108" s="10" t="inlineStr">
@@ -9022,7 +9022,7 @@
       </c>
       <c r="K110" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - B Mixed MUFC - Junior Boys U12B (Chris)</t>
+          <t>Manningham United Blues FC U12 Juniors - B Mixed (Chris)</t>
         </is>
       </c>
       <c r="L110" s="10" t="inlineStr">
@@ -9098,7 +9098,7 @@
       </c>
       <c r="K111" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - B Mixed MUFC - Junior Boys U12B (Andre)</t>
+          <t>Manningham United Blues FC U12 Juniors - B Mixed (Andre)</t>
         </is>
       </c>
       <c r="L111" s="12" t="inlineStr">
@@ -9326,7 +9326,7 @@
       </c>
       <c r="K114" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U10 MiniRoos - Kangaroos Mixed MUFC - Miniroos Boys U10 Kangas</t>
+          <t>Manningham United Blues FC U10 MiniRoos - Kangaroos Mixed</t>
         </is>
       </c>
       <c r="L114" s="10" t="inlineStr">
@@ -9402,7 +9402,7 @@
       </c>
       <c r="K115" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U9W (Souttar's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Souttar's)</t>
         </is>
       </c>
       <c r="L115" s="12" t="inlineStr">
@@ -9478,7 +9478,7 @@
       </c>
       <c r="K116" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - A Mixed MUFC - Junior Boys U12A (John)</t>
+          <t>Manningham United Blues FC U12 Juniors - A Mixed (John)</t>
         </is>
       </c>
       <c r="L116" s="10" t="inlineStr">
@@ -9554,7 +9554,7 @@
       </c>
       <c r="K117" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - A Female MUFC - Junior Girls U14A (Chloe)</t>
+          <t>Manningham United Blues FC U14 Juniors - A Female (Chloe)</t>
         </is>
       </c>
       <c r="L117" s="12" t="inlineStr">
@@ -9630,7 +9630,7 @@
       </c>
       <c r="K118" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U15 Juniors - A Mixed MUFC - Junior Boys U15A</t>
+          <t>Manningham United Blues FC U15 Juniors - A Mixed</t>
         </is>
       </c>
       <c r="L118" s="10" t="inlineStr">
@@ -9706,7 +9706,7 @@
       </c>
       <c r="K119" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U18 Juniors - A Male MUFC - Junior Boys U18A</t>
+          <t>Manningham United Blues FC U18 Juniors - A Male</t>
         </is>
       </c>
       <c r="L119" s="12" t="inlineStr">
@@ -9782,7 +9782,7 @@
       </c>
       <c r="K120" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U10 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U10J (Sainsbury's)</t>
+          <t>Manningham United Blues FC U10 MiniRoos - Joeys Mixed (Sainsbury's)</t>
         </is>
       </c>
       <c r="L120" s="10" t="inlineStr">
@@ -9858,7 +9858,7 @@
       </c>
       <c r="K121" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - B Mixed MUFC - Junior Boys U12B (Robert)</t>
+          <t>Manningham United Blues FC U12 Juniors - B Mixed (Robert)</t>
         </is>
       </c>
       <c r="L121" s="12" t="inlineStr">
@@ -9934,7 +9934,7 @@
       </c>
       <c r="K122" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - C Mixed MUFC - Junior Boys U13C (Martin)</t>
+          <t>Manningham United Blues FC U13 Juniors - C Mixed (Martin)</t>
         </is>
       </c>
       <c r="L122" s="10" t="inlineStr">
@@ -10010,7 +10010,7 @@
       </c>
       <c r="K123" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - B Mixed MUFC - Junior Boys U14B</t>
+          <t>Manningham United Blues FC U14 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="L123" s="12" t="inlineStr">
@@ -10086,7 +10086,7 @@
       </c>
       <c r="K124" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U16 Juniors - B Mixed MUFC - Junior Boys U16B</t>
+          <t>Manningham United Blues FC U16 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="L124" s="10" t="inlineStr">
@@ -10162,7 +10162,7 @@
       </c>
       <c r="K125" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U16 Juniors - A Mixed MUFC - Junior Boys U16A</t>
+          <t>Manningham United Blues FC U16 Juniors - A Mixed</t>
         </is>
       </c>
       <c r="L125" s="12" t="inlineStr">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="K127" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U7J (White)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (White)</t>
         </is>
       </c>
       <c r="L127" s="12" t="inlineStr">
@@ -10390,7 +10390,7 @@
       </c>
       <c r="K128" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U7J (Purple)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Purple)</t>
         </is>
       </c>
       <c r="L128" s="10" t="inlineStr">
@@ -10466,7 +10466,7 @@
       </c>
       <c r="K129" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U10 MiniRoos - Kangaroos Mixed MUFC - Miniroos Boys U10 Kangas</t>
+          <t>Manningham United Blues FC U10 MiniRoos - Kangaroos Mixed</t>
         </is>
       </c>
       <c r="L129" s="12" t="inlineStr">
@@ -10770,7 +10770,7 @@
       </c>
       <c r="K133" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U8J (Slater's)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed (Slater's)</t>
         </is>
       </c>
       <c r="L133" s="12" t="inlineStr">
@@ -10846,7 +10846,7 @@
       </c>
       <c r="K134" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U8J (Duke's)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed (Duke's)</t>
         </is>
       </c>
       <c r="L134" s="10" t="inlineStr">
@@ -10922,7 +10922,7 @@
       </c>
       <c r="K135" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U9W (Corica's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Corica's)</t>
         </is>
       </c>
       <c r="L135" s="12" t="inlineStr">
@@ -11682,7 +11682,7 @@
       </c>
       <c r="K145" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U11W (Culina's)</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Mixed (Culina's)</t>
         </is>
       </c>
       <c r="L145" s="12" t="inlineStr">
@@ -11758,7 +11758,7 @@
       </c>
       <c r="K146" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - B Mixed MUFC - Junior Boys U12B (Andre)</t>
+          <t>Manningham United Blues FC U12 Juniors - B Mixed (Andre)</t>
         </is>
       </c>
       <c r="L146" s="10" t="inlineStr">
@@ -11834,7 +11834,7 @@
       </c>
       <c r="K147" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - B Mixed MUFC - Junior Boys U12B (Chris)</t>
+          <t>Manningham United Blues FC U12 Juniors - B Mixed (Chris)</t>
         </is>
       </c>
       <c r="L147" s="12" t="inlineStr">
@@ -11910,12 +11910,12 @@
       </c>
       <c r="K148" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U9W (Souttar's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Souttar's)</t>
         </is>
       </c>
       <c r="L148" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U9W (Corica's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Corica's)</t>
         </is>
       </c>
       <c r="M148" s="10" t="inlineStr">
@@ -11986,12 +11986,12 @@
       </c>
       <c r="K149" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U7J (Red)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Red)</t>
         </is>
       </c>
       <c r="L149" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U7J (Green)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Green)</t>
         </is>
       </c>
       <c r="M149" s="12" t="inlineStr">
@@ -12062,7 +12062,7 @@
       </c>
       <c r="K150" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - C Female MUFC - Junior Girls U12C (Tahlia)</t>
+          <t>Manningham United Blues FC U12 Juniors - C Female (Tahlia)</t>
         </is>
       </c>
       <c r="L150" s="10" t="inlineStr">
@@ -12366,7 +12366,7 @@
       </c>
       <c r="K154" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - A Mixed MUFC - Junior Boys U12A (John)</t>
+          <t>Manningham United Blues FC U12 Juniors - A Mixed (John)</t>
         </is>
       </c>
       <c r="L154" s="10" t="inlineStr">
@@ -12442,7 +12442,7 @@
       </c>
       <c r="K155" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - A Female MUFC - Junior Girls U14A (Chloe)</t>
+          <t>Manningham United Blues FC U14 Juniors - A Female (Chloe)</t>
         </is>
       </c>
       <c r="L155" s="12" t="inlineStr">
@@ -12518,7 +12518,7 @@
       </c>
       <c r="K156" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC Seniors MUFC - State League Women's</t>
+          <t>Manningham United Blues FC Seniors</t>
         </is>
       </c>
       <c r="L156" s="10" t="inlineStr">
@@ -12670,7 +12670,7 @@
       </c>
       <c r="K158" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC Seniors MUFC - Women's Metro League</t>
+          <t>Manningham United Blues FC Seniors</t>
         </is>
       </c>
       <c r="L158" s="10" t="inlineStr">
@@ -12746,7 +12746,7 @@
       </c>
       <c r="K159" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U8J (Duke's)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed (Duke's)</t>
         </is>
       </c>
       <c r="L159" s="12" t="inlineStr">
@@ -12822,7 +12822,7 @@
       </c>
       <c r="K160" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U7J (White)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (White)</t>
         </is>
       </c>
       <c r="L160" s="10" t="inlineStr">
@@ -12898,7 +12898,7 @@
       </c>
       <c r="K161" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U7J (Purple)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Purple)</t>
         </is>
       </c>
       <c r="L161" s="12" t="inlineStr">
@@ -12974,7 +12974,7 @@
       </c>
       <c r="K162" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - B Mixed MUFC - Junior Boys U12B (Andre)</t>
+          <t>Manningham United Blues FC U12 Juniors - B Mixed (Andre)</t>
         </is>
       </c>
       <c r="L162" s="10" t="inlineStr">
@@ -13202,7 +13202,7 @@
       </c>
       <c r="K165" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U10 MiniRoos - Kangaroos Mixed MUFC - Miniroos Boys U10 Kangas</t>
+          <t>Manningham United Blues FC U10 MiniRoos - Kangaroos Mixed</t>
         </is>
       </c>
       <c r="L165" s="12" t="inlineStr">
@@ -13278,7 +13278,7 @@
       </c>
       <c r="K166" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U8J (Slater's)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed (Slater's)</t>
         </is>
       </c>
       <c r="L166" s="10" t="inlineStr">
@@ -13506,7 +13506,7 @@
       </c>
       <c r="K169" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U17/18 Juniors - B Female MUFC - Junior Girls 17/18 (Marilyn)</t>
+          <t>Manningham United Blues FC U17/18 Juniors - B Female (Marilyn)</t>
         </is>
       </c>
       <c r="L169" s="12" t="inlineStr">
@@ -13658,7 +13658,7 @@
       </c>
       <c r="K171" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - A Female MUFC - Junior Girls U12A (Sienna)</t>
+          <t>Manningham United Blues FC U12 Juniors - A Female (Sienna)</t>
         </is>
       </c>
       <c r="L171" s="12" t="inlineStr">
@@ -13886,7 +13886,7 @@
       </c>
       <c r="K174" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC Seniors MUFC - State League Women's</t>
+          <t>Manningham United Blues FC Seniors</t>
         </is>
       </c>
       <c r="L174" s="10" t="inlineStr">
@@ -14038,7 +14038,7 @@
       </c>
       <c r="K176" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC Seniors MUFC - State League Women's</t>
+          <t>Manningham United Blues FC Seniors</t>
         </is>
       </c>
       <c r="L176" s="10" t="inlineStr">
@@ -14114,12 +14114,12 @@
       </c>
       <c r="K177" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U8J (Slater's)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed (Slater's)</t>
         </is>
       </c>
       <c r="L177" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U8J (Duke's)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed (Duke's)</t>
         </is>
       </c>
       <c r="M177" s="12" t="inlineStr">
@@ -14190,7 +14190,7 @@
       </c>
       <c r="K178" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U10 MiniRoos - Kangaroos Mixed MUFC - Miniroos Boys U10 Kangas</t>
+          <t>Manningham United Blues FC U10 MiniRoos - Kangaroos Mixed</t>
         </is>
       </c>
       <c r="L178" s="10" t="inlineStr">
@@ -14266,7 +14266,7 @@
       </c>
       <c r="K179" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - B Mixed MUFC - Junior Boys U12B (Andre)</t>
+          <t>Manningham United Blues FC U12 Juniors - B Mixed (Andre)</t>
         </is>
       </c>
       <c r="L179" s="12" t="inlineStr">
@@ -14342,7 +14342,7 @@
       </c>
       <c r="K180" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - C Female MUFC - Junior Girls U14C (Christian)</t>
+          <t>Manningham United Blues FC U14 Juniors - C Female (Christian)</t>
         </is>
       </c>
       <c r="L180" s="10" t="inlineStr">
@@ -14418,7 +14418,7 @@
       </c>
       <c r="K181" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U15 Juniors - A Mixed MUFC - Junior Boys U15A</t>
+          <t>Manningham United Blues FC U15 Juniors - A Mixed</t>
         </is>
       </c>
       <c r="L181" s="12" t="inlineStr">
@@ -14494,7 +14494,7 @@
       </c>
       <c r="K182" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U16 Juniors - B Female MUFC - Junior Girls U16A (Eden)</t>
+          <t>Manningham United Blues FC U16 Juniors - B Female (Eden)</t>
         </is>
       </c>
       <c r="L182" s="10" t="inlineStr">
@@ -14570,7 +14570,7 @@
       </c>
       <c r="K183" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U16 Juniors - B Mixed MUFC - Junior Boys U16B</t>
+          <t>Manningham United Blues FC U16 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="L183" s="12" t="inlineStr">
@@ -14646,7 +14646,7 @@
       </c>
       <c r="K184" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - A Mixed MUFC - Junior Boys U12A (John)</t>
+          <t>Manningham United Blues FC U12 Juniors - A Mixed (John)</t>
         </is>
       </c>
       <c r="L184" s="10" t="inlineStr">
@@ -14722,7 +14722,7 @@
       </c>
       <c r="K185" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - A Mixed MUFC - Junior Boys U13A (George &amp; George)</t>
+          <t>Manningham United Blues FC U13 Juniors - A Mixed (George &amp; George)</t>
         </is>
       </c>
       <c r="L185" s="12" t="inlineStr">
@@ -14798,7 +14798,7 @@
       </c>
       <c r="K186" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - B Mixed MUFC - Junior Boys U14B</t>
+          <t>Manningham United Blues FC U14 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="L186" s="10" t="inlineStr">
@@ -14874,7 +14874,7 @@
       </c>
       <c r="K187" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U15 Juniors - B Mixed MUFC - Junior Boys U15B</t>
+          <t>Manningham United Blues FC U15 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="L187" s="12" t="inlineStr">
@@ -15026,7 +15026,7 @@
       </c>
       <c r="K189" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC Seniors MUFC - Women's Metro League</t>
+          <t>Manningham United Blues FC Seniors</t>
         </is>
       </c>
       <c r="L189" s="12" t="inlineStr">
@@ -15102,7 +15102,7 @@
       </c>
       <c r="K190" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U8J (Slater's)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed (Slater's)</t>
         </is>
       </c>
       <c r="L190" s="10" t="inlineStr">
@@ -15406,7 +15406,7 @@
       </c>
       <c r="K194" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U9W (Corica's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Corica's)</t>
         </is>
       </c>
       <c r="L194" s="10" t="inlineStr">
@@ -15482,7 +15482,7 @@
       </c>
       <c r="K195" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U7J (Purple)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Purple)</t>
         </is>
       </c>
       <c r="L195" s="12" t="inlineStr">
@@ -15558,7 +15558,7 @@
       </c>
       <c r="K196" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U8J (Duke's)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed (Duke's)</t>
         </is>
       </c>
       <c r="L196" s="10" t="inlineStr">
@@ -16394,7 +16394,7 @@
       </c>
       <c r="K207" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC Seniors MUFC - State League Women's</t>
+          <t>Manningham United Blues FC Seniors</t>
         </is>
       </c>
       <c r="L207" s="12" t="inlineStr">
@@ -16470,7 +16470,7 @@
       </c>
       <c r="K208" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U10 MiniRoos - Kangaroos Mixed MUFC - Miniroos Boys U10 Kangas</t>
+          <t>Manningham United Blues FC U10 MiniRoos - Kangaroos Mixed</t>
         </is>
       </c>
       <c r="L208" s="10" t="inlineStr">
@@ -16546,7 +16546,7 @@
       </c>
       <c r="K209" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U9W (Souttar's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Souttar's)</t>
         </is>
       </c>
       <c r="L209" s="12" t="inlineStr">
@@ -16622,7 +16622,7 @@
       </c>
       <c r="K210" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - B Mixed MUFC - Junior Boys U12B (Chris)</t>
+          <t>Manningham United Blues FC U12 Juniors - B Mixed (Chris)</t>
         </is>
       </c>
       <c r="L210" s="10" t="inlineStr">
@@ -16698,7 +16698,7 @@
       </c>
       <c r="K211" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - B Mixed MUFC - Junior Boys U12B (Andre)</t>
+          <t>Manningham United Blues FC U12 Juniors - B Mixed (Andre)</t>
         </is>
       </c>
       <c r="L211" s="12" t="inlineStr">
@@ -16774,7 +16774,7 @@
       </c>
       <c r="K212" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - C Female MUFC - Junior Girls U13C (Abigail)</t>
+          <t>Manningham United Blues FC U13 Juniors - C Female (Abigail)</t>
         </is>
       </c>
       <c r="L212" s="10" t="inlineStr">
@@ -16850,7 +16850,7 @@
       </c>
       <c r="K213" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - C Female MUFC - Junior Girls U12C (Tahlia)</t>
+          <t>Manningham United Blues FC U12 Juniors - C Female (Tahlia)</t>
         </is>
       </c>
       <c r="L213" s="12" t="inlineStr">
@@ -17078,7 +17078,7 @@
       </c>
       <c r="K216" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U16 Juniors - B Female MUFC - Junior Girls U16A (Eden)</t>
+          <t>Manningham United Blues FC U16 Juniors - B Female (Eden)</t>
         </is>
       </c>
       <c r="L216" s="10" t="inlineStr">
@@ -17230,7 +17230,7 @@
       </c>
       <c r="K218" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - A Mixed MUFC - Junior Boys U12A (John)</t>
+          <t>Manningham United Blues FC U12 Juniors - A Mixed (John)</t>
         </is>
       </c>
       <c r="L218" s="10" t="inlineStr">
@@ -17306,7 +17306,7 @@
       </c>
       <c r="K219" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - A Mixed MUFC - Junior Boys U13A (George &amp; George)</t>
+          <t>Manningham United Blues FC U13 Juniors - A Mixed (George &amp; George)</t>
         </is>
       </c>
       <c r="L219" s="12" t="inlineStr">
@@ -17382,7 +17382,7 @@
       </c>
       <c r="K220" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - A Female MUFC - Junior Girls U14A (Chloe)</t>
+          <t>Manningham United Blues FC U14 Juniors - A Female (Chloe)</t>
         </is>
       </c>
       <c r="L220" s="10" t="inlineStr">
@@ -17458,7 +17458,7 @@
       </c>
       <c r="K221" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - C Female MUFC - Junior Girls U14C (Christian)</t>
+          <t>Manningham United Blues FC U14 Juniors - C Female (Christian)</t>
         </is>
       </c>
       <c r="L221" s="12" t="inlineStr">
@@ -17534,7 +17534,7 @@
       </c>
       <c r="K222" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U15 Juniors - B Mixed MUFC - Junior Boys U15B</t>
+          <t>Manningham United Blues FC U15 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="L222" s="10" t="inlineStr">
@@ -17914,7 +17914,7 @@
       </c>
       <c r="K227" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U8J (Slater's)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed (Slater's)</t>
         </is>
       </c>
       <c r="L227" s="12" t="inlineStr">
@@ -17990,7 +17990,7 @@
       </c>
       <c r="K228" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U9W (Corica's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Corica's)</t>
         </is>
       </c>
       <c r="L228" s="10" t="inlineStr">
@@ -18066,7 +18066,7 @@
       </c>
       <c r="K229" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U7J (Purple)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Purple)</t>
         </is>
       </c>
       <c r="L229" s="12" t="inlineStr">
@@ -18142,7 +18142,7 @@
       </c>
       <c r="K230" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U8J (Duke's)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed (Duke's)</t>
         </is>
       </c>
       <c r="L230" s="10" t="inlineStr">
@@ -18598,7 +18598,7 @@
       </c>
       <c r="K236" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - A Mixed MUFC - Junior Boys U13A (Sam Z)</t>
+          <t>Manningham United Blues FC U13 Juniors - A Mixed (Sam Z)</t>
         </is>
       </c>
       <c r="L236" s="10" t="inlineStr">
@@ -18674,7 +18674,7 @@
       </c>
       <c r="K237" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U18 Juniors - A Male MUFC - Junior Boys U18A</t>
+          <t>Manningham United Blues FC U18 Juniors - A Male</t>
         </is>
       </c>
       <c r="L237" s="12" t="inlineStr">
@@ -18902,7 +18902,7 @@
       </c>
       <c r="K240" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U10 MiniRoos - Kangaroos Mixed MUFC - Miniroos Boys U10 Kangas</t>
+          <t>Manningham United Blues FC U10 MiniRoos - Kangaroos Mixed</t>
         </is>
       </c>
       <c r="L240" s="10" t="inlineStr">
@@ -18978,7 +18978,7 @@
       </c>
       <c r="K241" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U11W (Culina's)</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Mixed (Culina's)</t>
         </is>
       </c>
       <c r="L241" s="12" t="inlineStr">
@@ -19774,7 +19774,7 @@
       </c>
       <c r="K252" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U9W (Souttar's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Souttar's)</t>
         </is>
       </c>
       <c r="L252" s="10" t="inlineStr">
@@ -19850,7 +19850,7 @@
       </c>
       <c r="K253" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U9W (Corica's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Corica's)</t>
         </is>
       </c>
       <c r="L253" s="12" t="inlineStr">
@@ -19926,7 +19926,7 @@
       </c>
       <c r="K254" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - A Mixed MUFC - Junior Boys U13A (Sam Z)</t>
+          <t>Manningham United Blues FC U13 Juniors - A Mixed (Sam Z)</t>
         </is>
       </c>
       <c r="L254" s="10" t="inlineStr">
@@ -20002,7 +20002,7 @@
       </c>
       <c r="K255" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U15 Juniors - A Mixed MUFC - Junior Boys U15A</t>
+          <t>Manningham United Blues FC U15 Juniors - A Mixed</t>
         </is>
       </c>
       <c r="L255" s="12" t="inlineStr">
@@ -20078,7 +20078,7 @@
       </c>
       <c r="K256" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U16 Juniors - A Mixed MUFC - Junior Boys U16A</t>
+          <t>Manningham United Blues FC U16 Juniors - A Mixed</t>
         </is>
       </c>
       <c r="L256" s="10" t="inlineStr">
@@ -20230,7 +20230,7 @@
       </c>
       <c r="K258" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Joeys Female MUFC - Miniroos Girls U11J (Grace)</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Joeys Female (Grace)</t>
         </is>
       </c>
       <c r="L258" s="10" t="inlineStr">
@@ -20306,7 +20306,7 @@
       </c>
       <c r="K259" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - C Female MUFC - Junior Girls U13C (Abigail)</t>
+          <t>Manningham United Blues FC U13 Juniors - C Female (Abigail)</t>
         </is>
       </c>
       <c r="L259" s="12" t="inlineStr">
@@ -20382,7 +20382,7 @@
       </c>
       <c r="K260" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - B Mixed MUFC - Junior Boys U13B (Samir)</t>
+          <t>Manningham United Blues FC U13 Juniors - B Mixed (Samir)</t>
         </is>
       </c>
       <c r="L260" s="10" t="inlineStr">
@@ -20458,7 +20458,7 @@
       </c>
       <c r="K261" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - A Female MUFC - Junior Girls U14A (Chloe)</t>
+          <t>Manningham United Blues FC U14 Juniors - A Female (Chloe)</t>
         </is>
       </c>
       <c r="L261" s="12" t="inlineStr">
@@ -20534,7 +20534,7 @@
       </c>
       <c r="K262" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U15 Juniors - B Mixed MUFC - Junior Boys U15B</t>
+          <t>Manningham United Blues FC U15 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="L262" s="10" t="inlineStr">
@@ -20610,7 +20610,7 @@
       </c>
       <c r="K263" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U15 Juniors - B Female MUFC - Junior Girls U15B (Ethan)</t>
+          <t>Manningham United Blues FC U15 Juniors - B Female (Ethan)</t>
         </is>
       </c>
       <c r="L263" s="12" t="inlineStr">
@@ -20686,7 +20686,7 @@
       </c>
       <c r="K264" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC Seniors MUFC - State League Women's</t>
+          <t>Manningham United Blues FC Seniors</t>
         </is>
       </c>
       <c r="L264" s="10" t="inlineStr">
@@ -20762,7 +20762,7 @@
       </c>
       <c r="K265" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - B Mixed MUFC - Junior Boys U12B (Andre)</t>
+          <t>Manningham United Blues FC U12 Juniors - B Mixed (Andre)</t>
         </is>
       </c>
       <c r="L265" s="12" t="inlineStr">
@@ -20838,7 +20838,7 @@
       </c>
       <c r="K266" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U8J (Duke's)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed (Duke's)</t>
         </is>
       </c>
       <c r="L266" s="10" t="inlineStr">
@@ -20914,7 +20914,7 @@
       </c>
       <c r="K267" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U8J (Slater's)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed (Slater's)</t>
         </is>
       </c>
       <c r="L267" s="12" t="inlineStr">
@@ -21218,7 +21218,7 @@
       </c>
       <c r="K271" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U10 MiniRoos - Kangaroos Mixed MUFC - Miniroos Boys U10 Kangas</t>
+          <t>Manningham United Blues FC U10 MiniRoos - Kangaroos Mixed</t>
         </is>
       </c>
       <c r="L271" s="12" t="inlineStr">
@@ -21294,7 +21294,7 @@
       </c>
       <c r="K272" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U9W (Corica's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Corica's)</t>
         </is>
       </c>
       <c r="L272" s="10" t="inlineStr">
@@ -21750,7 +21750,7 @@
       </c>
       <c r="K278" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - A Female MUFC - Junior Girls U12A (Sienna)</t>
+          <t>Manningham United Blues FC U12 Juniors - A Female (Sienna)</t>
         </is>
       </c>
       <c r="L278" s="10" t="inlineStr">
@@ -21826,7 +21826,7 @@
       </c>
       <c r="K279" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - A Mixed MUFC - Junior Boys U12A (Hamid)</t>
+          <t>Manningham United Blues FC U12 Juniors - A Mixed (Hamid)</t>
         </is>
       </c>
       <c r="L279" s="12" t="inlineStr">
@@ -21902,7 +21902,7 @@
       </c>
       <c r="K280" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - A Mixed MUFC - Junior Boys U14A</t>
+          <t>Manningham United Blues FC U14 Juniors - A Mixed</t>
         </is>
       </c>
       <c r="L280" s="10" t="inlineStr">
@@ -21978,7 +21978,7 @@
       </c>
       <c r="K281" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U15 Juniors - B Mixed MUFC - Junior Boys U15B</t>
+          <t>Manningham United Blues FC U15 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="L281" s="12" t="inlineStr">
@@ -22130,7 +22130,7 @@
       </c>
       <c r="K283" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U11W (Culina's)</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Mixed (Culina's)</t>
         </is>
       </c>
       <c r="L283" s="12" t="inlineStr">
@@ -22206,12 +22206,12 @@
       </c>
       <c r="K284" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - B Mixed MUFC - Junior Boys U12B (Chris)</t>
+          <t>Manningham United Blues FC U12 Juniors - B Mixed (Chris)</t>
         </is>
       </c>
       <c r="L284" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - B Mixed MUFC - Junior Boys U12B (Andre)</t>
+          <t>Manningham United Blues FC U12 Juniors - B Mixed (Andre)</t>
         </is>
       </c>
       <c r="M284" s="10" t="inlineStr">
@@ -22510,7 +22510,7 @@
       </c>
       <c r="K288" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U9W (Souttar's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Souttar's)</t>
         </is>
       </c>
       <c r="L288" s="10" t="inlineStr">
@@ -22586,12 +22586,12 @@
       </c>
       <c r="K289" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U7J (White)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (White)</t>
         </is>
       </c>
       <c r="L289" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U7J (Purple)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Purple)</t>
         </is>
       </c>
       <c r="M289" s="12" t="inlineStr">
@@ -22662,7 +22662,7 @@
       </c>
       <c r="K290" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - A Female MUFC - Junior Girls U14A (Chloe)</t>
+          <t>Manningham United Blues FC U14 Juniors - A Female (Chloe)</t>
         </is>
       </c>
       <c r="L290" s="10" t="inlineStr">
@@ -23042,7 +23042,7 @@
       </c>
       <c r="K295" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - A Mixed MUFC - Junior Boys U12A (John)</t>
+          <t>Manningham United Blues FC U12 Juniors - A Mixed (John)</t>
         </is>
       </c>
       <c r="L295" s="12" t="inlineStr">
@@ -23118,7 +23118,7 @@
       </c>
       <c r="K296" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - A Mixed MUFC - Junior Boys U13A (Sam Z)</t>
+          <t>Manningham United Blues FC U13 Juniors - A Mixed (Sam Z)</t>
         </is>
       </c>
       <c r="L296" s="10" t="inlineStr">
@@ -23194,7 +23194,7 @@
       </c>
       <c r="K297" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U15 Juniors - B Female MUFC - Junior Girls U15B (Ethan)</t>
+          <t>Manningham United Blues FC U15 Juniors - B Female (Ethan)</t>
         </is>
       </c>
       <c r="L297" s="12" t="inlineStr">
@@ -23270,7 +23270,7 @@
       </c>
       <c r="K298" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U11W (Culina's)</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Mixed (Culina's)</t>
         </is>
       </c>
       <c r="L298" s="10" t="inlineStr">
@@ -23346,7 +23346,7 @@
       </c>
       <c r="K299" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - B Mixed MUFC - Junior Boys U12B (Chris)</t>
+          <t>Manningham United Blues FC U12 Juniors - B Mixed (Chris)</t>
         </is>
       </c>
       <c r="L299" s="12" t="inlineStr">
@@ -23422,12 +23422,12 @@
       </c>
       <c r="K300" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U8J (Duke's)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed (Duke's)</t>
         </is>
       </c>
       <c r="L300" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U8J (Slater's)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed (Slater's)</t>
         </is>
       </c>
       <c r="M300" s="10" t="inlineStr">
@@ -23650,7 +23650,7 @@
       </c>
       <c r="K303" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U10 MiniRoos - Kangaroos Mixed MUFC - Miniroos Boys U10 Kangas</t>
+          <t>Manningham United Blues FC U10 MiniRoos - Kangaroos Mixed</t>
         </is>
       </c>
       <c r="L303" s="12" t="inlineStr">
@@ -23726,7 +23726,7 @@
       </c>
       <c r="K304" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U9W (Corica's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Corica's)</t>
         </is>
       </c>
       <c r="L304" s="10" t="inlineStr">
@@ -23802,7 +23802,7 @@
       </c>
       <c r="K305" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U7J (Purple)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Purple)</t>
         </is>
       </c>
       <c r="L305" s="12" t="inlineStr">
@@ -24486,7 +24486,7 @@
       </c>
       <c r="K314" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U17/18 Juniors - B Female MUFC - Junior Girls 17/18 (Marilyn)</t>
+          <t>Manningham United Blues FC U17/18 Juniors - B Female (Marilyn)</t>
         </is>
       </c>
       <c r="L314" s="10" t="inlineStr">
@@ -24638,7 +24638,7 @@
       </c>
       <c r="K316" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC Seniors MUFC - State League Women's</t>
+          <t>Manningham United Blues FC Seniors</t>
         </is>
       </c>
       <c r="L316" s="10" t="inlineStr">
@@ -24714,7 +24714,7 @@
       </c>
       <c r="K317" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U7J (White)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (White)</t>
         </is>
       </c>
       <c r="L317" s="12" t="inlineStr">
@@ -24790,7 +24790,7 @@
       </c>
       <c r="K318" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - B Mixed MUFC - Junior Boys U12B (Andre)</t>
+          <t>Manningham United Blues FC U12 Juniors - B Mixed (Andre)</t>
         </is>
       </c>
       <c r="L318" s="10" t="inlineStr">
@@ -24866,12 +24866,12 @@
       </c>
       <c r="K319" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U9W (Souttar's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Souttar's)</t>
         </is>
       </c>
       <c r="L319" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U9W (Corica's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Corica's)</t>
         </is>
       </c>
       <c r="M319" s="12" t="inlineStr">
@@ -24942,7 +24942,7 @@
       </c>
       <c r="K320" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - B Mixed MUFC - Junior Boys U12B (Chris)</t>
+          <t>Manningham United Blues FC U12 Juniors - B Mixed (Chris)</t>
         </is>
       </c>
       <c r="L320" s="10" t="inlineStr">
@@ -25018,7 +25018,7 @@
       </c>
       <c r="K321" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - C Female MUFC - Junior Girls U13C (Abigail)</t>
+          <t>Manningham United Blues FC U13 Juniors - C Female (Abigail)</t>
         </is>
       </c>
       <c r="L321" s="12" t="inlineStr">
@@ -25094,7 +25094,7 @@
       </c>
       <c r="K322" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - B Mixed MUFC - Junior Boys U13B (Samir)</t>
+          <t>Manningham United Blues FC U13 Juniors - B Mixed (Samir)</t>
         </is>
       </c>
       <c r="L322" s="10" t="inlineStr">
@@ -25170,7 +25170,7 @@
       </c>
       <c r="K323" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - B Mixed MUFC - Junior Boys U14B</t>
+          <t>Manningham United Blues FC U14 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="L323" s="12" t="inlineStr">
@@ -25246,7 +25246,7 @@
       </c>
       <c r="K324" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - A Mixed MUFC - Junior Boys U14A</t>
+          <t>Manningham United Blues FC U14 Juniors - A Mixed</t>
         </is>
       </c>
       <c r="L324" s="10" t="inlineStr">
@@ -25322,7 +25322,7 @@
       </c>
       <c r="K325" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U16 Juniors - B Mixed MUFC - Junior Boys U16B</t>
+          <t>Manningham United Blues FC U16 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="L325" s="12" t="inlineStr">
@@ -25398,7 +25398,7 @@
       </c>
       <c r="K326" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Joeys Female MUFC - Miniroos Girls U8J (Yianna)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Joeys Female (Yianna)</t>
         </is>
       </c>
       <c r="L326" s="10" t="inlineStr">
@@ -25474,7 +25474,7 @@
       </c>
       <c r="K327" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U7J (Red)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Red)</t>
         </is>
       </c>
       <c r="L327" s="12" t="inlineStr">
@@ -25550,7 +25550,7 @@
       </c>
       <c r="K328" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U7J (Green)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Green)</t>
         </is>
       </c>
       <c r="L328" s="10" t="inlineStr">
@@ -25626,7 +25626,7 @@
       </c>
       <c r="K329" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Joeys Female MUFC - Miniroos Girls U11J (Grace)</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Joeys Female (Grace)</t>
         </is>
       </c>
       <c r="L329" s="12" t="inlineStr">
@@ -25702,7 +25702,7 @@
       </c>
       <c r="K330" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U9W (Cahill's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Cahill's)</t>
         </is>
       </c>
       <c r="L330" s="10" t="inlineStr">
@@ -25778,7 +25778,7 @@
       </c>
       <c r="K331" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Kangaroos Mixed MUFC - Miniroos Boys U9K (Emerton's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Kangaroos Mixed (Emerton's)</t>
         </is>
       </c>
       <c r="L331" s="12" t="inlineStr">
@@ -25854,7 +25854,7 @@
       </c>
       <c r="K332" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - A Female MUFC - Junior Girls U14A (Chloe)</t>
+          <t>Manningham United Blues FC U14 Juniors - A Female (Chloe)</t>
         </is>
       </c>
       <c r="L332" s="10" t="inlineStr">
@@ -25930,7 +25930,7 @@
       </c>
       <c r="K333" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U17/18 Juniors - B Female MUFC - Junior Girls 17/18 (Marilyn)</t>
+          <t>Manningham United Blues FC U17/18 Juniors - B Female (Marilyn)</t>
         </is>
       </c>
       <c r="L333" s="12" t="inlineStr">
@@ -26082,7 +26082,7 @@
       </c>
       <c r="K335" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U10 MiniRoos - Kangaroos Mixed MUFC - Miniroos Boys U10 Kangas</t>
+          <t>Manningham United Blues FC U10 MiniRoos - Kangaroos Mixed</t>
         </is>
       </c>
       <c r="L335" s="12" t="inlineStr">
@@ -26158,7 +26158,7 @@
       </c>
       <c r="K336" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U7J (Purple)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Purple)</t>
         </is>
       </c>
       <c r="L336" s="10" t="inlineStr">
@@ -26234,7 +26234,7 @@
       </c>
       <c r="K337" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U8J (Slater's)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed (Slater's)</t>
         </is>
       </c>
       <c r="L337" s="12" t="inlineStr">
@@ -26462,7 +26462,7 @@
       </c>
       <c r="K340" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U11W (Culina's)</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Mixed (Culina's)</t>
         </is>
       </c>
       <c r="L340" s="10" t="inlineStr">
@@ -26538,7 +26538,7 @@
       </c>
       <c r="K341" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U8J (Duke's)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed (Duke's)</t>
         </is>
       </c>
       <c r="L341" s="12" t="inlineStr">
@@ -26766,7 +26766,7 @@
       </c>
       <c r="K344" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U10 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U10J (Sainsbury's)</t>
+          <t>Manningham United Blues FC U10 MiniRoos - Joeys Mixed (Sainsbury's)</t>
         </is>
       </c>
       <c r="L344" s="10" t="inlineStr">
@@ -26842,7 +26842,7 @@
       </c>
       <c r="K345" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U10 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U10W (Tilio's)</t>
+          <t>Manningham United Blues FC U10 MiniRoos - Wallabies Mixed (Tilio's)</t>
         </is>
       </c>
       <c r="L345" s="12" t="inlineStr">
@@ -26918,7 +26918,7 @@
       </c>
       <c r="K346" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Kangaroos Mixed MUFC - Miniroos Boys U11 Kangas</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Kangaroos Mixed</t>
         </is>
       </c>
       <c r="L346" s="10" t="inlineStr">
@@ -26994,7 +26994,7 @@
       </c>
       <c r="K347" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U11W (Colosimo's)</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Mixed (Colosimo's)</t>
         </is>
       </c>
       <c r="L347" s="12" t="inlineStr">
@@ -27070,7 +27070,7 @@
       </c>
       <c r="K348" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U18 Juniors - A Male MUFC - Junior Boys U18A</t>
+          <t>Manningham United Blues FC U18 Juniors - A Male</t>
         </is>
       </c>
       <c r="L348" s="10" t="inlineStr">
@@ -27146,7 +27146,7 @@
       </c>
       <c r="K349" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - B Mixed MUFC - Junior Boys U12B (Andre)</t>
+          <t>Manningham United Blues FC U12 Juniors - B Mixed (Andre)</t>
         </is>
       </c>
       <c r="L349" s="12" t="inlineStr">
@@ -27222,7 +27222,7 @@
       </c>
       <c r="K350" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - B Mixed MUFC - Junior Boys U12B (Chris)</t>
+          <t>Manningham United Blues FC U12 Juniors - B Mixed (Chris)</t>
         </is>
       </c>
       <c r="L350" s="10" t="inlineStr">
@@ -27298,7 +27298,7 @@
       </c>
       <c r="K351" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U9W (Souttar's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Souttar's)</t>
         </is>
       </c>
       <c r="L351" s="12" t="inlineStr">
@@ -27374,7 +27374,7 @@
       </c>
       <c r="K352" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U9W (Corica's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Corica's)</t>
         </is>
       </c>
       <c r="L352" s="10" t="inlineStr">
@@ -27450,7 +27450,7 @@
       </c>
       <c r="K353" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U11W (Culina's)</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Mixed (Culina's)</t>
         </is>
       </c>
       <c r="L353" s="12" t="inlineStr">
@@ -27526,7 +27526,7 @@
       </c>
       <c r="K354" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U7J (White)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (White)</t>
         </is>
       </c>
       <c r="L354" s="10" t="inlineStr">
@@ -27982,7 +27982,7 @@
       </c>
       <c r="K360" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - A Mixed MUFC - Junior Boys U12A (John)</t>
+          <t>Manningham United Blues FC U12 Juniors - A Mixed (John)</t>
         </is>
       </c>
       <c r="L360" s="10" t="inlineStr">
@@ -28058,7 +28058,7 @@
       </c>
       <c r="K361" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - A Mixed MUFC - Junior Boys U13A (George &amp; George)</t>
+          <t>Manningham United Blues FC U13 Juniors - A Mixed (George &amp; George)</t>
         </is>
       </c>
       <c r="L361" s="12" t="inlineStr">
@@ -28134,7 +28134,7 @@
       </c>
       <c r="K362" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U15 Juniors - A Mixed MUFC - Junior Boys U15A</t>
+          <t>Manningham United Blues FC U15 Juniors - A Mixed</t>
         </is>
       </c>
       <c r="L362" s="10" t="inlineStr">
@@ -28590,7 +28590,7 @@
       </c>
       <c r="K368" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U7J (Red)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Red)</t>
         </is>
       </c>
       <c r="L368" s="10" t="inlineStr">
@@ -28666,7 +28666,7 @@
       </c>
       <c r="K369" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U9W (Cahill's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Cahill's)</t>
         </is>
       </c>
       <c r="L369" s="12" t="inlineStr">
@@ -28742,7 +28742,7 @@
       </c>
       <c r="K370" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U11W (Colosimo's)</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Mixed (Colosimo's)</t>
         </is>
       </c>
       <c r="L370" s="10" t="inlineStr">
@@ -28818,7 +28818,7 @@
       </c>
       <c r="K371" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U10 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U10J (Sainsbury's)</t>
+          <t>Manningham United Blues FC U10 MiniRoos - Joeys Mixed (Sainsbury's)</t>
         </is>
       </c>
       <c r="L371" s="12" t="inlineStr">
@@ -28894,7 +28894,7 @@
       </c>
       <c r="K372" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - A Mixed MUFC - Junior Boys U14A</t>
+          <t>Manningham United Blues FC U14 Juniors - A Mixed</t>
         </is>
       </c>
       <c r="L372" s="10" t="inlineStr">
@@ -28970,7 +28970,7 @@
       </c>
       <c r="K373" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U15 Juniors - A Mixed MUFC - Junior Boys U15A</t>
+          <t>Manningham United Blues FC U15 Juniors - A Mixed</t>
         </is>
       </c>
       <c r="L373" s="12" t="inlineStr">
@@ -29046,7 +29046,7 @@
       </c>
       <c r="K374" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U16 Juniors - A Mixed MUFC - Junior Boys U16A</t>
+          <t>Manningham United Blues FC U16 Juniors - A Mixed</t>
         </is>
       </c>
       <c r="L374" s="10" t="inlineStr">
@@ -29122,7 +29122,7 @@
       </c>
       <c r="K375" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - A Mixed MUFC - Junior Boys U12A (John)</t>
+          <t>Manningham United Blues FC U12 Juniors - A Mixed (John)</t>
         </is>
       </c>
       <c r="L375" s="12" t="inlineStr">
@@ -29198,7 +29198,7 @@
       </c>
       <c r="K376" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - A Mixed MUFC - Junior Boys U13A (Sam Z)</t>
+          <t>Manningham United Blues FC U13 Juniors - A Mixed (Sam Z)</t>
         </is>
       </c>
       <c r="L376" s="10" t="inlineStr">
@@ -29274,7 +29274,7 @@
       </c>
       <c r="K377" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - B Mixed MUFC - Junior Boys U14B</t>
+          <t>Manningham United Blues FC U14 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="L377" s="12" t="inlineStr">
@@ -29426,7 +29426,7 @@
       </c>
       <c r="K379" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Kangaroos Mixed MUFC - Miniroos Boys U11 Kangas</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Kangaroos Mixed</t>
         </is>
       </c>
       <c r="L379" s="12" t="inlineStr">
@@ -29502,7 +29502,7 @@
       </c>
       <c r="K380" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - C Mixed MUFC - Junior Boys U13C (Martin)</t>
+          <t>Manningham United Blues FC U13 Juniors - C Mixed (Martin)</t>
         </is>
       </c>
       <c r="L380" s="10" t="inlineStr">
@@ -29578,7 +29578,7 @@
       </c>
       <c r="K381" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - C Female MUFC - Junior Girls U13C (Abigail)</t>
+          <t>Manningham United Blues FC U13 Juniors - C Female (Abigail)</t>
         </is>
       </c>
       <c r="L381" s="12" t="inlineStr">
@@ -29654,7 +29654,7 @@
       </c>
       <c r="K382" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - B Mixed MUFC - Junior Boys U12B (Robert)</t>
+          <t>Manningham United Blues FC U12 Juniors - B Mixed (Robert)</t>
         </is>
       </c>
       <c r="L382" s="10" t="inlineStr">
@@ -29730,7 +29730,7 @@
       </c>
       <c r="K383" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U16 Juniors - B Mixed MUFC - Junior Boys U16B</t>
+          <t>Manningham United Blues FC U16 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="L383" s="12" t="inlineStr">
@@ -29806,7 +29806,7 @@
       </c>
       <c r="K384" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U18 Juniors - A Male MUFC - Junior Boys U18A</t>
+          <t>Manningham United Blues FC U18 Juniors - A Male</t>
         </is>
       </c>
       <c r="L384" s="10" t="inlineStr">
@@ -29882,7 +29882,7 @@
       </c>
       <c r="K385" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Kangaroos Mixed MUFC - Miniroos Boys U8K (Arnold's)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Kangaroos Mixed (Arnold's)</t>
         </is>
       </c>
       <c r="L385" s="12" t="inlineStr">
@@ -29958,7 +29958,7 @@
       </c>
       <c r="K386" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U8W (Coe's)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Wallabies Mixed (Coe's)</t>
         </is>
       </c>
       <c r="L386" s="10" t="inlineStr">
@@ -30034,7 +30034,7 @@
       </c>
       <c r="K387" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Kangaroos Mixed MUFC - Miniroos Boys U11 Kangas</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Kangaroos Mixed</t>
         </is>
       </c>
       <c r="L387" s="12" t="inlineStr">
@@ -30110,7 +30110,7 @@
       </c>
       <c r="K388" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U11W (Colosimo's)</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Mixed (Colosimo's)</t>
         </is>
       </c>
       <c r="L388" s="10" t="inlineStr">
@@ -30186,7 +30186,7 @@
       </c>
       <c r="K389" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Kangaroos Mixed MUFC - Miniroos Boys U9K (Emerton's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Kangaroos Mixed (Emerton's)</t>
         </is>
       </c>
       <c r="L389" s="12" t="inlineStr">
@@ -30262,7 +30262,7 @@
       </c>
       <c r="K390" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - A Mixed MUFC - Junior Boys U12A (Hamid)</t>
+          <t>Manningham United Blues FC U12 Juniors - A Mixed (Hamid)</t>
         </is>
       </c>
       <c r="L390" s="10" t="inlineStr">
@@ -30338,7 +30338,7 @@
       </c>
       <c r="K391" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - B Mixed MUFC - Junior Boys U13B (Samir)</t>
+          <t>Manningham United Blues FC U13 Juniors - B Mixed (Samir)</t>
         </is>
       </c>
       <c r="L391" s="12" t="inlineStr">
@@ -30414,7 +30414,7 @@
       </c>
       <c r="K392" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - A Mixed MUFC - Junior Boys U14A</t>
+          <t>Manningham United Blues FC U14 Juniors - A Mixed</t>
         </is>
       </c>
       <c r="L392" s="10" t="inlineStr">
@@ -30566,7 +30566,7 @@
       </c>
       <c r="K394" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U7J (Green)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Green)</t>
         </is>
       </c>
       <c r="L394" s="10" t="inlineStr">
@@ -30642,7 +30642,7 @@
       </c>
       <c r="K395" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U10 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U10W (Tilio's)</t>
+          <t>Manningham United Blues FC U10 MiniRoos - Wallabies Mixed (Tilio's)</t>
         </is>
       </c>
       <c r="L395" s="12" t="inlineStr">
@@ -30718,7 +30718,7 @@
       </c>
       <c r="K396" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U15 Juniors - B Mixed MUFC - Junior Boys U15B</t>
+          <t>Manningham United Blues FC U15 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="L396" s="10" t="inlineStr">
@@ -30794,7 +30794,7 @@
       </c>
       <c r="K397" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U15 Juniors - B Female MUFC - Junior Girls U15B (Ethan)</t>
+          <t>Manningham United Blues FC U15 Juniors - B Female (Ethan)</t>
         </is>
       </c>
       <c r="L397" s="12" t="inlineStr">
@@ -30870,7 +30870,7 @@
       </c>
       <c r="K398" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - C Female MUFC - Junior Girls U14C (Christian)</t>
+          <t>Manningham United Blues FC U14 Juniors - C Female (Christian)</t>
         </is>
       </c>
       <c r="L398" s="10" t="inlineStr">
@@ -30946,7 +30946,7 @@
       </c>
       <c r="K399" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U9W (Cahill's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Cahill's)</t>
         </is>
       </c>
       <c r="L399" s="12" t="inlineStr">
@@ -31022,7 +31022,7 @@
       </c>
       <c r="K400" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - C Female MUFC - Junior Girls U13C (Abigail)</t>
+          <t>Manningham United Blues FC U13 Juniors - C Female (Abigail)</t>
         </is>
       </c>
       <c r="L400" s="10" t="inlineStr">
@@ -31098,7 +31098,7 @@
       </c>
       <c r="K401" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - A Mixed MUFC - Junior Boys U13A (Sam Z)</t>
+          <t>Manningham United Blues FC U13 Juniors - A Mixed (Sam Z)</t>
         </is>
       </c>
       <c r="L401" s="12" t="inlineStr">
@@ -31250,7 +31250,7 @@
       </c>
       <c r="K403" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U7J (Red)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Red)</t>
         </is>
       </c>
       <c r="L403" s="12" t="inlineStr">
@@ -31326,7 +31326,7 @@
       </c>
       <c r="K404" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - A Mixed MUFC - Junior Boys U13A (George &amp; George)</t>
+          <t>Manningham United Blues FC U13 Juniors - A Mixed (George &amp; George)</t>
         </is>
       </c>
       <c r="L404" s="10" t="inlineStr">
@@ -31402,7 +31402,7 @@
       </c>
       <c r="K405" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Kangaroos Mixed MUFC - Miniroos Boys U8K (Arnold's)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Kangaroos Mixed (Arnold's)</t>
         </is>
       </c>
       <c r="L405" s="12" t="inlineStr">
@@ -31478,7 +31478,7 @@
       </c>
       <c r="K406" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U10 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U10W (Tilio's)</t>
+          <t>Manningham United Blues FC U10 MiniRoos - Wallabies Mixed (Tilio's)</t>
         </is>
       </c>
       <c r="L406" s="10" t="inlineStr">
@@ -31554,7 +31554,7 @@
       </c>
       <c r="K407" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U11W (Colosimo's)</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Mixed (Colosimo's)</t>
         </is>
       </c>
       <c r="L407" s="12" t="inlineStr">
@@ -31630,7 +31630,7 @@
       </c>
       <c r="K408" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - B Mixed MUFC - Junior Boys U13B (Samir)</t>
+          <t>Manningham United Blues FC U13 Juniors - B Mixed (Samir)</t>
         </is>
       </c>
       <c r="L408" s="10" t="inlineStr">
@@ -31706,7 +31706,7 @@
       </c>
       <c r="K409" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - A Female MUFC - Junior Girls U12A (Sienna)</t>
+          <t>Manningham United Blues FC U12 Juniors - A Female (Sienna)</t>
         </is>
       </c>
       <c r="L409" s="12" t="inlineStr">
@@ -31782,7 +31782,7 @@
       </c>
       <c r="K410" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - A Mixed MUFC - Junior Boys U14A</t>
+          <t>Manningham United Blues FC U14 Juniors - A Mixed</t>
         </is>
       </c>
       <c r="L410" s="10" t="inlineStr">
@@ -31858,7 +31858,7 @@
       </c>
       <c r="K411" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U16 Juniors - A Mixed MUFC - Junior Boys U16A</t>
+          <t>Manningham United Blues FC U16 Juniors - A Mixed</t>
         </is>
       </c>
       <c r="L411" s="12" t="inlineStr">
@@ -31934,7 +31934,7 @@
       </c>
       <c r="K412" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U7J (Green)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Green)</t>
         </is>
       </c>
       <c r="L412" s="10" t="inlineStr">
@@ -32010,7 +32010,7 @@
       </c>
       <c r="K413" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Kangaroos Mixed MUFC - Miniroos Boys U11 Kangas</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Kangaroos Mixed</t>
         </is>
       </c>
       <c r="L413" s="12" t="inlineStr">
@@ -32086,7 +32086,7 @@
       </c>
       <c r="K414" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U10 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U10J (Sainsbury's)</t>
+          <t>Manningham United Blues FC U10 MiniRoos - Joeys Mixed (Sainsbury's)</t>
         </is>
       </c>
       <c r="L414" s="10" t="inlineStr">
@@ -32162,7 +32162,7 @@
       </c>
       <c r="K415" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - B Mixed MUFC - Junior Boys U12B (Robert)</t>
+          <t>Manningham United Blues FC U12 Juniors - B Mixed (Robert)</t>
         </is>
       </c>
       <c r="L415" s="12" t="inlineStr">
@@ -32238,7 +32238,7 @@
       </c>
       <c r="K416" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - C Female MUFC - Junior Girls U14C (Christian)</t>
+          <t>Manningham United Blues FC U14 Juniors - C Female (Christian)</t>
         </is>
       </c>
       <c r="L416" s="10" t="inlineStr">
@@ -32314,7 +32314,7 @@
       </c>
       <c r="K417" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U15 Juniors - B Female MUFC - Junior Girls U15B (Ethan)</t>
+          <t>Manningham United Blues FC U15 Juniors - B Female (Ethan)</t>
         </is>
       </c>
       <c r="L417" s="12" t="inlineStr">
@@ -32390,7 +32390,7 @@
       </c>
       <c r="K418" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U9W (Cahill's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Cahill's)</t>
         </is>
       </c>
       <c r="L418" s="10" t="inlineStr">
@@ -32466,7 +32466,7 @@
       </c>
       <c r="K419" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U8W (Coe's)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Wallabies Mixed (Coe's)</t>
         </is>
       </c>
       <c r="L419" s="12" t="inlineStr">
@@ -32542,7 +32542,7 @@
       </c>
       <c r="K420" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U15 Juniors - A Mixed MUFC - Junior Boys U15A</t>
+          <t>Manningham United Blues FC U15 Juniors - A Mixed</t>
         </is>
       </c>
       <c r="L420" s="10" t="inlineStr">
@@ -32618,7 +32618,7 @@
       </c>
       <c r="K421" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U16 Juniors - B Mixed MUFC - Junior Boys U16B</t>
+          <t>Manningham United Blues FC U16 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="L421" s="12" t="inlineStr">
@@ -32694,7 +32694,7 @@
       </c>
       <c r="K422" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U17/18 Juniors - B Female MUFC - Junior Girls 17/18 (Marilyn)</t>
+          <t>Manningham United Blues FC U17/18 Juniors - B Female (Marilyn)</t>
         </is>
       </c>
       <c r="L422" s="10" t="inlineStr">
@@ -32770,7 +32770,7 @@
       </c>
       <c r="K423" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - C Mixed MUFC - Junior Boys U13C (Martin)</t>
+          <t>Manningham United Blues FC U13 Juniors - C Mixed (Martin)</t>
         </is>
       </c>
       <c r="L423" s="12" t="inlineStr">
@@ -32846,7 +32846,7 @@
       </c>
       <c r="K424" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - B Mixed MUFC - Junior Boys U14B</t>
+          <t>Manningham United Blues FC U14 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="L424" s="10" t="inlineStr">
@@ -32922,7 +32922,7 @@
       </c>
       <c r="K425" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U18 Juniors - A Male MUFC - Junior Boys U18A</t>
+          <t>Manningham United Blues FC U18 Juniors - A Male</t>
         </is>
       </c>
       <c r="L425" s="12" t="inlineStr">
@@ -32998,7 +32998,7 @@
       </c>
       <c r="K426" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - C Mixed MUFC - Junior Boys U14C (Phil)</t>
+          <t>Manningham United Blues FC U14 Juniors - C Mixed (Phil)</t>
         </is>
       </c>
       <c r="L426" s="10" t="inlineStr">
@@ -33074,7 +33074,7 @@
       </c>
       <c r="K427" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - A Mixed MUFC - Junior Boys U13A (George &amp; George)</t>
+          <t>Manningham United Blues FC U13 Juniors - A Mixed (George &amp; George)</t>
         </is>
       </c>
       <c r="L427" s="12" t="inlineStr">
@@ -33226,7 +33226,7 @@
       </c>
       <c r="K429" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Kangaroos Mixed MUFC - Miniroos Boys U11 Kangas</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Kangaroos Mixed</t>
         </is>
       </c>
       <c r="L429" s="12" t="inlineStr">
@@ -33302,7 +33302,7 @@
       </c>
       <c r="K430" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Kangaroos Mixed MUFC - Miniroos Boys U8K (Arnold's)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Kangaroos Mixed (Arnold's)</t>
         </is>
       </c>
       <c r="L430" s="10" t="inlineStr">
@@ -33378,7 +33378,7 @@
       </c>
       <c r="K431" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Kangaroos Mixed MUFC - Miniroos Boys U9K (Emerton's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Kangaroos Mixed (Emerton's)</t>
         </is>
       </c>
       <c r="L431" s="12" t="inlineStr">
@@ -33454,7 +33454,7 @@
       </c>
       <c r="K432" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U10 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U10W (Tilio's)</t>
+          <t>Manningham United Blues FC U10 MiniRoos - Wallabies Mixed (Tilio's)</t>
         </is>
       </c>
       <c r="L432" s="10" t="inlineStr">
@@ -33530,7 +33530,7 @@
       </c>
       <c r="K433" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U10 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U10J (Sainsbury's)</t>
+          <t>Manningham United Blues FC U10 MiniRoos - Joeys Mixed (Sainsbury's)</t>
         </is>
       </c>
       <c r="L433" s="12" t="inlineStr">
@@ -33606,7 +33606,7 @@
       </c>
       <c r="K434" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - A Mixed MUFC - Junior Boys U12A (Hamid)</t>
+          <t>Manningham United Blues FC U12 Juniors - A Mixed (Hamid)</t>
         </is>
       </c>
       <c r="L434" s="10" t="inlineStr">
@@ -33682,7 +33682,7 @@
       </c>
       <c r="K435" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - B Mixed MUFC - Junior Boys U13B (Samir)</t>
+          <t>Manningham United Blues FC U13 Juniors - B Mixed (Samir)</t>
         </is>
       </c>
       <c r="L435" s="12" t="inlineStr">
@@ -33758,7 +33758,7 @@
       </c>
       <c r="K436" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - B Mixed MUFC - Junior Boys U14B</t>
+          <t>Manningham United Blues FC U14 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="L436" s="10" t="inlineStr">
@@ -33834,7 +33834,7 @@
       </c>
       <c r="K437" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - A Mixed MUFC - Junior Boys U14A</t>
+          <t>Manningham United Blues FC U14 Juniors - A Mixed</t>
         </is>
       </c>
       <c r="L437" s="12" t="inlineStr">
@@ -33910,7 +33910,7 @@
       </c>
       <c r="K438" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U16 Juniors - A Mixed MUFC - Junior Boys U16A</t>
+          <t>Manningham United Blues FC U16 Juniors - A Mixed</t>
         </is>
       </c>
       <c r="L438" s="10" t="inlineStr">
@@ -33986,7 +33986,7 @@
       </c>
       <c r="K439" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - B Mixed MUFC - Junior Boys U12B (Robert)</t>
+          <t>Manningham United Blues FC U12 Juniors - B Mixed (Robert)</t>
         </is>
       </c>
       <c r="L439" s="12" t="inlineStr">
@@ -34062,7 +34062,7 @@
       </c>
       <c r="K440" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U11W (Colosimo's)</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Mixed (Colosimo's)</t>
         </is>
       </c>
       <c r="L440" s="10" t="inlineStr">
@@ -34138,7 +34138,7 @@
       </c>
       <c r="K441" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - C Mixed MUFC - Junior Boys U14C (Phil)</t>
+          <t>Manningham United Blues FC U14 Juniors - C Mixed (Phil)</t>
         </is>
       </c>
       <c r="L441" s="12" t="inlineStr">
@@ -34214,7 +34214,7 @@
       </c>
       <c r="K442" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U15 Juniors - B Mixed MUFC - Junior Boys U15B</t>
+          <t>Manningham United Blues FC U15 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="L442" s="10" t="inlineStr">
@@ -34366,7 +34366,7 @@
       </c>
       <c r="K444" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U7J (Green)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Green)</t>
         </is>
       </c>
       <c r="L444" s="10" t="inlineStr">
@@ -34442,7 +34442,7 @@
       </c>
       <c r="K445" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - C Female MUFC - Junior Girls U14C (Christian)</t>
+          <t>Manningham United Blues FC U14 Juniors - C Female (Christian)</t>
         </is>
       </c>
       <c r="L445" s="12" t="inlineStr">
@@ -34518,7 +34518,7 @@
       </c>
       <c r="K446" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U15 Juniors - B Female MUFC - Junior Girls U15B (Ethan)</t>
+          <t>Manningham United Blues FC U15 Juniors - B Female (Ethan)</t>
         </is>
       </c>
       <c r="L446" s="10" t="inlineStr">
@@ -34594,7 +34594,7 @@
       </c>
       <c r="K447" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Joeys Female MUFC - Miniroos Girls U8J (Yianna)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Joeys Female (Yianna)</t>
         </is>
       </c>
       <c r="L447" s="12" t="inlineStr">
@@ -34670,7 +34670,7 @@
       </c>
       <c r="K448" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U9W (Cahill's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Cahill's)</t>
         </is>
       </c>
       <c r="L448" s="10" t="inlineStr">
@@ -34746,7 +34746,7 @@
       </c>
       <c r="K449" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Kangaroos Mixed MUFC - Miniroos Boys U9K (Emerton's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Kangaroos Mixed (Emerton's)</t>
         </is>
       </c>
       <c r="L449" s="12" t="inlineStr">
@@ -34822,7 +34822,7 @@
       </c>
       <c r="K450" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - C Female MUFC - Junior Girls U13C (Abigail)</t>
+          <t>Manningham United Blues FC U13 Juniors - C Female (Abigail)</t>
         </is>
       </c>
       <c r="L450" s="10" t="inlineStr">
@@ -34898,7 +34898,7 @@
       </c>
       <c r="K451" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - C Female MUFC - Junior Girls U12C (Tahlia)</t>
+          <t>Manningham United Blues FC U12 Juniors - C Female (Tahlia)</t>
         </is>
       </c>
       <c r="L451" s="12" t="inlineStr">
@@ -34974,7 +34974,7 @@
       </c>
       <c r="K452" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - B Mixed MUFC - Junior Boys U13B (Samir)</t>
+          <t>Manningham United Blues FC U13 Juniors - B Mixed (Samir)</t>
         </is>
       </c>
       <c r="L452" s="10" t="inlineStr">
@@ -35050,7 +35050,7 @@
       </c>
       <c r="K453" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Kangaroos Mixed MUFC - Miniroos Boys U11 Kangas</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Kangaroos Mixed</t>
         </is>
       </c>
       <c r="L453" s="12" t="inlineStr">
@@ -35126,7 +35126,7 @@
       </c>
       <c r="K454" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U11W (Colosimo's)</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Mixed (Colosimo's)</t>
         </is>
       </c>
       <c r="L454" s="10" t="inlineStr">
@@ -35202,7 +35202,7 @@
       </c>
       <c r="K455" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Female MUFC - Miniroos Girls U9W (Nat &amp; Chloe)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Female (Nat &amp; Chloe)</t>
         </is>
       </c>
       <c r="L455" s="12" t="inlineStr">
@@ -35278,7 +35278,7 @@
       </c>
       <c r="K456" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Kangaroos Mixed MUFC - Miniroos Boys U8K (Arnold's)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Kangaroos Mixed (Arnold's)</t>
         </is>
       </c>
       <c r="L456" s="10" t="inlineStr">
@@ -35354,7 +35354,7 @@
       </c>
       <c r="K457" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U8W (Coe's)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Wallabies Mixed (Coe's)</t>
         </is>
       </c>
       <c r="L457" s="12" t="inlineStr">
@@ -35430,7 +35430,7 @@
       </c>
       <c r="K458" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U10 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U10W (Tilio's)</t>
+          <t>Manningham United Blues FC U10 MiniRoos - Wallabies Mixed (Tilio's)</t>
         </is>
       </c>
       <c r="L458" s="10" t="inlineStr">
@@ -35506,7 +35506,7 @@
       </c>
       <c r="K459" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U11W (Colosimo's)</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Mixed (Colosimo's)</t>
         </is>
       </c>
       <c r="L459" s="12" t="inlineStr">
@@ -35582,7 +35582,7 @@
       </c>
       <c r="K460" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - A Mixed MUFC - Junior Boys U12A (Hamid)</t>
+          <t>Manningham United Blues FC U12 Juniors - A Mixed (Hamid)</t>
         </is>
       </c>
       <c r="L460" s="10" t="inlineStr">
@@ -35658,7 +35658,7 @@
       </c>
       <c r="K461" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - A Mixed MUFC - Junior Boys U13A (Sam Z)</t>
+          <t>Manningham United Blues FC U13 Juniors - A Mixed (Sam Z)</t>
         </is>
       </c>
       <c r="L461" s="12" t="inlineStr">
@@ -35734,7 +35734,7 @@
       </c>
       <c r="K462" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U17/18 Juniors - B Female MUFC - Junior Girls 17/18 (Marilyn)</t>
+          <t>Manningham United Blues FC U17/18 Juniors - B Female (Marilyn)</t>
         </is>
       </c>
       <c r="L462" s="10" t="inlineStr">
@@ -35810,7 +35810,7 @@
       </c>
       <c r="K463" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U7J (Green)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Green)</t>
         </is>
       </c>
       <c r="L463" s="12" t="inlineStr">
@@ -35886,7 +35886,7 @@
       </c>
       <c r="K464" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Kangaroos Mixed MUFC - Miniroos Boys U11 Kangas</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Kangaroos Mixed</t>
         </is>
       </c>
       <c r="L464" s="10" t="inlineStr">
@@ -35962,7 +35962,7 @@
       </c>
       <c r="K465" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U10 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U10J (Sainsbury's)</t>
+          <t>Manningham United Blues FC U10 MiniRoos - Joeys Mixed (Sainsbury's)</t>
         </is>
       </c>
       <c r="L465" s="12" t="inlineStr">
@@ -36038,7 +36038,7 @@
       </c>
       <c r="K466" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - A Female MUFC - Junior Girls U12A (Sienna)</t>
+          <t>Manningham United Blues FC U12 Juniors - A Female (Sienna)</t>
         </is>
       </c>
       <c r="L466" s="10" t="inlineStr">
@@ -36114,7 +36114,7 @@
       </c>
       <c r="K467" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - B Mixed MUFC - Junior Boys U12B (Robert)</t>
+          <t>Manningham United Blues FC U12 Juniors - B Mixed (Robert)</t>
         </is>
       </c>
       <c r="L467" s="12" t="inlineStr">
@@ -36190,7 +36190,7 @@
       </c>
       <c r="K468" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - C Mixed MUFC - Junior Boys U14C (Phil)</t>
+          <t>Manningham United Blues FC U14 Juniors - C Mixed (Phil)</t>
         </is>
       </c>
       <c r="L468" s="10" t="inlineStr">
@@ -36266,7 +36266,7 @@
       </c>
       <c r="K469" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U16 Juniors - A Mixed MUFC - Junior Boys U16A</t>
+          <t>Manningham United Blues FC U16 Juniors - A Mixed</t>
         </is>
       </c>
       <c r="L469" s="12" t="inlineStr">
@@ -36342,7 +36342,7 @@
       </c>
       <c r="K470" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Joeys Female MUFC - Miniroos Girls U8J (Yianna)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Joeys Female (Yianna)</t>
         </is>
       </c>
       <c r="L470" s="10" t="inlineStr">
@@ -36418,7 +36418,7 @@
       </c>
       <c r="K471" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U7J (Red)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Red)</t>
         </is>
       </c>
       <c r="L471" s="12" t="inlineStr">
@@ -36494,7 +36494,7 @@
       </c>
       <c r="K472" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Kangaroos Mixed MUFC - Miniroos Boys U9K (Emerton's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Kangaroos Mixed (Emerton's)</t>
         </is>
       </c>
       <c r="L472" s="10" t="inlineStr">
@@ -36570,7 +36570,7 @@
       </c>
       <c r="K473" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Joeys Female MUFC - Miniroos Girls U11J (Grace)</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Joeys Female (Grace)</t>
         </is>
       </c>
       <c r="L473" s="12" t="inlineStr">
@@ -36646,7 +36646,7 @@
       </c>
       <c r="K474" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U9W (Cahill's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Cahill's)</t>
         </is>
       </c>
       <c r="L474" s="10" t="inlineStr">
@@ -36722,7 +36722,7 @@
       </c>
       <c r="K475" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - A Mixed MUFC - Junior Boys U13A (Sam Z)</t>
+          <t>Manningham United Blues FC U13 Juniors - A Mixed (Sam Z)</t>
         </is>
       </c>
       <c r="L475" s="12" t="inlineStr">
@@ -36798,7 +36798,7 @@
       </c>
       <c r="K476" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - C Mixed MUFC - Junior Boys U13C (Martin)</t>
+          <t>Manningham United Blues FC U13 Juniors - C Mixed (Martin)</t>
         </is>
       </c>
       <c r="L476" s="10" t="inlineStr">
@@ -36874,7 +36874,7 @@
       </c>
       <c r="K477" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - B Mixed MUFC - Junior Boys U13B (Samir)</t>
+          <t>Manningham United Blues FC U13 Juniors - B Mixed (Samir)</t>
         </is>
       </c>
       <c r="L477" s="12" t="inlineStr">
@@ -36950,7 +36950,7 @@
       </c>
       <c r="K478" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - B Mixed MUFC - Junior Boys U14B</t>
+          <t>Manningham United Blues FC U14 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="L478" s="10" t="inlineStr">
@@ -37026,7 +37026,7 @@
       </c>
       <c r="K479" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U16 Juniors - B Mixed MUFC - Junior Boys U16B</t>
+          <t>Manningham United Blues FC U16 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="L479" s="12" t="inlineStr">
@@ -37102,7 +37102,7 @@
       </c>
       <c r="K480" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC Seniors MUFC - Women's Metro League</t>
+          <t>Manningham United Blues FC Seniors</t>
         </is>
       </c>
       <c r="L480" s="10" t="inlineStr">
@@ -37178,7 +37178,7 @@
       </c>
       <c r="K481" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U15 Juniors - A Mixed MUFC - Junior Boys U15A</t>
+          <t>Manningham United Blues FC U15 Juniors - A Mixed</t>
         </is>
       </c>
       <c r="L481" s="12" t="inlineStr">
@@ -37254,7 +37254,7 @@
       </c>
       <c r="K482" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U18 Juniors - A Male MUFC - Junior Boys U18A</t>
+          <t>Manningham United Blues FC U18 Juniors - A Male</t>
         </is>
       </c>
       <c r="L482" s="10" t="inlineStr">
@@ -37330,7 +37330,7 @@
       </c>
       <c r="K483" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Joeys Female MUFC - Miniroos Girls U8J (Amelia &amp; Karina)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Joeys Female (Amelia &amp; Karina)</t>
         </is>
       </c>
       <c r="L483" s="12" t="inlineStr">
@@ -37406,7 +37406,7 @@
       </c>
       <c r="K484" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U10 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U10J (Sainsbury's)</t>
+          <t>Manningham United Blues FC U10 MiniRoos - Joeys Mixed (Sainsbury's)</t>
         </is>
       </c>
       <c r="L484" s="10" t="inlineStr">
@@ -37482,7 +37482,7 @@
       </c>
       <c r="K485" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U10 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U10W (Tilio's)</t>
+          <t>Manningham United Blues FC U10 MiniRoos - Wallabies Mixed (Tilio's)</t>
         </is>
       </c>
       <c r="L485" s="12" t="inlineStr">
@@ -37558,7 +37558,7 @@
       </c>
       <c r="K486" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - A Female MUFC - Junior Girls U12A (Sienna)</t>
+          <t>Manningham United Blues FC U12 Juniors - A Female (Sienna)</t>
         </is>
       </c>
       <c r="L486" s="10" t="inlineStr">
@@ -37634,7 +37634,7 @@
       </c>
       <c r="K487" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - A Mixed MUFC - Junior Boys U12A (Hamid)</t>
+          <t>Manningham United Blues FC U12 Juniors - A Mixed (Hamid)</t>
         </is>
       </c>
       <c r="L487" s="12" t="inlineStr">
@@ -37710,7 +37710,7 @@
       </c>
       <c r="K488" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - A Mixed MUFC - Junior Boys U14A</t>
+          <t>Manningham United Blues FC U14 Juniors - A Mixed</t>
         </is>
       </c>
       <c r="L488" s="10" t="inlineStr">
@@ -37786,7 +37786,7 @@
       </c>
       <c r="K489" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U16 Juniors - B Female MUFC - Junior Girls U16A (Eden)</t>
+          <t>Manningham United Blues FC U16 Juniors - B Female (Eden)</t>
         </is>
       </c>
       <c r="L489" s="12" t="inlineStr">
@@ -37862,7 +37862,7 @@
       </c>
       <c r="K490" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Kangaroos Mixed MUFC - Miniroos Boys U11 Kangas</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Kangaroos Mixed</t>
         </is>
       </c>
       <c r="L490" s="10" t="inlineStr">
@@ -37938,7 +37938,7 @@
       </c>
       <c r="K491" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U11W (Colosimo's)</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Mixed (Colosimo's)</t>
         </is>
       </c>
       <c r="L491" s="12" t="inlineStr">
@@ -38014,7 +38014,7 @@
       </c>
       <c r="K492" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - B Mixed MUFC - Junior Boys U12B (Robert)</t>
+          <t>Manningham United Blues FC U12 Juniors - B Mixed (Robert)</t>
         </is>
       </c>
       <c r="L492" s="10" t="inlineStr">
@@ -38166,7 +38166,7 @@
       </c>
       <c r="K494" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - C Female MUFC - Junior Girls U14C (Christian)</t>
+          <t>Manningham United Blues FC U14 Juniors - C Female (Christian)</t>
         </is>
       </c>
       <c r="L494" s="10" t="inlineStr">
@@ -38242,7 +38242,7 @@
       </c>
       <c r="K495" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U15 Juniors - B Female MUFC - Junior Girls U15B (Ethan)</t>
+          <t>Manningham United Blues FC U15 Juniors - B Female (Ethan)</t>
         </is>
       </c>
       <c r="L495" s="12" t="inlineStr">
@@ -38318,7 +38318,7 @@
       </c>
       <c r="K496" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Female MUFC - Miniroos Girls U9W (Nat &amp; Chloe)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Female (Nat &amp; Chloe)</t>
         </is>
       </c>
       <c r="L496" s="10" t="inlineStr">
@@ -38394,7 +38394,7 @@
       </c>
       <c r="K497" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U7J (Red)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Red)</t>
         </is>
       </c>
       <c r="L497" s="12" t="inlineStr">
@@ -38470,7 +38470,7 @@
       </c>
       <c r="K498" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U8W (Coe's)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Wallabies Mixed (Coe's)</t>
         </is>
       </c>
       <c r="L498" s="10" t="inlineStr">
@@ -38546,7 +38546,7 @@
       </c>
       <c r="K499" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Joeys Female MUFC - Miniroos Girls U8J (Yianna)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Joeys Female (Yianna)</t>
         </is>
       </c>
       <c r="L499" s="12" t="inlineStr">
@@ -38622,7 +38622,7 @@
       </c>
       <c r="K500" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U9W (Cahill's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Cahill's)</t>
         </is>
       </c>
       <c r="L500" s="10" t="inlineStr">
@@ -38698,7 +38698,7 @@
       </c>
       <c r="K501" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Kangaroos Mixed MUFC - Miniroos Boys U9K (Emerton's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Kangaroos Mixed (Emerton's)</t>
         </is>
       </c>
       <c r="L501" s="12" t="inlineStr">
@@ -38774,7 +38774,7 @@
       </c>
       <c r="K502" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - A Mixed MUFC - Junior Boys U12A (John)</t>
+          <t>Manningham United Blues FC U12 Juniors - A Mixed (John)</t>
         </is>
       </c>
       <c r="L502" s="10" t="inlineStr">
@@ -38850,7 +38850,7 @@
       </c>
       <c r="K503" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - B Mixed MUFC - Junior Boys U14B</t>
+          <t>Manningham United Blues FC U14 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="L503" s="12" t="inlineStr">
@@ -38926,7 +38926,7 @@
       </c>
       <c r="K504" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC Seniors MUFC - Women's Metro League</t>
+          <t>Manningham United Blues FC Seniors</t>
         </is>
       </c>
       <c r="L504" s="10" t="inlineStr">
@@ -39002,7 +39002,7 @@
       </c>
       <c r="K505" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - C Mixed MUFC - Junior Boys U13C (Martin)</t>
+          <t>Manningham United Blues FC U13 Juniors - C Mixed (Martin)</t>
         </is>
       </c>
       <c r="L505" s="12" t="inlineStr">
@@ -39078,7 +39078,7 @@
       </c>
       <c r="K506" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - A Mixed MUFC - Junior Boys U13A (George &amp; George)</t>
+          <t>Manningham United Blues FC U13 Juniors - A Mixed (George &amp; George)</t>
         </is>
       </c>
       <c r="L506" s="10" t="inlineStr">
@@ -39154,7 +39154,7 @@
       </c>
       <c r="K507" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U17/18 Juniors - B Female MUFC - Junior Girls 17/18 (Marilyn)</t>
+          <t>Manningham United Blues FC U17/18 Juniors - B Female (Marilyn)</t>
         </is>
       </c>
       <c r="L507" s="12" t="inlineStr">
@@ -39230,7 +39230,7 @@
       </c>
       <c r="K508" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Female MUFC - Miniroos Girls U9W (Nat &amp; Chloe)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Female (Nat &amp; Chloe)</t>
         </is>
       </c>
       <c r="L508" s="10" t="inlineStr">
@@ -39306,7 +39306,7 @@
       </c>
       <c r="K509" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Joeys Female MUFC - Miniroos Girls U8J (Amelia &amp; Karina)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Joeys Female (Amelia &amp; Karina)</t>
         </is>
       </c>
       <c r="L509" s="12" t="inlineStr">
@@ -39382,7 +39382,7 @@
       </c>
       <c r="K510" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Kangaroos Mixed MUFC - Miniroos Boys U9K (Emerton's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Kangaroos Mixed (Emerton's)</t>
         </is>
       </c>
       <c r="L510" s="10" t="inlineStr">
@@ -39458,7 +39458,7 @@
       </c>
       <c r="K511" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U10 MiniRoos - Kangaroos Female MUFC - Miniroos Girls U10K (Karl)</t>
+          <t>Manningham United Blues FC U10 MiniRoos - Kangaroos Female (Karl)</t>
         </is>
       </c>
       <c r="L511" s="12" t="inlineStr">
@@ -39534,7 +39534,7 @@
       </c>
       <c r="K512" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U7J (Green)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Green)</t>
         </is>
       </c>
       <c r="L512" s="10" t="inlineStr">
@@ -39610,7 +39610,7 @@
       </c>
       <c r="K513" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Kangaroos Mixed MUFC - Miniroos Boys U8K (Arnold's)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Kangaroos Mixed (Arnold's)</t>
         </is>
       </c>
       <c r="L513" s="12" t="inlineStr">
@@ -39686,7 +39686,7 @@
       </c>
       <c r="K514" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U16 Juniors - B Female MUFC - Junior Girls U16A (Eden)</t>
+          <t>Manningham United Blues FC U16 Juniors - B Female (Eden)</t>
         </is>
       </c>
       <c r="L514" s="10" t="inlineStr">
@@ -39762,7 +39762,7 @@
       </c>
       <c r="K515" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U17/18 Juniors - B Female MUFC - Junior Girls 17/18 (Marilyn)</t>
+          <t>Manningham United Blues FC U17/18 Juniors - B Female (Marilyn)</t>
         </is>
       </c>
       <c r="L515" s="12" t="inlineStr">
@@ -39914,7 +39914,7 @@
       </c>
       <c r="K517" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U10 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U10W (Tilio's)</t>
+          <t>Manningham United Blues FC U10 MiniRoos - Wallabies Mixed (Tilio's)</t>
         </is>
       </c>
       <c r="L517" s="12" t="inlineStr">
@@ -39990,7 +39990,7 @@
       </c>
       <c r="K518" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Kangaroos Mixed MUFC - Miniroos Boys U11 Kangas</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Kangaroos Mixed</t>
         </is>
       </c>
       <c r="L518" s="10" t="inlineStr">
@@ -40066,7 +40066,7 @@
       </c>
       <c r="K519" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U11W (Colosimo's)</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Mixed (Colosimo's)</t>
         </is>
       </c>
       <c r="L519" s="12" t="inlineStr">
@@ -40142,7 +40142,7 @@
       </c>
       <c r="K520" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - B Mixed MUFC - Junior Boys U14B</t>
+          <t>Manningham United Blues FC U14 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="L520" s="10" t="inlineStr">
@@ -40218,7 +40218,7 @@
       </c>
       <c r="K521" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - C Mixed MUFC - Junior Boys U14C (Phil)</t>
+          <t>Manningham United Blues FC U14 Juniors - C Mixed (Phil)</t>
         </is>
       </c>
       <c r="L521" s="12" t="inlineStr">
@@ -40294,7 +40294,7 @@
       </c>
       <c r="K522" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC Seniors MUFC - Women's Metro League</t>
+          <t>Manningham United Blues FC Seniors</t>
         </is>
       </c>
       <c r="L522" s="10" t="inlineStr">
@@ -40370,7 +40370,7 @@
       </c>
       <c r="K523" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - A Mixed MUFC - Junior Boys U13A (Sam Z)</t>
+          <t>Manningham United Blues FC U13 Juniors - A Mixed (Sam Z)</t>
         </is>
       </c>
       <c r="L523" s="12" t="inlineStr">
@@ -40446,7 +40446,7 @@
       </c>
       <c r="K524" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - C Female MUFC - Junior Girls U14C (Christian)</t>
+          <t>Manningham United Blues FC U14 Juniors - C Female (Christian)</t>
         </is>
       </c>
       <c r="L524" s="10" t="inlineStr">
@@ -40522,7 +40522,7 @@
       </c>
       <c r="K525" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Joeys Female MUFC - Miniroos Girls U8J (Yianna)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Joeys Female (Yianna)</t>
         </is>
       </c>
       <c r="L525" s="12" t="inlineStr">
@@ -40598,12 +40598,12 @@
       </c>
       <c r="K526" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U7J (Red)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Red)</t>
         </is>
       </c>
       <c r="L526" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U7J (Green)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Green)</t>
         </is>
       </c>
       <c r="M526" s="10" t="inlineStr">
@@ -40674,7 +40674,7 @@
       </c>
       <c r="K527" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U8W (Coe's)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Wallabies Mixed (Coe's)</t>
         </is>
       </c>
       <c r="L527" s="12" t="inlineStr">
@@ -40750,7 +40750,7 @@
       </c>
       <c r="K528" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U10 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U10J (Sainsbury's)</t>
+          <t>Manningham United Blues FC U10 MiniRoos - Joeys Mixed (Sainsbury's)</t>
         </is>
       </c>
       <c r="L528" s="10" t="inlineStr">
@@ -40826,7 +40826,7 @@
       </c>
       <c r="K529" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U9W (Cahill's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Cahill's)</t>
         </is>
       </c>
       <c r="L529" s="12" t="inlineStr">
@@ -40902,7 +40902,7 @@
       </c>
       <c r="K530" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - C Female MUFC - Junior Girls U12C (Tahlia)</t>
+          <t>Manningham United Blues FC U12 Juniors - C Female (Tahlia)</t>
         </is>
       </c>
       <c r="L530" s="10" t="inlineStr">
@@ -40978,7 +40978,7 @@
       </c>
       <c r="K531" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - B Mixed MUFC - Junior Boys U13B (Samir)</t>
+          <t>Manningham United Blues FC U13 Juniors - B Mixed (Samir)</t>
         </is>
       </c>
       <c r="L531" s="12" t="inlineStr">
@@ -41054,7 +41054,7 @@
       </c>
       <c r="K532" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U15 Juniors - A Mixed MUFC - Junior Boys U15A</t>
+          <t>Manningham United Blues FC U15 Juniors - A Mixed</t>
         </is>
       </c>
       <c r="L532" s="10" t="inlineStr">
@@ -41206,7 +41206,7 @@
       </c>
       <c r="K534" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Joeys Female MUFC - Miniroos Girls U11J (Grace)</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Joeys Female (Grace)</t>
         </is>
       </c>
       <c r="L534" s="10" t="inlineStr">
@@ -41282,7 +41282,7 @@
       </c>
       <c r="K535" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - C Female MUFC - Junior Girls U13C (Abigail)</t>
+          <t>Manningham United Blues FC U13 Juniors - C Female (Abigail)</t>
         </is>
       </c>
       <c r="L535" s="12" t="inlineStr">
@@ -41358,7 +41358,7 @@
       </c>
       <c r="K536" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - B Mixed MUFC - Junior Boys U12B (Robert)</t>
+          <t>Manningham United Blues FC U12 Juniors - B Mixed (Robert)</t>
         </is>
       </c>
       <c r="L536" s="10" t="inlineStr">
@@ -41434,7 +41434,7 @@
       </c>
       <c r="K537" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - C Mixed MUFC - Junior Boys U13C (Martin)</t>
+          <t>Manningham United Blues FC U13 Juniors - C Mixed (Martin)</t>
         </is>
       </c>
       <c r="L537" s="12" t="inlineStr">
@@ -41510,7 +41510,7 @@
       </c>
       <c r="K538" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - A Mixed MUFC - Junior Boys U13A (George &amp; George)</t>
+          <t>Manningham United Blues FC U13 Juniors - A Mixed (George &amp; George)</t>
         </is>
       </c>
       <c r="L538" s="10" t="inlineStr">
@@ -41586,7 +41586,7 @@
       </c>
       <c r="K539" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U16 Juniors - B Mixed MUFC - Junior Boys U16B</t>
+          <t>Manningham United Blues FC U16 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="L539" s="12" t="inlineStr">
@@ -41662,7 +41662,7 @@
       </c>
       <c r="K540" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Joeys Female MUFC - Miniroos Girls U8J (Yianna)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Joeys Female (Yianna)</t>
         </is>
       </c>
       <c r="L540" s="10" t="inlineStr">
@@ -41738,7 +41738,7 @@
       </c>
       <c r="K541" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Female MUFC - Miniroos Girls U9W (Nat &amp; Chloe)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Female (Nat &amp; Chloe)</t>
         </is>
       </c>
       <c r="L541" s="12" t="inlineStr">
@@ -41814,7 +41814,7 @@
       </c>
       <c r="K542" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Joeys Female MUFC - Miniroos Girls U8J (Amelia &amp; Karina)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Joeys Female (Amelia &amp; Karina)</t>
         </is>
       </c>
       <c r="L542" s="10" t="inlineStr">
@@ -41966,7 +41966,7 @@
       </c>
       <c r="K544" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Joeys Female MUFC - Miniroos Girls U11J (Grace)</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Joeys Female (Grace)</t>
         </is>
       </c>
       <c r="L544" s="10" t="inlineStr">
@@ -42042,7 +42042,7 @@
       </c>
       <c r="K545" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - A Female MUFC - Junior Girls U12A (Sienna)</t>
+          <t>Manningham United Blues FC U12 Juniors - A Female (Sienna)</t>
         </is>
       </c>
       <c r="L545" s="12" t="inlineStr">
@@ -42118,7 +42118,7 @@
       </c>
       <c r="K546" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - C Female MUFC - Junior Girls U12C (Tahlia)</t>
+          <t>Manningham United Blues FC U12 Juniors - C Female (Tahlia)</t>
         </is>
       </c>
       <c r="L546" s="10" t="inlineStr">
@@ -42194,7 +42194,7 @@
       </c>
       <c r="K547" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - A Mixed MUFC - Junior Boys U14A</t>
+          <t>Manningham United Blues FC U14 Juniors - A Mixed</t>
         </is>
       </c>
       <c r="L547" s="12" t="inlineStr">
@@ -42270,7 +42270,7 @@
       </c>
       <c r="K548" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U16 Juniors - B Female MUFC - Junior Girls U16A (Eden)</t>
+          <t>Manningham United Blues FC U16 Juniors - B Female (Eden)</t>
         </is>
       </c>
       <c r="L548" s="10" t="inlineStr">
@@ -42346,7 +42346,7 @@
       </c>
       <c r="K549" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U16 Juniors - A Mixed MUFC - Junior Boys U16A</t>
+          <t>Manningham United Blues FC U16 Juniors - A Mixed</t>
         </is>
       </c>
       <c r="L549" s="12" t="inlineStr">
@@ -42422,7 +42422,7 @@
       </c>
       <c r="K550" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - A Mixed MUFC - Junior Boys U12A (Hamid)</t>
+          <t>Manningham United Blues FC U12 Juniors - A Mixed (Hamid)</t>
         </is>
       </c>
       <c r="L550" s="10" t="inlineStr">
@@ -42498,7 +42498,7 @@
       </c>
       <c r="K551" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - B Mixed MUFC - Junior Boys U12B (Robert)</t>
+          <t>Manningham United Blues FC U12 Juniors - B Mixed (Robert)</t>
         </is>
       </c>
       <c r="L551" s="12" t="inlineStr">
@@ -42574,7 +42574,7 @@
       </c>
       <c r="K552" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - A Mixed MUFC - Junior Boys U12A (John)</t>
+          <t>Manningham United Blues FC U12 Juniors - A Mixed (John)</t>
         </is>
       </c>
       <c r="L552" s="10" t="inlineStr">
@@ -42650,7 +42650,7 @@
       </c>
       <c r="K553" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - A Female MUFC - Junior Girls U14A (Chloe)</t>
+          <t>Manningham United Blues FC U14 Juniors - A Female (Chloe)</t>
         </is>
       </c>
       <c r="L553" s="12" t="inlineStr">
@@ -42726,7 +42726,7 @@
       </c>
       <c r="K554" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - C Female MUFC - Junior Girls U14C (Christian)</t>
+          <t>Manningham United Blues FC U14 Juniors - C Female (Christian)</t>
         </is>
       </c>
       <c r="L554" s="10" t="inlineStr">
@@ -42802,7 +42802,7 @@
       </c>
       <c r="K555" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U16 Juniors - B Mixed MUFC - Junior Boys U16B</t>
+          <t>Manningham United Blues FC U16 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="L555" s="12" t="inlineStr">
@@ -42878,7 +42878,7 @@
       </c>
       <c r="K556" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U10 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U10W (Tilio's)</t>
+          <t>Manningham United Blues FC U10 MiniRoos - Wallabies Mixed (Tilio's)</t>
         </is>
       </c>
       <c r="L556" s="10" t="inlineStr">
@@ -42954,7 +42954,7 @@
       </c>
       <c r="K557" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - C Mixed MUFC - Junior Boys U14C (Phil)</t>
+          <t>Manningham United Blues FC U14 Juniors - C Mixed (Phil)</t>
         </is>
       </c>
       <c r="L557" s="12" t="inlineStr">
@@ -43030,7 +43030,7 @@
       </c>
       <c r="K558" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U15 Juniors - B Mixed MUFC - Junior Boys U15B</t>
+          <t>Manningham United Blues FC U15 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="L558" s="10" t="inlineStr">
@@ -43106,7 +43106,7 @@
       </c>
       <c r="K559" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Kangaroos Mixed MUFC - Miniroos Boys U8K (Arnold's)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Kangaroos Mixed (Arnold's)</t>
         </is>
       </c>
       <c r="L559" s="12" t="inlineStr">
@@ -43182,7 +43182,7 @@
       </c>
       <c r="K560" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U8W (Coe's)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Wallabies Mixed (Coe's)</t>
         </is>
       </c>
       <c r="L560" s="10" t="inlineStr">
@@ -43258,7 +43258,7 @@
       </c>
       <c r="K561" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - C Mixed MUFC - Junior Boys U13C (Martin)</t>
+          <t>Manningham United Blues FC U13 Juniors - C Mixed (Martin)</t>
         </is>
       </c>
       <c r="L561" s="12" t="inlineStr">
@@ -43334,7 +43334,7 @@
       </c>
       <c r="K562" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U10 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U10J (Sainsbury's)</t>
+          <t>Manningham United Blues FC U10 MiniRoos - Joeys Mixed (Sainsbury's)</t>
         </is>
       </c>
       <c r="L562" s="10" t="inlineStr">
@@ -43410,7 +43410,7 @@
       </c>
       <c r="K563" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - A Mixed MUFC - Junior Boys U13A (George &amp; George)</t>
+          <t>Manningham United Blues FC U13 Juniors - A Mixed (George &amp; George)</t>
         </is>
       </c>
       <c r="L563" s="12" t="inlineStr">
@@ -43486,7 +43486,7 @@
       </c>
       <c r="K564" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U15 Juniors - A Mixed MUFC - Junior Boys U15A</t>
+          <t>Manningham United Blues FC U15 Juniors - A Mixed</t>
         </is>
       </c>
       <c r="L564" s="10" t="inlineStr">
@@ -43562,7 +43562,7 @@
       </c>
       <c r="K565" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U18 Juniors - A Male MUFC - Junior Boys U18A</t>
+          <t>Manningham United Blues FC U18 Juniors - A Male</t>
         </is>
       </c>
       <c r="L565" s="12" t="inlineStr">
@@ -43638,7 +43638,7 @@
       </c>
       <c r="K566" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - A Mixed MUFC - Junior Boys U12A (Hamid)</t>
+          <t>Manningham United Blues FC U12 Juniors - A Mixed (Hamid)</t>
         </is>
       </c>
       <c r="L566" s="10" t="inlineStr">
@@ -43714,7 +43714,7 @@
       </c>
       <c r="K567" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Joeys Female MUFC - Miniroos Girls U8J (Yianna)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Joeys Female (Yianna)</t>
         </is>
       </c>
       <c r="L567" s="12" t="inlineStr">
@@ -43790,7 +43790,7 @@
       </c>
       <c r="K568" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U10 MiniRoos - Kangaroos Female MUFC - Miniroos Girls U10K (Karl)</t>
+          <t>Manningham United Blues FC U10 MiniRoos - Kangaroos Female (Karl)</t>
         </is>
       </c>
       <c r="L568" s="10" t="inlineStr">
@@ -43866,7 +43866,7 @@
       </c>
       <c r="K569" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Female MUFC - Miniroos Girls U9W (Nat &amp; Chloe)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Female (Nat &amp; Chloe)</t>
         </is>
       </c>
       <c r="L569" s="12" t="inlineStr">
@@ -43942,7 +43942,7 @@
       </c>
       <c r="K570" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - C Female MUFC - Junior Girls U12C (Tahlia)</t>
+          <t>Manningham United Blues FC U12 Juniors - C Female (Tahlia)</t>
         </is>
       </c>
       <c r="L570" s="10" t="inlineStr">
@@ -44018,7 +44018,7 @@
       </c>
       <c r="K571" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - B Mixed MUFC - Junior Boys U13B (Samir)</t>
+          <t>Manningham United Blues FC U13 Juniors - B Mixed (Samir)</t>
         </is>
       </c>
       <c r="L571" s="12" t="inlineStr">
@@ -44094,7 +44094,7 @@
       </c>
       <c r="K572" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U16 Juniors - B Female MUFC - Junior Girls U16A (Eden)</t>
+          <t>Manningham United Blues FC U16 Juniors - B Female (Eden)</t>
         </is>
       </c>
       <c r="L572" s="10" t="inlineStr">
@@ -44170,7 +44170,7 @@
       </c>
       <c r="K573" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - A Mixed MUFC - Junior Boys U14A</t>
+          <t>Manningham United Blues FC U14 Juniors - A Mixed</t>
         </is>
       </c>
       <c r="L573" s="12" t="inlineStr">
@@ -44246,7 +44246,7 @@
       </c>
       <c r="K574" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - C Female MUFC - Junior Girls U14C (Christian)</t>
+          <t>Manningham United Blues FC U14 Juniors - C Female (Christian)</t>
         </is>
       </c>
       <c r="L574" s="10" t="inlineStr">
@@ -44322,7 +44322,7 @@
       </c>
       <c r="K575" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - C Mixed MUFC - Junior Boys U14C (Phil)</t>
+          <t>Manningham United Blues FC U14 Juniors - C Mixed (Phil)</t>
         </is>
       </c>
       <c r="L575" s="12" t="inlineStr">
@@ -44398,7 +44398,7 @@
       </c>
       <c r="K576" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U15 Juniors - B Mixed MUFC - Junior Boys U15B</t>
+          <t>Manningham United Blues FC U15 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="L576" s="10" t="inlineStr">
@@ -44550,7 +44550,7 @@
       </c>
       <c r="K578" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Female MUFC - Miniroos Girls U9W (Nat &amp; Chloe)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Female (Nat &amp; Chloe)</t>
         </is>
       </c>
       <c r="L578" s="10" t="inlineStr">
@@ -44626,7 +44626,7 @@
       </c>
       <c r="K579" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Kangaroos Mixed MUFC - Miniroos Boys U8K (Arnold's)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Kangaroos Mixed (Arnold's)</t>
         </is>
       </c>
       <c r="L579" s="12" t="inlineStr">
@@ -44702,7 +44702,7 @@
       </c>
       <c r="K580" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U8W (Coe's)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Wallabies Mixed (Coe's)</t>
         </is>
       </c>
       <c r="L580" s="10" t="inlineStr">
@@ -44778,7 +44778,7 @@
       </c>
       <c r="K581" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Joeys Female MUFC - Miniroos Girls U11J (Grace)</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Joeys Female (Grace)</t>
         </is>
       </c>
       <c r="L581" s="12" t="inlineStr">
@@ -44854,7 +44854,7 @@
       </c>
       <c r="K582" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed MUFC - Miniroos Boys U9W (Cahill's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Cahill's)</t>
         </is>
       </c>
       <c r="L582" s="10" t="inlineStr">
@@ -44930,7 +44930,7 @@
       </c>
       <c r="K583" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Kangaroos Mixed MUFC - Miniroos Boys U9K (Emerton's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Kangaroos Mixed (Emerton's)</t>
         </is>
       </c>
       <c r="L583" s="12" t="inlineStr">
@@ -45006,7 +45006,7 @@
       </c>
       <c r="K584" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - C Mixed MUFC - Junior Boys U13C (Martin)</t>
+          <t>Manningham United Blues FC U13 Juniors - C Mixed (Martin)</t>
         </is>
       </c>
       <c r="L584" s="10" t="inlineStr">
@@ -45158,7 +45158,7 @@
       </c>
       <c r="K586" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - A Female MUFC - Junior Girls U14A (Chloe)</t>
+          <t>Manningham United Blues FC U14 Juniors - A Female (Chloe)</t>
         </is>
       </c>
       <c r="L586" s="10" t="inlineStr">
@@ -45234,7 +45234,7 @@
       </c>
       <c r="K587" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U17/18 Juniors - B Female MUFC - Junior Girls 17/18 (Marilyn)</t>
+          <t>Manningham United Blues FC U17/18 Juniors - B Female (Marilyn)</t>
         </is>
       </c>
       <c r="L587" s="12" t="inlineStr">
@@ -45310,7 +45310,7 @@
       </c>
       <c r="K588" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Kangaroos Mixed MUFC - Miniroos Boys U11 Kangas</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Kangaroos Mixed</t>
         </is>
       </c>
       <c r="L588" s="10" t="inlineStr">
@@ -45386,7 +45386,7 @@
       </c>
       <c r="K589" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U7J (Red)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Red)</t>
         </is>
       </c>
       <c r="L589" s="12" t="inlineStr">
@@ -45462,7 +45462,7 @@
       </c>
       <c r="K590" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U7J (Green)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Green)</t>
         </is>
       </c>
       <c r="L590" s="10" t="inlineStr">
@@ -45538,7 +45538,7 @@
       </c>
       <c r="K591" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - A Female MUFC - Junior Girls U12A (Sienna)</t>
+          <t>Manningham United Blues FC U12 Juniors - A Female (Sienna)</t>
         </is>
       </c>
       <c r="L591" s="12" t="inlineStr">
@@ -45614,7 +45614,7 @@
       </c>
       <c r="K592" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - C Female MUFC - Junior Girls U13C (Abigail)</t>
+          <t>Manningham United Blues FC U13 Juniors - C Female (Abigail)</t>
         </is>
       </c>
       <c r="L592" s="10" t="inlineStr">
@@ -45690,7 +45690,7 @@
       </c>
       <c r="K593" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - B Mixed MUFC - Junior Boys U14B</t>
+          <t>Manningham United Blues FC U14 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="L593" s="12" t="inlineStr">
@@ -45766,7 +45766,7 @@
       </c>
       <c r="K594" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U15 Juniors - B Female MUFC - Junior Girls U15B (Ethan)</t>
+          <t>Manningham United Blues FC U15 Juniors - B Female (Ethan)</t>
         </is>
       </c>
       <c r="L594" s="10" t="inlineStr">
@@ -45842,7 +45842,7 @@
       </c>
       <c r="K595" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC Seniors MUFC - State League Women's</t>
+          <t>Manningham United Blues FC Seniors</t>
         </is>
       </c>
       <c r="L595" s="12" t="inlineStr">
@@ -45918,7 +45918,7 @@
       </c>
       <c r="K596" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - C Female MUFC - Junior Girls U14C (Christian)</t>
+          <t>Manningham United Blues FC U14 Juniors - C Female (Christian)</t>
         </is>
       </c>
       <c r="L596" s="10" t="inlineStr">
@@ -45994,7 +45994,7 @@
       </c>
       <c r="K597" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U15 Juniors - B Female MUFC - Junior Girls U15B (Ethan)</t>
+          <t>Manningham United Blues FC U15 Juniors - B Female (Ethan)</t>
         </is>
       </c>
       <c r="L597" s="12" t="inlineStr">
@@ -46070,7 +46070,7 @@
       </c>
       <c r="K598" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed MUFC - Miniroos Boys U7J (White)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (White)</t>
         </is>
       </c>
       <c r="L598" s="10" t="inlineStr">
@@ -46146,7 +46146,7 @@
       </c>
       <c r="K599" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - B Mixed MUFC - Junior Boys U12B (Andre)</t>
+          <t>Manningham United Blues FC U12 Juniors - B Mixed (Andre)</t>
         </is>
       </c>
       <c r="L599" s="12" t="inlineStr">
@@ -46222,7 +46222,7 @@
       </c>
       <c r="K600" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - B Mixed MUFC - Junior Boys U12B (Chris)</t>
+          <t>Manningham United Blues FC U12 Juniors - B Mixed (Chris)</t>
         </is>
       </c>
       <c r="L600" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Refresh fixtures (30 Jul capture); call out FV-actioned overrides on clash page
- Fresh full-season Dribl capture for all grounds (17 Jul -> 06 Nov, 297 duty
  games, 701 fixtures, 0 clash issues).
- Dropped 6 overrides FV has now actioned in Dribl (verified each game appears
  at its requested ground in the new capture); 10 still-pending moves kept.
- New: the clash page now shows a prominent green banner whenever a saved
  override no longer matches any fixture (= FV actioned it), listing each
  move and prompting verification + removal from overrides.json.
- Also lands the GitHub Actions daily auto-refresh workflow and the
  server-side Dribl API capture script (build/capture_dribl.py).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019VnU9JLaRboFmx5SumRF89
</commit_message>
<xml_diff>
--- a/Manningham_fixtures_and_overlaps.xlsx
+++ b/Manningham_fixtures_and_overlaps.xlsx
@@ -596,7 +596,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Source: fv.dribl.com, 2026 season, generated 25 Jul 2026</t>
+          <t>Source: fv.dribl.com, 2026 season, generated 31 Jul 2026</t>
         </is>
       </c>
     </row>
@@ -8087,7 +8087,7 @@
       </c>
       <c r="K99" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Souttar's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Joeys Mixed (Souttar's)</t>
         </is>
       </c>
       <c r="L99" s="12" t="inlineStr">
@@ -11042,7 +11042,7 @@
       </c>
       <c r="K138" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Souttar's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Joeys Mixed (Souttar's)</t>
         </is>
       </c>
       <c r="L138" s="10" t="inlineStr">
@@ -13859,7 +13859,7 @@
       </c>
       <c r="K175" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Souttar's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Joeys Mixed (Souttar's)</t>
         </is>
       </c>
       <c r="L175" s="12" t="inlineStr">
@@ -19222,7 +19222,7 @@
       </c>
       <c r="K246" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Souttar's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Joeys Mixed (Souttar's)</t>
         </is>
       </c>
       <c r="L246" s="10" t="inlineStr">
@@ -22919,7 +22919,7 @@
       </c>
       <c r="K295" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Souttar's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Joeys Mixed (Souttar's)</t>
         </is>
       </c>
       <c r="L295" s="12" t="inlineStr">
@@ -26012,12 +26012,12 @@
       </c>
       <c r="K336" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Souttar's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Joeys Mixed (Souttar's)</t>
         </is>
       </c>
       <c r="L336" s="10" t="inlineStr">
         <is>
-          <t>East Malvern Junior SC U09 MiniRoos - Wallabies Mixed EMJSC U9 Saturday Red</t>
+          <t>Whitehorse United SC U09 MiniRoos - Joeys Mixed Ed</t>
         </is>
       </c>
       <c r="M336" s="10" t="inlineStr">
@@ -26027,7 +26027,7 @@
       </c>
       <c r="N336" s="9" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Saturday East 9 Wallabies Red</t>
+          <t>Coles MiniRoos Mixed Saturday East 9 Joeys Blue</t>
         </is>
       </c>
       <c r="O336" s="9" t="inlineStr">
@@ -28574,12 +28574,12 @@
       </c>
       <c r="K370" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Souttar's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Joeys Mixed (Souttar's)</t>
         </is>
       </c>
       <c r="L370" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Corica's)</t>
+          <t>Riversdale SC U09 MiniRoos - Joeys Mixed Riversdale U9 Boys - Blue</t>
         </is>
       </c>
       <c r="M370" s="10" t="inlineStr">
@@ -28589,7 +28589,7 @@
       </c>
       <c r="N370" s="9" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Saturday East 9 Wallabies Red</t>
+          <t>Coles MiniRoos Mixed Saturday East 9 Joeys Blue</t>
         </is>
       </c>
       <c r="O370" s="9" t="inlineStr">
@@ -31156,12 +31156,12 @@
       </c>
       <c r="K404" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Souttar's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Joeys Mixed (Souttar's)</t>
         </is>
       </c>
       <c r="L404" s="10" t="inlineStr">
         <is>
-          <t>East Malvern Junior SC U09 MiniRoos - Wallabies Mixed EMJSC U9 Saturday White</t>
+          <t>Oakleigh Cannons FC U09 MiniRoos - Joeys Mixed OCFC Ross</t>
         </is>
       </c>
       <c r="M404" s="10" t="inlineStr">
@@ -31171,7 +31171,7 @@
       </c>
       <c r="N404" s="9" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Saturday East 9 Wallabies Red</t>
+          <t>Coles MiniRoos Mixed Saturday East 9 Joeys Blue</t>
         </is>
       </c>
       <c r="O404" s="9" t="inlineStr">
@@ -49642,12 +49642,12 @@
       </c>
       <c r="H645" s="11" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Sub</t>
         </is>
       </c>
       <c r="I645" s="12" t="inlineStr">
         <is>
-          <t>Pitch 3</t>
+          <t>Pitch 3A</t>
         </is>
       </c>
       <c r="J645" s="11" t="inlineStr">
@@ -49681,11 +49681,7 @@
         </is>
       </c>
       <c r="P645" s="11" t="inlineStr"/>
-      <c r="Q645" s="12" t="inlineStr">
-        <is>
-          <t>Pettys Reserve Pitch 1B (Bottom Field)</t>
-        </is>
-      </c>
+      <c r="Q645" s="12" t="inlineStr"/>
     </row>
     <row r="646">
       <c r="A646" s="9" t="inlineStr">
@@ -53670,12 +53666,12 @@
       </c>
       <c r="H697" s="11" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Sub</t>
         </is>
       </c>
       <c r="I697" s="12" t="inlineStr">
         <is>
-          <t>Pitch 2</t>
+          <t>Pitch 2B</t>
         </is>
       </c>
       <c r="J697" s="11" t="inlineStr">
@@ -53709,11 +53705,7 @@
         </is>
       </c>
       <c r="P697" s="11" t="inlineStr"/>
-      <c r="Q697" s="12" t="inlineStr">
-        <is>
-          <t>Powerful Owl Park Pitch 1B</t>
-        </is>
-      </c>
+      <c r="Q697" s="12" t="inlineStr"/>
     </row>
     <row r="698">
       <c r="A698" s="9" t="inlineStr">
@@ -53751,12 +53743,12 @@
       </c>
       <c r="H698" s="9" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Sub</t>
         </is>
       </c>
       <c r="I698" s="10" t="inlineStr">
         <is>
-          <t>Pitch 1</t>
+          <t>Pitch 1E - Quarter Pitch 4v4</t>
         </is>
       </c>
       <c r="J698" s="9" t="inlineStr">
@@ -53790,11 +53782,7 @@
         </is>
       </c>
       <c r="P698" s="9" t="inlineStr"/>
-      <c r="Q698" s="10" t="inlineStr">
-        <is>
-          <t>Pettys Reserve Pitch 2E (Top Field) - Quarter Pitch 4v4</t>
-        </is>
-      </c>
+      <c r="Q698" s="10" t="inlineStr"/>
     </row>
     <row r="699">
       <c r="A699" s="11" t="inlineStr">
@@ -53832,12 +53820,12 @@
       </c>
       <c r="H699" s="11" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Sub</t>
         </is>
       </c>
       <c r="I699" s="12" t="inlineStr">
         <is>
-          <t>Pitch 2</t>
+          <t>Pitch 2A</t>
         </is>
       </c>
       <c r="J699" s="11" t="inlineStr">
@@ -53871,11 +53859,7 @@
         </is>
       </c>
       <c r="P699" s="11" t="inlineStr"/>
-      <c r="Q699" s="12" t="inlineStr">
-        <is>
-          <t>Pettys Reserve Pitch 2B (Top Field)</t>
-        </is>
-      </c>
+      <c r="Q699" s="12" t="inlineStr"/>
     </row>
     <row r="700">
       <c r="A700" s="9" t="inlineStr">
@@ -53913,12 +53897,12 @@
       </c>
       <c r="H700" s="9" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Sub</t>
         </is>
       </c>
       <c r="I700" s="10" t="inlineStr">
         <is>
-          <t>Pitch 1</t>
+          <t>Pitch 1A</t>
         </is>
       </c>
       <c r="J700" s="9" t="inlineStr">
@@ -53952,11 +53936,7 @@
         </is>
       </c>
       <c r="P700" s="9" t="inlineStr"/>
-      <c r="Q700" s="10" t="inlineStr">
-        <is>
-          <t>Pettys Reserve Pitch 1B (Bottom Field)</t>
-        </is>
-      </c>
+      <c r="Q700" s="10" t="inlineStr"/>
     </row>
     <row r="701">
       <c r="A701" s="11" t="inlineStr">
@@ -53994,12 +53974,12 @@
       </c>
       <c r="H701" s="11" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Sub</t>
         </is>
       </c>
       <c r="I701" s="12" t="inlineStr">
         <is>
-          <t>Pitch 2</t>
+          <t>Pitch 2A</t>
         </is>
       </c>
       <c r="J701" s="11" t="inlineStr">
@@ -54033,11 +54013,7 @@
         </is>
       </c>
       <c r="P701" s="11" t="inlineStr"/>
-      <c r="Q701" s="12" t="inlineStr">
-        <is>
-          <t>Pettys Reserve Pitch 2B (Top Field)</t>
-        </is>
-      </c>
+      <c r="Q701" s="12" t="inlineStr"/>
     </row>
     <row r="702">
       <c r="A702" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Refresh fixtures (30 Jul capture); call out FV-actioned overrides on clash page (#19)
- Fresh full-season Dribl capture for all grounds (17 Jul -> 06 Nov, 297 duty
  games, 701 fixtures, 0 clash issues).
- Dropped 6 overrides FV has now actioned in Dribl (verified each game appears
  at its requested ground in the new capture); 10 still-pending moves kept.
- New: the clash page now shows a prominent green banner whenever a saved
  override no longer matches any fixture (= FV actioned it), listing each
  move and prompting verification + removal from overrides.json.
- Also lands the GitHub Actions daily auto-refresh workflow and the
  server-side Dribl API capture script (build/capture_dribl.py).


Claude-Session: https://claude.ai/code/session_019VnU9JLaRboFmx5SumRF89

Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Manningham_fixtures_and_overlaps.xlsx
+++ b/Manningham_fixtures_and_overlaps.xlsx
@@ -596,7 +596,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Source: fv.dribl.com, 2026 season, generated 25 Jul 2026</t>
+          <t>Source: fv.dribl.com, 2026 season, generated 31 Jul 2026</t>
         </is>
       </c>
     </row>
@@ -8087,7 +8087,7 @@
       </c>
       <c r="K99" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Souttar's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Joeys Mixed (Souttar's)</t>
         </is>
       </c>
       <c r="L99" s="12" t="inlineStr">
@@ -11042,7 +11042,7 @@
       </c>
       <c r="K138" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Souttar's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Joeys Mixed (Souttar's)</t>
         </is>
       </c>
       <c r="L138" s="10" t="inlineStr">
@@ -13859,7 +13859,7 @@
       </c>
       <c r="K175" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Souttar's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Joeys Mixed (Souttar's)</t>
         </is>
       </c>
       <c r="L175" s="12" t="inlineStr">
@@ -19222,7 +19222,7 @@
       </c>
       <c r="K246" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Souttar's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Joeys Mixed (Souttar's)</t>
         </is>
       </c>
       <c r="L246" s="10" t="inlineStr">
@@ -22919,7 +22919,7 @@
       </c>
       <c r="K295" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Souttar's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Joeys Mixed (Souttar's)</t>
         </is>
       </c>
       <c r="L295" s="12" t="inlineStr">
@@ -26012,12 +26012,12 @@
       </c>
       <c r="K336" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Souttar's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Joeys Mixed (Souttar's)</t>
         </is>
       </c>
       <c r="L336" s="10" t="inlineStr">
         <is>
-          <t>East Malvern Junior SC U09 MiniRoos - Wallabies Mixed EMJSC U9 Saturday Red</t>
+          <t>Whitehorse United SC U09 MiniRoos - Joeys Mixed Ed</t>
         </is>
       </c>
       <c r="M336" s="10" t="inlineStr">
@@ -26027,7 +26027,7 @@
       </c>
       <c r="N336" s="9" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Saturday East 9 Wallabies Red</t>
+          <t>Coles MiniRoos Mixed Saturday East 9 Joeys Blue</t>
         </is>
       </c>
       <c r="O336" s="9" t="inlineStr">
@@ -28574,12 +28574,12 @@
       </c>
       <c r="K370" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Souttar's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Joeys Mixed (Souttar's)</t>
         </is>
       </c>
       <c r="L370" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Corica's)</t>
+          <t>Riversdale SC U09 MiniRoos - Joeys Mixed Riversdale U9 Boys - Blue</t>
         </is>
       </c>
       <c r="M370" s="10" t="inlineStr">
@@ -28589,7 +28589,7 @@
       </c>
       <c r="N370" s="9" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Saturday East 9 Wallabies Red</t>
+          <t>Coles MiniRoos Mixed Saturday East 9 Joeys Blue</t>
         </is>
       </c>
       <c r="O370" s="9" t="inlineStr">
@@ -31156,12 +31156,12 @@
       </c>
       <c r="K404" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Souttar's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Joeys Mixed (Souttar's)</t>
         </is>
       </c>
       <c r="L404" s="10" t="inlineStr">
         <is>
-          <t>East Malvern Junior SC U09 MiniRoos - Wallabies Mixed EMJSC U9 Saturday White</t>
+          <t>Oakleigh Cannons FC U09 MiniRoos - Joeys Mixed OCFC Ross</t>
         </is>
       </c>
       <c r="M404" s="10" t="inlineStr">
@@ -31171,7 +31171,7 @@
       </c>
       <c r="N404" s="9" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Saturday East 9 Wallabies Red</t>
+          <t>Coles MiniRoos Mixed Saturday East 9 Joeys Blue</t>
         </is>
       </c>
       <c r="O404" s="9" t="inlineStr">
@@ -49642,12 +49642,12 @@
       </c>
       <c r="H645" s="11" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Sub</t>
         </is>
       </c>
       <c r="I645" s="12" t="inlineStr">
         <is>
-          <t>Pitch 3</t>
+          <t>Pitch 3A</t>
         </is>
       </c>
       <c r="J645" s="11" t="inlineStr">
@@ -49681,11 +49681,7 @@
         </is>
       </c>
       <c r="P645" s="11" t="inlineStr"/>
-      <c r="Q645" s="12" t="inlineStr">
-        <is>
-          <t>Pettys Reserve Pitch 1B (Bottom Field)</t>
-        </is>
-      </c>
+      <c r="Q645" s="12" t="inlineStr"/>
     </row>
     <row r="646">
       <c r="A646" s="9" t="inlineStr">
@@ -53670,12 +53666,12 @@
       </c>
       <c r="H697" s="11" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Sub</t>
         </is>
       </c>
       <c r="I697" s="12" t="inlineStr">
         <is>
-          <t>Pitch 2</t>
+          <t>Pitch 2B</t>
         </is>
       </c>
       <c r="J697" s="11" t="inlineStr">
@@ -53709,11 +53705,7 @@
         </is>
       </c>
       <c r="P697" s="11" t="inlineStr"/>
-      <c r="Q697" s="12" t="inlineStr">
-        <is>
-          <t>Powerful Owl Park Pitch 1B</t>
-        </is>
-      </c>
+      <c r="Q697" s="12" t="inlineStr"/>
     </row>
     <row r="698">
       <c r="A698" s="9" t="inlineStr">
@@ -53751,12 +53743,12 @@
       </c>
       <c r="H698" s="9" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Sub</t>
         </is>
       </c>
       <c r="I698" s="10" t="inlineStr">
         <is>
-          <t>Pitch 1</t>
+          <t>Pitch 1E - Quarter Pitch 4v4</t>
         </is>
       </c>
       <c r="J698" s="9" t="inlineStr">
@@ -53790,11 +53782,7 @@
         </is>
       </c>
       <c r="P698" s="9" t="inlineStr"/>
-      <c r="Q698" s="10" t="inlineStr">
-        <is>
-          <t>Pettys Reserve Pitch 2E (Top Field) - Quarter Pitch 4v4</t>
-        </is>
-      </c>
+      <c r="Q698" s="10" t="inlineStr"/>
     </row>
     <row r="699">
       <c r="A699" s="11" t="inlineStr">
@@ -53832,12 +53820,12 @@
       </c>
       <c r="H699" s="11" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Sub</t>
         </is>
       </c>
       <c r="I699" s="12" t="inlineStr">
         <is>
-          <t>Pitch 2</t>
+          <t>Pitch 2A</t>
         </is>
       </c>
       <c r="J699" s="11" t="inlineStr">
@@ -53871,11 +53859,7 @@
         </is>
       </c>
       <c r="P699" s="11" t="inlineStr"/>
-      <c r="Q699" s="12" t="inlineStr">
-        <is>
-          <t>Pettys Reserve Pitch 2B (Top Field)</t>
-        </is>
-      </c>
+      <c r="Q699" s="12" t="inlineStr"/>
     </row>
     <row r="700">
       <c r="A700" s="9" t="inlineStr">
@@ -53913,12 +53897,12 @@
       </c>
       <c r="H700" s="9" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Sub</t>
         </is>
       </c>
       <c r="I700" s="10" t="inlineStr">
         <is>
-          <t>Pitch 1</t>
+          <t>Pitch 1A</t>
         </is>
       </c>
       <c r="J700" s="9" t="inlineStr">
@@ -53952,11 +53936,7 @@
         </is>
       </c>
       <c r="P700" s="9" t="inlineStr"/>
-      <c r="Q700" s="10" t="inlineStr">
-        <is>
-          <t>Pettys Reserve Pitch 1B (Bottom Field)</t>
-        </is>
-      </c>
+      <c r="Q700" s="10" t="inlineStr"/>
     </row>
     <row r="701">
       <c r="A701" s="11" t="inlineStr">
@@ -53994,12 +53974,12 @@
       </c>
       <c r="H701" s="11" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Sub</t>
         </is>
       </c>
       <c r="I701" s="12" t="inlineStr">
         <is>
-          <t>Pitch 2</t>
+          <t>Pitch 2A</t>
         </is>
       </c>
       <c r="J701" s="11" t="inlineStr">
@@ -54033,11 +54013,7 @@
         </is>
       </c>
       <c r="P701" s="11" t="inlineStr"/>
-      <c r="Q701" s="12" t="inlineStr">
-        <is>
-          <t>Pettys Reserve Pitch 2B (Top Field)</t>
-        </is>
-      </c>
+      <c r="Q701" s="12" t="inlineStr"/>
     </row>
     <row r="702">
       <c r="A702" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Auto-refresh fixtures from Dribl (2026-07-31)
</commit_message>
<xml_diff>
--- a/Manningham_fixtures_and_overlaps.xlsx
+++ b/Manningham_fixtures_and_overlaps.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Games" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overlaps &amp; Peak Load" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="All Games" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Overlaps &amp; Peak Load" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Games'!$A$1:$Q$702</definedName>

</xml_diff>

<commit_message>
Refresh fixtures from Dribl (7 Aug 2026 capture)
Full-season capture spans 17 Jul -> 06 Nov, 296 home games. All 10
pending overrides still match original Dribl placements and are kept.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019cjbt4XSbos5Seo7rdEqmn
</commit_message>
<xml_diff>
--- a/Manningham_fixtures_and_overlaps.xlsx
+++ b/Manningham_fixtures_and_overlaps.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="All Games" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Overlaps &amp; Peak Load" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Games" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overlaps &amp; Peak Load" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Games'!$A$1:$Q$701</definedName>
@@ -596,7 +596,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Source: fv.dribl.com, 2026 season, generated 05 Aug 2026</t>
+          <t>Source: fv.dribl.com, 2026 season, generated 07 Aug 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh fixtures from Dribl (7 Aug 2026 capture) (#20)
Full-season capture spans 17 Jul -> 06 Nov, 296 home games. All 10
pending overrides still match original Dribl placements and are kept.


Claude-Session: https://claude.ai/code/session_019cjbt4XSbos5Seo7rdEqmn

Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Manningham_fixtures_and_overlaps.xlsx
+++ b/Manningham_fixtures_and_overlaps.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="All Games" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Overlaps &amp; Peak Load" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Games" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overlaps &amp; Peak Load" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Games'!$A$1:$Q$701</definedName>
@@ -596,7 +596,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Source: fv.dribl.com, 2026 season, generated 05 Aug 2026</t>
+          <t>Source: fv.dribl.com, 2026 season, generated 07 Aug 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh fixtures from Dribl (2026-08-07)
</commit_message>
<xml_diff>
--- a/Manningham_fixtures_and_overlaps.xlsx
+++ b/Manningham_fixtures_and_overlaps.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Games" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overlaps &amp; Peak Load" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="All Games" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Overlaps &amp; Peak Load" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Games'!$A$1:$Q$701</definedName>

</xml_diff>

<commit_message>
Auto-refresh fixtures from Dribl (2026-08-13)
</commit_message>
<xml_diff>
--- a/Manningham_fixtures_and_overlaps.xlsx
+++ b/Manningham_fixtures_and_overlaps.xlsx
@@ -596,7 +596,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Source: fv.dribl.com, 2026 season, generated 12 Aug 2026</t>
+          <t>Source: fv.dribl.com, 2026 season, generated 13 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -21334,12 +21334,12 @@
       </c>
       <c r="C276" s="9" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="D276" s="9" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="E276" s="9" t="n">

</xml_diff>

<commit_message>
Refresh fixtures from Dribl (17 Aug 2026) + prune actioned/stale overrides
- Regenerated all outputs from the 16 Aug full-season Action capture
  (the 14 Aug hand capture was a partial 3-week window and was discarded)
- overrides.json pruned 8 -> 4: dropped the played 2/8/15/16 Aug moves;
  re-keyed the 23 Aug U13B (Samir) move to FV's new 12:10 kickoff
  (Pitch 3 move kept deliberately - the resulting U18 overlap is flagged
  on the clash page); kept 22 Aug, 5 Sep, 6 Sep pending moves
- Setup/pack-up page: collapsible ground-layouts section, duty controls
  moved to top

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Puq4Xn23NC4d6RhNQLZP1N
</commit_message>
<xml_diff>
--- a/Manningham_fixtures_and_overlaps.xlsx
+++ b/Manningham_fixtures_and_overlaps.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="All Games" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Overlaps &amp; Peak Load" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Games" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overlaps &amp; Peak Load" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Games'!$A$1:$Q$692</definedName>
@@ -596,7 +596,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Source: fv.dribl.com, 2026 season, generated 16 Aug 2026</t>
+          <t>Source: fv.dribl.com, 2026 season, generated 17 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
         </is>
       </c>
       <c r="B11" s="8" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -26270,235 +26270,247 @@
       <c r="Q339" s="12" t="inlineStr"/>
     </row>
     <row r="340">
-      <c r="A340" s="9" t="inlineStr">
+      <c r="A340" s="13" t="inlineStr">
         <is>
           <t>08 Aug 2026</t>
         </is>
       </c>
-      <c r="B340" s="9" t="inlineStr">
+      <c r="B340" s="13" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="C340" s="9" t="inlineStr">
+      <c r="C340" s="13" t="inlineStr">
         <is>
           <t>08:30</t>
         </is>
       </c>
-      <c r="D340" s="9" t="inlineStr">
+      <c r="D340" s="13" t="inlineStr">
         <is>
           <t>09:10</t>
         </is>
       </c>
-      <c r="E340" s="9" t="n">
+      <c r="E340" s="13" t="n">
         <v>40</v>
       </c>
-      <c r="F340" s="9" t="inlineStr">
+      <c r="F340" s="13" t="inlineStr">
         <is>
           <t>Pettys Reserve</t>
         </is>
       </c>
-      <c r="G340" s="9" t="inlineStr">
+      <c r="G340" s="13" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="H340" s="9" t="inlineStr">
+      <c r="H340" s="13" t="inlineStr">
         <is>
           <t>Sub</t>
         </is>
       </c>
-      <c r="I340" s="10" t="inlineStr">
+      <c r="I340" s="14" t="inlineStr">
         <is>
           <t>Pitch 1B (Bottom Field)</t>
         </is>
       </c>
-      <c r="J340" s="9" t="inlineStr">
+      <c r="J340" s="13" t="inlineStr">
         <is>
           <t>U11</t>
         </is>
       </c>
-      <c r="K340" s="10" t="inlineStr">
+      <c r="K340" s="14" t="inlineStr">
         <is>
           <t>Manningham United Blues FC U11 MiniRoos - Wallabies Mixed (Culina's)</t>
         </is>
       </c>
-      <c r="L340" s="10" t="inlineStr">
+      <c r="L340" s="14" t="inlineStr">
         <is>
           <t>Whitehorse United SC U11 MiniRoos - Wallabies Mixed Vanntha</t>
         </is>
       </c>
-      <c r="M340" s="10" t="inlineStr">
+      <c r="M340" s="14" t="inlineStr">
         <is>
           <t>Coles MiniRoos Mixed Saturday (U6 - U11)</t>
         </is>
       </c>
-      <c r="N340" s="9" t="inlineStr">
+      <c r="N340" s="13" t="inlineStr">
         <is>
           <t>Coles MiniRoos Mixed Saturday East 11 Wallabies Blue</t>
         </is>
       </c>
-      <c r="O340" s="9" t="inlineStr">
+      <c r="O340" s="13" t="inlineStr">
         <is>
           <t>R14</t>
         </is>
       </c>
-      <c r="P340" s="9" t="inlineStr"/>
-      <c r="Q340" s="10" t="inlineStr"/>
+      <c r="P340" s="15" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Q340" s="14" t="inlineStr"/>
     </row>
     <row r="341">
-      <c r="A341" s="11" t="inlineStr">
+      <c r="A341" s="13" t="inlineStr">
         <is>
           <t>08 Aug 2026</t>
         </is>
       </c>
-      <c r="B341" s="11" t="inlineStr">
+      <c r="B341" s="13" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="C341" s="11" t="inlineStr">
+      <c r="C341" s="13" t="inlineStr">
         <is>
           <t>08:30</t>
         </is>
       </c>
-      <c r="D341" s="11" t="inlineStr">
+      <c r="D341" s="13" t="inlineStr">
         <is>
           <t>09:30</t>
         </is>
       </c>
-      <c r="E341" s="11" t="n">
+      <c r="E341" s="13" t="n">
         <v>60</v>
       </c>
-      <c r="F341" s="11" t="inlineStr">
+      <c r="F341" s="13" t="inlineStr">
         <is>
           <t>Pettys Reserve</t>
         </is>
       </c>
-      <c r="G341" s="11" t="inlineStr">
+      <c r="G341" s="13" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="H341" s="11" t="inlineStr">
+      <c r="H341" s="13" t="inlineStr">
         <is>
           <t>Sub</t>
         </is>
       </c>
-      <c r="I341" s="12" t="inlineStr">
+      <c r="I341" s="14" t="inlineStr">
         <is>
           <t>Pitch 1A (Bottom Field)</t>
         </is>
       </c>
-      <c r="J341" s="11" t="inlineStr">
+      <c r="J341" s="13" t="inlineStr">
         <is>
           <t>U12</t>
         </is>
       </c>
-      <c r="K341" s="12" t="inlineStr">
+      <c r="K341" s="14" t="inlineStr">
         <is>
           <t>Manningham United Blues FC U12 Juniors - B Mixed (Chris)</t>
         </is>
       </c>
-      <c r="L341" s="12" t="inlineStr">
+      <c r="L341" s="14" t="inlineStr">
         <is>
           <t>Nunawading City FC U12 Juniors - B Mixed</t>
         </is>
       </c>
-      <c r="M341" s="12" t="inlineStr">
+      <c r="M341" s="14" t="inlineStr">
         <is>
           <t>Junior Mixed Saturday (U12 - U16)</t>
         </is>
       </c>
-      <c r="N341" s="11" t="inlineStr">
+      <c r="N341" s="13" t="inlineStr">
         <is>
           <t>Mixed Saturday East 12B</t>
         </is>
       </c>
-      <c r="O341" s="11" t="inlineStr">
+      <c r="O341" s="13" t="inlineStr">
         <is>
           <t>R14</t>
         </is>
       </c>
-      <c r="P341" s="11" t="inlineStr"/>
-      <c r="Q341" s="12" t="inlineStr"/>
+      <c r="P341" s="15" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Q341" s="14" t="inlineStr"/>
     </row>
     <row r="342">
-      <c r="A342" s="9" t="inlineStr">
+      <c r="A342" s="13" t="inlineStr">
         <is>
           <t>08 Aug 2026</t>
         </is>
       </c>
-      <c r="B342" s="9" t="inlineStr">
+      <c r="B342" s="13" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="C342" s="9" t="inlineStr">
-        <is>
-          <t>12:45</t>
-        </is>
-      </c>
-      <c r="D342" s="9" t="inlineStr">
-        <is>
-          <t>14:15</t>
-        </is>
-      </c>
-      <c r="E342" s="9" t="n">
-        <v>90</v>
-      </c>
-      <c r="F342" s="9" t="inlineStr">
+      <c r="C342" s="13" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="D342" s="13" t="inlineStr">
+        <is>
+          <t>09:40</t>
+        </is>
+      </c>
+      <c r="E342" s="13" t="n">
+        <v>40</v>
+      </c>
+      <c r="F342" s="13" t="inlineStr">
         <is>
           <t>Pettys Reserve</t>
         </is>
       </c>
-      <c r="G342" s="9" t="inlineStr">
+      <c r="G342" s="13" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="H342" s="9" t="inlineStr">
-        <is>
-          <t>Full</t>
-        </is>
-      </c>
-      <c r="I342" s="10" t="inlineStr">
-        <is>
-          <t>Pitch 1 (Bottom Field)</t>
-        </is>
-      </c>
-      <c r="J342" s="9" t="inlineStr">
-        <is>
-          <t>Reserves</t>
-        </is>
-      </c>
-      <c r="K342" s="10" t="inlineStr">
-        <is>
-          <t>Manningham United Blues FC Reserves</t>
-        </is>
-      </c>
-      <c r="L342" s="10" t="inlineStr">
-        <is>
-          <t>Geelong Galaxy United FC Reserves</t>
-        </is>
-      </c>
-      <c r="M342" s="10" t="inlineStr">
-        <is>
-          <t>VPL Women</t>
-        </is>
-      </c>
-      <c r="N342" s="9" t="inlineStr">
-        <is>
-          <t>VPL Women - Reserves</t>
-        </is>
-      </c>
-      <c r="O342" s="9" t="inlineStr">
-        <is>
-          <t>R19</t>
-        </is>
-      </c>
-      <c r="P342" s="9" t="inlineStr"/>
-      <c r="Q342" s="10" t="inlineStr"/>
+      <c r="H342" s="13" t="inlineStr">
+        <is>
+          <t>Sub</t>
+        </is>
+      </c>
+      <c r="I342" s="14" t="inlineStr">
+        <is>
+          <t>Pitch 1C (Bottom Field) - Quarter Pitch 7v7</t>
+        </is>
+      </c>
+      <c r="J342" s="13" t="inlineStr">
+        <is>
+          <t>U08</t>
+        </is>
+      </c>
+      <c r="K342" s="14" t="inlineStr">
+        <is>
+          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed (Duke's)</t>
+        </is>
+      </c>
+      <c r="L342" s="14" t="inlineStr">
+        <is>
+          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed (Slater's)</t>
+        </is>
+      </c>
+      <c r="M342" s="14" t="inlineStr">
+        <is>
+          <t>Coles MiniRoos Mixed Saturday (U6 - U11)</t>
+        </is>
+      </c>
+      <c r="N342" s="13" t="inlineStr">
+        <is>
+          <t>Coles MiniRoos Mixed Saturday East 8 Joeys Red</t>
+        </is>
+      </c>
+      <c r="O342" s="13" t="inlineStr">
+        <is>
+          <t>R14</t>
+        </is>
+      </c>
+      <c r="P342" s="15" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Q342" s="14" t="inlineStr"/>
     </row>
     <row r="343">
       <c r="A343" s="11" t="inlineStr">
@@ -26513,12 +26525,12 @@
       </c>
       <c r="C343" s="11" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>12:45</t>
         </is>
       </c>
       <c r="D343" s="11" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>14:15</t>
         </is>
       </c>
       <c r="E343" s="11" t="n">
@@ -26546,17 +26558,17 @@
       </c>
       <c r="J343" s="11" t="inlineStr">
         <is>
-          <t>Seniors</t>
+          <t>Reserves</t>
         </is>
       </c>
       <c r="K343" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC Seniors</t>
+          <t>Manningham United Blues FC Reserves</t>
         </is>
       </c>
       <c r="L343" s="12" t="inlineStr">
         <is>
-          <t>Geelong Galaxy United FC Seniors</t>
+          <t>Geelong Galaxy United FC Reserves</t>
         </is>
       </c>
       <c r="M343" s="12" t="inlineStr">
@@ -26566,7 +26578,7 @@
       </c>
       <c r="N343" s="11" t="inlineStr">
         <is>
-          <t>VPL Women</t>
+          <t>VPL Women - Reserves</t>
         </is>
       </c>
       <c r="O343" s="11" t="inlineStr">
@@ -26590,16 +26602,16 @@
       </c>
       <c r="C344" s="9" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="D344" s="9" t="inlineStr">
         <is>
-          <t>09:10</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="E344" s="9" t="n">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="F344" s="9" t="inlineStr">
         <is>
@@ -26608,47 +26620,47 @@
       </c>
       <c r="G344" s="9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H344" s="9" t="inlineStr">
         <is>
-          <t>Sub</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="I344" s="10" t="inlineStr">
         <is>
-          <t>Pitch 2C (Top Field) - Quarter Pitch 7v7</t>
+          <t>Pitch 1 (Bottom Field)</t>
         </is>
       </c>
       <c r="J344" s="9" t="inlineStr">
         <is>
-          <t>U09</t>
+          <t>Seniors</t>
         </is>
       </c>
       <c r="K344" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Corica's)</t>
+          <t>Manningham United Blues FC Seniors</t>
         </is>
       </c>
       <c r="L344" s="10" t="inlineStr">
         <is>
-          <t>East Malvern Junior SC U09 MiniRoos - Wallabies Mixed EMJSC U9 Saturday Red</t>
+          <t>Geelong Galaxy United FC Seniors</t>
         </is>
       </c>
       <c r="M344" s="10" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Saturday (U6 - U11)</t>
+          <t>VPL Women</t>
         </is>
       </c>
       <c r="N344" s="9" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Saturday East 9 Wallabies Red</t>
+          <t>VPL Women</t>
         </is>
       </c>
       <c r="O344" s="9" t="inlineStr">
         <is>
-          <t>R14</t>
+          <t>R19</t>
         </is>
       </c>
       <c r="P344" s="9" t="inlineStr"/>
@@ -26667,12 +26679,12 @@
       </c>
       <c r="C345" s="11" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:30</t>
         </is>
       </c>
       <c r="D345" s="11" t="inlineStr">
         <is>
-          <t>09:40</t>
+          <t>09:10</t>
         </is>
       </c>
       <c r="E345" s="11" t="n">
@@ -26690,27 +26702,27 @@
       </c>
       <c r="H345" s="11" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Sub</t>
         </is>
       </c>
       <c r="I345" s="12" t="inlineStr">
         <is>
-          <t>Pitch 2</t>
+          <t>Pitch 2C (Top Field) - Quarter Pitch 7v7</t>
         </is>
       </c>
       <c r="J345" s="11" t="inlineStr">
         <is>
-          <t>U08</t>
+          <t>U09</t>
         </is>
       </c>
       <c r="K345" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed (Duke's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Corica's)</t>
         </is>
       </c>
       <c r="L345" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed (Slater's)</t>
+          <t>East Malvern Junior SC U09 MiniRoos - Wallabies Mixed EMJSC U9 Saturday Red</t>
         </is>
       </c>
       <c r="M345" s="12" t="inlineStr">
@@ -26720,7 +26732,7 @@
       </c>
       <c r="N345" s="11" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Saturday East 8 Joeys Red</t>
+          <t>Coles MiniRoos Mixed Saturday East 9 Wallabies Red</t>
         </is>
       </c>
       <c r="O345" s="11" t="inlineStr">
@@ -26729,11 +26741,7 @@
         </is>
       </c>
       <c r="P345" s="11" t="inlineStr"/>
-      <c r="Q345" s="12" t="inlineStr">
-        <is>
-          <t>Pettys Reserve Pitch 1C (Bottom Field) - Quarter Pitch 7v7</t>
-        </is>
-      </c>
+      <c r="Q345" s="12" t="inlineStr"/>
     </row>
     <row r="346">
       <c r="A346" s="9" t="inlineStr">
@@ -27713,223 +27721,235 @@
       <c r="Q358" s="10" t="inlineStr"/>
     </row>
     <row r="359">
-      <c r="A359" s="11" t="inlineStr">
+      <c r="A359" s="13" t="inlineStr">
         <is>
           <t>15 Aug 2026</t>
         </is>
       </c>
-      <c r="B359" s="11" t="inlineStr">
+      <c r="B359" s="13" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="C359" s="11" t="inlineStr">
+      <c r="C359" s="13" t="inlineStr">
         <is>
           <t>08:30</t>
         </is>
       </c>
-      <c r="D359" s="11" t="inlineStr">
+      <c r="D359" s="13" t="inlineStr">
+        <is>
+          <t>09:10</t>
+        </is>
+      </c>
+      <c r="E359" s="13" t="n">
+        <v>40</v>
+      </c>
+      <c r="F359" s="13" t="inlineStr">
+        <is>
+          <t>Pettys Reserve</t>
+        </is>
+      </c>
+      <c r="G359" s="13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H359" s="13" t="inlineStr">
+        <is>
+          <t>Sub</t>
+        </is>
+      </c>
+      <c r="I359" s="14" t="inlineStr">
+        <is>
+          <t>Pitch 1E (Bottom Field) - Quarter Pitch 4v4</t>
+        </is>
+      </c>
+      <c r="J359" s="13" t="inlineStr">
+        <is>
+          <t>U07</t>
+        </is>
+      </c>
+      <c r="K359" s="14" t="inlineStr">
+        <is>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (White)</t>
+        </is>
+      </c>
+      <c r="L359" s="14" t="inlineStr">
+        <is>
+          <t>Oakleigh Cannons FC U07 MiniRoos - Joeys Mixed OCFC Chippa/Jason</t>
+        </is>
+      </c>
+      <c r="M359" s="14" t="inlineStr">
+        <is>
+          <t>Coles MiniRoos Mixed Saturday (U6 - U11)</t>
+        </is>
+      </c>
+      <c r="N359" s="13" t="inlineStr">
+        <is>
+          <t>Coles MiniRoos Mixed Saturday East 7 Joeys Red</t>
+        </is>
+      </c>
+      <c r="O359" s="13" t="inlineStr">
+        <is>
+          <t>R15</t>
+        </is>
+      </c>
+      <c r="P359" s="15" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Q359" s="14" t="inlineStr"/>
+    </row>
+    <row r="360">
+      <c r="A360" s="13" t="inlineStr">
+        <is>
+          <t>15 Aug 2026</t>
+        </is>
+      </c>
+      <c r="B360" s="13" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="C360" s="13" t="inlineStr">
+        <is>
+          <t>08:30</t>
+        </is>
+      </c>
+      <c r="D360" s="13" t="inlineStr">
         <is>
           <t>09:30</t>
         </is>
       </c>
-      <c r="E359" s="11" t="n">
+      <c r="E360" s="13" t="n">
         <v>60</v>
       </c>
-      <c r="F359" s="11" t="inlineStr">
+      <c r="F360" s="13" t="inlineStr">
         <is>
           <t>Pettys Reserve</t>
         </is>
       </c>
-      <c r="G359" s="11" t="inlineStr">
+      <c r="G360" s="13" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="H359" s="11" t="inlineStr">
+      <c r="H360" s="13" t="inlineStr">
         <is>
           <t>Sub</t>
         </is>
       </c>
-      <c r="I359" s="12" t="inlineStr">
+      <c r="I360" s="14" t="inlineStr">
         <is>
           <t>Pitch 1A (Bottom Field)</t>
         </is>
       </c>
-      <c r="J359" s="11" t="inlineStr">
+      <c r="J360" s="13" t="inlineStr">
         <is>
           <t>U12</t>
         </is>
       </c>
-      <c r="K359" s="12" t="inlineStr">
+      <c r="K360" s="14" t="inlineStr">
         <is>
           <t>Manningham United Blues FC U12 Juniors - B Mixed (Andre)</t>
         </is>
       </c>
-      <c r="L359" s="12" t="inlineStr">
+      <c r="L360" s="14" t="inlineStr">
         <is>
           <t>FC Bulleen Lions U12 Juniors - B Mixed</t>
         </is>
       </c>
-      <c r="M359" s="12" t="inlineStr">
+      <c r="M360" s="14" t="inlineStr">
         <is>
           <t>Junior Mixed Saturday (U12 - U16)</t>
         </is>
       </c>
-      <c r="N359" s="11" t="inlineStr">
+      <c r="N360" s="13" t="inlineStr">
         <is>
           <t>Mixed Saturday East 12B</t>
         </is>
       </c>
-      <c r="O359" s="11" t="inlineStr">
+      <c r="O360" s="13" t="inlineStr">
         <is>
           <t>R15</t>
         </is>
       </c>
-      <c r="P359" s="11" t="inlineStr"/>
-      <c r="Q359" s="12" t="inlineStr"/>
-    </row>
-    <row r="360">
-      <c r="A360" s="9" t="inlineStr">
+      <c r="P360" s="15" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Q360" s="14" t="inlineStr"/>
+    </row>
+    <row r="361">
+      <c r="A361" s="13" t="inlineStr">
         <is>
           <t>15 Aug 2026</t>
         </is>
       </c>
-      <c r="B360" s="9" t="inlineStr">
+      <c r="B361" s="13" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="C360" s="9" t="inlineStr">
+      <c r="C361" s="13" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="D360" s="9" t="inlineStr">
+      <c r="D361" s="13" t="inlineStr">
         <is>
           <t>10:00</t>
         </is>
       </c>
-      <c r="E360" s="9" t="n">
+      <c r="E361" s="13" t="n">
         <v>60</v>
       </c>
-      <c r="F360" s="9" t="inlineStr">
+      <c r="F361" s="13" t="inlineStr">
         <is>
           <t>Pettys Reserve</t>
         </is>
       </c>
-      <c r="G360" s="9" t="inlineStr">
+      <c r="G361" s="13" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="H360" s="9" t="inlineStr">
+      <c r="H361" s="13" t="inlineStr">
         <is>
           <t>Sub</t>
         </is>
       </c>
-      <c r="I360" s="10" t="inlineStr">
+      <c r="I361" s="14" t="inlineStr">
         <is>
           <t>Pitch 1B (Bottom Field)</t>
         </is>
       </c>
-      <c r="J360" s="9" t="inlineStr"/>
-      <c r="K360" s="10" t="inlineStr">
+      <c r="J361" s="13" t="inlineStr"/>
+      <c r="K361" s="14" t="inlineStr">
         <is>
           <t>Manningham United Blues FC Girls Clinic</t>
         </is>
       </c>
-      <c r="L360" s="10" t="inlineStr">
+      <c r="L361" s="14" t="inlineStr">
         <is>
           <t>[MANUAL ADD]</t>
         </is>
       </c>
-      <c r="M360" s="10" t="inlineStr">
+      <c r="M361" s="14" t="inlineStr">
         <is>
           <t>Girls Clinic</t>
         </is>
       </c>
-      <c r="N360" s="9" t="inlineStr"/>
-      <c r="O360" s="9" t="inlineStr"/>
-      <c r="P360" s="9" t="inlineStr"/>
-      <c r="Q360" s="10" t="inlineStr"/>
-    </row>
-    <row r="361">
-      <c r="A361" s="11" t="inlineStr">
-        <is>
-          <t>15 Aug 2026</t>
-        </is>
-      </c>
-      <c r="B361" s="11" t="inlineStr">
-        <is>
-          <t>Sat</t>
-        </is>
-      </c>
-      <c r="C361" s="11" t="inlineStr">
-        <is>
-          <t>08:30</t>
-        </is>
-      </c>
-      <c r="D361" s="11" t="inlineStr">
-        <is>
-          <t>09:10</t>
-        </is>
-      </c>
-      <c r="E361" s="11" t="n">
-        <v>40</v>
-      </c>
-      <c r="F361" s="11" t="inlineStr">
-        <is>
-          <t>Pettys Reserve</t>
-        </is>
-      </c>
-      <c r="G361" s="11" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="H361" s="11" t="inlineStr">
-        <is>
-          <t>Sub</t>
-        </is>
-      </c>
-      <c r="I361" s="12" t="inlineStr">
-        <is>
-          <t>Pitch 2D (Top Field) - Quarter Pitch 7v7</t>
-        </is>
-      </c>
-      <c r="J361" s="11" t="inlineStr">
-        <is>
-          <t>U09</t>
-        </is>
-      </c>
-      <c r="K361" s="12" t="inlineStr">
-        <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Joeys Mixed (Souttar's)</t>
-        </is>
-      </c>
-      <c r="L361" s="12" t="inlineStr">
-        <is>
-          <t>Riversdale SC U09 MiniRoos - Joeys Mixed Riversdale U9 Boys - Blue</t>
-        </is>
-      </c>
-      <c r="M361" s="12" t="inlineStr">
-        <is>
-          <t>Coles MiniRoos Mixed Saturday (U6 - U11)</t>
-        </is>
-      </c>
-      <c r="N361" s="11" t="inlineStr">
-        <is>
-          <t>Coles MiniRoos Mixed Saturday East 9 Joeys Blue</t>
-        </is>
-      </c>
-      <c r="O361" s="11" t="inlineStr">
-        <is>
-          <t>R15</t>
-        </is>
-      </c>
-      <c r="P361" s="11" t="inlineStr"/>
-      <c r="Q361" s="12" t="inlineStr"/>
+      <c r="N361" s="13" t="inlineStr"/>
+      <c r="O361" s="13" t="inlineStr"/>
+      <c r="P361" s="15" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Q361" s="14" t="inlineStr"/>
     </row>
     <row r="362">
       <c r="A362" s="9" t="inlineStr">
@@ -27967,27 +27987,27 @@
       </c>
       <c r="H362" s="9" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Sub</t>
         </is>
       </c>
       <c r="I362" s="10" t="inlineStr">
         <is>
-          <t>Pitch 2</t>
+          <t>Pitch 2D (Top Field) - Quarter Pitch 7v7</t>
         </is>
       </c>
       <c r="J362" s="9" t="inlineStr">
         <is>
-          <t>U07</t>
+          <t>U09</t>
         </is>
       </c>
       <c r="K362" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (White)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Joeys Mixed (Souttar's)</t>
         </is>
       </c>
       <c r="L362" s="10" t="inlineStr">
         <is>
-          <t>Oakleigh Cannons FC U07 MiniRoos - Joeys Mixed OCFC Chippa/Jason</t>
+          <t>Riversdale SC U09 MiniRoos - Joeys Mixed Riversdale U9 Boys - Blue</t>
         </is>
       </c>
       <c r="M362" s="10" t="inlineStr">
@@ -27997,7 +28017,7 @@
       </c>
       <c r="N362" s="9" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Saturday East 7 Joeys Red</t>
+          <t>Coles MiniRoos Mixed Saturday East 9 Joeys Blue</t>
         </is>
       </c>
       <c r="O362" s="9" t="inlineStr">
@@ -28006,11 +28026,7 @@
         </is>
       </c>
       <c r="P362" s="9" t="inlineStr"/>
-      <c r="Q362" s="10" t="inlineStr">
-        <is>
-          <t>Pettys Reserve Pitch 1E (Bottom Field) - Quarter Pitch 4v4</t>
-        </is>
-      </c>
+      <c r="Q362" s="10" t="inlineStr"/>
     </row>
     <row r="363">
       <c r="A363" s="11" t="inlineStr">
@@ -46559,16 +46575,16 @@
       </c>
       <c r="C605" s="11" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>11:45</t>
         </is>
       </c>
       <c r="D605" s="11" t="inlineStr">
         <is>
-          <t>14:10</t>
+          <t>12:45</t>
         </is>
       </c>
       <c r="E605" s="11" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="F605" s="11" t="inlineStr">
         <is>
@@ -46582,27 +46598,27 @@
       </c>
       <c r="H605" s="11" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Sub</t>
         </is>
       </c>
       <c r="I605" s="12" t="inlineStr">
         <is>
-          <t>Pitch 2</t>
+          <t>Pitch 2B</t>
         </is>
       </c>
       <c r="J605" s="11" t="inlineStr">
         <is>
-          <t>U16</t>
+          <t>U13</t>
         </is>
       </c>
       <c r="K605" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U16 Juniors - B Mixed</t>
+          <t>Manningham United Blues FC U13 Juniors - A Mixed (George &amp; George)</t>
         </is>
       </c>
       <c r="L605" s="12" t="inlineStr">
         <is>
-          <t>Monash City Villarreal FC U16 Juniors - B Mixed Monash City Villarreal FC U16 Blue</t>
+          <t>Burwood City FC U13 Juniors - A Mixed LTE</t>
         </is>
       </c>
       <c r="M605" s="12" t="inlineStr">
@@ -46612,7 +46628,7 @@
       </c>
       <c r="N605" s="11" t="inlineStr">
         <is>
-          <t>Mixed East 16B</t>
+          <t>Mixed Sunday East 13A</t>
         </is>
       </c>
       <c r="O605" s="11" t="inlineStr">
@@ -46636,16 +46652,16 @@
       </c>
       <c r="C606" s="9" t="inlineStr">
         <is>
-          <t>11:45</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="D606" s="9" t="inlineStr">
         <is>
-          <t>12:45</t>
+          <t>14:10</t>
         </is>
       </c>
       <c r="E606" s="9" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F606" s="9" t="inlineStr">
         <is>
@@ -46654,7 +46670,7 @@
       </c>
       <c r="G606" s="9" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H606" s="9" t="inlineStr">
@@ -46664,22 +46680,22 @@
       </c>
       <c r="I606" s="10" t="inlineStr">
         <is>
-          <t>Pitch 3</t>
+          <t>Pitch 2</t>
         </is>
       </c>
       <c r="J606" s="9" t="inlineStr">
         <is>
-          <t>U13</t>
+          <t>U16</t>
         </is>
       </c>
       <c r="K606" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - A Mixed (George &amp; George)</t>
+          <t>Manningham United Blues FC U16 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="L606" s="10" t="inlineStr">
         <is>
-          <t>Burwood City FC U13 Juniors - A Mixed LTE</t>
+          <t>Monash City Villarreal FC U16 Juniors - B Mixed Monash City Villarreal FC U16 Blue</t>
         </is>
       </c>
       <c r="M606" s="10" t="inlineStr">
@@ -46689,7 +46705,7 @@
       </c>
       <c r="N606" s="9" t="inlineStr">
         <is>
-          <t>Mixed Sunday East 13A</t>
+          <t>Mixed East 16B</t>
         </is>
       </c>
       <c r="O606" s="9" t="inlineStr">
@@ -46698,11 +46714,7 @@
         </is>
       </c>
       <c r="P606" s="9" t="inlineStr"/>
-      <c r="Q606" s="10" t="inlineStr">
-        <is>
-          <t>Powerful Owl Park Pitch 2B</t>
-        </is>
-      </c>
+      <c r="Q606" s="10" t="inlineStr"/>
     </row>
     <row r="607">
       <c r="A607" s="11" t="inlineStr">
@@ -48416,11 +48428,11 @@
       </c>
       <c r="D629" s="11" t="inlineStr">
         <is>
-          <t>11:20</t>
+          <t>11:40</t>
         </is>
       </c>
       <c r="E629" s="11" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="F629" s="11" t="inlineStr">
         <is>
@@ -48439,32 +48451,32 @@
       </c>
       <c r="I629" s="12" t="inlineStr">
         <is>
-          <t>Pitch 1 - Midi Field B</t>
+          <t>Pitch 1B</t>
         </is>
       </c>
       <c r="J629" s="11" t="inlineStr">
         <is>
-          <t>U10</t>
+          <t>U13</t>
         </is>
       </c>
       <c r="K629" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U10 MiniRoos - Joeys Mixed (Sainsbury's)</t>
+          <t>Manningham United Blues FC U13 Juniors - C Mixed (Martin)</t>
         </is>
       </c>
       <c r="L629" s="12" t="inlineStr">
         <is>
-          <t>East Malvern Junior SC U10 MiniRoos - Joeys Mixed EMJSC U10 Sunday</t>
+          <t>Malvern City FC U13 Juniors - C Mixed U13 Anthony - C</t>
         </is>
       </c>
       <c r="M629" s="12" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Sunday (U6 - U11)</t>
+          <t>Junior Mixed Sunday (U12 - U16)</t>
         </is>
       </c>
       <c r="N629" s="11" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Sunday East 10 Joeys Red</t>
+          <t>Mixed Sunday East 13C Red</t>
         </is>
       </c>
       <c r="O629" s="11" t="inlineStr">
@@ -48488,16 +48500,16 @@
       </c>
       <c r="C630" s="9" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>10:40</t>
         </is>
       </c>
       <c r="D630" s="9" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>11:20</t>
         </is>
       </c>
       <c r="E630" s="9" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="F630" s="9" t="inlineStr">
         <is>
@@ -48516,32 +48528,32 @@
       </c>
       <c r="I630" s="10" t="inlineStr">
         <is>
-          <t>Pitch 1B</t>
+          <t>Pitch 1 - Midi Field B</t>
         </is>
       </c>
       <c r="J630" s="9" t="inlineStr">
         <is>
-          <t>U13</t>
+          <t>U10</t>
         </is>
       </c>
       <c r="K630" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - A Mixed (George &amp; George)</t>
+          <t>Manningham United Blues FC U10 MiniRoos - Joeys Mixed (Sainsbury's)</t>
         </is>
       </c>
       <c r="L630" s="10" t="inlineStr">
         <is>
-          <t>Knox City FC U13 Juniors - A Mixed U13A</t>
+          <t>East Malvern Junior SC U10 MiniRoos - Joeys Mixed EMJSC U10 Sunday</t>
         </is>
       </c>
       <c r="M630" s="10" t="inlineStr">
         <is>
-          <t>Junior Mixed Sunday (U12 - U16)</t>
+          <t>Coles MiniRoos Mixed Sunday (U6 - U11)</t>
         </is>
       </c>
       <c r="N630" s="9" t="inlineStr">
         <is>
-          <t>Mixed Sunday East 13A</t>
+          <t>Coles MiniRoos Mixed Sunday East 10 Joeys Red</t>
         </is>
       </c>
       <c r="O630" s="9" t="inlineStr">
@@ -48565,16 +48577,16 @@
       </c>
       <c r="C631" s="11" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="D631" s="11" t="inlineStr">
         <is>
-          <t>14:40</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="E631" s="11" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="F631" s="11" t="inlineStr">
         <is>
@@ -48588,27 +48600,27 @@
       </c>
       <c r="H631" s="11" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Sub</t>
         </is>
       </c>
       <c r="I631" s="12" t="inlineStr">
         <is>
-          <t>Pitch 1</t>
+          <t>Pitch 1B</t>
         </is>
       </c>
       <c r="J631" s="11" t="inlineStr">
         <is>
-          <t>U15</t>
+          <t>U13</t>
         </is>
       </c>
       <c r="K631" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U15 Juniors - A Mixed</t>
+          <t>Manningham United Blues FC U13 Juniors - A Mixed (George &amp; George)</t>
         </is>
       </c>
       <c r="L631" s="12" t="inlineStr">
         <is>
-          <t>Mooroolbark SC U15 Juniors - A Mixed Mooroolbark SC - Under 15 John</t>
+          <t>Knox City FC U13 Juniors - A Mixed U13A</t>
         </is>
       </c>
       <c r="M631" s="12" t="inlineStr">
@@ -48618,7 +48630,7 @@
       </c>
       <c r="N631" s="11" t="inlineStr">
         <is>
-          <t>Mixed East 15A</t>
+          <t>Mixed Sunday East 13A</t>
         </is>
       </c>
       <c r="O631" s="11" t="inlineStr">
@@ -48642,12 +48654,12 @@
       </c>
       <c r="C632" s="9" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="D632" s="9" t="inlineStr">
         <is>
-          <t>16:25</t>
+          <t>14:40</t>
         </is>
       </c>
       <c r="E632" s="9" t="n">
@@ -48675,27 +48687,27 @@
       </c>
       <c r="J632" s="9" t="inlineStr">
         <is>
-          <t>U18</t>
+          <t>U15</t>
         </is>
       </c>
       <c r="K632" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U18 Juniors - A Male</t>
+          <t>Manningham United Blues FC U15 Juniors - A Mixed</t>
         </is>
       </c>
       <c r="L632" s="10" t="inlineStr">
         <is>
-          <t>Collingwood City FC U18 Juniors - A Male 18A</t>
+          <t>Mooroolbark SC U15 Juniors - A Mixed Mooroolbark SC - Under 15 John</t>
         </is>
       </c>
       <c r="M632" s="10" t="inlineStr">
         <is>
-          <t>Junior Boys Sunday (U17 - U18)</t>
+          <t>Junior Mixed Sunday (U12 - U16)</t>
         </is>
       </c>
       <c r="N632" s="9" t="inlineStr">
         <is>
-          <t>Boys North-East 18A</t>
+          <t>Mixed East 15A</t>
         </is>
       </c>
       <c r="O632" s="9" t="inlineStr">
@@ -48719,16 +48731,16 @@
       </c>
       <c r="C633" s="11" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>15:15</t>
         </is>
       </c>
       <c r="D633" s="11" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>16:25</t>
         </is>
       </c>
       <c r="E633" s="11" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F633" s="11" t="inlineStr">
         <is>
@@ -48737,42 +48749,42 @@
       </c>
       <c r="G633" s="11" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H633" s="11" t="inlineStr">
         <is>
-          <t>Sub</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="I633" s="12" t="inlineStr">
         <is>
-          <t>Pitch 2A</t>
+          <t>Pitch 1</t>
         </is>
       </c>
       <c r="J633" s="11" t="inlineStr">
         <is>
-          <t>U12</t>
+          <t>U18</t>
         </is>
       </c>
       <c r="K633" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - A Mixed (Hamid)</t>
+          <t>Manningham United Blues FC U18 Juniors - A Male</t>
         </is>
       </c>
       <c r="L633" s="12" t="inlineStr">
         <is>
-          <t>Nunawading City FC U12 Juniors - A Mixed</t>
+          <t>Collingwood City FC U18 Juniors - A Male 18A</t>
         </is>
       </c>
       <c r="M633" s="12" t="inlineStr">
         <is>
-          <t>Junior Mixed Sunday (U12 - U16)</t>
+          <t>Junior Boys Sunday (U17 - U18)</t>
         </is>
       </c>
       <c r="N633" s="11" t="inlineStr">
         <is>
-          <t>Mixed Sunday East 12A Blue</t>
+          <t>Boys North-East 18A</t>
         </is>
       </c>
       <c r="O633" s="11" t="inlineStr">
@@ -48796,12 +48808,12 @@
       </c>
       <c r="C634" s="9" t="inlineStr">
         <is>
-          <t>10:40</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="D634" s="9" t="inlineStr">
         <is>
-          <t>11:40</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="E634" s="9" t="n">
@@ -48814,32 +48826,32 @@
       </c>
       <c r="G634" s="9" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H634" s="9" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Sub</t>
         </is>
       </c>
       <c r="I634" s="10" t="inlineStr">
         <is>
-          <t>Pitch 3</t>
+          <t>Pitch 2A</t>
         </is>
       </c>
       <c r="J634" s="9" t="inlineStr">
         <is>
-          <t>U13</t>
+          <t>U12</t>
         </is>
       </c>
       <c r="K634" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - C Mixed (Martin)</t>
+          <t>Manningham United Blues FC U12 Juniors - A Mixed (Hamid)</t>
         </is>
       </c>
       <c r="L634" s="10" t="inlineStr">
         <is>
-          <t>Malvern City FC U13 Juniors - C Mixed U13 Anthony - C</t>
+          <t>Nunawading City FC U12 Juniors - A Mixed</t>
         </is>
       </c>
       <c r="M634" s="10" t="inlineStr">
@@ -48849,7 +48861,7 @@
       </c>
       <c r="N634" s="9" t="inlineStr">
         <is>
-          <t>Mixed Sunday East 13C Red</t>
+          <t>Mixed Sunday East 12A Blue</t>
         </is>
       </c>
       <c r="O634" s="9" t="inlineStr">
@@ -48858,11 +48870,7 @@
         </is>
       </c>
       <c r="P634" s="9" t="inlineStr"/>
-      <c r="Q634" s="10" t="inlineStr">
-        <is>
-          <t>Powerful Owl Park Pitch 1B</t>
-        </is>
-      </c>
+      <c r="Q634" s="10" t="inlineStr"/>
     </row>
     <row r="635">
       <c r="A635" s="11" t="inlineStr">
@@ -49262,16 +49270,16 @@
       </c>
       <c r="C640" s="9" t="inlineStr">
         <is>
-          <t>12:10</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D640" s="9" t="inlineStr">
         <is>
-          <t>13:10</t>
+          <t>15:10</t>
         </is>
       </c>
       <c r="E640" s="9" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F640" s="9" t="inlineStr">
         <is>
@@ -49285,37 +49293,37 @@
       </c>
       <c r="H640" s="9" t="inlineStr">
         <is>
-          <t>Sub</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="I640" s="10" t="inlineStr">
         <is>
-          <t>Pitch 1 - Midi Field B</t>
+          <t>Pitch 1</t>
         </is>
       </c>
       <c r="J640" s="9" t="inlineStr">
         <is>
-          <t>U13</t>
+          <t>U16</t>
         </is>
       </c>
       <c r="K640" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - B Mixed (Samir)</t>
+          <t>Manningham United Blues FC U16 Juniors - B Female (Eden)</t>
         </is>
       </c>
       <c r="L640" s="10" t="inlineStr">
         <is>
-          <t>Mazenod FC U13 Juniors - B Mixed</t>
+          <t>Glen Eira FC AAL - Junior Juniors - B Female Glen Eira FC - Van Egmonds</t>
         </is>
       </c>
       <c r="M640" s="10" t="inlineStr">
         <is>
-          <t>Junior Mixed Sunday (U12 - U16)</t>
+          <t>Junior Girls Sunday (U12 - U18)</t>
         </is>
       </c>
       <c r="N640" s="9" t="inlineStr">
         <is>
-          <t>Mixed Sunday East 13B</t>
+          <t>Girls' South-East 16B</t>
         </is>
       </c>
       <c r="O640" s="9" t="inlineStr">
@@ -49339,16 +49347,16 @@
       </c>
       <c r="C641" s="11" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>09:45</t>
         </is>
       </c>
       <c r="D641" s="11" t="inlineStr">
         <is>
-          <t>15:10</t>
+          <t>10:45</t>
         </is>
       </c>
       <c r="E641" s="11" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="F641" s="11" t="inlineStr">
         <is>
@@ -49357,7 +49365,7 @@
       </c>
       <c r="G641" s="11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H641" s="11" t="inlineStr">
@@ -49367,32 +49375,32 @@
       </c>
       <c r="I641" s="12" t="inlineStr">
         <is>
-          <t>Pitch 1</t>
+          <t>Pitch 2</t>
         </is>
       </c>
       <c r="J641" s="11" t="inlineStr">
         <is>
-          <t>U16</t>
+          <t>U14</t>
         </is>
       </c>
       <c r="K641" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U16 Juniors - B Female (Eden)</t>
+          <t>Manningham United Blues FC U14 Juniors - A Mixed</t>
         </is>
       </c>
       <c r="L641" s="12" t="inlineStr">
         <is>
-          <t>Glen Eira FC AAL - Junior Juniors - B Female Glen Eira FC - Van Egmonds</t>
+          <t>Boronia SC U14 Juniors - A Mixed Tristan</t>
         </is>
       </c>
       <c r="M641" s="12" t="inlineStr">
         <is>
-          <t>Junior Girls Sunday (U12 - U18)</t>
+          <t>Junior Mixed Sunday (U12 - U16)</t>
         </is>
       </c>
       <c r="N641" s="11" t="inlineStr">
         <is>
-          <t>Girls' South-East 16B</t>
+          <t>Mixed East 14A</t>
         </is>
       </c>
       <c r="O641" s="11" t="inlineStr">
@@ -49416,12 +49424,12 @@
       </c>
       <c r="C642" s="9" t="inlineStr">
         <is>
-          <t>09:45</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="D642" s="9" t="inlineStr">
         <is>
-          <t>10:45</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="E642" s="9" t="n">
@@ -49454,22 +49462,22 @@
       </c>
       <c r="K642" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - A Mixed</t>
+          <t>Manningham United Blues FC U14 Juniors - C Female (Christian)</t>
         </is>
       </c>
       <c r="L642" s="10" t="inlineStr">
         <is>
-          <t>Boronia SC U14 Juniors - A Mixed Tristan</t>
+          <t>Ashburton United SC U14 Juniors - C Female</t>
         </is>
       </c>
       <c r="M642" s="10" t="inlineStr">
         <is>
-          <t>Junior Mixed Sunday (U12 - U16)</t>
+          <t>Junior Girls Sunday (U12 - U18)</t>
         </is>
       </c>
       <c r="N642" s="9" t="inlineStr">
         <is>
-          <t>Mixed East 14A</t>
+          <t>Girls' South-East 14C</t>
         </is>
       </c>
       <c r="O642" s="9" t="inlineStr">
@@ -49493,12 +49501,12 @@
       </c>
       <c r="C643" s="11" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>13:15</t>
         </is>
       </c>
       <c r="D643" s="11" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>14:15</t>
         </is>
       </c>
       <c r="E643" s="11" t="n">
@@ -49531,22 +49539,22 @@
       </c>
       <c r="K643" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - C Female (Christian)</t>
+          <t>Manningham United Blues FC U14 Juniors - C Mixed (Phil)</t>
         </is>
       </c>
       <c r="L643" s="12" t="inlineStr">
         <is>
-          <t>Ashburton United SC U14 Juniors - C Female</t>
+          <t>Mazenod FC U14 Juniors - C Mixed</t>
         </is>
       </c>
       <c r="M643" s="12" t="inlineStr">
         <is>
-          <t>Junior Girls Sunday (U12 - U18)</t>
+          <t>Junior Mixed Sunday (U12 - U16)</t>
         </is>
       </c>
       <c r="N643" s="11" t="inlineStr">
         <is>
-          <t>Girls' South-East 14C</t>
+          <t>Mixed East 14C Red</t>
         </is>
       </c>
       <c r="O643" s="11" t="inlineStr">
@@ -49570,16 +49578,16 @@
       </c>
       <c r="C644" s="9" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="D644" s="9" t="inlineStr">
         <is>
-          <t>14:15</t>
+          <t>16:10</t>
         </is>
       </c>
       <c r="E644" s="9" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F644" s="9" t="inlineStr">
         <is>
@@ -49603,17 +49611,17 @@
       </c>
       <c r="J644" s="9" t="inlineStr">
         <is>
-          <t>U14</t>
+          <t>U15</t>
         </is>
       </c>
       <c r="K644" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - C Mixed (Phil)</t>
+          <t>Manningham United Blues FC U15 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="L644" s="10" t="inlineStr">
         <is>
-          <t>Mazenod FC U14 Juniors - C Mixed</t>
+          <t>Bunyip &amp; District SC U15 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="M644" s="10" t="inlineStr">
@@ -49623,7 +49631,7 @@
       </c>
       <c r="N644" s="9" t="inlineStr">
         <is>
-          <t>Mixed East 14C Red</t>
+          <t>Mixed South-East 15B</t>
         </is>
       </c>
       <c r="O644" s="9" t="inlineStr">
@@ -49635,158 +49643,170 @@
       <c r="Q644" s="10" t="inlineStr"/>
     </row>
     <row r="645">
-      <c r="A645" s="11" t="inlineStr">
+      <c r="A645" s="13" t="inlineStr">
         <is>
           <t>23 Aug 2026</t>
         </is>
       </c>
-      <c r="B645" s="11" t="inlineStr">
+      <c r="B645" s="13" t="inlineStr">
         <is>
           <t>Sun</t>
         </is>
       </c>
-      <c r="C645" s="11" t="inlineStr">
-        <is>
-          <t>15:00</t>
-        </is>
-      </c>
-      <c r="D645" s="11" t="inlineStr">
-        <is>
-          <t>16:10</t>
-        </is>
-      </c>
-      <c r="E645" s="11" t="n">
+      <c r="C645" s="13" t="inlineStr">
+        <is>
+          <t>12:10</t>
+        </is>
+      </c>
+      <c r="D645" s="13" t="inlineStr">
+        <is>
+          <t>13:10</t>
+        </is>
+      </c>
+      <c r="E645" s="13" t="n">
+        <v>60</v>
+      </c>
+      <c r="F645" s="13" t="inlineStr">
+        <is>
+          <t>Powerful Owl Park</t>
+        </is>
+      </c>
+      <c r="G645" s="13" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H645" s="13" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="I645" s="14" t="inlineStr">
+        <is>
+          <t>Pitch 3</t>
+        </is>
+      </c>
+      <c r="J645" s="13" t="inlineStr">
+        <is>
+          <t>U13</t>
+        </is>
+      </c>
+      <c r="K645" s="14" t="inlineStr">
+        <is>
+          <t>Manningham United Blues FC U13 Juniors - B Mixed (Samir)</t>
+        </is>
+      </c>
+      <c r="L645" s="14" t="inlineStr">
+        <is>
+          <t>Mazenod FC U13 Juniors - B Mixed</t>
+        </is>
+      </c>
+      <c r="M645" s="14" t="inlineStr">
+        <is>
+          <t>Junior Mixed Sunday (U12 - U16)</t>
+        </is>
+      </c>
+      <c r="N645" s="13" t="inlineStr">
+        <is>
+          <t>Mixed Sunday East 13B</t>
+        </is>
+      </c>
+      <c r="O645" s="13" t="inlineStr">
+        <is>
+          <t>R16</t>
+        </is>
+      </c>
+      <c r="P645" s="15" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Q645" s="14" t="inlineStr">
+        <is>
+          <t>Powerful Owl Park Pitch 1 - Midi Field B</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" s="13" t="inlineStr">
+        <is>
+          <t>23 Aug 2026</t>
+        </is>
+      </c>
+      <c r="B646" s="13" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
+      <c r="C646" s="13" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="D646" s="13" t="inlineStr">
+        <is>
+          <t>14:10</t>
+        </is>
+      </c>
+      <c r="E646" s="13" t="n">
         <v>70</v>
       </c>
-      <c r="F645" s="11" t="inlineStr">
+      <c r="F646" s="13" t="inlineStr">
         <is>
           <t>Powerful Owl Park</t>
         </is>
       </c>
-      <c r="G645" s="11" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="H645" s="11" t="inlineStr">
+      <c r="G646" s="13" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H646" s="13" t="inlineStr">
         <is>
           <t>Full</t>
         </is>
       </c>
-      <c r="I645" s="12" t="inlineStr">
-        <is>
-          <t>Pitch 2</t>
-        </is>
-      </c>
-      <c r="J645" s="11" t="inlineStr">
-        <is>
-          <t>U15</t>
-        </is>
-      </c>
-      <c r="K645" s="12" t="inlineStr">
-        <is>
-          <t>Manningham United Blues FC U15 Juniors - B Mixed</t>
-        </is>
-      </c>
-      <c r="L645" s="12" t="inlineStr">
-        <is>
-          <t>Bunyip &amp; District SC U15 Juniors - B Mixed</t>
-        </is>
-      </c>
-      <c r="M645" s="12" t="inlineStr">
-        <is>
-          <t>Junior Mixed Sunday (U12 - U16)</t>
-        </is>
-      </c>
-      <c r="N645" s="11" t="inlineStr">
-        <is>
-          <t>Mixed South-East 15B</t>
-        </is>
-      </c>
-      <c r="O645" s="11" t="inlineStr">
+      <c r="I646" s="14" t="inlineStr">
+        <is>
+          <t>Pitch 3</t>
+        </is>
+      </c>
+      <c r="J646" s="13" t="inlineStr">
+        <is>
+          <t>U18</t>
+        </is>
+      </c>
+      <c r="K646" s="14" t="inlineStr">
+        <is>
+          <t>Manningham United Blues FC U18 Juniors - A Male</t>
+        </is>
+      </c>
+      <c r="L646" s="14" t="inlineStr">
+        <is>
+          <t>West Preston SC U18 Juniors - A Male West Preston U/18A</t>
+        </is>
+      </c>
+      <c r="M646" s="14" t="inlineStr">
+        <is>
+          <t>Junior Boys Sunday (U17 - U18)</t>
+        </is>
+      </c>
+      <c r="N646" s="13" t="inlineStr">
+        <is>
+          <t>Boys North-East 18A</t>
+        </is>
+      </c>
+      <c r="O646" s="13" t="inlineStr">
         <is>
           <t>R16</t>
         </is>
       </c>
-      <c r="P645" s="11" t="inlineStr"/>
-      <c r="Q645" s="12" t="inlineStr"/>
-    </row>
-    <row r="646">
-      <c r="A646" s="9" t="inlineStr">
-        <is>
-          <t>23 Aug 2026</t>
-        </is>
-      </c>
-      <c r="B646" s="9" t="inlineStr">
-        <is>
-          <t>Sun</t>
-        </is>
-      </c>
-      <c r="C646" s="9" t="inlineStr">
-        <is>
-          <t>13:00</t>
-        </is>
-      </c>
-      <c r="D646" s="9" t="inlineStr">
-        <is>
-          <t>14:10</t>
-        </is>
-      </c>
-      <c r="E646" s="9" t="n">
-        <v>70</v>
-      </c>
-      <c r="F646" s="9" t="inlineStr">
-        <is>
-          <t>Powerful Owl Park</t>
-        </is>
-      </c>
-      <c r="G646" s="9" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="H646" s="9" t="inlineStr">
-        <is>
-          <t>Full</t>
-        </is>
-      </c>
-      <c r="I646" s="10" t="inlineStr">
-        <is>
-          <t>Pitch 3</t>
-        </is>
-      </c>
-      <c r="J646" s="9" t="inlineStr">
-        <is>
-          <t>U18</t>
-        </is>
-      </c>
-      <c r="K646" s="10" t="inlineStr">
-        <is>
-          <t>Manningham United Blues FC U18 Juniors - A Male</t>
-        </is>
-      </c>
-      <c r="L646" s="10" t="inlineStr">
-        <is>
-          <t>West Preston SC U18 Juniors - A Male West Preston U/18A</t>
-        </is>
-      </c>
-      <c r="M646" s="10" t="inlineStr">
-        <is>
-          <t>Junior Boys Sunday (U17 - U18)</t>
-        </is>
-      </c>
-      <c r="N646" s="9" t="inlineStr">
-        <is>
-          <t>Boys North-East 18A</t>
-        </is>
-      </c>
-      <c r="O646" s="9" t="inlineStr">
-        <is>
-          <t>R16</t>
-        </is>
-      </c>
-      <c r="P646" s="9" t="inlineStr"/>
-      <c r="Q646" s="10" t="inlineStr"/>
+      <c r="P646" s="15" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Q646" s="14" t="inlineStr"/>
     </row>
     <row r="647">
       <c r="A647" s="11" t="inlineStr">
@@ -50345,11 +50365,11 @@
       </c>
       <c r="D654" s="9" t="inlineStr">
         <is>
-          <t>12:10</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="E654" s="9" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="F654" s="9" t="inlineStr">
         <is>
@@ -50368,32 +50388,32 @@
       </c>
       <c r="I654" s="10" t="inlineStr">
         <is>
-          <t>Pitch 1 - Midi Field B</t>
+          <t>Pitch 1B</t>
         </is>
       </c>
       <c r="J654" s="9" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>U13</t>
         </is>
       </c>
       <c r="K654" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Female Miniroos Girls U11W (Holly &amp; Marina)</t>
+          <t>Manningham United Blues FC U13 Juniors - C Mixed (Martin)</t>
         </is>
       </c>
       <c r="L654" s="10" t="inlineStr">
         <is>
-          <t>Malvern City FC U11 MiniRoos - Wallabies Female U11 MCFC Girls</t>
+          <t>Whitehorse United SC U13 Juniors - C Mixed Shane</t>
         </is>
       </c>
       <c r="M654" s="10" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Girls' Sunday (U6 - U11)</t>
+          <t>Junior Mixed Sunday (U12 - U16)</t>
         </is>
       </c>
       <c r="N654" s="9" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Girls' East 11 Wallabies</t>
+          <t>Mixed Sunday East 13C Red</t>
         </is>
       </c>
       <c r="O654" s="9" t="inlineStr">
@@ -50417,16 +50437,16 @@
       </c>
       <c r="C655" s="11" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="D655" s="11" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>12:10</t>
         </is>
       </c>
       <c r="E655" s="11" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="F655" s="11" t="inlineStr">
         <is>
@@ -50440,37 +50460,37 @@
       </c>
       <c r="H655" s="11" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Sub</t>
         </is>
       </c>
       <c r="I655" s="12" t="inlineStr">
         <is>
-          <t>Pitch 1</t>
+          <t>Pitch 1 - Midi Field B</t>
         </is>
       </c>
       <c r="J655" s="11" t="inlineStr">
         <is>
-          <t>U14</t>
+          <t>U11</t>
         </is>
       </c>
       <c r="K655" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - A Female (Chloe)</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Female Miniroos Girls U11W (Holly &amp; Marina)</t>
         </is>
       </c>
       <c r="L655" s="12" t="inlineStr">
         <is>
-          <t>Alamein FC U14 Juniors - A Female</t>
+          <t>Malvern City FC U11 MiniRoos - Wallabies Female U11 MCFC Girls</t>
         </is>
       </c>
       <c r="M655" s="12" t="inlineStr">
         <is>
-          <t>Junior Girls Sunday (U12 - U18)</t>
+          <t>Coles MiniRoos Girls' Sunday (U6 - U11)</t>
         </is>
       </c>
       <c r="N655" s="11" t="inlineStr">
         <is>
-          <t>Girls' South-East 14A</t>
+          <t>Coles MiniRoos Girls' East 11 Wallabies</t>
         </is>
       </c>
       <c r="O655" s="11" t="inlineStr">
@@ -50494,16 +50514,16 @@
       </c>
       <c r="C656" s="9" t="inlineStr">
         <is>
-          <t>14:45</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="D656" s="9" t="inlineStr">
         <is>
-          <t>15:55</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="E656" s="9" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="F656" s="9" t="inlineStr">
         <is>
@@ -50527,17 +50547,17 @@
       </c>
       <c r="J656" s="9" t="inlineStr">
         <is>
-          <t>U17/18</t>
+          <t>U14</t>
         </is>
       </c>
       <c r="K656" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U17/18 Juniors - B Female (Marilyn)</t>
+          <t>Manningham United Blues FC U14 Juniors - A Female (Chloe)</t>
         </is>
       </c>
       <c r="L656" s="10" t="inlineStr">
         <is>
-          <t>Mount Eliza SC U17/18 Juniors - B Female Red</t>
+          <t>Alamein FC U14 Juniors - A Female</t>
         </is>
       </c>
       <c r="M656" s="10" t="inlineStr">
@@ -50547,7 +50567,7 @@
       </c>
       <c r="N656" s="9" t="inlineStr">
         <is>
-          <t>Girls' South-East 17/18B</t>
+          <t>Girls' South-East 14A</t>
         </is>
       </c>
       <c r="O656" s="9" t="inlineStr">
@@ -50571,16 +50591,16 @@
       </c>
       <c r="C657" s="11" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>14:45</t>
         </is>
       </c>
       <c r="D657" s="11" t="inlineStr">
         <is>
-          <t>09:40</t>
+          <t>15:55</t>
         </is>
       </c>
       <c r="E657" s="11" t="n">
-        <v>40</v>
+        <v>70</v>
       </c>
       <c r="F657" s="11" t="inlineStr">
         <is>
@@ -50589,42 +50609,42 @@
       </c>
       <c r="G657" s="11" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H657" s="11" t="inlineStr">
         <is>
-          <t>Sub</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="I657" s="12" t="inlineStr">
         <is>
-          <t>Pitch 2A</t>
+          <t>Pitch 1</t>
         </is>
       </c>
       <c r="J657" s="11" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>U17/18</t>
         </is>
       </c>
       <c r="K657" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Kangaroos Mixed</t>
+          <t>Manningham United Blues FC U17/18 Juniors - B Female (Marilyn)</t>
         </is>
       </c>
       <c r="L657" s="12" t="inlineStr">
         <is>
-          <t>FC Bulleen Lions U11 MiniRoos - Kangaroos Mixed Anthony &amp; Rob</t>
+          <t>Mount Eliza SC U17/18 Juniors - B Female Red</t>
         </is>
       </c>
       <c r="M657" s="12" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Sunday (U6 - U11)</t>
+          <t>Junior Girls Sunday (U12 - U18)</t>
         </is>
       </c>
       <c r="N657" s="11" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Sunday East 11 Kangaroos Red</t>
+          <t>Girls' South-East 17/18B</t>
         </is>
       </c>
       <c r="O657" s="11" t="inlineStr">
@@ -50676,22 +50696,22 @@
       </c>
       <c r="I658" s="10" t="inlineStr">
         <is>
-          <t>Pitch 2 - Midi B</t>
+          <t>Pitch 2A</t>
         </is>
       </c>
       <c r="J658" s="9" t="inlineStr">
         <is>
-          <t>U07</t>
+          <t>U11</t>
         </is>
       </c>
       <c r="K658" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Red)</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Kangaroos Mixed</t>
         </is>
       </c>
       <c r="L658" s="10" t="inlineStr">
         <is>
-          <t>East Malvern Junior SC U07 MiniRoos - Joeys Mixed EMJSC U7 Sunday Orange</t>
+          <t>FC Bulleen Lions U11 MiniRoos - Kangaroos Mixed Anthony &amp; Rob</t>
         </is>
       </c>
       <c r="M658" s="10" t="inlineStr">
@@ -50701,7 +50721,7 @@
       </c>
       <c r="N658" s="9" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Sunday East 7 Joeys Red</t>
+          <t>Coles MiniRoos Mixed Sunday East 11 Kangaroos Red</t>
         </is>
       </c>
       <c r="O658" s="9" t="inlineStr">
@@ -50753,7 +50773,7 @@
       </c>
       <c r="I659" s="12" t="inlineStr">
         <is>
-          <t>Pitch 2 - Midi A</t>
+          <t>Pitch 2 - Midi B</t>
         </is>
       </c>
       <c r="J659" s="11" t="inlineStr">
@@ -50763,12 +50783,12 @@
       </c>
       <c r="K659" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Green)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Red)</t>
         </is>
       </c>
       <c r="L659" s="12" t="inlineStr">
         <is>
-          <t>Doncaster Rovers SC U07 MiniRoos - Joeys Mixed</t>
+          <t>East Malvern Junior SC U07 MiniRoos - Joeys Mixed EMJSC U7 Sunday Orange</t>
         </is>
       </c>
       <c r="M659" s="12" t="inlineStr">
@@ -50802,16 +50822,16 @@
       </c>
       <c r="C660" s="9" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="D660" s="9" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>09:40</t>
         </is>
       </c>
       <c r="E660" s="9" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="F660" s="9" t="inlineStr">
         <is>
@@ -50830,32 +50850,32 @@
       </c>
       <c r="I660" s="10" t="inlineStr">
         <is>
-          <t>Pitch 2A</t>
+          <t>Pitch 2 - Midi A</t>
         </is>
       </c>
       <c r="J660" s="9" t="inlineStr">
         <is>
-          <t>U12</t>
+          <t>U07</t>
         </is>
       </c>
       <c r="K660" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - A Female (Sienna)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Green)</t>
         </is>
       </c>
       <c r="L660" s="10" t="inlineStr">
         <is>
-          <t>Alamein FC U12 Juniors - A Female</t>
+          <t>Doncaster Rovers SC U07 MiniRoos - Joeys Mixed</t>
         </is>
       </c>
       <c r="M660" s="10" t="inlineStr">
         <is>
-          <t>Junior Girls Sunday (U12 - U18)</t>
+          <t>Coles MiniRoos Mixed Sunday (U6 - U11)</t>
         </is>
       </c>
       <c r="N660" s="9" t="inlineStr">
         <is>
-          <t>Girls' South-East 12A</t>
+          <t>Coles MiniRoos Mixed Sunday East 7 Joeys Red</t>
         </is>
       </c>
       <c r="O660" s="9" t="inlineStr">
@@ -50879,12 +50899,12 @@
       </c>
       <c r="C661" s="11" t="inlineStr">
         <is>
-          <t>11:45</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="D661" s="11" t="inlineStr">
         <is>
-          <t>12:45</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="E661" s="11" t="n">
@@ -50902,37 +50922,37 @@
       </c>
       <c r="H661" s="11" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Sub</t>
         </is>
       </c>
       <c r="I661" s="12" t="inlineStr">
         <is>
-          <t>Pitch 2</t>
+          <t>Pitch 2A</t>
         </is>
       </c>
       <c r="J661" s="11" t="inlineStr">
         <is>
-          <t>U14</t>
+          <t>U12</t>
         </is>
       </c>
       <c r="K661" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - B Mixed</t>
+          <t>Manningham United Blues FC U12 Juniors - A Female (Sienna)</t>
         </is>
       </c>
       <c r="L661" s="12" t="inlineStr">
         <is>
-          <t>Malvern City FC U14 Juniors - B Mixed U14 - B</t>
+          <t>Alamein FC U12 Juniors - A Female</t>
         </is>
       </c>
       <c r="M661" s="12" t="inlineStr">
         <is>
-          <t>Junior Mixed Sunday (U12 - U16)</t>
+          <t>Junior Girls Sunday (U12 - U18)</t>
         </is>
       </c>
       <c r="N661" s="11" t="inlineStr">
         <is>
-          <t>Mixed East 14B</t>
+          <t>Girls' South-East 12A</t>
         </is>
       </c>
       <c r="O661" s="11" t="inlineStr">
@@ -50956,16 +50976,16 @@
       </c>
       <c r="C662" s="9" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="D662" s="9" t="inlineStr">
         <is>
-          <t>14:25</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="E662" s="9" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="F662" s="9" t="inlineStr">
         <is>
@@ -50979,27 +50999,27 @@
       </c>
       <c r="H662" s="9" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Sub</t>
         </is>
       </c>
       <c r="I662" s="10" t="inlineStr">
         <is>
-          <t>Pitch 2</t>
+          <t>Pitch 2B</t>
         </is>
       </c>
       <c r="J662" s="9" t="inlineStr">
         <is>
-          <t>U15</t>
+          <t>U13</t>
         </is>
       </c>
       <c r="K662" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U15 Juniors - B Female (Ethan)</t>
+          <t>Manningham United Blues FC U13 Juniors - C Female (Abigail)</t>
         </is>
       </c>
       <c r="L662" s="10" t="inlineStr">
         <is>
-          <t>Brighton SC U15 Juniors - B Female Apollos</t>
+          <t>Hampton East Brighton FC U13 Juniors - C Female u13 girls</t>
         </is>
       </c>
       <c r="M662" s="10" t="inlineStr">
@@ -51009,7 +51029,7 @@
       </c>
       <c r="N662" s="9" t="inlineStr">
         <is>
-          <t>Girls' South-East 15B</t>
+          <t>Girls' South-East 13C</t>
         </is>
       </c>
       <c r="O662" s="9" t="inlineStr">
@@ -51033,16 +51053,16 @@
       </c>
       <c r="C663" s="11" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>11:45</t>
         </is>
       </c>
       <c r="D663" s="11" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>12:45</t>
         </is>
       </c>
       <c r="E663" s="11" t="n">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="F663" s="11" t="inlineStr">
         <is>
@@ -51066,27 +51086,27 @@
       </c>
       <c r="J663" s="11" t="inlineStr">
         <is>
-          <t>Seniors</t>
+          <t>U14</t>
         </is>
       </c>
       <c r="K663" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC Seniors</t>
+          <t>Manningham United Blues FC U14 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="L663" s="12" t="inlineStr">
         <is>
-          <t>Mount Martha SC Seniors</t>
+          <t>Malvern City FC U14 Juniors - B Mixed U14 - B</t>
         </is>
       </c>
       <c r="M663" s="12" t="inlineStr">
         <is>
-          <t>VETO Sports State League Women's</t>
+          <t>Junior Mixed Sunday (U12 - U16)</t>
         </is>
       </c>
       <c r="N663" s="11" t="inlineStr">
         <is>
-          <t>State League 6 Women's - South-East</t>
+          <t>Mixed East 14B</t>
         </is>
       </c>
       <c r="O663" s="11" t="inlineStr">
@@ -51110,16 +51130,16 @@
       </c>
       <c r="C664" s="9" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>13:15</t>
         </is>
       </c>
       <c r="D664" s="9" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>14:25</t>
         </is>
       </c>
       <c r="E664" s="9" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F664" s="9" t="inlineStr">
         <is>
@@ -51128,7 +51148,7 @@
       </c>
       <c r="G664" s="9" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H664" s="9" t="inlineStr">
@@ -51138,22 +51158,22 @@
       </c>
       <c r="I664" s="10" t="inlineStr">
         <is>
-          <t>Pitch 3</t>
+          <t>Pitch 2</t>
         </is>
       </c>
       <c r="J664" s="9" t="inlineStr">
         <is>
-          <t>U13</t>
+          <t>U15</t>
         </is>
       </c>
       <c r="K664" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - C Female (Abigail)</t>
+          <t>Manningham United Blues FC U15 Juniors - B Female (Ethan)</t>
         </is>
       </c>
       <c r="L664" s="10" t="inlineStr">
         <is>
-          <t>Hampton East Brighton FC U13 Juniors - C Female u13 girls</t>
+          <t>Brighton SC U15 Juniors - B Female Apollos</t>
         </is>
       </c>
       <c r="M664" s="10" t="inlineStr">
@@ -51163,7 +51183,7 @@
       </c>
       <c r="N664" s="9" t="inlineStr">
         <is>
-          <t>Girls' South-East 13C</t>
+          <t>Girls' South-East 15B</t>
         </is>
       </c>
       <c r="O664" s="9" t="inlineStr">
@@ -51172,11 +51192,7 @@
         </is>
       </c>
       <c r="P664" s="9" t="inlineStr"/>
-      <c r="Q664" s="10" t="inlineStr">
-        <is>
-          <t>Powerful Owl Park Pitch 2B</t>
-        </is>
-      </c>
+      <c r="Q664" s="10" t="inlineStr"/>
     </row>
     <row r="665">
       <c r="A665" s="11" t="inlineStr">
@@ -51191,16 +51207,16 @@
       </c>
       <c r="C665" s="11" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="D665" s="11" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="E665" s="11" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F665" s="11" t="inlineStr">
         <is>
@@ -51209,7 +51225,7 @@
       </c>
       <c r="G665" s="11" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H665" s="11" t="inlineStr">
@@ -51219,32 +51235,32 @@
       </c>
       <c r="I665" s="12" t="inlineStr">
         <is>
-          <t>Pitch 3</t>
+          <t>Pitch 2</t>
         </is>
       </c>
       <c r="J665" s="11" t="inlineStr">
         <is>
-          <t>U13</t>
+          <t>Seniors</t>
         </is>
       </c>
       <c r="K665" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - C Mixed (Martin)</t>
+          <t>Manningham United Blues FC Seniors</t>
         </is>
       </c>
       <c r="L665" s="12" t="inlineStr">
         <is>
-          <t>Whitehorse United SC U13 Juniors - C Mixed Shane</t>
+          <t>Mount Martha SC Seniors</t>
         </is>
       </c>
       <c r="M665" s="12" t="inlineStr">
         <is>
-          <t>Junior Mixed Sunday (U12 - U16)</t>
+          <t>VETO Sports State League Women's</t>
         </is>
       </c>
       <c r="N665" s="11" t="inlineStr">
         <is>
-          <t>Mixed Sunday East 13C Red</t>
+          <t>State League 6 Women's - South-East</t>
         </is>
       </c>
       <c r="O665" s="11" t="inlineStr">
@@ -51253,11 +51269,7 @@
         </is>
       </c>
       <c r="P665" s="11" t="inlineStr"/>
-      <c r="Q665" s="12" t="inlineStr">
-        <is>
-          <t>Powerful Owl Park Pitch 1B</t>
-        </is>
-      </c>
+      <c r="Q665" s="12" t="inlineStr"/>
     </row>
     <row r="666">
       <c r="A666" s="9" t="inlineStr">
@@ -53354,7 +53366,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -53406,7 +53418,7 @@
     <row r="7">
       <c r="A7" s="17" t="inlineStr">
         <is>
-          <t>A.  Over-capacity moments: 7 found</t>
+          <t>A.  Over-capacity moments: 10 found</t>
         </is>
       </c>
     </row>
@@ -53772,130 +53784,265 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="20" t="n">
+        <v>8</v>
+      </c>
+      <c r="B16" s="20" t="inlineStr">
+        <is>
+          <t>08 Aug 2026</t>
+        </is>
+      </c>
+      <c r="C16" s="20" t="inlineStr">
+        <is>
+          <t>Pettys Reserve</t>
+        </is>
+      </c>
+      <c r="D16" s="20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E16" s="21" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="F16" s="20" t="inlineStr">
+        <is>
+          <t>09:10</t>
+        </is>
+      </c>
+      <c r="G16" s="21" t="inlineStr">
+        <is>
+          <t>Pitch over capacity</t>
+        </is>
+      </c>
+      <c r="H16" s="20" t="inlineStr">
+        <is>
+          <t>2×U10-13, 1×U8/9 = 1.25</t>
+        </is>
+      </c>
+      <c r="I16" s="20" t="inlineStr">
+        <is>
+          <t>08:30 U11 Pitch 1B (Bottom Field) (Manningham United Blues FC U11 MiniRoos - Wallabies Mixed (Culina's) v Whitehorse United SC U11 MiniRoos - Wallabies Mixed Vanntha)  |  08:30 U12 Pitch 1A (Bottom Field) (Manningham United Blues FC U12 Juniors - B Mixed (Chris) v Nunawading City FC U12 Juniors - B Mixed)  |  09:00 U08 Pitch 1C (Bottom Field) - Quarter Pitch 7v7 (Manningham United Blues FC U08 MiniRoos - Joeys Mixed (Duke's) v Manningham United Blues FC U08 MiniRoos - Joeys Mixed (Slater's))</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="18" t="n">
+        <v>9</v>
+      </c>
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>15 Aug 2026</t>
+        </is>
+      </c>
+      <c r="C17" s="18" t="inlineStr">
+        <is>
+          <t>Pettys Reserve</t>
+        </is>
+      </c>
+      <c r="D17" s="18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E17" s="19" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="F17" s="18" t="inlineStr">
+        <is>
+          <t>09:10</t>
+        </is>
+      </c>
+      <c r="G17" s="19" t="inlineStr">
+        <is>
+          <t>Pitch over capacity</t>
+        </is>
+      </c>
+      <c r="H17" s="18" t="inlineStr">
+        <is>
+          <t>2×U10-13, 1×U6/7 = 1.25</t>
+        </is>
+      </c>
+      <c r="I17" s="18" t="inlineStr">
+        <is>
+          <t>08:30 U07 Pitch 1E (Bottom Field) - Quarter Pitch 4v4 (Manningham United Blues FC U07 MiniRoos - Joeys Mixed (White) v Oakleigh Cannons FC U07 MiniRoos - Joeys Mixed OCFC Chippa/Jason)  |  08:30 U12 Pitch 1A (Bottom Field) (Manningham United Blues FC U12 Juniors - B Mixed (Andre) v FC Bulleen Lions U12 Juniors - B Mixed)  |  09:00  Pitch 1B (Bottom Field) (Manningham United Blues FC Girls Clinic v [MANUAL ADD])</t>
+        </is>
+      </c>
+    </row>
     <row r="18">
-      <c r="A18" s="22" t="inlineStr">
+      <c r="A18" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="B18" s="20" t="inlineStr">
+        <is>
+          <t>23 Aug 2026</t>
+        </is>
+      </c>
+      <c r="C18" s="20" t="inlineStr">
+        <is>
+          <t>Powerful Owl Park</t>
+        </is>
+      </c>
+      <c r="D18" s="20" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E18" s="21" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="F18" s="20" t="inlineStr">
+        <is>
+          <t>13:10</t>
+        </is>
+      </c>
+      <c r="G18" s="21" t="inlineStr">
+        <is>
+          <t>U14+ must have the pitch to itself</t>
+        </is>
+      </c>
+      <c r="H18" s="20" t="inlineStr">
+        <is>
+          <t>1×U14+, 1×U10-13 = 1.5</t>
+        </is>
+      </c>
+      <c r="I18" s="20" t="inlineStr">
+        <is>
+          <t>12:10 U13 Pitch 3 (Manningham United Blues FC U13 Juniors - B Mixed (Samir) v Mazenod FC U13 Juniors - B Mixed)  |  13:00 U18 Pitch 3 (Manningham United Blues FC U18 Juniors - A Male v West Preston SC U18 Juniors - A Male West Preston U/18A)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="22" t="inlineStr">
         <is>
           <t>B.  Peak simultaneous games per ground (busiest moment)</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>Ground</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>Max at once</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="D22" s="3" t="inlineStr">
         <is>
           <t>From</t>
         </is>
       </c>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="E22" s="3" t="inlineStr">
         <is>
           <t>Until</t>
         </is>
       </c>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="F22" s="3" t="inlineStr">
         <is>
           <t>Pitches in use then</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="21" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="19" t="inlineStr">
         <is>
           <t>Pettys Reserve</t>
         </is>
       </c>
-      <c r="B20" s="20" t="n">
+      <c r="B23" s="18" t="n">
         <v>7</v>
       </c>
-      <c r="C20" s="20" t="inlineStr">
+      <c r="C23" s="18" t="inlineStr">
         <is>
           <t>Sat 16 May 2026</t>
         </is>
       </c>
-      <c r="D20" s="20" t="inlineStr">
+      <c r="D23" s="18" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="E20" s="20" t="inlineStr">
+      <c r="E23" s="18" t="inlineStr">
         <is>
           <t>09:10</t>
         </is>
       </c>
-      <c r="F20" s="21" t="inlineStr">
+      <c r="F23" s="19" t="inlineStr">
         <is>
           <t>Pitch 1A (Bottom Field), Pitch 1B (Bottom Field), Pitch 1E (Bottom Field) - Quarter Pitch 4v4, Pitch 1F (Bottom Field) - Quarter Pitch 4v4, Pitch 2A (Top Field), Pitch 2C (Top Field) - Quarter Pitch 7v7, Pitch 2D (Top Field) - Quarter Pitch 7v7</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="19" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="21" t="inlineStr">
         <is>
           <t>Powerful Owl Park</t>
         </is>
       </c>
-      <c r="B21" s="18" t="n">
+      <c r="B24" s="20" t="n">
         <v>7</v>
       </c>
-      <c r="C21" s="18" t="inlineStr">
+      <c r="C24" s="20" t="inlineStr">
         <is>
           <t>Sun 09 Aug 2026</t>
         </is>
       </c>
-      <c r="D21" s="18" t="inlineStr">
+      <c r="D24" s="20" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="E21" s="18" t="inlineStr">
+      <c r="E24" s="20" t="inlineStr">
         <is>
           <t>09:10</t>
         </is>
       </c>
-      <c r="F21" s="19" t="inlineStr">
+      <c r="F24" s="21" t="inlineStr">
         <is>
           <t>Pitch 1 - Midi Field A, Pitch 1 - Midi Field B, Pitch 1B, Pitch 2A, Pitch 2B, Pitch 3A, Pitch 3B</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="21" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="19" t="inlineStr">
         <is>
           <t>Timber Ridge Reserve</t>
         </is>
       </c>
-      <c r="B22" s="20" t="n">
+      <c r="B25" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="C22" s="20" t="inlineStr">
+      <c r="C25" s="18" t="inlineStr">
         <is>
           <t>Sat 18 Jul 2026</t>
         </is>
       </c>
-      <c r="D22" s="20" t="inlineStr">
+      <c r="D25" s="18" t="inlineStr">
         <is>
           <t>09:40</t>
         </is>
       </c>
-      <c r="E22" s="20" t="inlineStr">
+      <c r="E25" s="18" t="inlineStr">
         <is>
           <t>10:40</t>
         </is>
       </c>
-      <c r="F22" s="21" t="inlineStr">
+      <c r="F25" s="19" t="inlineStr">
         <is>
           <t>Pitch 1A, Pitch 1B</t>
         </is>

</xml_diff>

<commit_message>
Refresh fixtures from Dribl (17 Aug 2026) + prune actioned/stale overrides (#21)
- Regenerated all outputs from the 16 Aug full-season Action capture
  (the 14 Aug hand capture was a partial 3-week window and was discarded)
- overrides.json pruned 8 -> 4: dropped the played 2/8/15/16 Aug moves;
  re-keyed the 23 Aug U13B (Samir) move to FV's new 12:10 kickoff
  (Pitch 3 move kept deliberately - the resulting U18 overlap is flagged
  on the clash page); kept 22 Aug, 5 Sep, 6 Sep pending moves
- Setup/pack-up page: collapsible ground-layouts section, duty controls
  moved to top


Claude-Session: https://claude.ai/code/session_01Puq4Xn23NC4d6RhNQLZP1N

Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Manningham_fixtures_and_overlaps.xlsx
+++ b/Manningham_fixtures_and_overlaps.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="All Games" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Overlaps &amp; Peak Load" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Games" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overlaps &amp; Peak Load" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Games'!$A$1:$Q$692</definedName>
@@ -596,7 +596,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Source: fv.dribl.com, 2026 season, generated 16 Aug 2026</t>
+          <t>Source: fv.dribl.com, 2026 season, generated 17 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
         </is>
       </c>
       <c r="B11" s="8" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -26270,235 +26270,247 @@
       <c r="Q339" s="12" t="inlineStr"/>
     </row>
     <row r="340">
-      <c r="A340" s="9" t="inlineStr">
+      <c r="A340" s="13" t="inlineStr">
         <is>
           <t>08 Aug 2026</t>
         </is>
       </c>
-      <c r="B340" s="9" t="inlineStr">
+      <c r="B340" s="13" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="C340" s="9" t="inlineStr">
+      <c r="C340" s="13" t="inlineStr">
         <is>
           <t>08:30</t>
         </is>
       </c>
-      <c r="D340" s="9" t="inlineStr">
+      <c r="D340" s="13" t="inlineStr">
         <is>
           <t>09:10</t>
         </is>
       </c>
-      <c r="E340" s="9" t="n">
+      <c r="E340" s="13" t="n">
         <v>40</v>
       </c>
-      <c r="F340" s="9" t="inlineStr">
+      <c r="F340" s="13" t="inlineStr">
         <is>
           <t>Pettys Reserve</t>
         </is>
       </c>
-      <c r="G340" s="9" t="inlineStr">
+      <c r="G340" s="13" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="H340" s="9" t="inlineStr">
+      <c r="H340" s="13" t="inlineStr">
         <is>
           <t>Sub</t>
         </is>
       </c>
-      <c r="I340" s="10" t="inlineStr">
+      <c r="I340" s="14" t="inlineStr">
         <is>
           <t>Pitch 1B (Bottom Field)</t>
         </is>
       </c>
-      <c r="J340" s="9" t="inlineStr">
+      <c r="J340" s="13" t="inlineStr">
         <is>
           <t>U11</t>
         </is>
       </c>
-      <c r="K340" s="10" t="inlineStr">
+      <c r="K340" s="14" t="inlineStr">
         <is>
           <t>Manningham United Blues FC U11 MiniRoos - Wallabies Mixed (Culina's)</t>
         </is>
       </c>
-      <c r="L340" s="10" t="inlineStr">
+      <c r="L340" s="14" t="inlineStr">
         <is>
           <t>Whitehorse United SC U11 MiniRoos - Wallabies Mixed Vanntha</t>
         </is>
       </c>
-      <c r="M340" s="10" t="inlineStr">
+      <c r="M340" s="14" t="inlineStr">
         <is>
           <t>Coles MiniRoos Mixed Saturday (U6 - U11)</t>
         </is>
       </c>
-      <c r="N340" s="9" t="inlineStr">
+      <c r="N340" s="13" t="inlineStr">
         <is>
           <t>Coles MiniRoos Mixed Saturday East 11 Wallabies Blue</t>
         </is>
       </c>
-      <c r="O340" s="9" t="inlineStr">
+      <c r="O340" s="13" t="inlineStr">
         <is>
           <t>R14</t>
         </is>
       </c>
-      <c r="P340" s="9" t="inlineStr"/>
-      <c r="Q340" s="10" t="inlineStr"/>
+      <c r="P340" s="15" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Q340" s="14" t="inlineStr"/>
     </row>
     <row r="341">
-      <c r="A341" s="11" t="inlineStr">
+      <c r="A341" s="13" t="inlineStr">
         <is>
           <t>08 Aug 2026</t>
         </is>
       </c>
-      <c r="B341" s="11" t="inlineStr">
+      <c r="B341" s="13" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="C341" s="11" t="inlineStr">
+      <c r="C341" s="13" t="inlineStr">
         <is>
           <t>08:30</t>
         </is>
       </c>
-      <c r="D341" s="11" t="inlineStr">
+      <c r="D341" s="13" t="inlineStr">
         <is>
           <t>09:30</t>
         </is>
       </c>
-      <c r="E341" s="11" t="n">
+      <c r="E341" s="13" t="n">
         <v>60</v>
       </c>
-      <c r="F341" s="11" t="inlineStr">
+      <c r="F341" s="13" t="inlineStr">
         <is>
           <t>Pettys Reserve</t>
         </is>
       </c>
-      <c r="G341" s="11" t="inlineStr">
+      <c r="G341" s="13" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="H341" s="11" t="inlineStr">
+      <c r="H341" s="13" t="inlineStr">
         <is>
           <t>Sub</t>
         </is>
       </c>
-      <c r="I341" s="12" t="inlineStr">
+      <c r="I341" s="14" t="inlineStr">
         <is>
           <t>Pitch 1A (Bottom Field)</t>
         </is>
       </c>
-      <c r="J341" s="11" t="inlineStr">
+      <c r="J341" s="13" t="inlineStr">
         <is>
           <t>U12</t>
         </is>
       </c>
-      <c r="K341" s="12" t="inlineStr">
+      <c r="K341" s="14" t="inlineStr">
         <is>
           <t>Manningham United Blues FC U12 Juniors - B Mixed (Chris)</t>
         </is>
       </c>
-      <c r="L341" s="12" t="inlineStr">
+      <c r="L341" s="14" t="inlineStr">
         <is>
           <t>Nunawading City FC U12 Juniors - B Mixed</t>
         </is>
       </c>
-      <c r="M341" s="12" t="inlineStr">
+      <c r="M341" s="14" t="inlineStr">
         <is>
           <t>Junior Mixed Saturday (U12 - U16)</t>
         </is>
       </c>
-      <c r="N341" s="11" t="inlineStr">
+      <c r="N341" s="13" t="inlineStr">
         <is>
           <t>Mixed Saturday East 12B</t>
         </is>
       </c>
-      <c r="O341" s="11" t="inlineStr">
+      <c r="O341" s="13" t="inlineStr">
         <is>
           <t>R14</t>
         </is>
       </c>
-      <c r="P341" s="11" t="inlineStr"/>
-      <c r="Q341" s="12" t="inlineStr"/>
+      <c r="P341" s="15" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Q341" s="14" t="inlineStr"/>
     </row>
     <row r="342">
-      <c r="A342" s="9" t="inlineStr">
+      <c r="A342" s="13" t="inlineStr">
         <is>
           <t>08 Aug 2026</t>
         </is>
       </c>
-      <c r="B342" s="9" t="inlineStr">
+      <c r="B342" s="13" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="C342" s="9" t="inlineStr">
-        <is>
-          <t>12:45</t>
-        </is>
-      </c>
-      <c r="D342" s="9" t="inlineStr">
-        <is>
-          <t>14:15</t>
-        </is>
-      </c>
-      <c r="E342" s="9" t="n">
-        <v>90</v>
-      </c>
-      <c r="F342" s="9" t="inlineStr">
+      <c r="C342" s="13" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="D342" s="13" t="inlineStr">
+        <is>
+          <t>09:40</t>
+        </is>
+      </c>
+      <c r="E342" s="13" t="n">
+        <v>40</v>
+      </c>
+      <c r="F342" s="13" t="inlineStr">
         <is>
           <t>Pettys Reserve</t>
         </is>
       </c>
-      <c r="G342" s="9" t="inlineStr">
+      <c r="G342" s="13" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="H342" s="9" t="inlineStr">
-        <is>
-          <t>Full</t>
-        </is>
-      </c>
-      <c r="I342" s="10" t="inlineStr">
-        <is>
-          <t>Pitch 1 (Bottom Field)</t>
-        </is>
-      </c>
-      <c r="J342" s="9" t="inlineStr">
-        <is>
-          <t>Reserves</t>
-        </is>
-      </c>
-      <c r="K342" s="10" t="inlineStr">
-        <is>
-          <t>Manningham United Blues FC Reserves</t>
-        </is>
-      </c>
-      <c r="L342" s="10" t="inlineStr">
-        <is>
-          <t>Geelong Galaxy United FC Reserves</t>
-        </is>
-      </c>
-      <c r="M342" s="10" t="inlineStr">
-        <is>
-          <t>VPL Women</t>
-        </is>
-      </c>
-      <c r="N342" s="9" t="inlineStr">
-        <is>
-          <t>VPL Women - Reserves</t>
-        </is>
-      </c>
-      <c r="O342" s="9" t="inlineStr">
-        <is>
-          <t>R19</t>
-        </is>
-      </c>
-      <c r="P342" s="9" t="inlineStr"/>
-      <c r="Q342" s="10" t="inlineStr"/>
+      <c r="H342" s="13" t="inlineStr">
+        <is>
+          <t>Sub</t>
+        </is>
+      </c>
+      <c r="I342" s="14" t="inlineStr">
+        <is>
+          <t>Pitch 1C (Bottom Field) - Quarter Pitch 7v7</t>
+        </is>
+      </c>
+      <c r="J342" s="13" t="inlineStr">
+        <is>
+          <t>U08</t>
+        </is>
+      </c>
+      <c r="K342" s="14" t="inlineStr">
+        <is>
+          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed (Duke's)</t>
+        </is>
+      </c>
+      <c r="L342" s="14" t="inlineStr">
+        <is>
+          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed (Slater's)</t>
+        </is>
+      </c>
+      <c r="M342" s="14" t="inlineStr">
+        <is>
+          <t>Coles MiniRoos Mixed Saturday (U6 - U11)</t>
+        </is>
+      </c>
+      <c r="N342" s="13" t="inlineStr">
+        <is>
+          <t>Coles MiniRoos Mixed Saturday East 8 Joeys Red</t>
+        </is>
+      </c>
+      <c r="O342" s="13" t="inlineStr">
+        <is>
+          <t>R14</t>
+        </is>
+      </c>
+      <c r="P342" s="15" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Q342" s="14" t="inlineStr"/>
     </row>
     <row r="343">
       <c r="A343" s="11" t="inlineStr">
@@ -26513,12 +26525,12 @@
       </c>
       <c r="C343" s="11" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>12:45</t>
         </is>
       </c>
       <c r="D343" s="11" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>14:15</t>
         </is>
       </c>
       <c r="E343" s="11" t="n">
@@ -26546,17 +26558,17 @@
       </c>
       <c r="J343" s="11" t="inlineStr">
         <is>
-          <t>Seniors</t>
+          <t>Reserves</t>
         </is>
       </c>
       <c r="K343" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC Seniors</t>
+          <t>Manningham United Blues FC Reserves</t>
         </is>
       </c>
       <c r="L343" s="12" t="inlineStr">
         <is>
-          <t>Geelong Galaxy United FC Seniors</t>
+          <t>Geelong Galaxy United FC Reserves</t>
         </is>
       </c>
       <c r="M343" s="12" t="inlineStr">
@@ -26566,7 +26578,7 @@
       </c>
       <c r="N343" s="11" t="inlineStr">
         <is>
-          <t>VPL Women</t>
+          <t>VPL Women - Reserves</t>
         </is>
       </c>
       <c r="O343" s="11" t="inlineStr">
@@ -26590,16 +26602,16 @@
       </c>
       <c r="C344" s="9" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="D344" s="9" t="inlineStr">
         <is>
-          <t>09:10</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="E344" s="9" t="n">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="F344" s="9" t="inlineStr">
         <is>
@@ -26608,47 +26620,47 @@
       </c>
       <c r="G344" s="9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H344" s="9" t="inlineStr">
         <is>
-          <t>Sub</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="I344" s="10" t="inlineStr">
         <is>
-          <t>Pitch 2C (Top Field) - Quarter Pitch 7v7</t>
+          <t>Pitch 1 (Bottom Field)</t>
         </is>
       </c>
       <c r="J344" s="9" t="inlineStr">
         <is>
-          <t>U09</t>
+          <t>Seniors</t>
         </is>
       </c>
       <c r="K344" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Corica's)</t>
+          <t>Manningham United Blues FC Seniors</t>
         </is>
       </c>
       <c r="L344" s="10" t="inlineStr">
         <is>
-          <t>East Malvern Junior SC U09 MiniRoos - Wallabies Mixed EMJSC U9 Saturday Red</t>
+          <t>Geelong Galaxy United FC Seniors</t>
         </is>
       </c>
       <c r="M344" s="10" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Saturday (U6 - U11)</t>
+          <t>VPL Women</t>
         </is>
       </c>
       <c r="N344" s="9" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Saturday East 9 Wallabies Red</t>
+          <t>VPL Women</t>
         </is>
       </c>
       <c r="O344" s="9" t="inlineStr">
         <is>
-          <t>R14</t>
+          <t>R19</t>
         </is>
       </c>
       <c r="P344" s="9" t="inlineStr"/>
@@ -26667,12 +26679,12 @@
       </c>
       <c r="C345" s="11" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:30</t>
         </is>
       </c>
       <c r="D345" s="11" t="inlineStr">
         <is>
-          <t>09:40</t>
+          <t>09:10</t>
         </is>
       </c>
       <c r="E345" s="11" t="n">
@@ -26690,27 +26702,27 @@
       </c>
       <c r="H345" s="11" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Sub</t>
         </is>
       </c>
       <c r="I345" s="12" t="inlineStr">
         <is>
-          <t>Pitch 2</t>
+          <t>Pitch 2C (Top Field) - Quarter Pitch 7v7</t>
         </is>
       </c>
       <c r="J345" s="11" t="inlineStr">
         <is>
-          <t>U08</t>
+          <t>U09</t>
         </is>
       </c>
       <c r="K345" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed (Duke's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Corica's)</t>
         </is>
       </c>
       <c r="L345" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Joeys Mixed (Slater's)</t>
+          <t>East Malvern Junior SC U09 MiniRoos - Wallabies Mixed EMJSC U9 Saturday Red</t>
         </is>
       </c>
       <c r="M345" s="12" t="inlineStr">
@@ -26720,7 +26732,7 @@
       </c>
       <c r="N345" s="11" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Saturday East 8 Joeys Red</t>
+          <t>Coles MiniRoos Mixed Saturday East 9 Wallabies Red</t>
         </is>
       </c>
       <c r="O345" s="11" t="inlineStr">
@@ -26729,11 +26741,7 @@
         </is>
       </c>
       <c r="P345" s="11" t="inlineStr"/>
-      <c r="Q345" s="12" t="inlineStr">
-        <is>
-          <t>Pettys Reserve Pitch 1C (Bottom Field) - Quarter Pitch 7v7</t>
-        </is>
-      </c>
+      <c r="Q345" s="12" t="inlineStr"/>
     </row>
     <row r="346">
       <c r="A346" s="9" t="inlineStr">
@@ -27713,223 +27721,235 @@
       <c r="Q358" s="10" t="inlineStr"/>
     </row>
     <row r="359">
-      <c r="A359" s="11" t="inlineStr">
+      <c r="A359" s="13" t="inlineStr">
         <is>
           <t>15 Aug 2026</t>
         </is>
       </c>
-      <c r="B359" s="11" t="inlineStr">
+      <c r="B359" s="13" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="C359" s="11" t="inlineStr">
+      <c r="C359" s="13" t="inlineStr">
         <is>
           <t>08:30</t>
         </is>
       </c>
-      <c r="D359" s="11" t="inlineStr">
+      <c r="D359" s="13" t="inlineStr">
+        <is>
+          <t>09:10</t>
+        </is>
+      </c>
+      <c r="E359" s="13" t="n">
+        <v>40</v>
+      </c>
+      <c r="F359" s="13" t="inlineStr">
+        <is>
+          <t>Pettys Reserve</t>
+        </is>
+      </c>
+      <c r="G359" s="13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H359" s="13" t="inlineStr">
+        <is>
+          <t>Sub</t>
+        </is>
+      </c>
+      <c r="I359" s="14" t="inlineStr">
+        <is>
+          <t>Pitch 1E (Bottom Field) - Quarter Pitch 4v4</t>
+        </is>
+      </c>
+      <c r="J359" s="13" t="inlineStr">
+        <is>
+          <t>U07</t>
+        </is>
+      </c>
+      <c r="K359" s="14" t="inlineStr">
+        <is>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (White)</t>
+        </is>
+      </c>
+      <c r="L359" s="14" t="inlineStr">
+        <is>
+          <t>Oakleigh Cannons FC U07 MiniRoos - Joeys Mixed OCFC Chippa/Jason</t>
+        </is>
+      </c>
+      <c r="M359" s="14" t="inlineStr">
+        <is>
+          <t>Coles MiniRoos Mixed Saturday (U6 - U11)</t>
+        </is>
+      </c>
+      <c r="N359" s="13" t="inlineStr">
+        <is>
+          <t>Coles MiniRoos Mixed Saturday East 7 Joeys Red</t>
+        </is>
+      </c>
+      <c r="O359" s="13" t="inlineStr">
+        <is>
+          <t>R15</t>
+        </is>
+      </c>
+      <c r="P359" s="15" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Q359" s="14" t="inlineStr"/>
+    </row>
+    <row r="360">
+      <c r="A360" s="13" t="inlineStr">
+        <is>
+          <t>15 Aug 2026</t>
+        </is>
+      </c>
+      <c r="B360" s="13" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="C360" s="13" t="inlineStr">
+        <is>
+          <t>08:30</t>
+        </is>
+      </c>
+      <c r="D360" s="13" t="inlineStr">
         <is>
           <t>09:30</t>
         </is>
       </c>
-      <c r="E359" s="11" t="n">
+      <c r="E360" s="13" t="n">
         <v>60</v>
       </c>
-      <c r="F359" s="11" t="inlineStr">
+      <c r="F360" s="13" t="inlineStr">
         <is>
           <t>Pettys Reserve</t>
         </is>
       </c>
-      <c r="G359" s="11" t="inlineStr">
+      <c r="G360" s="13" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="H359" s="11" t="inlineStr">
+      <c r="H360" s="13" t="inlineStr">
         <is>
           <t>Sub</t>
         </is>
       </c>
-      <c r="I359" s="12" t="inlineStr">
+      <c r="I360" s="14" t="inlineStr">
         <is>
           <t>Pitch 1A (Bottom Field)</t>
         </is>
       </c>
-      <c r="J359" s="11" t="inlineStr">
+      <c r="J360" s="13" t="inlineStr">
         <is>
           <t>U12</t>
         </is>
       </c>
-      <c r="K359" s="12" t="inlineStr">
+      <c r="K360" s="14" t="inlineStr">
         <is>
           <t>Manningham United Blues FC U12 Juniors - B Mixed (Andre)</t>
         </is>
       </c>
-      <c r="L359" s="12" t="inlineStr">
+      <c r="L360" s="14" t="inlineStr">
         <is>
           <t>FC Bulleen Lions U12 Juniors - B Mixed</t>
         </is>
       </c>
-      <c r="M359" s="12" t="inlineStr">
+      <c r="M360" s="14" t="inlineStr">
         <is>
           <t>Junior Mixed Saturday (U12 - U16)</t>
         </is>
       </c>
-      <c r="N359" s="11" t="inlineStr">
+      <c r="N360" s="13" t="inlineStr">
         <is>
           <t>Mixed Saturday East 12B</t>
         </is>
       </c>
-      <c r="O359" s="11" t="inlineStr">
+      <c r="O360" s="13" t="inlineStr">
         <is>
           <t>R15</t>
         </is>
       </c>
-      <c r="P359" s="11" t="inlineStr"/>
-      <c r="Q359" s="12" t="inlineStr"/>
-    </row>
-    <row r="360">
-      <c r="A360" s="9" t="inlineStr">
+      <c r="P360" s="15" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Q360" s="14" t="inlineStr"/>
+    </row>
+    <row r="361">
+      <c r="A361" s="13" t="inlineStr">
         <is>
           <t>15 Aug 2026</t>
         </is>
       </c>
-      <c r="B360" s="9" t="inlineStr">
+      <c r="B361" s="13" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="C360" s="9" t="inlineStr">
+      <c r="C361" s="13" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="D360" s="9" t="inlineStr">
+      <c r="D361" s="13" t="inlineStr">
         <is>
           <t>10:00</t>
         </is>
       </c>
-      <c r="E360" s="9" t="n">
+      <c r="E361" s="13" t="n">
         <v>60</v>
       </c>
-      <c r="F360" s="9" t="inlineStr">
+      <c r="F361" s="13" t="inlineStr">
         <is>
           <t>Pettys Reserve</t>
         </is>
       </c>
-      <c r="G360" s="9" t="inlineStr">
+      <c r="G361" s="13" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="H360" s="9" t="inlineStr">
+      <c r="H361" s="13" t="inlineStr">
         <is>
           <t>Sub</t>
         </is>
       </c>
-      <c r="I360" s="10" t="inlineStr">
+      <c r="I361" s="14" t="inlineStr">
         <is>
           <t>Pitch 1B (Bottom Field)</t>
         </is>
       </c>
-      <c r="J360" s="9" t="inlineStr"/>
-      <c r="K360" s="10" t="inlineStr">
+      <c r="J361" s="13" t="inlineStr"/>
+      <c r="K361" s="14" t="inlineStr">
         <is>
           <t>Manningham United Blues FC Girls Clinic</t>
         </is>
       </c>
-      <c r="L360" s="10" t="inlineStr">
+      <c r="L361" s="14" t="inlineStr">
         <is>
           <t>[MANUAL ADD]</t>
         </is>
       </c>
-      <c r="M360" s="10" t="inlineStr">
+      <c r="M361" s="14" t="inlineStr">
         <is>
           <t>Girls Clinic</t>
         </is>
       </c>
-      <c r="N360" s="9" t="inlineStr"/>
-      <c r="O360" s="9" t="inlineStr"/>
-      <c r="P360" s="9" t="inlineStr"/>
-      <c r="Q360" s="10" t="inlineStr"/>
-    </row>
-    <row r="361">
-      <c r="A361" s="11" t="inlineStr">
-        <is>
-          <t>15 Aug 2026</t>
-        </is>
-      </c>
-      <c r="B361" s="11" t="inlineStr">
-        <is>
-          <t>Sat</t>
-        </is>
-      </c>
-      <c r="C361" s="11" t="inlineStr">
-        <is>
-          <t>08:30</t>
-        </is>
-      </c>
-      <c r="D361" s="11" t="inlineStr">
-        <is>
-          <t>09:10</t>
-        </is>
-      </c>
-      <c r="E361" s="11" t="n">
-        <v>40</v>
-      </c>
-      <c r="F361" s="11" t="inlineStr">
-        <is>
-          <t>Pettys Reserve</t>
-        </is>
-      </c>
-      <c r="G361" s="11" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="H361" s="11" t="inlineStr">
-        <is>
-          <t>Sub</t>
-        </is>
-      </c>
-      <c r="I361" s="12" t="inlineStr">
-        <is>
-          <t>Pitch 2D (Top Field) - Quarter Pitch 7v7</t>
-        </is>
-      </c>
-      <c r="J361" s="11" t="inlineStr">
-        <is>
-          <t>U09</t>
-        </is>
-      </c>
-      <c r="K361" s="12" t="inlineStr">
-        <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Joeys Mixed (Souttar's)</t>
-        </is>
-      </c>
-      <c r="L361" s="12" t="inlineStr">
-        <is>
-          <t>Riversdale SC U09 MiniRoos - Joeys Mixed Riversdale U9 Boys - Blue</t>
-        </is>
-      </c>
-      <c r="M361" s="12" t="inlineStr">
-        <is>
-          <t>Coles MiniRoos Mixed Saturday (U6 - U11)</t>
-        </is>
-      </c>
-      <c r="N361" s="11" t="inlineStr">
-        <is>
-          <t>Coles MiniRoos Mixed Saturday East 9 Joeys Blue</t>
-        </is>
-      </c>
-      <c r="O361" s="11" t="inlineStr">
-        <is>
-          <t>R15</t>
-        </is>
-      </c>
-      <c r="P361" s="11" t="inlineStr"/>
-      <c r="Q361" s="12" t="inlineStr"/>
+      <c r="N361" s="13" t="inlineStr"/>
+      <c r="O361" s="13" t="inlineStr"/>
+      <c r="P361" s="15" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Q361" s="14" t="inlineStr"/>
     </row>
     <row r="362">
       <c r="A362" s="9" t="inlineStr">
@@ -27967,27 +27987,27 @@
       </c>
       <c r="H362" s="9" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Sub</t>
         </is>
       </c>
       <c r="I362" s="10" t="inlineStr">
         <is>
-          <t>Pitch 2</t>
+          <t>Pitch 2D (Top Field) - Quarter Pitch 7v7</t>
         </is>
       </c>
       <c r="J362" s="9" t="inlineStr">
         <is>
-          <t>U07</t>
+          <t>U09</t>
         </is>
       </c>
       <c r="K362" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (White)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Joeys Mixed (Souttar's)</t>
         </is>
       </c>
       <c r="L362" s="10" t="inlineStr">
         <is>
-          <t>Oakleigh Cannons FC U07 MiniRoos - Joeys Mixed OCFC Chippa/Jason</t>
+          <t>Riversdale SC U09 MiniRoos - Joeys Mixed Riversdale U9 Boys - Blue</t>
         </is>
       </c>
       <c r="M362" s="10" t="inlineStr">
@@ -27997,7 +28017,7 @@
       </c>
       <c r="N362" s="9" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Saturday East 7 Joeys Red</t>
+          <t>Coles MiniRoos Mixed Saturday East 9 Joeys Blue</t>
         </is>
       </c>
       <c r="O362" s="9" t="inlineStr">
@@ -28006,11 +28026,7 @@
         </is>
       </c>
       <c r="P362" s="9" t="inlineStr"/>
-      <c r="Q362" s="10" t="inlineStr">
-        <is>
-          <t>Pettys Reserve Pitch 1E (Bottom Field) - Quarter Pitch 4v4</t>
-        </is>
-      </c>
+      <c r="Q362" s="10" t="inlineStr"/>
     </row>
     <row r="363">
       <c r="A363" s="11" t="inlineStr">
@@ -46559,16 +46575,16 @@
       </c>
       <c r="C605" s="11" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>11:45</t>
         </is>
       </c>
       <c r="D605" s="11" t="inlineStr">
         <is>
-          <t>14:10</t>
+          <t>12:45</t>
         </is>
       </c>
       <c r="E605" s="11" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="F605" s="11" t="inlineStr">
         <is>
@@ -46582,27 +46598,27 @@
       </c>
       <c r="H605" s="11" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Sub</t>
         </is>
       </c>
       <c r="I605" s="12" t="inlineStr">
         <is>
-          <t>Pitch 2</t>
+          <t>Pitch 2B</t>
         </is>
       </c>
       <c r="J605" s="11" t="inlineStr">
         <is>
-          <t>U16</t>
+          <t>U13</t>
         </is>
       </c>
       <c r="K605" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U16 Juniors - B Mixed</t>
+          <t>Manningham United Blues FC U13 Juniors - A Mixed (George &amp; George)</t>
         </is>
       </c>
       <c r="L605" s="12" t="inlineStr">
         <is>
-          <t>Monash City Villarreal FC U16 Juniors - B Mixed Monash City Villarreal FC U16 Blue</t>
+          <t>Burwood City FC U13 Juniors - A Mixed LTE</t>
         </is>
       </c>
       <c r="M605" s="12" t="inlineStr">
@@ -46612,7 +46628,7 @@
       </c>
       <c r="N605" s="11" t="inlineStr">
         <is>
-          <t>Mixed East 16B</t>
+          <t>Mixed Sunday East 13A</t>
         </is>
       </c>
       <c r="O605" s="11" t="inlineStr">
@@ -46636,16 +46652,16 @@
       </c>
       <c r="C606" s="9" t="inlineStr">
         <is>
-          <t>11:45</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="D606" s="9" t="inlineStr">
         <is>
-          <t>12:45</t>
+          <t>14:10</t>
         </is>
       </c>
       <c r="E606" s="9" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F606" s="9" t="inlineStr">
         <is>
@@ -46654,7 +46670,7 @@
       </c>
       <c r="G606" s="9" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H606" s="9" t="inlineStr">
@@ -46664,22 +46680,22 @@
       </c>
       <c r="I606" s="10" t="inlineStr">
         <is>
-          <t>Pitch 3</t>
+          <t>Pitch 2</t>
         </is>
       </c>
       <c r="J606" s="9" t="inlineStr">
         <is>
-          <t>U13</t>
+          <t>U16</t>
         </is>
       </c>
       <c r="K606" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - A Mixed (George &amp; George)</t>
+          <t>Manningham United Blues FC U16 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="L606" s="10" t="inlineStr">
         <is>
-          <t>Burwood City FC U13 Juniors - A Mixed LTE</t>
+          <t>Monash City Villarreal FC U16 Juniors - B Mixed Monash City Villarreal FC U16 Blue</t>
         </is>
       </c>
       <c r="M606" s="10" t="inlineStr">
@@ -46689,7 +46705,7 @@
       </c>
       <c r="N606" s="9" t="inlineStr">
         <is>
-          <t>Mixed Sunday East 13A</t>
+          <t>Mixed East 16B</t>
         </is>
       </c>
       <c r="O606" s="9" t="inlineStr">
@@ -46698,11 +46714,7 @@
         </is>
       </c>
       <c r="P606" s="9" t="inlineStr"/>
-      <c r="Q606" s="10" t="inlineStr">
-        <is>
-          <t>Powerful Owl Park Pitch 2B</t>
-        </is>
-      </c>
+      <c r="Q606" s="10" t="inlineStr"/>
     </row>
     <row r="607">
       <c r="A607" s="11" t="inlineStr">
@@ -48416,11 +48428,11 @@
       </c>
       <c r="D629" s="11" t="inlineStr">
         <is>
-          <t>11:20</t>
+          <t>11:40</t>
         </is>
       </c>
       <c r="E629" s="11" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="F629" s="11" t="inlineStr">
         <is>
@@ -48439,32 +48451,32 @@
       </c>
       <c r="I629" s="12" t="inlineStr">
         <is>
-          <t>Pitch 1 - Midi Field B</t>
+          <t>Pitch 1B</t>
         </is>
       </c>
       <c r="J629" s="11" t="inlineStr">
         <is>
-          <t>U10</t>
+          <t>U13</t>
         </is>
       </c>
       <c r="K629" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U10 MiniRoos - Joeys Mixed (Sainsbury's)</t>
+          <t>Manningham United Blues FC U13 Juniors - C Mixed (Martin)</t>
         </is>
       </c>
       <c r="L629" s="12" t="inlineStr">
         <is>
-          <t>East Malvern Junior SC U10 MiniRoos - Joeys Mixed EMJSC U10 Sunday</t>
+          <t>Malvern City FC U13 Juniors - C Mixed U13 Anthony - C</t>
         </is>
       </c>
       <c r="M629" s="12" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Sunday (U6 - U11)</t>
+          <t>Junior Mixed Sunday (U12 - U16)</t>
         </is>
       </c>
       <c r="N629" s="11" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Sunday East 10 Joeys Red</t>
+          <t>Mixed Sunday East 13C Red</t>
         </is>
       </c>
       <c r="O629" s="11" t="inlineStr">
@@ -48488,16 +48500,16 @@
       </c>
       <c r="C630" s="9" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>10:40</t>
         </is>
       </c>
       <c r="D630" s="9" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>11:20</t>
         </is>
       </c>
       <c r="E630" s="9" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="F630" s="9" t="inlineStr">
         <is>
@@ -48516,32 +48528,32 @@
       </c>
       <c r="I630" s="10" t="inlineStr">
         <is>
-          <t>Pitch 1B</t>
+          <t>Pitch 1 - Midi Field B</t>
         </is>
       </c>
       <c r="J630" s="9" t="inlineStr">
         <is>
-          <t>U13</t>
+          <t>U10</t>
         </is>
       </c>
       <c r="K630" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - A Mixed (George &amp; George)</t>
+          <t>Manningham United Blues FC U10 MiniRoos - Joeys Mixed (Sainsbury's)</t>
         </is>
       </c>
       <c r="L630" s="10" t="inlineStr">
         <is>
-          <t>Knox City FC U13 Juniors - A Mixed U13A</t>
+          <t>East Malvern Junior SC U10 MiniRoos - Joeys Mixed EMJSC U10 Sunday</t>
         </is>
       </c>
       <c r="M630" s="10" t="inlineStr">
         <is>
-          <t>Junior Mixed Sunday (U12 - U16)</t>
+          <t>Coles MiniRoos Mixed Sunday (U6 - U11)</t>
         </is>
       </c>
       <c r="N630" s="9" t="inlineStr">
         <is>
-          <t>Mixed Sunday East 13A</t>
+          <t>Coles MiniRoos Mixed Sunday East 10 Joeys Red</t>
         </is>
       </c>
       <c r="O630" s="9" t="inlineStr">
@@ -48565,16 +48577,16 @@
       </c>
       <c r="C631" s="11" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="D631" s="11" t="inlineStr">
         <is>
-          <t>14:40</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="E631" s="11" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="F631" s="11" t="inlineStr">
         <is>
@@ -48588,27 +48600,27 @@
       </c>
       <c r="H631" s="11" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Sub</t>
         </is>
       </c>
       <c r="I631" s="12" t="inlineStr">
         <is>
-          <t>Pitch 1</t>
+          <t>Pitch 1B</t>
         </is>
       </c>
       <c r="J631" s="11" t="inlineStr">
         <is>
-          <t>U15</t>
+          <t>U13</t>
         </is>
       </c>
       <c r="K631" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U15 Juniors - A Mixed</t>
+          <t>Manningham United Blues FC U13 Juniors - A Mixed (George &amp; George)</t>
         </is>
       </c>
       <c r="L631" s="12" t="inlineStr">
         <is>
-          <t>Mooroolbark SC U15 Juniors - A Mixed Mooroolbark SC - Under 15 John</t>
+          <t>Knox City FC U13 Juniors - A Mixed U13A</t>
         </is>
       </c>
       <c r="M631" s="12" t="inlineStr">
@@ -48618,7 +48630,7 @@
       </c>
       <c r="N631" s="11" t="inlineStr">
         <is>
-          <t>Mixed East 15A</t>
+          <t>Mixed Sunday East 13A</t>
         </is>
       </c>
       <c r="O631" s="11" t="inlineStr">
@@ -48642,12 +48654,12 @@
       </c>
       <c r="C632" s="9" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="D632" s="9" t="inlineStr">
         <is>
-          <t>16:25</t>
+          <t>14:40</t>
         </is>
       </c>
       <c r="E632" s="9" t="n">
@@ -48675,27 +48687,27 @@
       </c>
       <c r="J632" s="9" t="inlineStr">
         <is>
-          <t>U18</t>
+          <t>U15</t>
         </is>
       </c>
       <c r="K632" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U18 Juniors - A Male</t>
+          <t>Manningham United Blues FC U15 Juniors - A Mixed</t>
         </is>
       </c>
       <c r="L632" s="10" t="inlineStr">
         <is>
-          <t>Collingwood City FC U18 Juniors - A Male 18A</t>
+          <t>Mooroolbark SC U15 Juniors - A Mixed Mooroolbark SC - Under 15 John</t>
         </is>
       </c>
       <c r="M632" s="10" t="inlineStr">
         <is>
-          <t>Junior Boys Sunday (U17 - U18)</t>
+          <t>Junior Mixed Sunday (U12 - U16)</t>
         </is>
       </c>
       <c r="N632" s="9" t="inlineStr">
         <is>
-          <t>Boys North-East 18A</t>
+          <t>Mixed East 15A</t>
         </is>
       </c>
       <c r="O632" s="9" t="inlineStr">
@@ -48719,16 +48731,16 @@
       </c>
       <c r="C633" s="11" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>15:15</t>
         </is>
       </c>
       <c r="D633" s="11" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>16:25</t>
         </is>
       </c>
       <c r="E633" s="11" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F633" s="11" t="inlineStr">
         <is>
@@ -48737,42 +48749,42 @@
       </c>
       <c r="G633" s="11" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H633" s="11" t="inlineStr">
         <is>
-          <t>Sub</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="I633" s="12" t="inlineStr">
         <is>
-          <t>Pitch 2A</t>
+          <t>Pitch 1</t>
         </is>
       </c>
       <c r="J633" s="11" t="inlineStr">
         <is>
-          <t>U12</t>
+          <t>U18</t>
         </is>
       </c>
       <c r="K633" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - A Mixed (Hamid)</t>
+          <t>Manningham United Blues FC U18 Juniors - A Male</t>
         </is>
       </c>
       <c r="L633" s="12" t="inlineStr">
         <is>
-          <t>Nunawading City FC U12 Juniors - A Mixed</t>
+          <t>Collingwood City FC U18 Juniors - A Male 18A</t>
         </is>
       </c>
       <c r="M633" s="12" t="inlineStr">
         <is>
-          <t>Junior Mixed Sunday (U12 - U16)</t>
+          <t>Junior Boys Sunday (U17 - U18)</t>
         </is>
       </c>
       <c r="N633" s="11" t="inlineStr">
         <is>
-          <t>Mixed Sunday East 12A Blue</t>
+          <t>Boys North-East 18A</t>
         </is>
       </c>
       <c r="O633" s="11" t="inlineStr">
@@ -48796,12 +48808,12 @@
       </c>
       <c r="C634" s="9" t="inlineStr">
         <is>
-          <t>10:40</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="D634" s="9" t="inlineStr">
         <is>
-          <t>11:40</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="E634" s="9" t="n">
@@ -48814,32 +48826,32 @@
       </c>
       <c r="G634" s="9" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H634" s="9" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Sub</t>
         </is>
       </c>
       <c r="I634" s="10" t="inlineStr">
         <is>
-          <t>Pitch 3</t>
+          <t>Pitch 2A</t>
         </is>
       </c>
       <c r="J634" s="9" t="inlineStr">
         <is>
-          <t>U13</t>
+          <t>U12</t>
         </is>
       </c>
       <c r="K634" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - C Mixed (Martin)</t>
+          <t>Manningham United Blues FC U12 Juniors - A Mixed (Hamid)</t>
         </is>
       </c>
       <c r="L634" s="10" t="inlineStr">
         <is>
-          <t>Malvern City FC U13 Juniors - C Mixed U13 Anthony - C</t>
+          <t>Nunawading City FC U12 Juniors - A Mixed</t>
         </is>
       </c>
       <c r="M634" s="10" t="inlineStr">
@@ -48849,7 +48861,7 @@
       </c>
       <c r="N634" s="9" t="inlineStr">
         <is>
-          <t>Mixed Sunday East 13C Red</t>
+          <t>Mixed Sunday East 12A Blue</t>
         </is>
       </c>
       <c r="O634" s="9" t="inlineStr">
@@ -48858,11 +48870,7 @@
         </is>
       </c>
       <c r="P634" s="9" t="inlineStr"/>
-      <c r="Q634" s="10" t="inlineStr">
-        <is>
-          <t>Powerful Owl Park Pitch 1B</t>
-        </is>
-      </c>
+      <c r="Q634" s="10" t="inlineStr"/>
     </row>
     <row r="635">
       <c r="A635" s="11" t="inlineStr">
@@ -49262,16 +49270,16 @@
       </c>
       <c r="C640" s="9" t="inlineStr">
         <is>
-          <t>12:10</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D640" s="9" t="inlineStr">
         <is>
-          <t>13:10</t>
+          <t>15:10</t>
         </is>
       </c>
       <c r="E640" s="9" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F640" s="9" t="inlineStr">
         <is>
@@ -49285,37 +49293,37 @@
       </c>
       <c r="H640" s="9" t="inlineStr">
         <is>
-          <t>Sub</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="I640" s="10" t="inlineStr">
         <is>
-          <t>Pitch 1 - Midi Field B</t>
+          <t>Pitch 1</t>
         </is>
       </c>
       <c r="J640" s="9" t="inlineStr">
         <is>
-          <t>U13</t>
+          <t>U16</t>
         </is>
       </c>
       <c r="K640" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - B Mixed (Samir)</t>
+          <t>Manningham United Blues FC U16 Juniors - B Female (Eden)</t>
         </is>
       </c>
       <c r="L640" s="10" t="inlineStr">
         <is>
-          <t>Mazenod FC U13 Juniors - B Mixed</t>
+          <t>Glen Eira FC AAL - Junior Juniors - B Female Glen Eira FC - Van Egmonds</t>
         </is>
       </c>
       <c r="M640" s="10" t="inlineStr">
         <is>
-          <t>Junior Mixed Sunday (U12 - U16)</t>
+          <t>Junior Girls Sunday (U12 - U18)</t>
         </is>
       </c>
       <c r="N640" s="9" t="inlineStr">
         <is>
-          <t>Mixed Sunday East 13B</t>
+          <t>Girls' South-East 16B</t>
         </is>
       </c>
       <c r="O640" s="9" t="inlineStr">
@@ -49339,16 +49347,16 @@
       </c>
       <c r="C641" s="11" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>09:45</t>
         </is>
       </c>
       <c r="D641" s="11" t="inlineStr">
         <is>
-          <t>15:10</t>
+          <t>10:45</t>
         </is>
       </c>
       <c r="E641" s="11" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="F641" s="11" t="inlineStr">
         <is>
@@ -49357,7 +49365,7 @@
       </c>
       <c r="G641" s="11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H641" s="11" t="inlineStr">
@@ -49367,32 +49375,32 @@
       </c>
       <c r="I641" s="12" t="inlineStr">
         <is>
-          <t>Pitch 1</t>
+          <t>Pitch 2</t>
         </is>
       </c>
       <c r="J641" s="11" t="inlineStr">
         <is>
-          <t>U16</t>
+          <t>U14</t>
         </is>
       </c>
       <c r="K641" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U16 Juniors - B Female (Eden)</t>
+          <t>Manningham United Blues FC U14 Juniors - A Mixed</t>
         </is>
       </c>
       <c r="L641" s="12" t="inlineStr">
         <is>
-          <t>Glen Eira FC AAL - Junior Juniors - B Female Glen Eira FC - Van Egmonds</t>
+          <t>Boronia SC U14 Juniors - A Mixed Tristan</t>
         </is>
       </c>
       <c r="M641" s="12" t="inlineStr">
         <is>
-          <t>Junior Girls Sunday (U12 - U18)</t>
+          <t>Junior Mixed Sunday (U12 - U16)</t>
         </is>
       </c>
       <c r="N641" s="11" t="inlineStr">
         <is>
-          <t>Girls' South-East 16B</t>
+          <t>Mixed East 14A</t>
         </is>
       </c>
       <c r="O641" s="11" t="inlineStr">
@@ -49416,12 +49424,12 @@
       </c>
       <c r="C642" s="9" t="inlineStr">
         <is>
-          <t>09:45</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="D642" s="9" t="inlineStr">
         <is>
-          <t>10:45</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="E642" s="9" t="n">
@@ -49454,22 +49462,22 @@
       </c>
       <c r="K642" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - A Mixed</t>
+          <t>Manningham United Blues FC U14 Juniors - C Female (Christian)</t>
         </is>
       </c>
       <c r="L642" s="10" t="inlineStr">
         <is>
-          <t>Boronia SC U14 Juniors - A Mixed Tristan</t>
+          <t>Ashburton United SC U14 Juniors - C Female</t>
         </is>
       </c>
       <c r="M642" s="10" t="inlineStr">
         <is>
-          <t>Junior Mixed Sunday (U12 - U16)</t>
+          <t>Junior Girls Sunday (U12 - U18)</t>
         </is>
       </c>
       <c r="N642" s="9" t="inlineStr">
         <is>
-          <t>Mixed East 14A</t>
+          <t>Girls' South-East 14C</t>
         </is>
       </c>
       <c r="O642" s="9" t="inlineStr">
@@ -49493,12 +49501,12 @@
       </c>
       <c r="C643" s="11" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>13:15</t>
         </is>
       </c>
       <c r="D643" s="11" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>14:15</t>
         </is>
       </c>
       <c r="E643" s="11" t="n">
@@ -49531,22 +49539,22 @@
       </c>
       <c r="K643" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - C Female (Christian)</t>
+          <t>Manningham United Blues FC U14 Juniors - C Mixed (Phil)</t>
         </is>
       </c>
       <c r="L643" s="12" t="inlineStr">
         <is>
-          <t>Ashburton United SC U14 Juniors - C Female</t>
+          <t>Mazenod FC U14 Juniors - C Mixed</t>
         </is>
       </c>
       <c r="M643" s="12" t="inlineStr">
         <is>
-          <t>Junior Girls Sunday (U12 - U18)</t>
+          <t>Junior Mixed Sunday (U12 - U16)</t>
         </is>
       </c>
       <c r="N643" s="11" t="inlineStr">
         <is>
-          <t>Girls' South-East 14C</t>
+          <t>Mixed East 14C Red</t>
         </is>
       </c>
       <c r="O643" s="11" t="inlineStr">
@@ -49570,16 +49578,16 @@
       </c>
       <c r="C644" s="9" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="D644" s="9" t="inlineStr">
         <is>
-          <t>14:15</t>
+          <t>16:10</t>
         </is>
       </c>
       <c r="E644" s="9" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F644" s="9" t="inlineStr">
         <is>
@@ -49603,17 +49611,17 @@
       </c>
       <c r="J644" s="9" t="inlineStr">
         <is>
-          <t>U14</t>
+          <t>U15</t>
         </is>
       </c>
       <c r="K644" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - C Mixed (Phil)</t>
+          <t>Manningham United Blues FC U15 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="L644" s="10" t="inlineStr">
         <is>
-          <t>Mazenod FC U14 Juniors - C Mixed</t>
+          <t>Bunyip &amp; District SC U15 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="M644" s="10" t="inlineStr">
@@ -49623,7 +49631,7 @@
       </c>
       <c r="N644" s="9" t="inlineStr">
         <is>
-          <t>Mixed East 14C Red</t>
+          <t>Mixed South-East 15B</t>
         </is>
       </c>
       <c r="O644" s="9" t="inlineStr">
@@ -49635,158 +49643,170 @@
       <c r="Q644" s="10" t="inlineStr"/>
     </row>
     <row r="645">
-      <c r="A645" s="11" t="inlineStr">
+      <c r="A645" s="13" t="inlineStr">
         <is>
           <t>23 Aug 2026</t>
         </is>
       </c>
-      <c r="B645" s="11" t="inlineStr">
+      <c r="B645" s="13" t="inlineStr">
         <is>
           <t>Sun</t>
         </is>
       </c>
-      <c r="C645" s="11" t="inlineStr">
-        <is>
-          <t>15:00</t>
-        </is>
-      </c>
-      <c r="D645" s="11" t="inlineStr">
-        <is>
-          <t>16:10</t>
-        </is>
-      </c>
-      <c r="E645" s="11" t="n">
+      <c r="C645" s="13" t="inlineStr">
+        <is>
+          <t>12:10</t>
+        </is>
+      </c>
+      <c r="D645" s="13" t="inlineStr">
+        <is>
+          <t>13:10</t>
+        </is>
+      </c>
+      <c r="E645" s="13" t="n">
+        <v>60</v>
+      </c>
+      <c r="F645" s="13" t="inlineStr">
+        <is>
+          <t>Powerful Owl Park</t>
+        </is>
+      </c>
+      <c r="G645" s="13" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H645" s="13" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="I645" s="14" t="inlineStr">
+        <is>
+          <t>Pitch 3</t>
+        </is>
+      </c>
+      <c r="J645" s="13" t="inlineStr">
+        <is>
+          <t>U13</t>
+        </is>
+      </c>
+      <c r="K645" s="14" t="inlineStr">
+        <is>
+          <t>Manningham United Blues FC U13 Juniors - B Mixed (Samir)</t>
+        </is>
+      </c>
+      <c r="L645" s="14" t="inlineStr">
+        <is>
+          <t>Mazenod FC U13 Juniors - B Mixed</t>
+        </is>
+      </c>
+      <c r="M645" s="14" t="inlineStr">
+        <is>
+          <t>Junior Mixed Sunday (U12 - U16)</t>
+        </is>
+      </c>
+      <c r="N645" s="13" t="inlineStr">
+        <is>
+          <t>Mixed Sunday East 13B</t>
+        </is>
+      </c>
+      <c r="O645" s="13" t="inlineStr">
+        <is>
+          <t>R16</t>
+        </is>
+      </c>
+      <c r="P645" s="15" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Q645" s="14" t="inlineStr">
+        <is>
+          <t>Powerful Owl Park Pitch 1 - Midi Field B</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" s="13" t="inlineStr">
+        <is>
+          <t>23 Aug 2026</t>
+        </is>
+      </c>
+      <c r="B646" s="13" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
+      <c r="C646" s="13" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="D646" s="13" t="inlineStr">
+        <is>
+          <t>14:10</t>
+        </is>
+      </c>
+      <c r="E646" s="13" t="n">
         <v>70</v>
       </c>
-      <c r="F645" s="11" t="inlineStr">
+      <c r="F646" s="13" t="inlineStr">
         <is>
           <t>Powerful Owl Park</t>
         </is>
       </c>
-      <c r="G645" s="11" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="H645" s="11" t="inlineStr">
+      <c r="G646" s="13" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H646" s="13" t="inlineStr">
         <is>
           <t>Full</t>
         </is>
       </c>
-      <c r="I645" s="12" t="inlineStr">
-        <is>
-          <t>Pitch 2</t>
-        </is>
-      </c>
-      <c r="J645" s="11" t="inlineStr">
-        <is>
-          <t>U15</t>
-        </is>
-      </c>
-      <c r="K645" s="12" t="inlineStr">
-        <is>
-          <t>Manningham United Blues FC U15 Juniors - B Mixed</t>
-        </is>
-      </c>
-      <c r="L645" s="12" t="inlineStr">
-        <is>
-          <t>Bunyip &amp; District SC U15 Juniors - B Mixed</t>
-        </is>
-      </c>
-      <c r="M645" s="12" t="inlineStr">
-        <is>
-          <t>Junior Mixed Sunday (U12 - U16)</t>
-        </is>
-      </c>
-      <c r="N645" s="11" t="inlineStr">
-        <is>
-          <t>Mixed South-East 15B</t>
-        </is>
-      </c>
-      <c r="O645" s="11" t="inlineStr">
+      <c r="I646" s="14" t="inlineStr">
+        <is>
+          <t>Pitch 3</t>
+        </is>
+      </c>
+      <c r="J646" s="13" t="inlineStr">
+        <is>
+          <t>U18</t>
+        </is>
+      </c>
+      <c r="K646" s="14" t="inlineStr">
+        <is>
+          <t>Manningham United Blues FC U18 Juniors - A Male</t>
+        </is>
+      </c>
+      <c r="L646" s="14" t="inlineStr">
+        <is>
+          <t>West Preston SC U18 Juniors - A Male West Preston U/18A</t>
+        </is>
+      </c>
+      <c r="M646" s="14" t="inlineStr">
+        <is>
+          <t>Junior Boys Sunday (U17 - U18)</t>
+        </is>
+      </c>
+      <c r="N646" s="13" t="inlineStr">
+        <is>
+          <t>Boys North-East 18A</t>
+        </is>
+      </c>
+      <c r="O646" s="13" t="inlineStr">
         <is>
           <t>R16</t>
         </is>
       </c>
-      <c r="P645" s="11" t="inlineStr"/>
-      <c r="Q645" s="12" t="inlineStr"/>
-    </row>
-    <row r="646">
-      <c r="A646" s="9" t="inlineStr">
-        <is>
-          <t>23 Aug 2026</t>
-        </is>
-      </c>
-      <c r="B646" s="9" t="inlineStr">
-        <is>
-          <t>Sun</t>
-        </is>
-      </c>
-      <c r="C646" s="9" t="inlineStr">
-        <is>
-          <t>13:00</t>
-        </is>
-      </c>
-      <c r="D646" s="9" t="inlineStr">
-        <is>
-          <t>14:10</t>
-        </is>
-      </c>
-      <c r="E646" s="9" t="n">
-        <v>70</v>
-      </c>
-      <c r="F646" s="9" t="inlineStr">
-        <is>
-          <t>Powerful Owl Park</t>
-        </is>
-      </c>
-      <c r="G646" s="9" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="H646" s="9" t="inlineStr">
-        <is>
-          <t>Full</t>
-        </is>
-      </c>
-      <c r="I646" s="10" t="inlineStr">
-        <is>
-          <t>Pitch 3</t>
-        </is>
-      </c>
-      <c r="J646" s="9" t="inlineStr">
-        <is>
-          <t>U18</t>
-        </is>
-      </c>
-      <c r="K646" s="10" t="inlineStr">
-        <is>
-          <t>Manningham United Blues FC U18 Juniors - A Male</t>
-        </is>
-      </c>
-      <c r="L646" s="10" t="inlineStr">
-        <is>
-          <t>West Preston SC U18 Juniors - A Male West Preston U/18A</t>
-        </is>
-      </c>
-      <c r="M646" s="10" t="inlineStr">
-        <is>
-          <t>Junior Boys Sunday (U17 - U18)</t>
-        </is>
-      </c>
-      <c r="N646" s="9" t="inlineStr">
-        <is>
-          <t>Boys North-East 18A</t>
-        </is>
-      </c>
-      <c r="O646" s="9" t="inlineStr">
-        <is>
-          <t>R16</t>
-        </is>
-      </c>
-      <c r="P646" s="9" t="inlineStr"/>
-      <c r="Q646" s="10" t="inlineStr"/>
+      <c r="P646" s="15" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Q646" s="14" t="inlineStr"/>
     </row>
     <row r="647">
       <c r="A647" s="11" t="inlineStr">
@@ -50345,11 +50365,11 @@
       </c>
       <c r="D654" s="9" t="inlineStr">
         <is>
-          <t>12:10</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="E654" s="9" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="F654" s="9" t="inlineStr">
         <is>
@@ -50368,32 +50388,32 @@
       </c>
       <c r="I654" s="10" t="inlineStr">
         <is>
-          <t>Pitch 1 - Midi Field B</t>
+          <t>Pitch 1B</t>
         </is>
       </c>
       <c r="J654" s="9" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>U13</t>
         </is>
       </c>
       <c r="K654" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Female Miniroos Girls U11W (Holly &amp; Marina)</t>
+          <t>Manningham United Blues FC U13 Juniors - C Mixed (Martin)</t>
         </is>
       </c>
       <c r="L654" s="10" t="inlineStr">
         <is>
-          <t>Malvern City FC U11 MiniRoos - Wallabies Female U11 MCFC Girls</t>
+          <t>Whitehorse United SC U13 Juniors - C Mixed Shane</t>
         </is>
       </c>
       <c r="M654" s="10" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Girls' Sunday (U6 - U11)</t>
+          <t>Junior Mixed Sunday (U12 - U16)</t>
         </is>
       </c>
       <c r="N654" s="9" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Girls' East 11 Wallabies</t>
+          <t>Mixed Sunday East 13C Red</t>
         </is>
       </c>
       <c r="O654" s="9" t="inlineStr">
@@ -50417,16 +50437,16 @@
       </c>
       <c r="C655" s="11" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="D655" s="11" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>12:10</t>
         </is>
       </c>
       <c r="E655" s="11" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="F655" s="11" t="inlineStr">
         <is>
@@ -50440,37 +50460,37 @@
       </c>
       <c r="H655" s="11" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Sub</t>
         </is>
       </c>
       <c r="I655" s="12" t="inlineStr">
         <is>
-          <t>Pitch 1</t>
+          <t>Pitch 1 - Midi Field B</t>
         </is>
       </c>
       <c r="J655" s="11" t="inlineStr">
         <is>
-          <t>U14</t>
+          <t>U11</t>
         </is>
       </c>
       <c r="K655" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - A Female (Chloe)</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Female Miniroos Girls U11W (Holly &amp; Marina)</t>
         </is>
       </c>
       <c r="L655" s="12" t="inlineStr">
         <is>
-          <t>Alamein FC U14 Juniors - A Female</t>
+          <t>Malvern City FC U11 MiniRoos - Wallabies Female U11 MCFC Girls</t>
         </is>
       </c>
       <c r="M655" s="12" t="inlineStr">
         <is>
-          <t>Junior Girls Sunday (U12 - U18)</t>
+          <t>Coles MiniRoos Girls' Sunday (U6 - U11)</t>
         </is>
       </c>
       <c r="N655" s="11" t="inlineStr">
         <is>
-          <t>Girls' South-East 14A</t>
+          <t>Coles MiniRoos Girls' East 11 Wallabies</t>
         </is>
       </c>
       <c r="O655" s="11" t="inlineStr">
@@ -50494,16 +50514,16 @@
       </c>
       <c r="C656" s="9" t="inlineStr">
         <is>
-          <t>14:45</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="D656" s="9" t="inlineStr">
         <is>
-          <t>15:55</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="E656" s="9" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="F656" s="9" t="inlineStr">
         <is>
@@ -50527,17 +50547,17 @@
       </c>
       <c r="J656" s="9" t="inlineStr">
         <is>
-          <t>U17/18</t>
+          <t>U14</t>
         </is>
       </c>
       <c r="K656" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U17/18 Juniors - B Female (Marilyn)</t>
+          <t>Manningham United Blues FC U14 Juniors - A Female (Chloe)</t>
         </is>
       </c>
       <c r="L656" s="10" t="inlineStr">
         <is>
-          <t>Mount Eliza SC U17/18 Juniors - B Female Red</t>
+          <t>Alamein FC U14 Juniors - A Female</t>
         </is>
       </c>
       <c r="M656" s="10" t="inlineStr">
@@ -50547,7 +50567,7 @@
       </c>
       <c r="N656" s="9" t="inlineStr">
         <is>
-          <t>Girls' South-East 17/18B</t>
+          <t>Girls' South-East 14A</t>
         </is>
       </c>
       <c r="O656" s="9" t="inlineStr">
@@ -50571,16 +50591,16 @@
       </c>
       <c r="C657" s="11" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>14:45</t>
         </is>
       </c>
       <c r="D657" s="11" t="inlineStr">
         <is>
-          <t>09:40</t>
+          <t>15:55</t>
         </is>
       </c>
       <c r="E657" s="11" t="n">
-        <v>40</v>
+        <v>70</v>
       </c>
       <c r="F657" s="11" t="inlineStr">
         <is>
@@ -50589,42 +50609,42 @@
       </c>
       <c r="G657" s="11" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H657" s="11" t="inlineStr">
         <is>
-          <t>Sub</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="I657" s="12" t="inlineStr">
         <is>
-          <t>Pitch 2A</t>
+          <t>Pitch 1</t>
         </is>
       </c>
       <c r="J657" s="11" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>U17/18</t>
         </is>
       </c>
       <c r="K657" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Kangaroos Mixed</t>
+          <t>Manningham United Blues FC U17/18 Juniors - B Female (Marilyn)</t>
         </is>
       </c>
       <c r="L657" s="12" t="inlineStr">
         <is>
-          <t>FC Bulleen Lions U11 MiniRoos - Kangaroos Mixed Anthony &amp; Rob</t>
+          <t>Mount Eliza SC U17/18 Juniors - B Female Red</t>
         </is>
       </c>
       <c r="M657" s="12" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Sunday (U6 - U11)</t>
+          <t>Junior Girls Sunday (U12 - U18)</t>
         </is>
       </c>
       <c r="N657" s="11" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Sunday East 11 Kangaroos Red</t>
+          <t>Girls' South-East 17/18B</t>
         </is>
       </c>
       <c r="O657" s="11" t="inlineStr">
@@ -50676,22 +50696,22 @@
       </c>
       <c r="I658" s="10" t="inlineStr">
         <is>
-          <t>Pitch 2 - Midi B</t>
+          <t>Pitch 2A</t>
         </is>
       </c>
       <c r="J658" s="9" t="inlineStr">
         <is>
-          <t>U07</t>
+          <t>U11</t>
         </is>
       </c>
       <c r="K658" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Red)</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Kangaroos Mixed</t>
         </is>
       </c>
       <c r="L658" s="10" t="inlineStr">
         <is>
-          <t>East Malvern Junior SC U07 MiniRoos - Joeys Mixed EMJSC U7 Sunday Orange</t>
+          <t>FC Bulleen Lions U11 MiniRoos - Kangaroos Mixed Anthony &amp; Rob</t>
         </is>
       </c>
       <c r="M658" s="10" t="inlineStr">
@@ -50701,7 +50721,7 @@
       </c>
       <c r="N658" s="9" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Sunday East 7 Joeys Red</t>
+          <t>Coles MiniRoos Mixed Sunday East 11 Kangaroos Red</t>
         </is>
       </c>
       <c r="O658" s="9" t="inlineStr">
@@ -50753,7 +50773,7 @@
       </c>
       <c r="I659" s="12" t="inlineStr">
         <is>
-          <t>Pitch 2 - Midi A</t>
+          <t>Pitch 2 - Midi B</t>
         </is>
       </c>
       <c r="J659" s="11" t="inlineStr">
@@ -50763,12 +50783,12 @@
       </c>
       <c r="K659" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Green)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Red)</t>
         </is>
       </c>
       <c r="L659" s="12" t="inlineStr">
         <is>
-          <t>Doncaster Rovers SC U07 MiniRoos - Joeys Mixed</t>
+          <t>East Malvern Junior SC U07 MiniRoos - Joeys Mixed EMJSC U7 Sunday Orange</t>
         </is>
       </c>
       <c r="M659" s="12" t="inlineStr">
@@ -50802,16 +50822,16 @@
       </c>
       <c r="C660" s="9" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="D660" s="9" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>09:40</t>
         </is>
       </c>
       <c r="E660" s="9" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="F660" s="9" t="inlineStr">
         <is>
@@ -50830,32 +50850,32 @@
       </c>
       <c r="I660" s="10" t="inlineStr">
         <is>
-          <t>Pitch 2A</t>
+          <t>Pitch 2 - Midi A</t>
         </is>
       </c>
       <c r="J660" s="9" t="inlineStr">
         <is>
-          <t>U12</t>
+          <t>U07</t>
         </is>
       </c>
       <c r="K660" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - A Female (Sienna)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Green)</t>
         </is>
       </c>
       <c r="L660" s="10" t="inlineStr">
         <is>
-          <t>Alamein FC U12 Juniors - A Female</t>
+          <t>Doncaster Rovers SC U07 MiniRoos - Joeys Mixed</t>
         </is>
       </c>
       <c r="M660" s="10" t="inlineStr">
         <is>
-          <t>Junior Girls Sunday (U12 - U18)</t>
+          <t>Coles MiniRoos Mixed Sunday (U6 - U11)</t>
         </is>
       </c>
       <c r="N660" s="9" t="inlineStr">
         <is>
-          <t>Girls' South-East 12A</t>
+          <t>Coles MiniRoos Mixed Sunday East 7 Joeys Red</t>
         </is>
       </c>
       <c r="O660" s="9" t="inlineStr">
@@ -50879,12 +50899,12 @@
       </c>
       <c r="C661" s="11" t="inlineStr">
         <is>
-          <t>11:45</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="D661" s="11" t="inlineStr">
         <is>
-          <t>12:45</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="E661" s="11" t="n">
@@ -50902,37 +50922,37 @@
       </c>
       <c r="H661" s="11" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Sub</t>
         </is>
       </c>
       <c r="I661" s="12" t="inlineStr">
         <is>
-          <t>Pitch 2</t>
+          <t>Pitch 2A</t>
         </is>
       </c>
       <c r="J661" s="11" t="inlineStr">
         <is>
-          <t>U14</t>
+          <t>U12</t>
         </is>
       </c>
       <c r="K661" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - B Mixed</t>
+          <t>Manningham United Blues FC U12 Juniors - A Female (Sienna)</t>
         </is>
       </c>
       <c r="L661" s="12" t="inlineStr">
         <is>
-          <t>Malvern City FC U14 Juniors - B Mixed U14 - B</t>
+          <t>Alamein FC U12 Juniors - A Female</t>
         </is>
       </c>
       <c r="M661" s="12" t="inlineStr">
         <is>
-          <t>Junior Mixed Sunday (U12 - U16)</t>
+          <t>Junior Girls Sunday (U12 - U18)</t>
         </is>
       </c>
       <c r="N661" s="11" t="inlineStr">
         <is>
-          <t>Mixed East 14B</t>
+          <t>Girls' South-East 12A</t>
         </is>
       </c>
       <c r="O661" s="11" t="inlineStr">
@@ -50956,16 +50976,16 @@
       </c>
       <c r="C662" s="9" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="D662" s="9" t="inlineStr">
         <is>
-          <t>14:25</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="E662" s="9" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="F662" s="9" t="inlineStr">
         <is>
@@ -50979,27 +50999,27 @@
       </c>
       <c r="H662" s="9" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Sub</t>
         </is>
       </c>
       <c r="I662" s="10" t="inlineStr">
         <is>
-          <t>Pitch 2</t>
+          <t>Pitch 2B</t>
         </is>
       </c>
       <c r="J662" s="9" t="inlineStr">
         <is>
-          <t>U15</t>
+          <t>U13</t>
         </is>
       </c>
       <c r="K662" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U15 Juniors - B Female (Ethan)</t>
+          <t>Manningham United Blues FC U13 Juniors - C Female (Abigail)</t>
         </is>
       </c>
       <c r="L662" s="10" t="inlineStr">
         <is>
-          <t>Brighton SC U15 Juniors - B Female Apollos</t>
+          <t>Hampton East Brighton FC U13 Juniors - C Female u13 girls</t>
         </is>
       </c>
       <c r="M662" s="10" t="inlineStr">
@@ -51009,7 +51029,7 @@
       </c>
       <c r="N662" s="9" t="inlineStr">
         <is>
-          <t>Girls' South-East 15B</t>
+          <t>Girls' South-East 13C</t>
         </is>
       </c>
       <c r="O662" s="9" t="inlineStr">
@@ -51033,16 +51053,16 @@
       </c>
       <c r="C663" s="11" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>11:45</t>
         </is>
       </c>
       <c r="D663" s="11" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>12:45</t>
         </is>
       </c>
       <c r="E663" s="11" t="n">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="F663" s="11" t="inlineStr">
         <is>
@@ -51066,27 +51086,27 @@
       </c>
       <c r="J663" s="11" t="inlineStr">
         <is>
-          <t>Seniors</t>
+          <t>U14</t>
         </is>
       </c>
       <c r="K663" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC Seniors</t>
+          <t>Manningham United Blues FC U14 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="L663" s="12" t="inlineStr">
         <is>
-          <t>Mount Martha SC Seniors</t>
+          <t>Malvern City FC U14 Juniors - B Mixed U14 - B</t>
         </is>
       </c>
       <c r="M663" s="12" t="inlineStr">
         <is>
-          <t>VETO Sports State League Women's</t>
+          <t>Junior Mixed Sunday (U12 - U16)</t>
         </is>
       </c>
       <c r="N663" s="11" t="inlineStr">
         <is>
-          <t>State League 6 Women's - South-East</t>
+          <t>Mixed East 14B</t>
         </is>
       </c>
       <c r="O663" s="11" t="inlineStr">
@@ -51110,16 +51130,16 @@
       </c>
       <c r="C664" s="9" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>13:15</t>
         </is>
       </c>
       <c r="D664" s="9" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>14:25</t>
         </is>
       </c>
       <c r="E664" s="9" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F664" s="9" t="inlineStr">
         <is>
@@ -51128,7 +51148,7 @@
       </c>
       <c r="G664" s="9" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H664" s="9" t="inlineStr">
@@ -51138,22 +51158,22 @@
       </c>
       <c r="I664" s="10" t="inlineStr">
         <is>
-          <t>Pitch 3</t>
+          <t>Pitch 2</t>
         </is>
       </c>
       <c r="J664" s="9" t="inlineStr">
         <is>
-          <t>U13</t>
+          <t>U15</t>
         </is>
       </c>
       <c r="K664" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - C Female (Abigail)</t>
+          <t>Manningham United Blues FC U15 Juniors - B Female (Ethan)</t>
         </is>
       </c>
       <c r="L664" s="10" t="inlineStr">
         <is>
-          <t>Hampton East Brighton FC U13 Juniors - C Female u13 girls</t>
+          <t>Brighton SC U15 Juniors - B Female Apollos</t>
         </is>
       </c>
       <c r="M664" s="10" t="inlineStr">
@@ -51163,7 +51183,7 @@
       </c>
       <c r="N664" s="9" t="inlineStr">
         <is>
-          <t>Girls' South-East 13C</t>
+          <t>Girls' South-East 15B</t>
         </is>
       </c>
       <c r="O664" s="9" t="inlineStr">
@@ -51172,11 +51192,7 @@
         </is>
       </c>
       <c r="P664" s="9" t="inlineStr"/>
-      <c r="Q664" s="10" t="inlineStr">
-        <is>
-          <t>Powerful Owl Park Pitch 2B</t>
-        </is>
-      </c>
+      <c r="Q664" s="10" t="inlineStr"/>
     </row>
     <row r="665">
       <c r="A665" s="11" t="inlineStr">
@@ -51191,16 +51207,16 @@
       </c>
       <c r="C665" s="11" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="D665" s="11" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="E665" s="11" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F665" s="11" t="inlineStr">
         <is>
@@ -51209,7 +51225,7 @@
       </c>
       <c r="G665" s="11" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H665" s="11" t="inlineStr">
@@ -51219,32 +51235,32 @@
       </c>
       <c r="I665" s="12" t="inlineStr">
         <is>
-          <t>Pitch 3</t>
+          <t>Pitch 2</t>
         </is>
       </c>
       <c r="J665" s="11" t="inlineStr">
         <is>
-          <t>U13</t>
+          <t>Seniors</t>
         </is>
       </c>
       <c r="K665" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - C Mixed (Martin)</t>
+          <t>Manningham United Blues FC Seniors</t>
         </is>
       </c>
       <c r="L665" s="12" t="inlineStr">
         <is>
-          <t>Whitehorse United SC U13 Juniors - C Mixed Shane</t>
+          <t>Mount Martha SC Seniors</t>
         </is>
       </c>
       <c r="M665" s="12" t="inlineStr">
         <is>
-          <t>Junior Mixed Sunday (U12 - U16)</t>
+          <t>VETO Sports State League Women's</t>
         </is>
       </c>
       <c r="N665" s="11" t="inlineStr">
         <is>
-          <t>Mixed Sunday East 13C Red</t>
+          <t>State League 6 Women's - South-East</t>
         </is>
       </c>
       <c r="O665" s="11" t="inlineStr">
@@ -51253,11 +51269,7 @@
         </is>
       </c>
       <c r="P665" s="11" t="inlineStr"/>
-      <c r="Q665" s="12" t="inlineStr">
-        <is>
-          <t>Powerful Owl Park Pitch 1B</t>
-        </is>
-      </c>
+      <c r="Q665" s="12" t="inlineStr"/>
     </row>
     <row r="666">
       <c r="A666" s="9" t="inlineStr">
@@ -53354,7 +53366,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -53406,7 +53418,7 @@
     <row r="7">
       <c r="A7" s="17" t="inlineStr">
         <is>
-          <t>A.  Over-capacity moments: 7 found</t>
+          <t>A.  Over-capacity moments: 10 found</t>
         </is>
       </c>
     </row>
@@ -53772,130 +53784,265 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="20" t="n">
+        <v>8</v>
+      </c>
+      <c r="B16" s="20" t="inlineStr">
+        <is>
+          <t>08 Aug 2026</t>
+        </is>
+      </c>
+      <c r="C16" s="20" t="inlineStr">
+        <is>
+          <t>Pettys Reserve</t>
+        </is>
+      </c>
+      <c r="D16" s="20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E16" s="21" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="F16" s="20" t="inlineStr">
+        <is>
+          <t>09:10</t>
+        </is>
+      </c>
+      <c r="G16" s="21" t="inlineStr">
+        <is>
+          <t>Pitch over capacity</t>
+        </is>
+      </c>
+      <c r="H16" s="20" t="inlineStr">
+        <is>
+          <t>2×U10-13, 1×U8/9 = 1.25</t>
+        </is>
+      </c>
+      <c r="I16" s="20" t="inlineStr">
+        <is>
+          <t>08:30 U11 Pitch 1B (Bottom Field) (Manningham United Blues FC U11 MiniRoos - Wallabies Mixed (Culina's) v Whitehorse United SC U11 MiniRoos - Wallabies Mixed Vanntha)  |  08:30 U12 Pitch 1A (Bottom Field) (Manningham United Blues FC U12 Juniors - B Mixed (Chris) v Nunawading City FC U12 Juniors - B Mixed)  |  09:00 U08 Pitch 1C (Bottom Field) - Quarter Pitch 7v7 (Manningham United Blues FC U08 MiniRoos - Joeys Mixed (Duke's) v Manningham United Blues FC U08 MiniRoos - Joeys Mixed (Slater's))</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="18" t="n">
+        <v>9</v>
+      </c>
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>15 Aug 2026</t>
+        </is>
+      </c>
+      <c r="C17" s="18" t="inlineStr">
+        <is>
+          <t>Pettys Reserve</t>
+        </is>
+      </c>
+      <c r="D17" s="18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E17" s="19" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="F17" s="18" t="inlineStr">
+        <is>
+          <t>09:10</t>
+        </is>
+      </c>
+      <c r="G17" s="19" t="inlineStr">
+        <is>
+          <t>Pitch over capacity</t>
+        </is>
+      </c>
+      <c r="H17" s="18" t="inlineStr">
+        <is>
+          <t>2×U10-13, 1×U6/7 = 1.25</t>
+        </is>
+      </c>
+      <c r="I17" s="18" t="inlineStr">
+        <is>
+          <t>08:30 U07 Pitch 1E (Bottom Field) - Quarter Pitch 4v4 (Manningham United Blues FC U07 MiniRoos - Joeys Mixed (White) v Oakleigh Cannons FC U07 MiniRoos - Joeys Mixed OCFC Chippa/Jason)  |  08:30 U12 Pitch 1A (Bottom Field) (Manningham United Blues FC U12 Juniors - B Mixed (Andre) v FC Bulleen Lions U12 Juniors - B Mixed)  |  09:00  Pitch 1B (Bottom Field) (Manningham United Blues FC Girls Clinic v [MANUAL ADD])</t>
+        </is>
+      </c>
+    </row>
     <row r="18">
-      <c r="A18" s="22" t="inlineStr">
+      <c r="A18" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="B18" s="20" t="inlineStr">
+        <is>
+          <t>23 Aug 2026</t>
+        </is>
+      </c>
+      <c r="C18" s="20" t="inlineStr">
+        <is>
+          <t>Powerful Owl Park</t>
+        </is>
+      </c>
+      <c r="D18" s="20" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E18" s="21" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="F18" s="20" t="inlineStr">
+        <is>
+          <t>13:10</t>
+        </is>
+      </c>
+      <c r="G18" s="21" t="inlineStr">
+        <is>
+          <t>U14+ must have the pitch to itself</t>
+        </is>
+      </c>
+      <c r="H18" s="20" t="inlineStr">
+        <is>
+          <t>1×U14+, 1×U10-13 = 1.5</t>
+        </is>
+      </c>
+      <c r="I18" s="20" t="inlineStr">
+        <is>
+          <t>12:10 U13 Pitch 3 (Manningham United Blues FC U13 Juniors - B Mixed (Samir) v Mazenod FC U13 Juniors - B Mixed)  |  13:00 U18 Pitch 3 (Manningham United Blues FC U18 Juniors - A Male v West Preston SC U18 Juniors - A Male West Preston U/18A)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="22" t="inlineStr">
         <is>
           <t>B.  Peak simultaneous games per ground (busiest moment)</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>Ground</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>Max at once</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="D22" s="3" t="inlineStr">
         <is>
           <t>From</t>
         </is>
       </c>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="E22" s="3" t="inlineStr">
         <is>
           <t>Until</t>
         </is>
       </c>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="F22" s="3" t="inlineStr">
         <is>
           <t>Pitches in use then</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="21" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="19" t="inlineStr">
         <is>
           <t>Pettys Reserve</t>
         </is>
       </c>
-      <c r="B20" s="20" t="n">
+      <c r="B23" s="18" t="n">
         <v>7</v>
       </c>
-      <c r="C20" s="20" t="inlineStr">
+      <c r="C23" s="18" t="inlineStr">
         <is>
           <t>Sat 16 May 2026</t>
         </is>
       </c>
-      <c r="D20" s="20" t="inlineStr">
+      <c r="D23" s="18" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="E20" s="20" t="inlineStr">
+      <c r="E23" s="18" t="inlineStr">
         <is>
           <t>09:10</t>
         </is>
       </c>
-      <c r="F20" s="21" t="inlineStr">
+      <c r="F23" s="19" t="inlineStr">
         <is>
           <t>Pitch 1A (Bottom Field), Pitch 1B (Bottom Field), Pitch 1E (Bottom Field) - Quarter Pitch 4v4, Pitch 1F (Bottom Field) - Quarter Pitch 4v4, Pitch 2A (Top Field), Pitch 2C (Top Field) - Quarter Pitch 7v7, Pitch 2D (Top Field) - Quarter Pitch 7v7</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="19" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="21" t="inlineStr">
         <is>
           <t>Powerful Owl Park</t>
         </is>
       </c>
-      <c r="B21" s="18" t="n">
+      <c r="B24" s="20" t="n">
         <v>7</v>
       </c>
-      <c r="C21" s="18" t="inlineStr">
+      <c r="C24" s="20" t="inlineStr">
         <is>
           <t>Sun 09 Aug 2026</t>
         </is>
       </c>
-      <c r="D21" s="18" t="inlineStr">
+      <c r="D24" s="20" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="E21" s="18" t="inlineStr">
+      <c r="E24" s="20" t="inlineStr">
         <is>
           <t>09:10</t>
         </is>
       </c>
-      <c r="F21" s="19" t="inlineStr">
+      <c r="F24" s="21" t="inlineStr">
         <is>
           <t>Pitch 1 - Midi Field A, Pitch 1 - Midi Field B, Pitch 1B, Pitch 2A, Pitch 2B, Pitch 3A, Pitch 3B</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="21" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="19" t="inlineStr">
         <is>
           <t>Timber Ridge Reserve</t>
         </is>
       </c>
-      <c r="B22" s="20" t="n">
+      <c r="B25" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="C22" s="20" t="inlineStr">
+      <c r="C25" s="18" t="inlineStr">
         <is>
           <t>Sat 18 Jul 2026</t>
         </is>
       </c>
-      <c r="D22" s="20" t="inlineStr">
+      <c r="D25" s="18" t="inlineStr">
         <is>
           <t>09:40</t>
         </is>
       </c>
-      <c r="E22" s="20" t="inlineStr">
+      <c r="E25" s="18" t="inlineStr">
         <is>
           <t>10:40</t>
         </is>
       </c>
-      <c r="F22" s="21" t="inlineStr">
+      <c r="F25" s="19" t="inlineStr">
         <is>
           <t>Pitch 1A, Pitch 1B</t>
         </is>

</xml_diff>

<commit_message>
Move 23 Aug U13B (Samir) override to Powl Pitch 1, resolving the U18 clash
Vince re-targeted the 23 Aug 12:10 game from Pitch 3 to Pitch 1 (full pitch,
free at that time). Rewritten as a single override from the game's Dribl
location (Pitch 1 - Midi Field B) since overrides match raw fixtures and
don't chain. Clash count drops 2 -> 1; only the 30 Aug 5-min capacity blip
remains.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Puq4Xn23NC4d6RhNQLZP1N
</commit_message>
<xml_diff>
--- a/Manningham_fixtures_and_overlaps.xlsx
+++ b/Manningham_fixtures_and_overlaps.xlsx
@@ -680,7 +680,7 @@
         </is>
       </c>
       <c r="B11" s="8" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -49270,16 +49270,16 @@
       </c>
       <c r="C640" s="9" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>12:10</t>
         </is>
       </c>
       <c r="D640" s="9" t="inlineStr">
         <is>
-          <t>15:10</t>
+          <t>13:10</t>
         </is>
       </c>
       <c r="E640" s="9" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="F640" s="9" t="inlineStr">
         <is>
@@ -49303,27 +49303,27 @@
       </c>
       <c r="J640" s="9" t="inlineStr">
         <is>
-          <t>U16</t>
+          <t>U13</t>
         </is>
       </c>
       <c r="K640" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U16 Juniors - B Female (Eden)</t>
+          <t>Manningham United Blues FC U13 Juniors - B Mixed (Samir)</t>
         </is>
       </c>
       <c r="L640" s="10" t="inlineStr">
         <is>
-          <t>Glen Eira FC AAL - Junior Juniors - B Female Glen Eira FC - Van Egmonds</t>
+          <t>Mazenod FC U13 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="M640" s="10" t="inlineStr">
         <is>
-          <t>Junior Girls Sunday (U12 - U18)</t>
+          <t>Junior Mixed Sunday (U12 - U16)</t>
         </is>
       </c>
       <c r="N640" s="9" t="inlineStr">
         <is>
-          <t>Girls' South-East 16B</t>
+          <t>Mixed Sunday East 13B</t>
         </is>
       </c>
       <c r="O640" s="9" t="inlineStr">
@@ -49332,7 +49332,11 @@
         </is>
       </c>
       <c r="P640" s="9" t="inlineStr"/>
-      <c r="Q640" s="10" t="inlineStr"/>
+      <c r="Q640" s="10" t="inlineStr">
+        <is>
+          <t>Powerful Owl Park Pitch 1 - Midi Field B</t>
+        </is>
+      </c>
     </row>
     <row r="641">
       <c r="A641" s="11" t="inlineStr">
@@ -49347,16 +49351,16 @@
       </c>
       <c r="C641" s="11" t="inlineStr">
         <is>
-          <t>09:45</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D641" s="11" t="inlineStr">
         <is>
-          <t>10:45</t>
+          <t>15:10</t>
         </is>
       </c>
       <c r="E641" s="11" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F641" s="11" t="inlineStr">
         <is>
@@ -49365,7 +49369,7 @@
       </c>
       <c r="G641" s="11" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H641" s="11" t="inlineStr">
@@ -49375,32 +49379,32 @@
       </c>
       <c r="I641" s="12" t="inlineStr">
         <is>
-          <t>Pitch 2</t>
+          <t>Pitch 1</t>
         </is>
       </c>
       <c r="J641" s="11" t="inlineStr">
         <is>
-          <t>U14</t>
+          <t>U16</t>
         </is>
       </c>
       <c r="K641" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - A Mixed</t>
+          <t>Manningham United Blues FC U16 Juniors - B Female (Eden)</t>
         </is>
       </c>
       <c r="L641" s="12" t="inlineStr">
         <is>
-          <t>Boronia SC U14 Juniors - A Mixed Tristan</t>
+          <t>Glen Eira FC AAL - Junior Juniors - B Female Glen Eira FC - Van Egmonds</t>
         </is>
       </c>
       <c r="M641" s="12" t="inlineStr">
         <is>
-          <t>Junior Mixed Sunday (U12 - U16)</t>
+          <t>Junior Girls Sunday (U12 - U18)</t>
         </is>
       </c>
       <c r="N641" s="11" t="inlineStr">
         <is>
-          <t>Mixed East 14A</t>
+          <t>Girls' South-East 16B</t>
         </is>
       </c>
       <c r="O641" s="11" t="inlineStr">
@@ -49424,12 +49428,12 @@
       </c>
       <c r="C642" s="9" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>09:45</t>
         </is>
       </c>
       <c r="D642" s="9" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>10:45</t>
         </is>
       </c>
       <c r="E642" s="9" t="n">
@@ -49462,22 +49466,22 @@
       </c>
       <c r="K642" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - C Female (Christian)</t>
+          <t>Manningham United Blues FC U14 Juniors - A Mixed</t>
         </is>
       </c>
       <c r="L642" s="10" t="inlineStr">
         <is>
-          <t>Ashburton United SC U14 Juniors - C Female</t>
+          <t>Boronia SC U14 Juniors - A Mixed Tristan</t>
         </is>
       </c>
       <c r="M642" s="10" t="inlineStr">
         <is>
-          <t>Junior Girls Sunday (U12 - U18)</t>
+          <t>Junior Mixed Sunday (U12 - U16)</t>
         </is>
       </c>
       <c r="N642" s="9" t="inlineStr">
         <is>
-          <t>Girls' South-East 14C</t>
+          <t>Mixed East 14A</t>
         </is>
       </c>
       <c r="O642" s="9" t="inlineStr">
@@ -49501,12 +49505,12 @@
       </c>
       <c r="C643" s="11" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="D643" s="11" t="inlineStr">
         <is>
-          <t>14:15</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="E643" s="11" t="n">
@@ -49539,22 +49543,22 @@
       </c>
       <c r="K643" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - C Mixed (Phil)</t>
+          <t>Manningham United Blues FC U14 Juniors - C Female (Christian)</t>
         </is>
       </c>
       <c r="L643" s="12" t="inlineStr">
         <is>
-          <t>Mazenod FC U14 Juniors - C Mixed</t>
+          <t>Ashburton United SC U14 Juniors - C Female</t>
         </is>
       </c>
       <c r="M643" s="12" t="inlineStr">
         <is>
-          <t>Junior Mixed Sunday (U12 - U16)</t>
+          <t>Junior Girls Sunday (U12 - U18)</t>
         </is>
       </c>
       <c r="N643" s="11" t="inlineStr">
         <is>
-          <t>Mixed East 14C Red</t>
+          <t>Girls' South-East 14C</t>
         </is>
       </c>
       <c r="O643" s="11" t="inlineStr">
@@ -49578,16 +49582,16 @@
       </c>
       <c r="C644" s="9" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>13:15</t>
         </is>
       </c>
       <c r="D644" s="9" t="inlineStr">
         <is>
-          <t>16:10</t>
+          <t>14:15</t>
         </is>
       </c>
       <c r="E644" s="9" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="F644" s="9" t="inlineStr">
         <is>
@@ -49611,17 +49615,17 @@
       </c>
       <c r="J644" s="9" t="inlineStr">
         <is>
-          <t>U15</t>
+          <t>U14</t>
         </is>
       </c>
       <c r="K644" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U15 Juniors - B Mixed</t>
+          <t>Manningham United Blues FC U14 Juniors - C Mixed (Phil)</t>
         </is>
       </c>
       <c r="L644" s="10" t="inlineStr">
         <is>
-          <t>Bunyip &amp; District SC U15 Juniors - B Mixed</t>
+          <t>Mazenod FC U14 Juniors - C Mixed</t>
         </is>
       </c>
       <c r="M644" s="10" t="inlineStr">
@@ -49631,7 +49635,7 @@
       </c>
       <c r="N644" s="9" t="inlineStr">
         <is>
-          <t>Mixed South-East 15B</t>
+          <t>Mixed East 14C Red</t>
         </is>
       </c>
       <c r="O644" s="9" t="inlineStr">
@@ -49643,170 +49647,158 @@
       <c r="Q644" s="10" t="inlineStr"/>
     </row>
     <row r="645">
-      <c r="A645" s="13" t="inlineStr">
+      <c r="A645" s="11" t="inlineStr">
         <is>
           <t>23 Aug 2026</t>
         </is>
       </c>
-      <c r="B645" s="13" t="inlineStr">
+      <c r="B645" s="11" t="inlineStr">
         <is>
           <t>Sun</t>
         </is>
       </c>
-      <c r="C645" s="13" t="inlineStr">
-        <is>
-          <t>12:10</t>
-        </is>
-      </c>
-      <c r="D645" s="13" t="inlineStr">
-        <is>
-          <t>13:10</t>
-        </is>
-      </c>
-      <c r="E645" s="13" t="n">
-        <v>60</v>
-      </c>
-      <c r="F645" s="13" t="inlineStr">
+      <c r="C645" s="11" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D645" s="11" t="inlineStr">
+        <is>
+          <t>16:10</t>
+        </is>
+      </c>
+      <c r="E645" s="11" t="n">
+        <v>70</v>
+      </c>
+      <c r="F645" s="11" t="inlineStr">
         <is>
           <t>Powerful Owl Park</t>
         </is>
       </c>
-      <c r="G645" s="13" t="inlineStr">
+      <c r="G645" s="11" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H645" s="11" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="I645" s="12" t="inlineStr">
+        <is>
+          <t>Pitch 2</t>
+        </is>
+      </c>
+      <c r="J645" s="11" t="inlineStr">
+        <is>
+          <t>U15</t>
+        </is>
+      </c>
+      <c r="K645" s="12" t="inlineStr">
+        <is>
+          <t>Manningham United Blues FC U15 Juniors - B Mixed</t>
+        </is>
+      </c>
+      <c r="L645" s="12" t="inlineStr">
+        <is>
+          <t>Bunyip &amp; District SC U15 Juniors - B Mixed</t>
+        </is>
+      </c>
+      <c r="M645" s="12" t="inlineStr">
+        <is>
+          <t>Junior Mixed Sunday (U12 - U16)</t>
+        </is>
+      </c>
+      <c r="N645" s="11" t="inlineStr">
+        <is>
+          <t>Mixed South-East 15B</t>
+        </is>
+      </c>
+      <c r="O645" s="11" t="inlineStr">
+        <is>
+          <t>R16</t>
+        </is>
+      </c>
+      <c r="P645" s="11" t="inlineStr"/>
+      <c r="Q645" s="12" t="inlineStr"/>
+    </row>
+    <row r="646">
+      <c r="A646" s="9" t="inlineStr">
+        <is>
+          <t>23 Aug 2026</t>
+        </is>
+      </c>
+      <c r="B646" s="9" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
+      <c r="C646" s="9" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="D646" s="9" t="inlineStr">
+        <is>
+          <t>14:10</t>
+        </is>
+      </c>
+      <c r="E646" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F646" s="9" t="inlineStr">
+        <is>
+          <t>Powerful Owl Park</t>
+        </is>
+      </c>
+      <c r="G646" s="9" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="H645" s="13" t="inlineStr">
+      <c r="H646" s="9" t="inlineStr">
         <is>
           <t>Full</t>
         </is>
       </c>
-      <c r="I645" s="14" t="inlineStr">
+      <c r="I646" s="10" t="inlineStr">
         <is>
           <t>Pitch 3</t>
         </is>
       </c>
-      <c r="J645" s="13" t="inlineStr">
-        <is>
-          <t>U13</t>
-        </is>
-      </c>
-      <c r="K645" s="14" t="inlineStr">
-        <is>
-          <t>Manningham United Blues FC U13 Juniors - B Mixed (Samir)</t>
-        </is>
-      </c>
-      <c r="L645" s="14" t="inlineStr">
-        <is>
-          <t>Mazenod FC U13 Juniors - B Mixed</t>
-        </is>
-      </c>
-      <c r="M645" s="14" t="inlineStr">
-        <is>
-          <t>Junior Mixed Sunday (U12 - U16)</t>
-        </is>
-      </c>
-      <c r="N645" s="13" t="inlineStr">
-        <is>
-          <t>Mixed Sunday East 13B</t>
-        </is>
-      </c>
-      <c r="O645" s="13" t="inlineStr">
+      <c r="J646" s="9" t="inlineStr">
+        <is>
+          <t>U18</t>
+        </is>
+      </c>
+      <c r="K646" s="10" t="inlineStr">
+        <is>
+          <t>Manningham United Blues FC U18 Juniors - A Male</t>
+        </is>
+      </c>
+      <c r="L646" s="10" t="inlineStr">
+        <is>
+          <t>West Preston SC U18 Juniors - A Male West Preston U/18A</t>
+        </is>
+      </c>
+      <c r="M646" s="10" t="inlineStr">
+        <is>
+          <t>Junior Boys Sunday (U17 - U18)</t>
+        </is>
+      </c>
+      <c r="N646" s="9" t="inlineStr">
+        <is>
+          <t>Boys North-East 18A</t>
+        </is>
+      </c>
+      <c r="O646" s="9" t="inlineStr">
         <is>
           <t>R16</t>
         </is>
       </c>
-      <c r="P645" s="15" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="Q645" s="14" t="inlineStr">
-        <is>
-          <t>Powerful Owl Park Pitch 1 - Midi Field B</t>
-        </is>
-      </c>
-    </row>
-    <row r="646">
-      <c r="A646" s="13" t="inlineStr">
-        <is>
-          <t>23 Aug 2026</t>
-        </is>
-      </c>
-      <c r="B646" s="13" t="inlineStr">
-        <is>
-          <t>Sun</t>
-        </is>
-      </c>
-      <c r="C646" s="13" t="inlineStr">
-        <is>
-          <t>13:00</t>
-        </is>
-      </c>
-      <c r="D646" s="13" t="inlineStr">
-        <is>
-          <t>14:10</t>
-        </is>
-      </c>
-      <c r="E646" s="13" t="n">
-        <v>70</v>
-      </c>
-      <c r="F646" s="13" t="inlineStr">
-        <is>
-          <t>Powerful Owl Park</t>
-        </is>
-      </c>
-      <c r="G646" s="13" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="H646" s="13" t="inlineStr">
-        <is>
-          <t>Full</t>
-        </is>
-      </c>
-      <c r="I646" s="14" t="inlineStr">
-        <is>
-          <t>Pitch 3</t>
-        </is>
-      </c>
-      <c r="J646" s="13" t="inlineStr">
-        <is>
-          <t>U18</t>
-        </is>
-      </c>
-      <c r="K646" s="14" t="inlineStr">
-        <is>
-          <t>Manningham United Blues FC U18 Juniors - A Male</t>
-        </is>
-      </c>
-      <c r="L646" s="14" t="inlineStr">
-        <is>
-          <t>West Preston SC U18 Juniors - A Male West Preston U/18A</t>
-        </is>
-      </c>
-      <c r="M646" s="14" t="inlineStr">
-        <is>
-          <t>Junior Boys Sunday (U17 - U18)</t>
-        </is>
-      </c>
-      <c r="N646" s="13" t="inlineStr">
-        <is>
-          <t>Boys North-East 18A</t>
-        </is>
-      </c>
-      <c r="O646" s="13" t="inlineStr">
-        <is>
-          <t>R16</t>
-        </is>
-      </c>
-      <c r="P646" s="15" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="Q646" s="14" t="inlineStr"/>
+      <c r="P646" s="9" t="inlineStr"/>
+      <c r="Q646" s="10" t="inlineStr"/>
     </row>
     <row r="647">
       <c r="A647" s="11" t="inlineStr">
@@ -53366,7 +53358,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -53418,7 +53410,7 @@
     <row r="7">
       <c r="A7" s="17" t="inlineStr">
         <is>
-          <t>A.  Over-capacity moments: 10 found</t>
+          <t>A.  Over-capacity moments: 9 found</t>
         </is>
       </c>
     </row>
@@ -53874,94 +53866,79 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="20" t="n">
-        <v>10</v>
-      </c>
-      <c r="B18" s="20" t="inlineStr">
-        <is>
-          <t>23 Aug 2026</t>
-        </is>
-      </c>
-      <c r="C18" s="20" t="inlineStr">
-        <is>
-          <t>Powerful Owl Park</t>
-        </is>
-      </c>
-      <c r="D18" s="20" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E18" s="21" t="inlineStr">
-        <is>
-          <t>13:00</t>
-        </is>
-      </c>
-      <c r="F18" s="20" t="inlineStr">
-        <is>
-          <t>13:10</t>
-        </is>
-      </c>
-      <c r="G18" s="21" t="inlineStr">
-        <is>
-          <t>U14+ must have the pitch to itself</t>
-        </is>
-      </c>
-      <c r="H18" s="20" t="inlineStr">
-        <is>
-          <t>1×U14+, 1×U10-13 = 1.5</t>
-        </is>
-      </c>
-      <c r="I18" s="20" t="inlineStr">
-        <is>
-          <t>12:10 U13 Pitch 3 (Manningham United Blues FC U13 Juniors - B Mixed (Samir) v Mazenod FC U13 Juniors - B Mixed)  |  13:00 U18 Pitch 3 (Manningham United Blues FC U18 Juniors - A Male v West Preston SC U18 Juniors - A Male West Preston U/18A)</t>
+    <row r="20">
+      <c r="A20" s="22" t="inlineStr">
+        <is>
+          <t>B.  Peak simultaneous games per ground (busiest moment)</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="22" t="inlineStr">
-        <is>
-          <t>B.  Peak simultaneous games per ground (busiest moment)</t>
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Ground</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Max at once</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>From</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Until</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Pitches in use then</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>Ground</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>Max at once</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>From</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>Until</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>Pitches in use then</t>
+      <c r="A22" s="21" t="inlineStr">
+        <is>
+          <t>Pettys Reserve</t>
+        </is>
+      </c>
+      <c r="B22" s="20" t="n">
+        <v>7</v>
+      </c>
+      <c r="C22" s="20" t="inlineStr">
+        <is>
+          <t>Sat 16 May 2026</t>
+        </is>
+      </c>
+      <c r="D22" s="20" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="E22" s="20" t="inlineStr">
+        <is>
+          <t>09:10</t>
+        </is>
+      </c>
+      <c r="F22" s="21" t="inlineStr">
+        <is>
+          <t>Pitch 1A (Bottom Field), Pitch 1B (Bottom Field), Pitch 1E (Bottom Field) - Quarter Pitch 4v4, Pitch 1F (Bottom Field) - Quarter Pitch 4v4, Pitch 2A (Top Field), Pitch 2C (Top Field) - Quarter Pitch 7v7, Pitch 2D (Top Field) - Quarter Pitch 7v7</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="19" t="inlineStr">
         <is>
-          <t>Pettys Reserve</t>
+          <t>Powerful Owl Park</t>
         </is>
       </c>
       <c r="B23" s="18" t="n">
@@ -53969,7 +53946,7 @@
       </c>
       <c r="C23" s="18" t="inlineStr">
         <is>
-          <t>Sat 16 May 2026</t>
+          <t>Sun 09 Aug 2026</t>
         </is>
       </c>
       <c r="D23" s="18" t="inlineStr">
@@ -53984,65 +53961,35 @@
       </c>
       <c r="F23" s="19" t="inlineStr">
         <is>
-          <t>Pitch 1A (Bottom Field), Pitch 1B (Bottom Field), Pitch 1E (Bottom Field) - Quarter Pitch 4v4, Pitch 1F (Bottom Field) - Quarter Pitch 4v4, Pitch 2A (Top Field), Pitch 2C (Top Field) - Quarter Pitch 7v7, Pitch 2D (Top Field) - Quarter Pitch 7v7</t>
+          <t>Pitch 1 - Midi Field A, Pitch 1 - Midi Field B, Pitch 1B, Pitch 2A, Pitch 2B, Pitch 3A, Pitch 3B</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="21" t="inlineStr">
         <is>
-          <t>Powerful Owl Park</t>
+          <t>Timber Ridge Reserve</t>
         </is>
       </c>
       <c r="B24" s="20" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C24" s="20" t="inlineStr">
         <is>
-          <t>Sun 09 Aug 2026</t>
+          <t>Sat 18 Jul 2026</t>
         </is>
       </c>
       <c r="D24" s="20" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>09:40</t>
         </is>
       </c>
       <c r="E24" s="20" t="inlineStr">
         <is>
-          <t>09:10</t>
+          <t>10:40</t>
         </is>
       </c>
       <c r="F24" s="21" t="inlineStr">
-        <is>
-          <t>Pitch 1 - Midi Field A, Pitch 1 - Midi Field B, Pitch 1B, Pitch 2A, Pitch 2B, Pitch 3A, Pitch 3B</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="19" t="inlineStr">
-        <is>
-          <t>Timber Ridge Reserve</t>
-        </is>
-      </c>
-      <c r="B25" s="18" t="n">
-        <v>2</v>
-      </c>
-      <c r="C25" s="18" t="inlineStr">
-        <is>
-          <t>Sat 18 Jul 2026</t>
-        </is>
-      </c>
-      <c r="D25" s="18" t="inlineStr">
-        <is>
-          <t>09:40</t>
-        </is>
-      </c>
-      <c r="E25" s="18" t="inlineStr">
-        <is>
-          <t>10:40</t>
-        </is>
-      </c>
-      <c r="F25" s="19" t="inlineStr">
         <is>
           <t>Pitch 1A, Pitch 1B</t>
         </is>

</xml_diff>

<commit_message>
Move 23 Aug U13B (Samir) override to Powl Pitch 1, resolving the U18 clash (#22)
Vince re-targeted the 23 Aug 12:10 game from Pitch 3 to Pitch 1 (full pitch,
free at that time). Rewritten as a single override from the game's Dribl
location (Pitch 1 - Midi Field B) since overrides match raw fixtures and
don't chain. Clash count drops 2 -> 1; only the 30 Aug 5-min capacity blip
remains.


Claude-Session: https://claude.ai/code/session_01Puq4Xn23NC4d6RhNQLZP1N

Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Manningham_fixtures_and_overlaps.xlsx
+++ b/Manningham_fixtures_and_overlaps.xlsx
@@ -680,7 +680,7 @@
         </is>
       </c>
       <c r="B11" s="8" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -49270,16 +49270,16 @@
       </c>
       <c r="C640" s="9" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>12:10</t>
         </is>
       </c>
       <c r="D640" s="9" t="inlineStr">
         <is>
-          <t>15:10</t>
+          <t>13:10</t>
         </is>
       </c>
       <c r="E640" s="9" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="F640" s="9" t="inlineStr">
         <is>
@@ -49303,27 +49303,27 @@
       </c>
       <c r="J640" s="9" t="inlineStr">
         <is>
-          <t>U16</t>
+          <t>U13</t>
         </is>
       </c>
       <c r="K640" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U16 Juniors - B Female (Eden)</t>
+          <t>Manningham United Blues FC U13 Juniors - B Mixed (Samir)</t>
         </is>
       </c>
       <c r="L640" s="10" t="inlineStr">
         <is>
-          <t>Glen Eira FC AAL - Junior Juniors - B Female Glen Eira FC - Van Egmonds</t>
+          <t>Mazenod FC U13 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="M640" s="10" t="inlineStr">
         <is>
-          <t>Junior Girls Sunday (U12 - U18)</t>
+          <t>Junior Mixed Sunday (U12 - U16)</t>
         </is>
       </c>
       <c r="N640" s="9" t="inlineStr">
         <is>
-          <t>Girls' South-East 16B</t>
+          <t>Mixed Sunday East 13B</t>
         </is>
       </c>
       <c r="O640" s="9" t="inlineStr">
@@ -49332,7 +49332,11 @@
         </is>
       </c>
       <c r="P640" s="9" t="inlineStr"/>
-      <c r="Q640" s="10" t="inlineStr"/>
+      <c r="Q640" s="10" t="inlineStr">
+        <is>
+          <t>Powerful Owl Park Pitch 1 - Midi Field B</t>
+        </is>
+      </c>
     </row>
     <row r="641">
       <c r="A641" s="11" t="inlineStr">
@@ -49347,16 +49351,16 @@
       </c>
       <c r="C641" s="11" t="inlineStr">
         <is>
-          <t>09:45</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D641" s="11" t="inlineStr">
         <is>
-          <t>10:45</t>
+          <t>15:10</t>
         </is>
       </c>
       <c r="E641" s="11" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F641" s="11" t="inlineStr">
         <is>
@@ -49365,7 +49369,7 @@
       </c>
       <c r="G641" s="11" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H641" s="11" t="inlineStr">
@@ -49375,32 +49379,32 @@
       </c>
       <c r="I641" s="12" t="inlineStr">
         <is>
-          <t>Pitch 2</t>
+          <t>Pitch 1</t>
         </is>
       </c>
       <c r="J641" s="11" t="inlineStr">
         <is>
-          <t>U14</t>
+          <t>U16</t>
         </is>
       </c>
       <c r="K641" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - A Mixed</t>
+          <t>Manningham United Blues FC U16 Juniors - B Female (Eden)</t>
         </is>
       </c>
       <c r="L641" s="12" t="inlineStr">
         <is>
-          <t>Boronia SC U14 Juniors - A Mixed Tristan</t>
+          <t>Glen Eira FC AAL - Junior Juniors - B Female Glen Eira FC - Van Egmonds</t>
         </is>
       </c>
       <c r="M641" s="12" t="inlineStr">
         <is>
-          <t>Junior Mixed Sunday (U12 - U16)</t>
+          <t>Junior Girls Sunday (U12 - U18)</t>
         </is>
       </c>
       <c r="N641" s="11" t="inlineStr">
         <is>
-          <t>Mixed East 14A</t>
+          <t>Girls' South-East 16B</t>
         </is>
       </c>
       <c r="O641" s="11" t="inlineStr">
@@ -49424,12 +49428,12 @@
       </c>
       <c r="C642" s="9" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>09:45</t>
         </is>
       </c>
       <c r="D642" s="9" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>10:45</t>
         </is>
       </c>
       <c r="E642" s="9" t="n">
@@ -49462,22 +49466,22 @@
       </c>
       <c r="K642" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - C Female (Christian)</t>
+          <t>Manningham United Blues FC U14 Juniors - A Mixed</t>
         </is>
       </c>
       <c r="L642" s="10" t="inlineStr">
         <is>
-          <t>Ashburton United SC U14 Juniors - C Female</t>
+          <t>Boronia SC U14 Juniors - A Mixed Tristan</t>
         </is>
       </c>
       <c r="M642" s="10" t="inlineStr">
         <is>
-          <t>Junior Girls Sunday (U12 - U18)</t>
+          <t>Junior Mixed Sunday (U12 - U16)</t>
         </is>
       </c>
       <c r="N642" s="9" t="inlineStr">
         <is>
-          <t>Girls' South-East 14C</t>
+          <t>Mixed East 14A</t>
         </is>
       </c>
       <c r="O642" s="9" t="inlineStr">
@@ -49501,12 +49505,12 @@
       </c>
       <c r="C643" s="11" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="D643" s="11" t="inlineStr">
         <is>
-          <t>14:15</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="E643" s="11" t="n">
@@ -49539,22 +49543,22 @@
       </c>
       <c r="K643" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - C Mixed (Phil)</t>
+          <t>Manningham United Blues FC U14 Juniors - C Female (Christian)</t>
         </is>
       </c>
       <c r="L643" s="12" t="inlineStr">
         <is>
-          <t>Mazenod FC U14 Juniors - C Mixed</t>
+          <t>Ashburton United SC U14 Juniors - C Female</t>
         </is>
       </c>
       <c r="M643" s="12" t="inlineStr">
         <is>
-          <t>Junior Mixed Sunday (U12 - U16)</t>
+          <t>Junior Girls Sunday (U12 - U18)</t>
         </is>
       </c>
       <c r="N643" s="11" t="inlineStr">
         <is>
-          <t>Mixed East 14C Red</t>
+          <t>Girls' South-East 14C</t>
         </is>
       </c>
       <c r="O643" s="11" t="inlineStr">
@@ -49578,16 +49582,16 @@
       </c>
       <c r="C644" s="9" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>13:15</t>
         </is>
       </c>
       <c r="D644" s="9" t="inlineStr">
         <is>
-          <t>16:10</t>
+          <t>14:15</t>
         </is>
       </c>
       <c r="E644" s="9" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="F644" s="9" t="inlineStr">
         <is>
@@ -49611,17 +49615,17 @@
       </c>
       <c r="J644" s="9" t="inlineStr">
         <is>
-          <t>U15</t>
+          <t>U14</t>
         </is>
       </c>
       <c r="K644" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U15 Juniors - B Mixed</t>
+          <t>Manningham United Blues FC U14 Juniors - C Mixed (Phil)</t>
         </is>
       </c>
       <c r="L644" s="10" t="inlineStr">
         <is>
-          <t>Bunyip &amp; District SC U15 Juniors - B Mixed</t>
+          <t>Mazenod FC U14 Juniors - C Mixed</t>
         </is>
       </c>
       <c r="M644" s="10" t="inlineStr">
@@ -49631,7 +49635,7 @@
       </c>
       <c r="N644" s="9" t="inlineStr">
         <is>
-          <t>Mixed South-East 15B</t>
+          <t>Mixed East 14C Red</t>
         </is>
       </c>
       <c r="O644" s="9" t="inlineStr">
@@ -49643,170 +49647,158 @@
       <c r="Q644" s="10" t="inlineStr"/>
     </row>
     <row r="645">
-      <c r="A645" s="13" t="inlineStr">
+      <c r="A645" s="11" t="inlineStr">
         <is>
           <t>23 Aug 2026</t>
         </is>
       </c>
-      <c r="B645" s="13" t="inlineStr">
+      <c r="B645" s="11" t="inlineStr">
         <is>
           <t>Sun</t>
         </is>
       </c>
-      <c r="C645" s="13" t="inlineStr">
-        <is>
-          <t>12:10</t>
-        </is>
-      </c>
-      <c r="D645" s="13" t="inlineStr">
-        <is>
-          <t>13:10</t>
-        </is>
-      </c>
-      <c r="E645" s="13" t="n">
-        <v>60</v>
-      </c>
-      <c r="F645" s="13" t="inlineStr">
+      <c r="C645" s="11" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D645" s="11" t="inlineStr">
+        <is>
+          <t>16:10</t>
+        </is>
+      </c>
+      <c r="E645" s="11" t="n">
+        <v>70</v>
+      </c>
+      <c r="F645" s="11" t="inlineStr">
         <is>
           <t>Powerful Owl Park</t>
         </is>
       </c>
-      <c r="G645" s="13" t="inlineStr">
+      <c r="G645" s="11" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H645" s="11" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="I645" s="12" t="inlineStr">
+        <is>
+          <t>Pitch 2</t>
+        </is>
+      </c>
+      <c r="J645" s="11" t="inlineStr">
+        <is>
+          <t>U15</t>
+        </is>
+      </c>
+      <c r="K645" s="12" t="inlineStr">
+        <is>
+          <t>Manningham United Blues FC U15 Juniors - B Mixed</t>
+        </is>
+      </c>
+      <c r="L645" s="12" t="inlineStr">
+        <is>
+          <t>Bunyip &amp; District SC U15 Juniors - B Mixed</t>
+        </is>
+      </c>
+      <c r="M645" s="12" t="inlineStr">
+        <is>
+          <t>Junior Mixed Sunday (U12 - U16)</t>
+        </is>
+      </c>
+      <c r="N645" s="11" t="inlineStr">
+        <is>
+          <t>Mixed South-East 15B</t>
+        </is>
+      </c>
+      <c r="O645" s="11" t="inlineStr">
+        <is>
+          <t>R16</t>
+        </is>
+      </c>
+      <c r="P645" s="11" t="inlineStr"/>
+      <c r="Q645" s="12" t="inlineStr"/>
+    </row>
+    <row r="646">
+      <c r="A646" s="9" t="inlineStr">
+        <is>
+          <t>23 Aug 2026</t>
+        </is>
+      </c>
+      <c r="B646" s="9" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
+      <c r="C646" s="9" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="D646" s="9" t="inlineStr">
+        <is>
+          <t>14:10</t>
+        </is>
+      </c>
+      <c r="E646" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="F646" s="9" t="inlineStr">
+        <is>
+          <t>Powerful Owl Park</t>
+        </is>
+      </c>
+      <c r="G646" s="9" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="H645" s="13" t="inlineStr">
+      <c r="H646" s="9" t="inlineStr">
         <is>
           <t>Full</t>
         </is>
       </c>
-      <c r="I645" s="14" t="inlineStr">
+      <c r="I646" s="10" t="inlineStr">
         <is>
           <t>Pitch 3</t>
         </is>
       </c>
-      <c r="J645" s="13" t="inlineStr">
-        <is>
-          <t>U13</t>
-        </is>
-      </c>
-      <c r="K645" s="14" t="inlineStr">
-        <is>
-          <t>Manningham United Blues FC U13 Juniors - B Mixed (Samir)</t>
-        </is>
-      </c>
-      <c r="L645" s="14" t="inlineStr">
-        <is>
-          <t>Mazenod FC U13 Juniors - B Mixed</t>
-        </is>
-      </c>
-      <c r="M645" s="14" t="inlineStr">
-        <is>
-          <t>Junior Mixed Sunday (U12 - U16)</t>
-        </is>
-      </c>
-      <c r="N645" s="13" t="inlineStr">
-        <is>
-          <t>Mixed Sunday East 13B</t>
-        </is>
-      </c>
-      <c r="O645" s="13" t="inlineStr">
+      <c r="J646" s="9" t="inlineStr">
+        <is>
+          <t>U18</t>
+        </is>
+      </c>
+      <c r="K646" s="10" t="inlineStr">
+        <is>
+          <t>Manningham United Blues FC U18 Juniors - A Male</t>
+        </is>
+      </c>
+      <c r="L646" s="10" t="inlineStr">
+        <is>
+          <t>West Preston SC U18 Juniors - A Male West Preston U/18A</t>
+        </is>
+      </c>
+      <c r="M646" s="10" t="inlineStr">
+        <is>
+          <t>Junior Boys Sunday (U17 - U18)</t>
+        </is>
+      </c>
+      <c r="N646" s="9" t="inlineStr">
+        <is>
+          <t>Boys North-East 18A</t>
+        </is>
+      </c>
+      <c r="O646" s="9" t="inlineStr">
         <is>
           <t>R16</t>
         </is>
       </c>
-      <c r="P645" s="15" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="Q645" s="14" t="inlineStr">
-        <is>
-          <t>Powerful Owl Park Pitch 1 - Midi Field B</t>
-        </is>
-      </c>
-    </row>
-    <row r="646">
-      <c r="A646" s="13" t="inlineStr">
-        <is>
-          <t>23 Aug 2026</t>
-        </is>
-      </c>
-      <c r="B646" s="13" t="inlineStr">
-        <is>
-          <t>Sun</t>
-        </is>
-      </c>
-      <c r="C646" s="13" t="inlineStr">
-        <is>
-          <t>13:00</t>
-        </is>
-      </c>
-      <c r="D646" s="13" t="inlineStr">
-        <is>
-          <t>14:10</t>
-        </is>
-      </c>
-      <c r="E646" s="13" t="n">
-        <v>70</v>
-      </c>
-      <c r="F646" s="13" t="inlineStr">
-        <is>
-          <t>Powerful Owl Park</t>
-        </is>
-      </c>
-      <c r="G646" s="13" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="H646" s="13" t="inlineStr">
-        <is>
-          <t>Full</t>
-        </is>
-      </c>
-      <c r="I646" s="14" t="inlineStr">
-        <is>
-          <t>Pitch 3</t>
-        </is>
-      </c>
-      <c r="J646" s="13" t="inlineStr">
-        <is>
-          <t>U18</t>
-        </is>
-      </c>
-      <c r="K646" s="14" t="inlineStr">
-        <is>
-          <t>Manningham United Blues FC U18 Juniors - A Male</t>
-        </is>
-      </c>
-      <c r="L646" s="14" t="inlineStr">
-        <is>
-          <t>West Preston SC U18 Juniors - A Male West Preston U/18A</t>
-        </is>
-      </c>
-      <c r="M646" s="14" t="inlineStr">
-        <is>
-          <t>Junior Boys Sunday (U17 - U18)</t>
-        </is>
-      </c>
-      <c r="N646" s="13" t="inlineStr">
-        <is>
-          <t>Boys North-East 18A</t>
-        </is>
-      </c>
-      <c r="O646" s="13" t="inlineStr">
-        <is>
-          <t>R16</t>
-        </is>
-      </c>
-      <c r="P646" s="15" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="Q646" s="14" t="inlineStr"/>
+      <c r="P646" s="9" t="inlineStr"/>
+      <c r="Q646" s="10" t="inlineStr"/>
     </row>
     <row r="647">
       <c r="A647" s="11" t="inlineStr">
@@ -53366,7 +53358,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -53418,7 +53410,7 @@
     <row r="7">
       <c r="A7" s="17" t="inlineStr">
         <is>
-          <t>A.  Over-capacity moments: 10 found</t>
+          <t>A.  Over-capacity moments: 9 found</t>
         </is>
       </c>
     </row>
@@ -53874,94 +53866,79 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="20" t="n">
-        <v>10</v>
-      </c>
-      <c r="B18" s="20" t="inlineStr">
-        <is>
-          <t>23 Aug 2026</t>
-        </is>
-      </c>
-      <c r="C18" s="20" t="inlineStr">
-        <is>
-          <t>Powerful Owl Park</t>
-        </is>
-      </c>
-      <c r="D18" s="20" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E18" s="21" t="inlineStr">
-        <is>
-          <t>13:00</t>
-        </is>
-      </c>
-      <c r="F18" s="20" t="inlineStr">
-        <is>
-          <t>13:10</t>
-        </is>
-      </c>
-      <c r="G18" s="21" t="inlineStr">
-        <is>
-          <t>U14+ must have the pitch to itself</t>
-        </is>
-      </c>
-      <c r="H18" s="20" t="inlineStr">
-        <is>
-          <t>1×U14+, 1×U10-13 = 1.5</t>
-        </is>
-      </c>
-      <c r="I18" s="20" t="inlineStr">
-        <is>
-          <t>12:10 U13 Pitch 3 (Manningham United Blues FC U13 Juniors - B Mixed (Samir) v Mazenod FC U13 Juniors - B Mixed)  |  13:00 U18 Pitch 3 (Manningham United Blues FC U18 Juniors - A Male v West Preston SC U18 Juniors - A Male West Preston U/18A)</t>
+    <row r="20">
+      <c r="A20" s="22" t="inlineStr">
+        <is>
+          <t>B.  Peak simultaneous games per ground (busiest moment)</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="22" t="inlineStr">
-        <is>
-          <t>B.  Peak simultaneous games per ground (busiest moment)</t>
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Ground</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Max at once</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>From</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Until</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Pitches in use then</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>Ground</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>Max at once</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>From</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>Until</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>Pitches in use then</t>
+      <c r="A22" s="21" t="inlineStr">
+        <is>
+          <t>Pettys Reserve</t>
+        </is>
+      </c>
+      <c r="B22" s="20" t="n">
+        <v>7</v>
+      </c>
+      <c r="C22" s="20" t="inlineStr">
+        <is>
+          <t>Sat 16 May 2026</t>
+        </is>
+      </c>
+      <c r="D22" s="20" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="E22" s="20" t="inlineStr">
+        <is>
+          <t>09:10</t>
+        </is>
+      </c>
+      <c r="F22" s="21" t="inlineStr">
+        <is>
+          <t>Pitch 1A (Bottom Field), Pitch 1B (Bottom Field), Pitch 1E (Bottom Field) - Quarter Pitch 4v4, Pitch 1F (Bottom Field) - Quarter Pitch 4v4, Pitch 2A (Top Field), Pitch 2C (Top Field) - Quarter Pitch 7v7, Pitch 2D (Top Field) - Quarter Pitch 7v7</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="19" t="inlineStr">
         <is>
-          <t>Pettys Reserve</t>
+          <t>Powerful Owl Park</t>
         </is>
       </c>
       <c r="B23" s="18" t="n">
@@ -53969,7 +53946,7 @@
       </c>
       <c r="C23" s="18" t="inlineStr">
         <is>
-          <t>Sat 16 May 2026</t>
+          <t>Sun 09 Aug 2026</t>
         </is>
       </c>
       <c r="D23" s="18" t="inlineStr">
@@ -53984,65 +53961,35 @@
       </c>
       <c r="F23" s="19" t="inlineStr">
         <is>
-          <t>Pitch 1A (Bottom Field), Pitch 1B (Bottom Field), Pitch 1E (Bottom Field) - Quarter Pitch 4v4, Pitch 1F (Bottom Field) - Quarter Pitch 4v4, Pitch 2A (Top Field), Pitch 2C (Top Field) - Quarter Pitch 7v7, Pitch 2D (Top Field) - Quarter Pitch 7v7</t>
+          <t>Pitch 1 - Midi Field A, Pitch 1 - Midi Field B, Pitch 1B, Pitch 2A, Pitch 2B, Pitch 3A, Pitch 3B</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="21" t="inlineStr">
         <is>
-          <t>Powerful Owl Park</t>
+          <t>Timber Ridge Reserve</t>
         </is>
       </c>
       <c r="B24" s="20" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C24" s="20" t="inlineStr">
         <is>
-          <t>Sun 09 Aug 2026</t>
+          <t>Sat 18 Jul 2026</t>
         </is>
       </c>
       <c r="D24" s="20" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>09:40</t>
         </is>
       </c>
       <c r="E24" s="20" t="inlineStr">
         <is>
-          <t>09:10</t>
+          <t>10:40</t>
         </is>
       </c>
       <c r="F24" s="21" t="inlineStr">
-        <is>
-          <t>Pitch 1 - Midi Field A, Pitch 1 - Midi Field B, Pitch 1B, Pitch 2A, Pitch 2B, Pitch 3A, Pitch 3B</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="19" t="inlineStr">
-        <is>
-          <t>Timber Ridge Reserve</t>
-        </is>
-      </c>
-      <c r="B25" s="18" t="n">
-        <v>2</v>
-      </c>
-      <c r="C25" s="18" t="inlineStr">
-        <is>
-          <t>Sat 18 Jul 2026</t>
-        </is>
-      </c>
-      <c r="D25" s="18" t="inlineStr">
-        <is>
-          <t>09:40</t>
-        </is>
-      </c>
-      <c r="E25" s="18" t="inlineStr">
-        <is>
-          <t>10:40</t>
-        </is>
-      </c>
-      <c r="F25" s="19" t="inlineStr">
         <is>
           <t>Pitch 1A, Pitch 1B</t>
         </is>

</xml_diff>

<commit_message>
Auto-refresh fixtures from Dribl (2026-08-17)
</commit_message>
<xml_diff>
--- a/Manningham_fixtures_and_overlaps.xlsx
+++ b/Manningham_fixtures_and_overlaps.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Games" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overlaps &amp; Peak Load" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="All Games" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Overlaps &amp; Peak Load" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Games'!$A$1:$Q$692</definedName>

</xml_diff>

<commit_message>
Auto-refresh fixtures from Dribl (2026-08-20)
</commit_message>
<xml_diff>
--- a/Manningham_fixtures_and_overlaps.xlsx
+++ b/Manningham_fixtures_and_overlaps.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Overlaps &amp; Peak Load" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Games'!$A$1:$Q$692</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Games'!$A$1:$Q$691</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -596,7 +596,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Source: fv.dribl.com, 2026 season, generated 19 Aug 2026</t>
+          <t>Source: fv.dribl.com, 2026 season, generated 20 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
@@ -669,7 +669,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="C9" s="7" t="inlineStr"/>
     </row>
@@ -694,7 +694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q692"/>
+  <dimension ref="A1:Q691"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -49505,12 +49505,12 @@
       </c>
       <c r="C643" s="11" t="inlineStr">
         <is>
-          <t>09:45</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="D643" s="11" t="inlineStr">
         <is>
-          <t>10:45</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="E643" s="11" t="n">
@@ -49543,22 +49543,22 @@
       </c>
       <c r="K643" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - A Mixed</t>
+          <t>Manningham United Blues FC U14 Juniors - C Female (Christian)</t>
         </is>
       </c>
       <c r="L643" s="12" t="inlineStr">
         <is>
-          <t>Boronia SC U14 Juniors - A Mixed Tristan</t>
+          <t>Ashburton United SC U14 Juniors - C Female</t>
         </is>
       </c>
       <c r="M643" s="12" t="inlineStr">
         <is>
-          <t>Junior Mixed Sunday (U12 - U16)</t>
+          <t>Junior Girls Sunday (U12 - U18)</t>
         </is>
       </c>
       <c r="N643" s="11" t="inlineStr">
         <is>
-          <t>Mixed East 14A</t>
+          <t>Girls' South-East 14C</t>
         </is>
       </c>
       <c r="O643" s="11" t="inlineStr">
@@ -49582,12 +49582,12 @@
       </c>
       <c r="C644" s="9" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>13:15</t>
         </is>
       </c>
       <c r="D644" s="9" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>14:15</t>
         </is>
       </c>
       <c r="E644" s="9" t="n">
@@ -49620,22 +49620,22 @@
       </c>
       <c r="K644" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - C Female (Christian)</t>
+          <t>Manningham United Blues FC U14 Juniors - C Mixed (Phil)</t>
         </is>
       </c>
       <c r="L644" s="10" t="inlineStr">
         <is>
-          <t>Ashburton United SC U14 Juniors - C Female</t>
+          <t>Mazenod FC U14 Juniors - C Mixed</t>
         </is>
       </c>
       <c r="M644" s="10" t="inlineStr">
         <is>
-          <t>Junior Girls Sunday (U12 - U18)</t>
+          <t>Junior Mixed Sunday (U12 - U16)</t>
         </is>
       </c>
       <c r="N644" s="9" t="inlineStr">
         <is>
-          <t>Girls' South-East 14C</t>
+          <t>Mixed East 14C Red</t>
         </is>
       </c>
       <c r="O644" s="9" t="inlineStr">
@@ -49659,16 +49659,16 @@
       </c>
       <c r="C645" s="11" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="D645" s="11" t="inlineStr">
         <is>
-          <t>14:15</t>
+          <t>16:10</t>
         </is>
       </c>
       <c r="E645" s="11" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F645" s="11" t="inlineStr">
         <is>
@@ -49692,17 +49692,17 @@
       </c>
       <c r="J645" s="11" t="inlineStr">
         <is>
-          <t>U14</t>
+          <t>U15</t>
         </is>
       </c>
       <c r="K645" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - C Mixed (Phil)</t>
+          <t>Manningham United Blues FC U15 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="L645" s="12" t="inlineStr">
         <is>
-          <t>Mazenod FC U14 Juniors - C Mixed</t>
+          <t>Bunyip &amp; District SC U15 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="M645" s="12" t="inlineStr">
@@ -49712,7 +49712,7 @@
       </c>
       <c r="N645" s="11" t="inlineStr">
         <is>
-          <t>Mixed East 14C Red</t>
+          <t>Mixed South-East 15B</t>
         </is>
       </c>
       <c r="O645" s="11" t="inlineStr">
@@ -49736,12 +49736,12 @@
       </c>
       <c r="C646" s="9" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="D646" s="9" t="inlineStr">
         <is>
-          <t>16:10</t>
+          <t>14:10</t>
         </is>
       </c>
       <c r="E646" s="9" t="n">
@@ -49754,7 +49754,7 @@
       </c>
       <c r="G646" s="9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H646" s="9" t="inlineStr">
@@ -49764,32 +49764,32 @@
       </c>
       <c r="I646" s="10" t="inlineStr">
         <is>
-          <t>Pitch 2</t>
+          <t>Pitch 3</t>
         </is>
       </c>
       <c r="J646" s="9" t="inlineStr">
         <is>
-          <t>U15</t>
+          <t>U18</t>
         </is>
       </c>
       <c r="K646" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U15 Juniors - B Mixed</t>
+          <t>Manningham United Blues FC U18 Juniors - A Male</t>
         </is>
       </c>
       <c r="L646" s="10" t="inlineStr">
         <is>
-          <t>Bunyip &amp; District SC U15 Juniors - B Mixed</t>
+          <t>West Preston SC U18 Juniors - A Male West Preston U/18A</t>
         </is>
       </c>
       <c r="M646" s="10" t="inlineStr">
         <is>
-          <t>Junior Mixed Sunday (U12 - U16)</t>
+          <t>Junior Boys Sunday (U17 - U18)</t>
         </is>
       </c>
       <c r="N646" s="9" t="inlineStr">
         <is>
-          <t>Mixed South-East 15B</t>
+          <t>Boys North-East 18A</t>
         </is>
       </c>
       <c r="O646" s="9" t="inlineStr">
@@ -49813,16 +49813,16 @@
       </c>
       <c r="C647" s="11" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="D647" s="11" t="inlineStr">
         <is>
-          <t>14:10</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="E647" s="11" t="n">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="F647" s="11" t="inlineStr">
         <is>
@@ -49846,27 +49846,27 @@
       </c>
       <c r="J647" s="11" t="inlineStr">
         <is>
-          <t>U18</t>
+          <t>U21</t>
         </is>
       </c>
       <c r="K647" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U18 Juniors - A Male</t>
+          <t>Manningham United Blues FC U21 Reilly</t>
         </is>
       </c>
       <c r="L647" s="12" t="inlineStr">
         <is>
-          <t>West Preston SC U18 Juniors - A Male West Preston U/18A</t>
+          <t>FC Bulleen Lions U21</t>
         </is>
       </c>
       <c r="M647" s="12" t="inlineStr">
         <is>
-          <t>Junior Boys Sunday (U17 - U18)</t>
+          <t>Men's Metropolitan Under 21</t>
         </is>
       </c>
       <c r="N647" s="11" t="inlineStr">
         <is>
-          <t>Boys North-East 18A</t>
+          <t>Men's Metropolitan League U21 - North-East</t>
         </is>
       </c>
       <c r="O647" s="11" t="inlineStr">
@@ -49880,7 +49880,7 @@
     <row r="648">
       <c r="A648" s="9" t="inlineStr">
         <is>
-          <t>23 Aug 2026</t>
+          <t>30 Aug 2026</t>
         </is>
       </c>
       <c r="B648" s="9" t="inlineStr">
@@ -49890,16 +49890,16 @@
       </c>
       <c r="C648" s="9" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="D648" s="9" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>09:40</t>
         </is>
       </c>
       <c r="E648" s="9" t="n">
-        <v>90</v>
+        <v>40</v>
       </c>
       <c r="F648" s="9" t="inlineStr">
         <is>
@@ -49908,47 +49908,47 @@
       </c>
       <c r="G648" s="9" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H648" s="9" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Sub</t>
         </is>
       </c>
       <c r="I648" s="10" t="inlineStr">
         <is>
-          <t>Pitch 3</t>
+          <t>Pitch 1 - Midi Field B</t>
         </is>
       </c>
       <c r="J648" s="9" t="inlineStr">
         <is>
-          <t>U21</t>
+          <t>U09</t>
         </is>
       </c>
       <c r="K648" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U21 Reilly</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Female (Nat &amp; Chloe)</t>
         </is>
       </c>
       <c r="L648" s="10" t="inlineStr">
         <is>
-          <t>FC Bulleen Lions U21</t>
+          <t>Essendon Royals SC U09 MiniRoos - Wallabies Female U9 RED</t>
         </is>
       </c>
       <c r="M648" s="10" t="inlineStr">
         <is>
-          <t>Men's Metropolitan Under 21</t>
+          <t>Coles MiniRoos Girls' Sunday (U6 - U11)</t>
         </is>
       </c>
       <c r="N648" s="9" t="inlineStr">
         <is>
-          <t>Men's Metropolitan League U21 - North-East</t>
+          <t>Coles MiniRoos Girls' North-East 9 Wallabies</t>
         </is>
       </c>
       <c r="O648" s="9" t="inlineStr">
         <is>
-          <t>R16</t>
+          <t>R17</t>
         </is>
       </c>
       <c r="P648" s="9" t="inlineStr"/>
@@ -49995,32 +49995,32 @@
       </c>
       <c r="I649" s="12" t="inlineStr">
         <is>
-          <t>Pitch 1 - Midi Field B</t>
+          <t>Pitch 1B</t>
         </is>
       </c>
       <c r="J649" s="11" t="inlineStr">
         <is>
-          <t>U09</t>
+          <t>U08</t>
         </is>
       </c>
       <c r="K649" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Female (Nat &amp; Chloe)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Kangaroos Mixed (Arnold's)</t>
         </is>
       </c>
       <c r="L649" s="12" t="inlineStr">
         <is>
-          <t>Essendon Royals SC U09 MiniRoos - Wallabies Female U9 RED</t>
+          <t>Mazenod FC U08 MiniRoos - Kangaroos Mixed</t>
         </is>
       </c>
       <c r="M649" s="12" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Girls' Sunday (U6 - U11)</t>
+          <t>Coles MiniRoos Mixed Sunday (U6 - U11)</t>
         </is>
       </c>
       <c r="N649" s="11" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Girls' North-East 9 Wallabies</t>
+          <t>Coles MiniRoos Mixed Sunday South-East 8 Kangaroos</t>
         </is>
       </c>
       <c r="O649" s="11" t="inlineStr">
@@ -50072,7 +50072,7 @@
       </c>
       <c r="I650" s="10" t="inlineStr">
         <is>
-          <t>Pitch 1B</t>
+          <t>Pitch 1 - Midi Field A</t>
         </is>
       </c>
       <c r="J650" s="9" t="inlineStr">
@@ -50082,12 +50082,12 @@
       </c>
       <c r="K650" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Kangaroos Mixed (Arnold's)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Wallabies Mixed (Coe's)</t>
         </is>
       </c>
       <c r="L650" s="10" t="inlineStr">
         <is>
-          <t>Mazenod FC U08 MiniRoos - Kangaroos Mixed</t>
+          <t>East Malvern Junior SC U08 MiniRoos - Wallabies Mixed EMJSC U8 Sunday Red</t>
         </is>
       </c>
       <c r="M650" s="10" t="inlineStr">
@@ -50097,7 +50097,7 @@
       </c>
       <c r="N650" s="9" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Sunday South-East 8 Kangaroos</t>
+          <t>Coles MiniRoos Mixed Sunday East 8 Wallabies</t>
         </is>
       </c>
       <c r="O650" s="9" t="inlineStr">
@@ -50121,12 +50121,12 @@
       </c>
       <c r="C651" s="11" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>10:10</t>
         </is>
       </c>
       <c r="D651" s="11" t="inlineStr">
         <is>
-          <t>09:40</t>
+          <t>10:50</t>
         </is>
       </c>
       <c r="E651" s="11" t="n">
@@ -50154,27 +50154,27 @@
       </c>
       <c r="J651" s="11" t="inlineStr">
         <is>
-          <t>U08</t>
+          <t>U11</t>
         </is>
       </c>
       <c r="K651" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Wallabies Mixed (Coe's)</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Joeys Female (Grace)</t>
         </is>
       </c>
       <c r="L651" s="12" t="inlineStr">
         <is>
-          <t>East Malvern Junior SC U08 MiniRoos - Wallabies Mixed EMJSC U8 Sunday Red</t>
+          <t>Croydon City SC U11 MiniRoos - Joeys Female U11 - CCSC</t>
         </is>
       </c>
       <c r="M651" s="12" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Sunday (U6 - U11)</t>
+          <t>Coles MiniRoos Girls' Sunday (U6 - U11)</t>
         </is>
       </c>
       <c r="N651" s="11" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Sunday East 8 Wallabies</t>
+          <t>Coles MiniRoos Girls' East 11 Joeys</t>
         </is>
       </c>
       <c r="O651" s="11" t="inlineStr">
@@ -50226,32 +50226,32 @@
       </c>
       <c r="I652" s="10" t="inlineStr">
         <is>
-          <t>Pitch 1 - Midi Field A</t>
+          <t>Pitch 1 - Midi Field B</t>
         </is>
       </c>
       <c r="J652" s="9" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>U09</t>
         </is>
       </c>
       <c r="K652" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Joeys Female (Grace)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Cahill's)</t>
         </is>
       </c>
       <c r="L652" s="10" t="inlineStr">
         <is>
-          <t>Croydon City SC U11 MiniRoos - Joeys Female U11 - CCSC</t>
+          <t>Ashburton United SC U09 MiniRoos - Wallabies Mixed (Leo)</t>
         </is>
       </c>
       <c r="M652" s="10" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Girls' Sunday (U6 - U11)</t>
+          <t>Coles MiniRoos Mixed Sunday (U6 - U11)</t>
         </is>
       </c>
       <c r="N652" s="9" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Girls' East 11 Joeys</t>
+          <t>Coles MiniRoos Mixed Sunday East 9 Wallabies</t>
         </is>
       </c>
       <c r="O652" s="9" t="inlineStr">
@@ -50303,7 +50303,7 @@
       </c>
       <c r="I653" s="12" t="inlineStr">
         <is>
-          <t>Pitch 1 - Midi Field B</t>
+          <t>Pitch 1B</t>
         </is>
       </c>
       <c r="J653" s="11" t="inlineStr">
@@ -50313,12 +50313,12 @@
       </c>
       <c r="K653" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Cahill's)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Kangaroos Mixed (Emerton's)</t>
         </is>
       </c>
       <c r="L653" s="12" t="inlineStr">
         <is>
-          <t>Ashburton United SC U09 MiniRoos - Wallabies Mixed (Leo)</t>
+          <t>Monash City Villarreal FC U09 MiniRoos - Kangaroos Mixed Monash City Villarreal FC U8 Yellow</t>
         </is>
       </c>
       <c r="M653" s="12" t="inlineStr">
@@ -50328,7 +50328,7 @@
       </c>
       <c r="N653" s="11" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Sunday East 9 Wallabies</t>
+          <t>Coles MiniRoos Mixed Sunday East 9 Kangaroos Red</t>
         </is>
       </c>
       <c r="O653" s="11" t="inlineStr">
@@ -50352,16 +50352,16 @@
       </c>
       <c r="C654" s="9" t="inlineStr">
         <is>
-          <t>10:10</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="D654" s="9" t="inlineStr">
         <is>
-          <t>10:50</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="E654" s="9" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="F654" s="9" t="inlineStr">
         <is>
@@ -50385,27 +50385,27 @@
       </c>
       <c r="J654" s="9" t="inlineStr">
         <is>
-          <t>U09</t>
+          <t>U13</t>
         </is>
       </c>
       <c r="K654" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Kangaroos Mixed (Emerton's)</t>
+          <t>Manningham United Blues FC U13 Juniors - C Mixed (Martin)</t>
         </is>
       </c>
       <c r="L654" s="10" t="inlineStr">
         <is>
-          <t>Monash City Villarreal FC U09 MiniRoos - Kangaroos Mixed Monash City Villarreal FC U8 Yellow</t>
+          <t>Whitehorse United SC U13 Juniors - C Mixed Shane</t>
         </is>
       </c>
       <c r="M654" s="10" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Sunday (U6 - U11)</t>
+          <t>Junior Mixed Sunday (U12 - U16)</t>
         </is>
       </c>
       <c r="N654" s="9" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Sunday East 9 Kangaroos Red</t>
+          <t>Mixed Sunday East 13C Red</t>
         </is>
       </c>
       <c r="O654" s="9" t="inlineStr">
@@ -50434,11 +50434,11 @@
       </c>
       <c r="D655" s="11" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>12:10</t>
         </is>
       </c>
       <c r="E655" s="11" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="F655" s="11" t="inlineStr">
         <is>
@@ -50457,32 +50457,32 @@
       </c>
       <c r="I655" s="12" t="inlineStr">
         <is>
-          <t>Pitch 1B</t>
+          <t>Pitch 1 - Midi Field B</t>
         </is>
       </c>
       <c r="J655" s="11" t="inlineStr">
         <is>
-          <t>U13</t>
+          <t>U11</t>
         </is>
       </c>
       <c r="K655" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - C Mixed (Martin)</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Female Miniroos Girls U11W (Holly &amp; Marina)</t>
         </is>
       </c>
       <c r="L655" s="12" t="inlineStr">
         <is>
-          <t>Whitehorse United SC U13 Juniors - C Mixed Shane</t>
+          <t>Malvern City FC U11 MiniRoos - Wallabies Female U11 MCFC Girls</t>
         </is>
       </c>
       <c r="M655" s="12" t="inlineStr">
         <is>
-          <t>Junior Mixed Sunday (U12 - U16)</t>
+          <t>Coles MiniRoos Girls' Sunday (U6 - U11)</t>
         </is>
       </c>
       <c r="N655" s="11" t="inlineStr">
         <is>
-          <t>Mixed Sunday East 13C Red</t>
+          <t>Coles MiniRoos Girls' East 11 Wallabies</t>
         </is>
       </c>
       <c r="O655" s="11" t="inlineStr">
@@ -50506,16 +50506,16 @@
       </c>
       <c r="C656" s="9" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="D656" s="9" t="inlineStr">
         <is>
-          <t>12:10</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="E656" s="9" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="F656" s="9" t="inlineStr">
         <is>
@@ -50529,37 +50529,37 @@
       </c>
       <c r="H656" s="9" t="inlineStr">
         <is>
-          <t>Sub</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="I656" s="10" t="inlineStr">
         <is>
-          <t>Pitch 1 - Midi Field B</t>
+          <t>Pitch 1</t>
         </is>
       </c>
       <c r="J656" s="9" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>U14</t>
         </is>
       </c>
       <c r="K656" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Female Miniroos Girls U11W (Holly &amp; Marina)</t>
+          <t>Manningham United Blues FC U14 Juniors - A Female (Chloe)</t>
         </is>
       </c>
       <c r="L656" s="10" t="inlineStr">
         <is>
-          <t>Malvern City FC U11 MiniRoos - Wallabies Female U11 MCFC Girls</t>
+          <t>Alamein FC U14 Juniors - A Female</t>
         </is>
       </c>
       <c r="M656" s="10" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Girls' Sunday (U6 - U11)</t>
+          <t>Junior Girls Sunday (U12 - U18)</t>
         </is>
       </c>
       <c r="N656" s="9" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Girls' East 11 Wallabies</t>
+          <t>Girls' South-East 14A</t>
         </is>
       </c>
       <c r="O656" s="9" t="inlineStr">
@@ -50583,16 +50583,16 @@
       </c>
       <c r="C657" s="11" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>14:45</t>
         </is>
       </c>
       <c r="D657" s="11" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>15:55</t>
         </is>
       </c>
       <c r="E657" s="11" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F657" s="11" t="inlineStr">
         <is>
@@ -50616,17 +50616,17 @@
       </c>
       <c r="J657" s="11" t="inlineStr">
         <is>
-          <t>U14</t>
+          <t>U17/18</t>
         </is>
       </c>
       <c r="K657" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - A Female (Chloe)</t>
+          <t>Manningham United Blues FC U17/18 Juniors - B Female (Marilyn)</t>
         </is>
       </c>
       <c r="L657" s="12" t="inlineStr">
         <is>
-          <t>Alamein FC U14 Juniors - A Female</t>
+          <t>Mount Eliza SC U17/18 Juniors - B Female Red</t>
         </is>
       </c>
       <c r="M657" s="12" t="inlineStr">
@@ -50636,7 +50636,7 @@
       </c>
       <c r="N657" s="11" t="inlineStr">
         <is>
-          <t>Girls' South-East 14A</t>
+          <t>Girls' South-East 17/18B</t>
         </is>
       </c>
       <c r="O657" s="11" t="inlineStr">
@@ -50660,16 +50660,16 @@
       </c>
       <c r="C658" s="9" t="inlineStr">
         <is>
-          <t>14:45</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="D658" s="9" t="inlineStr">
         <is>
-          <t>15:55</t>
+          <t>09:40</t>
         </is>
       </c>
       <c r="E658" s="9" t="n">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="F658" s="9" t="inlineStr">
         <is>
@@ -50678,42 +50678,42 @@
       </c>
       <c r="G658" s="9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H658" s="9" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Sub</t>
         </is>
       </c>
       <c r="I658" s="10" t="inlineStr">
         <is>
-          <t>Pitch 1</t>
+          <t>Pitch 2A</t>
         </is>
       </c>
       <c r="J658" s="9" t="inlineStr">
         <is>
-          <t>U17/18</t>
+          <t>U11</t>
         </is>
       </c>
       <c r="K658" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U17/18 Juniors - B Female (Marilyn)</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Kangaroos Mixed</t>
         </is>
       </c>
       <c r="L658" s="10" t="inlineStr">
         <is>
-          <t>Mount Eliza SC U17/18 Juniors - B Female Red</t>
+          <t>FC Bulleen Lions U11 MiniRoos - Kangaroos Mixed Anthony &amp; Rob</t>
         </is>
       </c>
       <c r="M658" s="10" t="inlineStr">
         <is>
-          <t>Junior Girls Sunday (U12 - U18)</t>
+          <t>Coles MiniRoos Mixed Sunday (U6 - U11)</t>
         </is>
       </c>
       <c r="N658" s="9" t="inlineStr">
         <is>
-          <t>Girls' South-East 17/18B</t>
+          <t>Coles MiniRoos Mixed Sunday East 11 Kangaroos Red</t>
         </is>
       </c>
       <c r="O658" s="9" t="inlineStr">
@@ -50765,22 +50765,22 @@
       </c>
       <c r="I659" s="12" t="inlineStr">
         <is>
-          <t>Pitch 2A</t>
+          <t>Pitch 2 - Midi B</t>
         </is>
       </c>
       <c r="J659" s="11" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>U07</t>
         </is>
       </c>
       <c r="K659" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Kangaroos Mixed</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Red)</t>
         </is>
       </c>
       <c r="L659" s="12" t="inlineStr">
         <is>
-          <t>FC Bulleen Lions U11 MiniRoos - Kangaroos Mixed Anthony &amp; Rob</t>
+          <t>East Malvern Junior SC U07 MiniRoos - Joeys Mixed EMJSC U7 Sunday Orange</t>
         </is>
       </c>
       <c r="M659" s="12" t="inlineStr">
@@ -50790,7 +50790,7 @@
       </c>
       <c r="N659" s="11" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Sunday East 11 Kangaroos Red</t>
+          <t>Coles MiniRoos Mixed Sunday East 7 Joeys Red</t>
         </is>
       </c>
       <c r="O659" s="11" t="inlineStr">
@@ -50842,7 +50842,7 @@
       </c>
       <c r="I660" s="10" t="inlineStr">
         <is>
-          <t>Pitch 2 - Midi B</t>
+          <t>Pitch 2 - Midi A</t>
         </is>
       </c>
       <c r="J660" s="9" t="inlineStr">
@@ -50852,12 +50852,12 @@
       </c>
       <c r="K660" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Red)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Green)</t>
         </is>
       </c>
       <c r="L660" s="10" t="inlineStr">
         <is>
-          <t>East Malvern Junior SC U07 MiniRoos - Joeys Mixed EMJSC U7 Sunday Orange</t>
+          <t>Doncaster Rovers SC U07 MiniRoos - Joeys Mixed</t>
         </is>
       </c>
       <c r="M660" s="10" t="inlineStr">
@@ -50891,16 +50891,16 @@
       </c>
       <c r="C661" s="11" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="D661" s="11" t="inlineStr">
         <is>
-          <t>09:40</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="E661" s="11" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="F661" s="11" t="inlineStr">
         <is>
@@ -50919,32 +50919,32 @@
       </c>
       <c r="I661" s="12" t="inlineStr">
         <is>
-          <t>Pitch 2 - Midi A</t>
+          <t>Pitch 2A</t>
         </is>
       </c>
       <c r="J661" s="11" t="inlineStr">
         <is>
-          <t>U07</t>
+          <t>U12</t>
         </is>
       </c>
       <c r="K661" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Green)</t>
+          <t>Manningham United Blues FC U12 Juniors - A Female (Sienna)</t>
         </is>
       </c>
       <c r="L661" s="12" t="inlineStr">
         <is>
-          <t>Doncaster Rovers SC U07 MiniRoos - Joeys Mixed</t>
+          <t>Alamein FC U12 Juniors - A Female</t>
         </is>
       </c>
       <c r="M661" s="12" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Sunday (U6 - U11)</t>
+          <t>Junior Girls Sunday (U12 - U18)</t>
         </is>
       </c>
       <c r="N661" s="11" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Sunday East 7 Joeys Red</t>
+          <t>Girls' South-East 12A</t>
         </is>
       </c>
       <c r="O661" s="11" t="inlineStr">
@@ -50996,22 +50996,22 @@
       </c>
       <c r="I662" s="10" t="inlineStr">
         <is>
-          <t>Pitch 2A</t>
+          <t>Pitch 2B</t>
         </is>
       </c>
       <c r="J662" s="9" t="inlineStr">
         <is>
-          <t>U12</t>
+          <t>U13</t>
         </is>
       </c>
       <c r="K662" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - A Female (Sienna)</t>
+          <t>Manningham United Blues FC U13 Juniors - C Female (Abigail)</t>
         </is>
       </c>
       <c r="L662" s="10" t="inlineStr">
         <is>
-          <t>Alamein FC U12 Juniors - A Female</t>
+          <t>Hampton East Brighton FC U13 Juniors - C Female u13 girls</t>
         </is>
       </c>
       <c r="M662" s="10" t="inlineStr">
@@ -51021,7 +51021,7 @@
       </c>
       <c r="N662" s="9" t="inlineStr">
         <is>
-          <t>Girls' South-East 12A</t>
+          <t>Girls' South-East 13C</t>
         </is>
       </c>
       <c r="O662" s="9" t="inlineStr">
@@ -51045,12 +51045,12 @@
       </c>
       <c r="C663" s="11" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>11:45</t>
         </is>
       </c>
       <c r="D663" s="11" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>12:45</t>
         </is>
       </c>
       <c r="E663" s="11" t="n">
@@ -51068,37 +51068,37 @@
       </c>
       <c r="H663" s="11" t="inlineStr">
         <is>
-          <t>Sub</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="I663" s="12" t="inlineStr">
         <is>
-          <t>Pitch 2B</t>
+          <t>Pitch 2</t>
         </is>
       </c>
       <c r="J663" s="11" t="inlineStr">
         <is>
-          <t>U13</t>
+          <t>U14</t>
         </is>
       </c>
       <c r="K663" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - C Female (Abigail)</t>
+          <t>Manningham United Blues FC U14 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="L663" s="12" t="inlineStr">
         <is>
-          <t>Hampton East Brighton FC U13 Juniors - C Female u13 girls</t>
+          <t>Malvern City FC U14 Juniors - B Mixed U14 - B</t>
         </is>
       </c>
       <c r="M663" s="12" t="inlineStr">
         <is>
-          <t>Junior Girls Sunday (U12 - U18)</t>
+          <t>Junior Mixed Sunday (U12 - U16)</t>
         </is>
       </c>
       <c r="N663" s="11" t="inlineStr">
         <is>
-          <t>Girls' South-East 13C</t>
+          <t>Mixed East 14B</t>
         </is>
       </c>
       <c r="O663" s="11" t="inlineStr">
@@ -51122,16 +51122,16 @@
       </c>
       <c r="C664" s="9" t="inlineStr">
         <is>
-          <t>11:45</t>
+          <t>13:15</t>
         </is>
       </c>
       <c r="D664" s="9" t="inlineStr">
         <is>
-          <t>12:45</t>
+          <t>14:25</t>
         </is>
       </c>
       <c r="E664" s="9" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F664" s="9" t="inlineStr">
         <is>
@@ -51155,27 +51155,27 @@
       </c>
       <c r="J664" s="9" t="inlineStr">
         <is>
-          <t>U14</t>
+          <t>U15</t>
         </is>
       </c>
       <c r="K664" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - B Mixed</t>
+          <t>Manningham United Blues FC U15 Juniors - B Female (Ethan)</t>
         </is>
       </c>
       <c r="L664" s="10" t="inlineStr">
         <is>
-          <t>Malvern City FC U14 Juniors - B Mixed U14 - B</t>
+          <t>Brighton SC U15 Juniors - B Female Apollos</t>
         </is>
       </c>
       <c r="M664" s="10" t="inlineStr">
         <is>
-          <t>Junior Mixed Sunday (U12 - U16)</t>
+          <t>Junior Girls Sunday (U12 - U18)</t>
         </is>
       </c>
       <c r="N664" s="9" t="inlineStr">
         <is>
-          <t>Mixed East 14B</t>
+          <t>Girls' South-East 15B</t>
         </is>
       </c>
       <c r="O664" s="9" t="inlineStr">
@@ -51199,16 +51199,16 @@
       </c>
       <c r="C665" s="11" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="D665" s="11" t="inlineStr">
         <is>
-          <t>14:25</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="E665" s="11" t="n">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="F665" s="11" t="inlineStr">
         <is>
@@ -51232,27 +51232,27 @@
       </c>
       <c r="J665" s="11" t="inlineStr">
         <is>
-          <t>U15</t>
+          <t>Seniors</t>
         </is>
       </c>
       <c r="K665" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U15 Juniors - B Female (Ethan)</t>
+          <t>Manningham United Blues FC Seniors</t>
         </is>
       </c>
       <c r="L665" s="12" t="inlineStr">
         <is>
-          <t>Brighton SC U15 Juniors - B Female Apollos</t>
+          <t>Mount Martha SC Seniors</t>
         </is>
       </c>
       <c r="M665" s="12" t="inlineStr">
         <is>
-          <t>Junior Girls Sunday (U12 - U18)</t>
+          <t>VETO Sports State League Women's</t>
         </is>
       </c>
       <c r="N665" s="11" t="inlineStr">
         <is>
-          <t>Girls' South-East 15B</t>
+          <t>State League 6 Women's - South-East</t>
         </is>
       </c>
       <c r="O665" s="11" t="inlineStr">
@@ -51266,7 +51266,7 @@
     <row r="666">
       <c r="A666" s="9" t="inlineStr">
         <is>
-          <t>30 Aug 2026</t>
+          <t>06 Sep 2026</t>
         </is>
       </c>
       <c r="B666" s="9" t="inlineStr">
@@ -51276,16 +51276,16 @@
       </c>
       <c r="C666" s="9" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="D666" s="9" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>10:10</t>
         </is>
       </c>
       <c r="E666" s="9" t="n">
-        <v>90</v>
+        <v>40</v>
       </c>
       <c r="F666" s="9" t="inlineStr">
         <is>
@@ -51294,47 +51294,47 @@
       </c>
       <c r="G666" s="9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H666" s="9" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Sub</t>
         </is>
       </c>
       <c r="I666" s="10" t="inlineStr">
         <is>
-          <t>Pitch 2</t>
+          <t>Pitch 1 - Midi Field B</t>
         </is>
       </c>
       <c r="J666" s="9" t="inlineStr">
         <is>
-          <t>Seniors</t>
+          <t>U08</t>
         </is>
       </c>
       <c r="K666" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC Seniors</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Joeys Female (Yianna)</t>
         </is>
       </c>
       <c r="L666" s="10" t="inlineStr">
         <is>
-          <t>Mount Martha SC Seniors</t>
+          <t>East Malvern Junior SC U08 MiniRoos - Joeys Female EMJSC Girls U8 Red</t>
         </is>
       </c>
       <c r="M666" s="10" t="inlineStr">
         <is>
-          <t>VETO Sports State League Women's</t>
+          <t>Coles MiniRoos Girls' Sunday (U6 - U11)</t>
         </is>
       </c>
       <c r="N666" s="9" t="inlineStr">
         <is>
-          <t>State League 6 Women's - South-East</t>
+          <t>Coles MiniRoos Girls' East 8 Joeys</t>
         </is>
       </c>
       <c r="O666" s="9" t="inlineStr">
         <is>
-          <t>R17</t>
+          <t>R18</t>
         </is>
       </c>
       <c r="P666" s="9" t="inlineStr"/>
@@ -51381,7 +51381,7 @@
       </c>
       <c r="I667" s="12" t="inlineStr">
         <is>
-          <t>Pitch 1 - Midi Field B</t>
+          <t>Pitch 1B</t>
         </is>
       </c>
       <c r="J667" s="11" t="inlineStr">
@@ -51391,22 +51391,22 @@
       </c>
       <c r="K667" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Joeys Female (Yianna)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Kangaroos Mixed (Arnold's)</t>
         </is>
       </c>
       <c r="L667" s="12" t="inlineStr">
         <is>
-          <t>East Malvern Junior SC U08 MiniRoos - Joeys Female EMJSC Girls U8 Red</t>
+          <t>Eastern Lions SC U08 MiniRoos - Kangaroos Mixed</t>
         </is>
       </c>
       <c r="M667" s="12" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Girls' Sunday (U6 - U11)</t>
+          <t>Coles MiniRoos Mixed Sunday (U6 - U11)</t>
         </is>
       </c>
       <c r="N667" s="11" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Girls' East 8 Joeys</t>
+          <t>Coles MiniRoos Mixed Sunday South-East 8 Kangaroos</t>
         </is>
       </c>
       <c r="O667" s="11" t="inlineStr">
@@ -51458,7 +51458,7 @@
       </c>
       <c r="I668" s="10" t="inlineStr">
         <is>
-          <t>Pitch 1B</t>
+          <t>Pitch 1 - Midi Field A</t>
         </is>
       </c>
       <c r="J668" s="9" t="inlineStr">
@@ -51468,12 +51468,12 @@
       </c>
       <c r="K668" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Kangaroos Mixed (Arnold's)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Wallabies Mixed (Coe's)</t>
         </is>
       </c>
       <c r="L668" s="10" t="inlineStr">
         <is>
-          <t>Eastern Lions SC U08 MiniRoos - Kangaroos Mixed</t>
+          <t>Malvern City FC U08 MiniRoos - Wallabies Mixed U8 Blue Wallabies</t>
         </is>
       </c>
       <c r="M668" s="10" t="inlineStr">
@@ -51483,7 +51483,7 @@
       </c>
       <c r="N668" s="9" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Sunday South-East 8 Kangaroos</t>
+          <t>Coles MiniRoos Mixed Sunday East 8 Wallabies</t>
         </is>
       </c>
       <c r="O668" s="9" t="inlineStr">
@@ -51507,12 +51507,12 @@
       </c>
       <c r="C669" s="11" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="D669" s="11" t="inlineStr">
         <is>
-          <t>10:10</t>
+          <t>11:10</t>
         </is>
       </c>
       <c r="E669" s="11" t="n">
@@ -51545,22 +51545,22 @@
       </c>
       <c r="K669" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Wallabies Mixed (Coe's)</t>
+          <t>Manningham United Blues FC U08 MiniRoos - Joeys Female (Amelia &amp; Karina)</t>
         </is>
       </c>
       <c r="L669" s="12" t="inlineStr">
         <is>
-          <t>Malvern City FC U08 MiniRoos - Wallabies Mixed U8 Blue Wallabies</t>
+          <t>Fitzroy Lions SC U08 MiniRoos - Joeys Female</t>
         </is>
       </c>
       <c r="M669" s="12" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Sunday (U6 - U11)</t>
+          <t>Coles MiniRoos Girls' Sunday (U6 - U11)</t>
         </is>
       </c>
       <c r="N669" s="11" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Sunday East 8 Wallabies</t>
+          <t>Coles MiniRoos Girls' North-East 8 Joeys</t>
         </is>
       </c>
       <c r="O669" s="11" t="inlineStr">
@@ -51612,32 +51612,32 @@
       </c>
       <c r="I670" s="10" t="inlineStr">
         <is>
-          <t>Pitch 1 - Midi Field A</t>
+          <t>Pitch 1 - Midi Field B</t>
         </is>
       </c>
       <c r="J670" s="9" t="inlineStr">
         <is>
-          <t>U08</t>
+          <t>U07</t>
         </is>
       </c>
       <c r="K670" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U08 MiniRoos - Joeys Female (Amelia &amp; Karina)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Green)</t>
         </is>
       </c>
       <c r="L670" s="10" t="inlineStr">
         <is>
-          <t>Fitzroy Lions SC U08 MiniRoos - Joeys Female</t>
+          <t>Old Ivanhoe SC U07 MiniRoos - Joeys Mixed Grey</t>
         </is>
       </c>
       <c r="M670" s="10" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Girls' Sunday (U6 - U11)</t>
+          <t>Coles MiniRoos Mixed Sunday (U6 - U11)</t>
         </is>
       </c>
       <c r="N670" s="9" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Girls' North-East 8 Joeys</t>
+          <t>Coles MiniRoos Mixed Sunday East 7 Joeys Red</t>
         </is>
       </c>
       <c r="O670" s="9" t="inlineStr">
@@ -51689,22 +51689,22 @@
       </c>
       <c r="I671" s="12" t="inlineStr">
         <is>
-          <t>Pitch 1 - Midi Field B</t>
+          <t>Pitch 1B</t>
         </is>
       </c>
       <c r="J671" s="11" t="inlineStr">
         <is>
-          <t>U07</t>
+          <t>U10</t>
         </is>
       </c>
       <c r="K671" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Green)</t>
+          <t>Manningham United Blues FC U10 MiniRoos - Wallabies Mixed (Tilio's)</t>
         </is>
       </c>
       <c r="L671" s="12" t="inlineStr">
         <is>
-          <t>Old Ivanhoe SC U07 MiniRoos - Joeys Mixed Grey</t>
+          <t>Maccabi FC Caulfield U10 MiniRoos - Wallabies Mixed Maccabi FC Caulfield U10 Blue Wasps</t>
         </is>
       </c>
       <c r="M671" s="12" t="inlineStr">
@@ -51714,7 +51714,7 @@
       </c>
       <c r="N671" s="11" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Sunday East 7 Joeys Red</t>
+          <t>Coles MiniRoos Mixed Sunday East 10 Wallabies</t>
         </is>
       </c>
       <c r="O671" s="11" t="inlineStr">
@@ -51738,12 +51738,12 @@
       </c>
       <c r="C672" s="9" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>11:40</t>
         </is>
       </c>
       <c r="D672" s="9" t="inlineStr">
         <is>
-          <t>11:10</t>
+          <t>12:20</t>
         </is>
       </c>
       <c r="E672" s="9" t="n">
@@ -51771,27 +51771,27 @@
       </c>
       <c r="J672" s="9" t="inlineStr">
         <is>
-          <t>U10</t>
+          <t>U11</t>
         </is>
       </c>
       <c r="K672" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U10 MiniRoos - Wallabies Mixed (Tilio's)</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Joeys Female (Grace)</t>
         </is>
       </c>
       <c r="L672" s="10" t="inlineStr">
         <is>
-          <t>Maccabi FC Caulfield U10 MiniRoos - Wallabies Mixed Maccabi FC Caulfield U10 Blue Wasps</t>
+          <t>Collingwood City FC U11 MiniRoos - Joeys Female 11J girls</t>
         </is>
       </c>
       <c r="M672" s="10" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Sunday (U6 - U11)</t>
+          <t>Coles MiniRoos Girls' Sunday (U6 - U11)</t>
         </is>
       </c>
       <c r="N672" s="9" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Sunday East 10 Wallabies</t>
+          <t>Coles MiniRoos Girls' East 11 Joeys</t>
         </is>
       </c>
       <c r="O672" s="9" t="inlineStr">
@@ -51815,16 +51815,16 @@
       </c>
       <c r="C673" s="11" t="inlineStr">
         <is>
-          <t>11:40</t>
+          <t>13:15</t>
         </is>
       </c>
       <c r="D673" s="11" t="inlineStr">
         <is>
-          <t>12:20</t>
+          <t>14:25</t>
         </is>
       </c>
       <c r="E673" s="11" t="n">
-        <v>40</v>
+        <v>70</v>
       </c>
       <c r="F673" s="11" t="inlineStr">
         <is>
@@ -51838,37 +51838,37 @@
       </c>
       <c r="H673" s="11" t="inlineStr">
         <is>
-          <t>Sub</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="I673" s="12" t="inlineStr">
         <is>
-          <t>Pitch 1B</t>
+          <t>Pitch 1</t>
         </is>
       </c>
       <c r="J673" s="11" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>U16</t>
         </is>
       </c>
       <c r="K673" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Joeys Female (Grace)</t>
+          <t>Manningham United Blues FC U16 Juniors - A Mixed</t>
         </is>
       </c>
       <c r="L673" s="12" t="inlineStr">
         <is>
-          <t>Collingwood City FC U11 MiniRoos - Joeys Female 11J girls</t>
+          <t>Oakleigh Cannons FC U16 Juniors - A Mixed OCFC Michael E</t>
         </is>
       </c>
       <c r="M673" s="12" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Girls' Sunday (U6 - U11)</t>
+          <t>Junior Mixed Sunday (U12 - U16)</t>
         </is>
       </c>
       <c r="N673" s="11" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Girls' East 11 Joeys</t>
+          <t>Mixed South-East 16A</t>
         </is>
       </c>
       <c r="O673" s="11" t="inlineStr">
@@ -51892,12 +51892,12 @@
       </c>
       <c r="C674" s="9" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="D674" s="9" t="inlineStr">
         <is>
-          <t>14:25</t>
+          <t>16:10</t>
         </is>
       </c>
       <c r="E674" s="9" t="n">
@@ -51925,27 +51925,27 @@
       </c>
       <c r="J674" s="9" t="inlineStr">
         <is>
-          <t>U16</t>
+          <t>U18</t>
         </is>
       </c>
       <c r="K674" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U16 Juniors - A Mixed</t>
+          <t>Manningham United Blues FC U18 Juniors - A Male</t>
         </is>
       </c>
       <c r="L674" s="10" t="inlineStr">
         <is>
-          <t>Oakleigh Cannons FC U16 Juniors - A Mixed OCFC Michael E</t>
+          <t>Malvern City FC U18 Juniors - A Male U18 HP - A</t>
         </is>
       </c>
       <c r="M674" s="10" t="inlineStr">
         <is>
-          <t>Junior Mixed Sunday (U12 - U16)</t>
+          <t>Junior Boys Sunday (U17 - U18)</t>
         </is>
       </c>
       <c r="N674" s="9" t="inlineStr">
         <is>
-          <t>Mixed South-East 16A</t>
+          <t>Boys North-East 18A</t>
         </is>
       </c>
       <c r="O674" s="9" t="inlineStr">
@@ -51969,16 +51969,16 @@
       </c>
       <c r="C675" s="11" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="D675" s="11" t="inlineStr">
         <is>
-          <t>16:10</t>
+          <t>09:40</t>
         </is>
       </c>
       <c r="E675" s="11" t="n">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="F675" s="11" t="inlineStr">
         <is>
@@ -51987,42 +51987,42 @@
       </c>
       <c r="G675" s="11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H675" s="11" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Sub</t>
         </is>
       </c>
       <c r="I675" s="12" t="inlineStr">
         <is>
-          <t>Pitch 1</t>
+          <t>Pitch 2B</t>
         </is>
       </c>
       <c r="J675" s="11" t="inlineStr">
         <is>
-          <t>U18</t>
+          <t>U11</t>
         </is>
       </c>
       <c r="K675" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U18 Juniors - A Male</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Kangaroos Mixed</t>
         </is>
       </c>
       <c r="L675" s="12" t="inlineStr">
         <is>
-          <t>Malvern City FC U18 Juniors - A Male U18 HP - A</t>
+          <t>Malvern City FC U11 MiniRoos - Kangaroos Mixed U11 HP White Kangaroos</t>
         </is>
       </c>
       <c r="M675" s="12" t="inlineStr">
         <is>
-          <t>Junior Boys Sunday (U17 - U18)</t>
+          <t>Coles MiniRoos Mixed Sunday (U6 - U11)</t>
         </is>
       </c>
       <c r="N675" s="11" t="inlineStr">
         <is>
-          <t>Boys North-East 18A</t>
+          <t>Coles MiniRoos Mixed Sunday East 11 Kangaroos Red</t>
         </is>
       </c>
       <c r="O675" s="11" t="inlineStr">
@@ -52074,7 +52074,7 @@
       </c>
       <c r="I676" s="10" t="inlineStr">
         <is>
-          <t>Pitch 2B</t>
+          <t>Pitch 2A</t>
         </is>
       </c>
       <c r="J676" s="9" t="inlineStr">
@@ -52084,12 +52084,12 @@
       </c>
       <c r="K676" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Kangaroos Mixed</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Mixed (Colosimo's)</t>
         </is>
       </c>
       <c r="L676" s="10" t="inlineStr">
         <is>
-          <t>Malvern City FC U11 MiniRoos - Kangaroos Mixed U11 HP White Kangaroos</t>
+          <t>Malvern City FC U11 MiniRoos - Wallabies Mixed U11 White Wallabies</t>
         </is>
       </c>
       <c r="M676" s="10" t="inlineStr">
@@ -52099,7 +52099,7 @@
       </c>
       <c r="N676" s="9" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Sunday East 11 Kangaroos Red</t>
+          <t>Coles MiniRoos Mixed Sunday East 11 Wallabies Red</t>
         </is>
       </c>
       <c r="O676" s="9" t="inlineStr">
@@ -52123,16 +52123,16 @@
       </c>
       <c r="C677" s="11" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>10:10</t>
         </is>
       </c>
       <c r="D677" s="11" t="inlineStr">
         <is>
-          <t>09:40</t>
+          <t>11:10</t>
         </is>
       </c>
       <c r="E677" s="11" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="F677" s="11" t="inlineStr">
         <is>
@@ -52151,32 +52151,32 @@
       </c>
       <c r="I677" s="12" t="inlineStr">
         <is>
-          <t>Pitch 2A</t>
+          <t>Pitch 2B</t>
         </is>
       </c>
       <c r="J677" s="11" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>U12</t>
         </is>
       </c>
       <c r="K677" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Mixed (Colosimo's)</t>
+          <t>Manningham United Blues FC U12 Juniors - B Mixed (Robert)</t>
         </is>
       </c>
       <c r="L677" s="12" t="inlineStr">
         <is>
-          <t>Malvern City FC U11 MiniRoos - Wallabies Mixed U11 White Wallabies</t>
+          <t>Mazenod FC U12 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="M677" s="12" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Sunday (U6 - U11)</t>
+          <t>Junior Mixed Sunday (U12 - U16)</t>
         </is>
       </c>
       <c r="N677" s="11" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Sunday East 11 Wallabies Red</t>
+          <t>Mixed Sunday East 12B Blue</t>
         </is>
       </c>
       <c r="O677" s="11" t="inlineStr">
@@ -52200,16 +52200,16 @@
       </c>
       <c r="C678" s="9" t="inlineStr">
         <is>
-          <t>10:10</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="D678" s="9" t="inlineStr">
         <is>
-          <t>11:10</t>
+          <t>13:10</t>
         </is>
       </c>
       <c r="E678" s="9" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F678" s="9" t="inlineStr">
         <is>
@@ -52223,37 +52223,37 @@
       </c>
       <c r="H678" s="9" t="inlineStr">
         <is>
-          <t>Sub</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="I678" s="10" t="inlineStr">
         <is>
-          <t>Pitch 2B</t>
+          <t>Pitch 2</t>
         </is>
       </c>
       <c r="J678" s="9" t="inlineStr">
         <is>
-          <t>U12</t>
+          <t>U15</t>
         </is>
       </c>
       <c r="K678" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - B Mixed (Robert)</t>
+          <t>Manningham United Blues FC U15 Juniors - B Female (Ethan)</t>
         </is>
       </c>
       <c r="L678" s="10" t="inlineStr">
         <is>
-          <t>Mazenod FC U12 Juniors - B Mixed</t>
+          <t>Ringwood City FC U15 Juniors - B Female 15DC</t>
         </is>
       </c>
       <c r="M678" s="10" t="inlineStr">
         <is>
-          <t>Junior Mixed Sunday (U12 - U16)</t>
+          <t>Junior Girls Sunday (U12 - U18)</t>
         </is>
       </c>
       <c r="N678" s="9" t="inlineStr">
         <is>
-          <t>Mixed Sunday East 12B Blue</t>
+          <t>Girls' South-East 15B</t>
         </is>
       </c>
       <c r="O678" s="9" t="inlineStr">
@@ -52277,16 +52277,16 @@
       </c>
       <c r="C679" s="11" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="D679" s="11" t="inlineStr">
         <is>
-          <t>13:10</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="E679" s="11" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="F679" s="11" t="inlineStr">
         <is>
@@ -52295,7 +52295,7 @@
       </c>
       <c r="G679" s="11" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H679" s="11" t="inlineStr">
@@ -52305,22 +52305,22 @@
       </c>
       <c r="I679" s="12" t="inlineStr">
         <is>
-          <t>Pitch 2</t>
+          <t>Pitch 3</t>
         </is>
       </c>
       <c r="J679" s="11" t="inlineStr">
         <is>
-          <t>U15</t>
+          <t>U14</t>
         </is>
       </c>
       <c r="K679" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U15 Juniors - B Female (Ethan)</t>
+          <t>Manningham United Blues FC U14 Juniors - C Female (Christian)</t>
         </is>
       </c>
       <c r="L679" s="12" t="inlineStr">
         <is>
-          <t>Ringwood City FC U15 Juniors - B Female 15DC</t>
+          <t>Pakenham United FC U14 Juniors - C Female G13 Purple PUFC</t>
         </is>
       </c>
       <c r="M679" s="12" t="inlineStr">
@@ -52330,7 +52330,7 @@
       </c>
       <c r="N679" s="11" t="inlineStr">
         <is>
-          <t>Girls' South-East 15B</t>
+          <t>Girls' South-East 14C</t>
         </is>
       </c>
       <c r="O679" s="11" t="inlineStr">
@@ -52354,12 +52354,12 @@
       </c>
       <c r="C680" s="9" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>11:40</t>
         </is>
       </c>
       <c r="D680" s="9" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>12:40</t>
         </is>
       </c>
       <c r="E680" s="9" t="n">
@@ -52387,27 +52387,27 @@
       </c>
       <c r="J680" s="9" t="inlineStr">
         <is>
-          <t>U14</t>
+          <t>U13</t>
         </is>
       </c>
       <c r="K680" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - C Female (Christian)</t>
+          <t>Manningham United Blues FC U13 Juniors - B Mixed (Samir)</t>
         </is>
       </c>
       <c r="L680" s="10" t="inlineStr">
         <is>
-          <t>Pakenham United FC U14 Juniors - C Female G13 Purple PUFC</t>
+          <t>Croydon Ranges SC U13 Juniors - B Mixed Croydon Ranges U13 Sundays Blue</t>
         </is>
       </c>
       <c r="M680" s="10" t="inlineStr">
         <is>
-          <t>Junior Girls Sunday (U12 - U18)</t>
+          <t>Junior Mixed Sunday (U12 - U16)</t>
         </is>
       </c>
       <c r="N680" s="9" t="inlineStr">
         <is>
-          <t>Girls' South-East 14C</t>
+          <t>Mixed Sunday East 13B</t>
         </is>
       </c>
       <c r="O680" s="9" t="inlineStr">
@@ -52416,12 +52416,16 @@
         </is>
       </c>
       <c r="P680" s="9" t="inlineStr"/>
-      <c r="Q680" s="10" t="inlineStr"/>
+      <c r="Q680" s="10" t="inlineStr">
+        <is>
+          <t>Powerful Owl Park Pitch 1 - Midi Field B</t>
+        </is>
+      </c>
     </row>
     <row r="681">
       <c r="A681" s="11" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>26 Apr 2026</t>
         </is>
       </c>
       <c r="B681" s="11" t="inlineStr">
@@ -52431,12 +52435,12 @@
       </c>
       <c r="C681" s="11" t="inlineStr">
         <is>
-          <t>11:40</t>
+          <t>11:15</t>
         </is>
       </c>
       <c r="D681" s="11" t="inlineStr">
         <is>
-          <t>12:40</t>
+          <t>12:15</t>
         </is>
       </c>
       <c r="E681" s="11" t="n">
@@ -52444,12 +52448,12 @@
       </c>
       <c r="F681" s="11" t="inlineStr">
         <is>
-          <t>Powerful Owl Park</t>
+          <t>Timber Ridge Reserve</t>
         </is>
       </c>
       <c r="G681" s="11" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H681" s="11" t="inlineStr">
@@ -52459,45 +52463,41 @@
       </c>
       <c r="I681" s="12" t="inlineStr">
         <is>
-          <t>Pitch 3</t>
+          <t>Pitch 1</t>
         </is>
       </c>
       <c r="J681" s="11" t="inlineStr">
         <is>
-          <t>U13</t>
+          <t>U14</t>
         </is>
       </c>
       <c r="K681" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - B Mixed (Samir)</t>
+          <t>Manningham United Blues FC U14 Juniors - C Female (Christian)</t>
         </is>
       </c>
       <c r="L681" s="12" t="inlineStr">
         <is>
-          <t>Croydon Ranges SC U13 Juniors - B Mixed Croydon Ranges U13 Sundays Blue</t>
+          <t>East Bentleigh SC U14 Juniors - C Female Girls U14 Strikers</t>
         </is>
       </c>
       <c r="M681" s="12" t="inlineStr">
         <is>
-          <t>Junior Mixed Sunday (U12 - U16)</t>
+          <t>Junior Girls Sunday (U12 - U18)</t>
         </is>
       </c>
       <c r="N681" s="11" t="inlineStr">
         <is>
-          <t>Mixed Sunday East 13B</t>
+          <t>Girls' South-East 14C</t>
         </is>
       </c>
       <c r="O681" s="11" t="inlineStr">
         <is>
-          <t>R18</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="P681" s="11" t="inlineStr"/>
-      <c r="Q681" s="12" t="inlineStr">
-        <is>
-          <t>Powerful Owl Park Pitch 1 - Midi Field B</t>
-        </is>
-      </c>
+      <c r="Q681" s="12" t="inlineStr"/>
     </row>
     <row r="682">
       <c r="A682" s="9" t="inlineStr">
@@ -52512,16 +52512,16 @@
       </c>
       <c r="C682" s="9" t="inlineStr">
         <is>
-          <t>11:15</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="D682" s="9" t="inlineStr">
         <is>
-          <t>12:15</t>
+          <t>13:40</t>
         </is>
       </c>
       <c r="E682" s="9" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F682" s="9" t="inlineStr">
         <is>
@@ -52530,7 +52530,7 @@
       </c>
       <c r="G682" s="9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H682" s="9" t="inlineStr">
@@ -52540,22 +52540,22 @@
       </c>
       <c r="I682" s="10" t="inlineStr">
         <is>
-          <t>Pitch 1</t>
+          <t>Pitch 2</t>
         </is>
       </c>
       <c r="J682" s="9" t="inlineStr">
         <is>
-          <t>U14</t>
+          <t>U15</t>
         </is>
       </c>
       <c r="K682" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - C Female (Christian)</t>
+          <t>Manningham United Blues FC U15 Juniors - B Female (Ethan)</t>
         </is>
       </c>
       <c r="L682" s="10" t="inlineStr">
         <is>
-          <t>East Bentleigh SC U14 Juniors - C Female Girls U14 Strikers</t>
+          <t>Bayside Argonauts FC U15 Juniors - B Female</t>
         </is>
       </c>
       <c r="M682" s="10" t="inlineStr">
@@ -52565,7 +52565,7 @@
       </c>
       <c r="N682" s="9" t="inlineStr">
         <is>
-          <t>Girls' South-East 14C</t>
+          <t>Girls' South-East 15B</t>
         </is>
       </c>
       <c r="O682" s="9" t="inlineStr">
@@ -52579,26 +52579,26 @@
     <row r="683">
       <c r="A683" s="11" t="inlineStr">
         <is>
-          <t>26 Apr 2026</t>
+          <t>18 Jul 2026</t>
         </is>
       </c>
       <c r="B683" s="11" t="inlineStr">
         <is>
-          <t>Sun</t>
+          <t>Sat</t>
         </is>
       </c>
       <c r="C683" s="11" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>08:30</t>
         </is>
       </c>
       <c r="D683" s="11" t="inlineStr">
         <is>
-          <t>13:40</t>
+          <t>09:10</t>
         </is>
       </c>
       <c r="E683" s="11" t="n">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="F683" s="11" t="inlineStr">
         <is>
@@ -52607,47 +52607,47 @@
       </c>
       <c r="G683" s="11" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H683" s="11" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Sub</t>
         </is>
       </c>
       <c r="I683" s="12" t="inlineStr">
         <is>
-          <t>Pitch 2</t>
+          <t>Pitch 1E - Quarter Pitch 4v4</t>
         </is>
       </c>
       <c r="J683" s="11" t="inlineStr">
         <is>
-          <t>U15</t>
+          <t>U07</t>
         </is>
       </c>
       <c r="K683" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U15 Juniors - B Female (Ethan)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (White)</t>
         </is>
       </c>
       <c r="L683" s="12" t="inlineStr">
         <is>
-          <t>Bayside Argonauts FC U15 Juniors - B Female</t>
+          <t>Lilydale Montrose United FC U07 MiniRoos - Joeys Mixed Sat U7 Red</t>
         </is>
       </c>
       <c r="M683" s="12" t="inlineStr">
         <is>
-          <t>Junior Girls Sunday (U12 - U18)</t>
+          <t>Coles MiniRoos Mixed Saturday (U6 - U11)</t>
         </is>
       </c>
       <c r="N683" s="11" t="inlineStr">
         <is>
-          <t>Girls' South-East 15B</t>
+          <t>Coles MiniRoos Mixed Saturday East 7 Joeys Red</t>
         </is>
       </c>
       <c r="O683" s="11" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R11</t>
         </is>
       </c>
       <c r="P683" s="11" t="inlineStr"/>
@@ -52666,16 +52666,16 @@
       </c>
       <c r="C684" s="9" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>09:40</t>
         </is>
       </c>
       <c r="D684" s="9" t="inlineStr">
         <is>
-          <t>09:10</t>
+          <t>10:40</t>
         </is>
       </c>
       <c r="E684" s="9" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="F684" s="9" t="inlineStr">
         <is>
@@ -52694,32 +52694,32 @@
       </c>
       <c r="I684" s="10" t="inlineStr">
         <is>
-          <t>Pitch 1E - Quarter Pitch 4v4</t>
+          <t>Pitch 1A</t>
         </is>
       </c>
       <c r="J684" s="9" t="inlineStr">
         <is>
-          <t>U07</t>
+          <t>U12</t>
         </is>
       </c>
       <c r="K684" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (White)</t>
+          <t>Manningham United Blues FC U12 Juniors - B Mixed (Andre)</t>
         </is>
       </c>
       <c r="L684" s="10" t="inlineStr">
         <is>
-          <t>Lilydale Montrose United FC U07 MiniRoos - Joeys Mixed Sat U7 Red</t>
+          <t>Boroondara Eagles FC U12 Juniors - B Mixed Boroondara Eagles FC (CK)</t>
         </is>
       </c>
       <c r="M684" s="10" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Saturday (U6 - U11)</t>
+          <t>Junior Mixed Saturday (U12 - U16)</t>
         </is>
       </c>
       <c r="N684" s="9" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Saturday East 7 Joeys Red</t>
+          <t>Mixed Saturday East 12B</t>
         </is>
       </c>
       <c r="O684" s="9" t="inlineStr">
@@ -52771,7 +52771,7 @@
       </c>
       <c r="I685" s="12" t="inlineStr">
         <is>
-          <t>Pitch 1A</t>
+          <t>Pitch 1B</t>
         </is>
       </c>
       <c r="J685" s="11" t="inlineStr">
@@ -52781,12 +52781,12 @@
       </c>
       <c r="K685" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - B Mixed (Andre)</t>
+          <t>Manningham United Blues FC U12 Juniors - B Mixed (Chris)</t>
         </is>
       </c>
       <c r="L685" s="12" t="inlineStr">
         <is>
-          <t>Boroondara Eagles FC U12 Juniors - B Mixed Boroondara Eagles FC (CK)</t>
+          <t>South Yarra SC U12 Juniors - B Mixed South Yarra SC - U12 Mixed</t>
         </is>
       </c>
       <c r="M685" s="12" t="inlineStr">
@@ -52810,7 +52810,7 @@
     <row r="686">
       <c r="A686" s="9" t="inlineStr">
         <is>
-          <t>18 Jul 2026</t>
+          <t>25 Jul 2026</t>
         </is>
       </c>
       <c r="B686" s="9" t="inlineStr">
@@ -52820,12 +52820,12 @@
       </c>
       <c r="C686" s="9" t="inlineStr">
         <is>
-          <t>09:40</t>
+          <t>08:30</t>
         </is>
       </c>
       <c r="D686" s="9" t="inlineStr">
         <is>
-          <t>10:40</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="E686" s="9" t="n">
@@ -52848,7 +52848,7 @@
       </c>
       <c r="I686" s="10" t="inlineStr">
         <is>
-          <t>Pitch 1B</t>
+          <t>Pitch 1A</t>
         </is>
       </c>
       <c r="J686" s="9" t="inlineStr">
@@ -52858,12 +52858,12 @@
       </c>
       <c r="K686" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - B Mixed (Chris)</t>
+          <t>Manningham United Blues FC U12 Juniors - B Mixed (Andre)</t>
         </is>
       </c>
       <c r="L686" s="10" t="inlineStr">
         <is>
-          <t>South Yarra SC U12 Juniors - B Mixed South Yarra SC - U12 Mixed</t>
+          <t>Nunawading City FC U12 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="M686" s="10" t="inlineStr">
@@ -52878,7 +52878,7 @@
       </c>
       <c r="O686" s="9" t="inlineStr">
         <is>
-          <t>R11</t>
+          <t>R12</t>
         </is>
       </c>
       <c r="P686" s="9" t="inlineStr"/>
@@ -52887,22 +52887,22 @@
     <row r="687">
       <c r="A687" s="11" t="inlineStr">
         <is>
-          <t>25 Jul 2026</t>
+          <t>02 Aug 2026</t>
         </is>
       </c>
       <c r="B687" s="11" t="inlineStr">
         <is>
-          <t>Sat</t>
+          <t>Sun</t>
         </is>
       </c>
       <c r="C687" s="11" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>11:40</t>
         </is>
       </c>
       <c r="D687" s="11" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>12:40</t>
         </is>
       </c>
       <c r="E687" s="11" t="n">
@@ -52915,7 +52915,7 @@
       </c>
       <c r="G687" s="11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H687" s="11" t="inlineStr">
@@ -52925,37 +52925,37 @@
       </c>
       <c r="I687" s="12" t="inlineStr">
         <is>
-          <t>Pitch 1A</t>
+          <t>Pitch 2B</t>
         </is>
       </c>
       <c r="J687" s="11" t="inlineStr">
         <is>
-          <t>U12</t>
+          <t>U13</t>
         </is>
       </c>
       <c r="K687" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U12 Juniors - B Mixed (Andre)</t>
+          <t>Manningham United Blues FC U13 Juniors - B Mixed (Samir)</t>
         </is>
       </c>
       <c r="L687" s="12" t="inlineStr">
         <is>
-          <t>Nunawading City FC U12 Juniors - B Mixed</t>
+          <t>Eastern Lions SC U13 Juniors - B Mixed</t>
         </is>
       </c>
       <c r="M687" s="12" t="inlineStr">
         <is>
-          <t>Junior Mixed Saturday (U12 - U16)</t>
+          <t>Junior Mixed Sunday (U12 - U16)</t>
         </is>
       </c>
       <c r="N687" s="11" t="inlineStr">
         <is>
-          <t>Mixed Saturday East 12B</t>
+          <t>Mixed Sunday East 13B</t>
         </is>
       </c>
       <c r="O687" s="11" t="inlineStr">
         <is>
-          <t>R12</t>
+          <t>R13</t>
         </is>
       </c>
       <c r="P687" s="11" t="inlineStr"/>
@@ -52964,26 +52964,26 @@
     <row r="688">
       <c r="A688" s="9" t="inlineStr">
         <is>
-          <t>02 Aug 2026</t>
+          <t>08 Aug 2026</t>
         </is>
       </c>
       <c r="B688" s="9" t="inlineStr">
         <is>
-          <t>Sun</t>
+          <t>Sat</t>
         </is>
       </c>
       <c r="C688" s="9" t="inlineStr">
         <is>
-          <t>11:40</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="D688" s="9" t="inlineStr">
         <is>
-          <t>12:40</t>
+          <t>10:10</t>
         </is>
       </c>
       <c r="E688" s="9" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="F688" s="9" t="inlineStr">
         <is>
@@ -52992,7 +52992,7 @@
       </c>
       <c r="G688" s="9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H688" s="9" t="inlineStr">
@@ -53002,37 +53002,37 @@
       </c>
       <c r="I688" s="10" t="inlineStr">
         <is>
-          <t>Pitch 2B</t>
+          <t>Pitch 1E - Quarter Pitch 4v4</t>
         </is>
       </c>
       <c r="J688" s="9" t="inlineStr">
         <is>
-          <t>U13</t>
+          <t>U07</t>
         </is>
       </c>
       <c r="K688" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - B Mixed (Samir)</t>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Purple)</t>
         </is>
       </c>
       <c r="L688" s="10" t="inlineStr">
         <is>
-          <t>Eastern Lions SC U13 Juniors - B Mixed</t>
+          <t>Doncaster Rovers SC U07 MiniRoos - Joeys Mixed Daryl</t>
         </is>
       </c>
       <c r="M688" s="10" t="inlineStr">
         <is>
-          <t>Junior Mixed Sunday (U12 - U16)</t>
+          <t>Coles MiniRoos Mixed Saturday (U6 - U11)</t>
         </is>
       </c>
       <c r="N688" s="9" t="inlineStr">
         <is>
-          <t>Mixed Sunday East 13B</t>
+          <t>Coles MiniRoos Mixed Saturday East 7 Joeys Red</t>
         </is>
       </c>
       <c r="O688" s="9" t="inlineStr">
         <is>
-          <t>R13</t>
+          <t>R14</t>
         </is>
       </c>
       <c r="P688" s="9" t="inlineStr"/>
@@ -53051,12 +53051,12 @@
       </c>
       <c r="C689" s="11" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>08:30</t>
         </is>
       </c>
       <c r="D689" s="11" t="inlineStr">
         <is>
-          <t>10:10</t>
+          <t>09:10</t>
         </is>
       </c>
       <c r="E689" s="11" t="n">
@@ -53069,7 +53069,7 @@
       </c>
       <c r="G689" s="11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H689" s="11" t="inlineStr">
@@ -53079,22 +53079,22 @@
       </c>
       <c r="I689" s="12" t="inlineStr">
         <is>
-          <t>Pitch 1E - Quarter Pitch 4v4</t>
+          <t>Pitch 2A</t>
         </is>
       </c>
       <c r="J689" s="11" t="inlineStr">
         <is>
-          <t>U07</t>
+          <t>U10</t>
         </is>
       </c>
       <c r="K689" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Purple)</t>
+          <t>Manningham United Blues FC U10 MiniRoos - Kangaroos Mixed</t>
         </is>
       </c>
       <c r="L689" s="12" t="inlineStr">
         <is>
-          <t>Doncaster Rovers SC U07 MiniRoos - Joeys Mixed Daryl</t>
+          <t>Ringwood City FC U10 MiniRoos - Kangaroos Mixed 10BD</t>
         </is>
       </c>
       <c r="M689" s="12" t="inlineStr">
@@ -53104,7 +53104,7 @@
       </c>
       <c r="N689" s="11" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Saturday East 7 Joeys Red</t>
+          <t>Coles MiniRoos Mixed Saturday East 10 Kangaroos</t>
         </is>
       </c>
       <c r="O689" s="11" t="inlineStr">
@@ -53118,7 +53118,7 @@
     <row r="690">
       <c r="A690" s="9" t="inlineStr">
         <is>
-          <t>08 Aug 2026</t>
+          <t>29 Aug 2026</t>
         </is>
       </c>
       <c r="B690" s="9" t="inlineStr">
@@ -53161,17 +53161,17 @@
       </c>
       <c r="J690" s="9" t="inlineStr">
         <is>
-          <t>U10</t>
+          <t>U11</t>
         </is>
       </c>
       <c r="K690" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U10 MiniRoos - Kangaroos Mixed</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Mixed (Culina's)</t>
         </is>
       </c>
       <c r="L690" s="10" t="inlineStr">
         <is>
-          <t>Ringwood City FC U10 MiniRoos - Kangaroos Mixed 10BD</t>
+          <t>Doncaster Rovers SC U11 MiniRoos - Wallabies Mixed</t>
         </is>
       </c>
       <c r="M690" s="10" t="inlineStr">
@@ -53181,12 +53181,12 @@
       </c>
       <c r="N690" s="9" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Saturday East 10 Kangaroos</t>
+          <t>Coles MiniRoos Mixed Saturday East 11 Wallabies Blue</t>
         </is>
       </c>
       <c r="O690" s="9" t="inlineStr">
         <is>
-          <t>R14</t>
+          <t>R17</t>
         </is>
       </c>
       <c r="P690" s="9" t="inlineStr"/>
@@ -53195,26 +53195,26 @@
     <row r="691">
       <c r="A691" s="11" t="inlineStr">
         <is>
-          <t>29 Aug 2026</t>
+          <t>30 Aug 2026</t>
         </is>
       </c>
       <c r="B691" s="11" t="inlineStr">
         <is>
-          <t>Sat</t>
+          <t>Sun</t>
         </is>
       </c>
       <c r="C691" s="11" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="D691" s="11" t="inlineStr">
         <is>
-          <t>09:10</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="E691" s="11" t="n">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="F691" s="11" t="inlineStr">
         <is>
@@ -53223,42 +53223,42 @@
       </c>
       <c r="G691" s="11" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H691" s="11" t="inlineStr">
         <is>
-          <t>Sub</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="I691" s="12" t="inlineStr">
         <is>
-          <t>Pitch 2A</t>
+          <t>Pitch 1</t>
         </is>
       </c>
       <c r="J691" s="11" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>Seniors</t>
         </is>
       </c>
       <c r="K691" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Mixed (Culina's)</t>
+          <t>Keysborough District FC Seniors Keysborough District FC</t>
         </is>
       </c>
       <c r="L691" s="12" t="inlineStr">
         <is>
-          <t>Doncaster Rovers SC U11 MiniRoos - Wallabies Mixed</t>
+          <t>Manningham United Blues FC Seniors</t>
         </is>
       </c>
       <c r="M691" s="12" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Saturday (U6 - U11)</t>
+          <t>Men's Metropolitan League</t>
         </is>
       </c>
       <c r="N691" s="11" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Saturday East 11 Wallabies Blue</t>
+          <t>Men's Metropolitan League 7 South-East</t>
         </is>
       </c>
       <c r="O691" s="11" t="inlineStr">
@@ -53269,85 +53269,8 @@
       <c r="P691" s="11" t="inlineStr"/>
       <c r="Q691" s="12" t="inlineStr"/>
     </row>
-    <row r="692">
-      <c r="A692" s="9" t="inlineStr">
-        <is>
-          <t>30 Aug 2026</t>
-        </is>
-      </c>
-      <c r="B692" s="9" t="inlineStr">
-        <is>
-          <t>Sun</t>
-        </is>
-      </c>
-      <c r="C692" s="9" t="inlineStr">
-        <is>
-          <t>15:00</t>
-        </is>
-      </c>
-      <c r="D692" s="9" t="inlineStr">
-        <is>
-          <t>16:30</t>
-        </is>
-      </c>
-      <c r="E692" s="9" t="n">
-        <v>90</v>
-      </c>
-      <c r="F692" s="9" t="inlineStr">
-        <is>
-          <t>Timber Ridge Reserve</t>
-        </is>
-      </c>
-      <c r="G692" s="9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H692" s="9" t="inlineStr">
-        <is>
-          <t>Full</t>
-        </is>
-      </c>
-      <c r="I692" s="10" t="inlineStr">
-        <is>
-          <t>Pitch 1</t>
-        </is>
-      </c>
-      <c r="J692" s="9" t="inlineStr">
-        <is>
-          <t>Seniors</t>
-        </is>
-      </c>
-      <c r="K692" s="10" t="inlineStr">
-        <is>
-          <t>Keysborough District FC Seniors Keysborough District FC</t>
-        </is>
-      </c>
-      <c r="L692" s="10" t="inlineStr">
-        <is>
-          <t>Manningham United Blues FC Seniors</t>
-        </is>
-      </c>
-      <c r="M692" s="10" t="inlineStr">
-        <is>
-          <t>Men's Metropolitan League</t>
-        </is>
-      </c>
-      <c r="N692" s="9" t="inlineStr">
-        <is>
-          <t>Men's Metropolitan League 7 South-East</t>
-        </is>
-      </c>
-      <c r="O692" s="9" t="inlineStr">
-        <is>
-          <t>R17</t>
-        </is>
-      </c>
-      <c r="P692" s="9" t="inlineStr"/>
-      <c r="Q692" s="10" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:Q692"/>
+  <autoFilter ref="A1:Q691"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Auto-refresh fixtures from Dribl (2026-08-25)
</commit_message>
<xml_diff>
--- a/Manningham_fixtures_and_overlaps.xlsx
+++ b/Manningham_fixtures_and_overlaps.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Overlaps &amp; Peak Load" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Games'!$A$1:$Q$691</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Games'!$A$1:$Q$690</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -596,7 +596,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Source: fv.dribl.com, 2026 season, generated 24 Aug 2026</t>
+          <t>Source: fv.dribl.com, 2026 season, generated 25 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -654,11 +654,11 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>26 Apr - 30 Aug 2026</t>
+          <t>26 Apr - 29 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -669,7 +669,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="C9" s="7" t="inlineStr"/>
     </row>
@@ -694,7 +694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q691"/>
+  <dimension ref="A1:Q690"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -53192,85 +53192,8 @@
       <c r="P690" s="9" t="inlineStr"/>
       <c r="Q690" s="10" t="inlineStr"/>
     </row>
-    <row r="691">
-      <c r="A691" s="11" t="inlineStr">
-        <is>
-          <t>30 Aug 2026</t>
-        </is>
-      </c>
-      <c r="B691" s="11" t="inlineStr">
-        <is>
-          <t>Sun</t>
-        </is>
-      </c>
-      <c r="C691" s="11" t="inlineStr">
-        <is>
-          <t>15:00</t>
-        </is>
-      </c>
-      <c r="D691" s="11" t="inlineStr">
-        <is>
-          <t>16:30</t>
-        </is>
-      </c>
-      <c r="E691" s="11" t="n">
-        <v>90</v>
-      </c>
-      <c r="F691" s="11" t="inlineStr">
-        <is>
-          <t>Timber Ridge Reserve</t>
-        </is>
-      </c>
-      <c r="G691" s="11" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H691" s="11" t="inlineStr">
-        <is>
-          <t>Full</t>
-        </is>
-      </c>
-      <c r="I691" s="12" t="inlineStr">
-        <is>
-          <t>Pitch 1</t>
-        </is>
-      </c>
-      <c r="J691" s="11" t="inlineStr">
-        <is>
-          <t>Seniors</t>
-        </is>
-      </c>
-      <c r="K691" s="12" t="inlineStr">
-        <is>
-          <t>Keysborough District FC Seniors Keysborough District FC</t>
-        </is>
-      </c>
-      <c r="L691" s="12" t="inlineStr">
-        <is>
-          <t>Manningham United Blues FC Seniors</t>
-        </is>
-      </c>
-      <c r="M691" s="12" t="inlineStr">
-        <is>
-          <t>Men's Metropolitan League</t>
-        </is>
-      </c>
-      <c r="N691" s="11" t="inlineStr">
-        <is>
-          <t>Men's Metropolitan League 7 South-East</t>
-        </is>
-      </c>
-      <c r="O691" s="11" t="inlineStr">
-        <is>
-          <t>R17</t>
-        </is>
-      </c>
-      <c r="P691" s="11" t="inlineStr"/>
-      <c r="Q691" s="12" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:Q691"/>
+  <autoFilter ref="A1:Q690"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Auto-refresh fixtures from Dribl (2026-08-27)
</commit_message>
<xml_diff>
--- a/Manningham_fixtures_and_overlaps.xlsx
+++ b/Manningham_fixtures_and_overlaps.xlsx
@@ -596,7 +596,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Source: fv.dribl.com, 2026 season, generated 25 Aug 2026</t>
+          <t>Source: fv.dribl.com, 2026 season, generated 27 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
         </is>
       </c>
       <c r="B11" s="8" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -50275,16 +50275,16 @@
       </c>
       <c r="C653" s="11" t="inlineStr">
         <is>
-          <t>10:10</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="D653" s="11" t="inlineStr">
         <is>
-          <t>10:50</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="E653" s="11" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="F653" s="11" t="inlineStr">
         <is>
@@ -50308,27 +50308,27 @@
       </c>
       <c r="J653" s="11" t="inlineStr">
         <is>
-          <t>U09</t>
+          <t>U13</t>
         </is>
       </c>
       <c r="K653" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Kangaroos Mixed (Emerton's)</t>
+          <t>Manningham United Blues FC U13 Juniors - C Mixed (Martin)</t>
         </is>
       </c>
       <c r="L653" s="12" t="inlineStr">
         <is>
-          <t>Monash City Villarreal FC U09 MiniRoos - Kangaroos Mixed Monash City Villarreal FC U8 Yellow</t>
+          <t>Whitehorse United SC U13 Juniors - C Mixed Shane</t>
         </is>
       </c>
       <c r="M653" s="12" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Sunday (U6 - U11)</t>
+          <t>Junior Mixed Sunday (U12 - U16)</t>
         </is>
       </c>
       <c r="N653" s="11" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Sunday East 9 Kangaroos Red</t>
+          <t>Mixed Sunday East 13C Red</t>
         </is>
       </c>
       <c r="O653" s="11" t="inlineStr">
@@ -50357,11 +50357,11 @@
       </c>
       <c r="D654" s="9" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>12:10</t>
         </is>
       </c>
       <c r="E654" s="9" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="F654" s="9" t="inlineStr">
         <is>
@@ -50380,32 +50380,32 @@
       </c>
       <c r="I654" s="10" t="inlineStr">
         <is>
-          <t>Pitch 1B</t>
+          <t>Pitch 1 - Midi Field B</t>
         </is>
       </c>
       <c r="J654" s="9" t="inlineStr">
         <is>
-          <t>U13</t>
+          <t>U11</t>
         </is>
       </c>
       <c r="K654" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - C Mixed (Martin)</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Female Miniroos Girls U11W (Holly &amp; Marina)</t>
         </is>
       </c>
       <c r="L654" s="10" t="inlineStr">
         <is>
-          <t>Whitehorse United SC U13 Juniors - C Mixed Shane</t>
+          <t>Malvern City FC U11 MiniRoos - Wallabies Female U11 MCFC Girls</t>
         </is>
       </c>
       <c r="M654" s="10" t="inlineStr">
         <is>
-          <t>Junior Mixed Sunday (U12 - U16)</t>
+          <t>Coles MiniRoos Girls' Sunday (U6 - U11)</t>
         </is>
       </c>
       <c r="N654" s="9" t="inlineStr">
         <is>
-          <t>Mixed Sunday East 13C Red</t>
+          <t>Coles MiniRoos Girls' East 11 Wallabies</t>
         </is>
       </c>
       <c r="O654" s="9" t="inlineStr">
@@ -50429,16 +50429,16 @@
       </c>
       <c r="C655" s="11" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="D655" s="11" t="inlineStr">
         <is>
-          <t>12:10</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="E655" s="11" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="F655" s="11" t="inlineStr">
         <is>
@@ -50452,37 +50452,37 @@
       </c>
       <c r="H655" s="11" t="inlineStr">
         <is>
-          <t>Sub</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="I655" s="12" t="inlineStr">
         <is>
-          <t>Pitch 1 - Midi Field B</t>
+          <t>Pitch 1</t>
         </is>
       </c>
       <c r="J655" s="11" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>U14</t>
         </is>
       </c>
       <c r="K655" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Female Miniroos Girls U11W (Holly &amp; Marina)</t>
+          <t>Manningham United Blues FC U14 Juniors - A Female (Chloe)</t>
         </is>
       </c>
       <c r="L655" s="12" t="inlineStr">
         <is>
-          <t>Malvern City FC U11 MiniRoos - Wallabies Female U11 MCFC Girls</t>
+          <t>Alamein FC U14 Juniors - A Female</t>
         </is>
       </c>
       <c r="M655" s="12" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Girls' Sunday (U6 - U11)</t>
+          <t>Junior Girls Sunday (U12 - U18)</t>
         </is>
       </c>
       <c r="N655" s="11" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Girls' East 11 Wallabies</t>
+          <t>Girls' South-East 14A</t>
         </is>
       </c>
       <c r="O655" s="11" t="inlineStr">
@@ -50506,16 +50506,16 @@
       </c>
       <c r="C656" s="9" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>14:45</t>
         </is>
       </c>
       <c r="D656" s="9" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>15:55</t>
         </is>
       </c>
       <c r="E656" s="9" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F656" s="9" t="inlineStr">
         <is>
@@ -50539,17 +50539,17 @@
       </c>
       <c r="J656" s="9" t="inlineStr">
         <is>
-          <t>U14</t>
+          <t>U17/18</t>
         </is>
       </c>
       <c r="K656" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - A Female (Chloe)</t>
+          <t>Manningham United Blues FC U17/18 Juniors - B Female (Marilyn)</t>
         </is>
       </c>
       <c r="L656" s="10" t="inlineStr">
         <is>
-          <t>Alamein FC U14 Juniors - A Female</t>
+          <t>Mount Eliza SC U17/18 Juniors - B Female Red</t>
         </is>
       </c>
       <c r="M656" s="10" t="inlineStr">
@@ -50559,7 +50559,7 @@
       </c>
       <c r="N656" s="9" t="inlineStr">
         <is>
-          <t>Girls' South-East 14A</t>
+          <t>Girls' South-East 17/18B</t>
         </is>
       </c>
       <c r="O656" s="9" t="inlineStr">
@@ -50571,312 +50571,328 @@
       <c r="Q656" s="10" t="inlineStr"/>
     </row>
     <row r="657">
-      <c r="A657" s="11" t="inlineStr">
+      <c r="A657" s="13" t="inlineStr">
         <is>
           <t>30 Aug 2026</t>
         </is>
       </c>
-      <c r="B657" s="11" t="inlineStr">
+      <c r="B657" s="13" t="inlineStr">
         <is>
           <t>Sun</t>
         </is>
       </c>
-      <c r="C657" s="11" t="inlineStr">
-        <is>
-          <t>14:45</t>
-        </is>
-      </c>
-      <c r="D657" s="11" t="inlineStr">
-        <is>
-          <t>15:55</t>
-        </is>
-      </c>
-      <c r="E657" s="11" t="n">
-        <v>70</v>
-      </c>
-      <c r="F657" s="11" t="inlineStr">
+      <c r="C657" s="13" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="D657" s="13" t="inlineStr">
+        <is>
+          <t>09:40</t>
+        </is>
+      </c>
+      <c r="E657" s="13" t="n">
+        <v>40</v>
+      </c>
+      <c r="F657" s="13" t="inlineStr">
         <is>
           <t>Powerful Owl Park</t>
         </is>
       </c>
-      <c r="G657" s="11" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H657" s="11" t="inlineStr">
-        <is>
-          <t>Full</t>
-        </is>
-      </c>
-      <c r="I657" s="12" t="inlineStr">
-        <is>
-          <t>Pitch 1</t>
-        </is>
-      </c>
-      <c r="J657" s="11" t="inlineStr">
-        <is>
-          <t>U17/18</t>
-        </is>
-      </c>
-      <c r="K657" s="12" t="inlineStr">
-        <is>
-          <t>Manningham United Blues FC U17/18 Juniors - B Female (Marilyn)</t>
-        </is>
-      </c>
-      <c r="L657" s="12" t="inlineStr">
-        <is>
-          <t>Mount Eliza SC U17/18 Juniors - B Female Red</t>
-        </is>
-      </c>
-      <c r="M657" s="12" t="inlineStr">
-        <is>
-          <t>Junior Girls Sunday (U12 - U18)</t>
-        </is>
-      </c>
-      <c r="N657" s="11" t="inlineStr">
-        <is>
-          <t>Girls' South-East 17/18B</t>
-        </is>
-      </c>
-      <c r="O657" s="11" t="inlineStr">
+      <c r="G657" s="13" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H657" s="13" t="inlineStr">
+        <is>
+          <t>Sub</t>
+        </is>
+      </c>
+      <c r="I657" s="14" t="inlineStr">
+        <is>
+          <t>Pitch 2A</t>
+        </is>
+      </c>
+      <c r="J657" s="13" t="inlineStr">
+        <is>
+          <t>U11</t>
+        </is>
+      </c>
+      <c r="K657" s="14" t="inlineStr">
+        <is>
+          <t>Manningham United Blues FC U11 MiniRoos - Kangaroos Mixed</t>
+        </is>
+      </c>
+      <c r="L657" s="14" t="inlineStr">
+        <is>
+          <t>FC Bulleen Lions U11 MiniRoos - Kangaroos Mixed Anthony &amp; Rob</t>
+        </is>
+      </c>
+      <c r="M657" s="14" t="inlineStr">
+        <is>
+          <t>Coles MiniRoos Mixed Sunday (U6 - U11)</t>
+        </is>
+      </c>
+      <c r="N657" s="13" t="inlineStr">
+        <is>
+          <t>Coles MiniRoos Mixed Sunday East 11 Kangaroos Red</t>
+        </is>
+      </c>
+      <c r="O657" s="13" t="inlineStr">
         <is>
           <t>R17</t>
         </is>
       </c>
-      <c r="P657" s="11" t="inlineStr"/>
-      <c r="Q657" s="12" t="inlineStr"/>
+      <c r="P657" s="15" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Q657" s="14" t="inlineStr"/>
     </row>
     <row r="658">
-      <c r="A658" s="9" t="inlineStr">
+      <c r="A658" s="13" t="inlineStr">
         <is>
           <t>30 Aug 2026</t>
         </is>
       </c>
-      <c r="B658" s="9" t="inlineStr">
+      <c r="B658" s="13" t="inlineStr">
         <is>
           <t>Sun</t>
         </is>
       </c>
-      <c r="C658" s="9" t="inlineStr">
+      <c r="C658" s="13" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="D658" s="9" t="inlineStr">
+      <c r="D658" s="13" t="inlineStr">
         <is>
           <t>09:40</t>
         </is>
       </c>
-      <c r="E658" s="9" t="n">
+      <c r="E658" s="13" t="n">
         <v>40</v>
       </c>
-      <c r="F658" s="9" t="inlineStr">
+      <c r="F658" s="13" t="inlineStr">
         <is>
           <t>Powerful Owl Park</t>
         </is>
       </c>
-      <c r="G658" s="9" t="inlineStr">
+      <c r="G658" s="13" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="H658" s="9" t="inlineStr">
+      <c r="H658" s="13" t="inlineStr">
         <is>
           <t>Sub</t>
         </is>
       </c>
-      <c r="I658" s="10" t="inlineStr">
-        <is>
-          <t>Pitch 2A</t>
-        </is>
-      </c>
-      <c r="J658" s="9" t="inlineStr">
-        <is>
-          <t>U11</t>
-        </is>
-      </c>
-      <c r="K658" s="10" t="inlineStr">
-        <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Kangaroos Mixed</t>
-        </is>
-      </c>
-      <c r="L658" s="10" t="inlineStr">
-        <is>
-          <t>FC Bulleen Lions U11 MiniRoos - Kangaroos Mixed Anthony &amp; Rob</t>
-        </is>
-      </c>
-      <c r="M658" s="10" t="inlineStr">
+      <c r="I658" s="14" t="inlineStr">
+        <is>
+          <t>Pitch 2 - Midi B</t>
+        </is>
+      </c>
+      <c r="J658" s="13" t="inlineStr">
+        <is>
+          <t>U07</t>
+        </is>
+      </c>
+      <c r="K658" s="14" t="inlineStr">
+        <is>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Red)</t>
+        </is>
+      </c>
+      <c r="L658" s="14" t="inlineStr">
+        <is>
+          <t>East Malvern Junior SC U07 MiniRoos - Joeys Mixed EMJSC U7 Sunday Orange</t>
+        </is>
+      </c>
+      <c r="M658" s="14" t="inlineStr">
         <is>
           <t>Coles MiniRoos Mixed Sunday (U6 - U11)</t>
         </is>
       </c>
-      <c r="N658" s="9" t="inlineStr">
-        <is>
-          <t>Coles MiniRoos Mixed Sunday East 11 Kangaroos Red</t>
-        </is>
-      </c>
-      <c r="O658" s="9" t="inlineStr">
+      <c r="N658" s="13" t="inlineStr">
+        <is>
+          <t>Coles MiniRoos Mixed Sunday East 7 Joeys Red</t>
+        </is>
+      </c>
+      <c r="O658" s="13" t="inlineStr">
         <is>
           <t>R17</t>
         </is>
       </c>
-      <c r="P658" s="9" t="inlineStr"/>
-      <c r="Q658" s="10" t="inlineStr"/>
+      <c r="P658" s="15" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Q658" s="14" t="inlineStr"/>
     </row>
     <row r="659">
-      <c r="A659" s="11" t="inlineStr">
+      <c r="A659" s="13" t="inlineStr">
         <is>
           <t>30 Aug 2026</t>
         </is>
       </c>
-      <c r="B659" s="11" t="inlineStr">
+      <c r="B659" s="13" t="inlineStr">
         <is>
           <t>Sun</t>
         </is>
       </c>
-      <c r="C659" s="11" t="inlineStr">
+      <c r="C659" s="13" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="D659" s="11" t="inlineStr">
+      <c r="D659" s="13" t="inlineStr">
         <is>
           <t>09:40</t>
         </is>
       </c>
-      <c r="E659" s="11" t="n">
+      <c r="E659" s="13" t="n">
         <v>40</v>
       </c>
-      <c r="F659" s="11" t="inlineStr">
+      <c r="F659" s="13" t="inlineStr">
         <is>
           <t>Powerful Owl Park</t>
         </is>
       </c>
-      <c r="G659" s="11" t="inlineStr">
+      <c r="G659" s="13" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="H659" s="11" t="inlineStr">
+      <c r="H659" s="13" t="inlineStr">
         <is>
           <t>Sub</t>
         </is>
       </c>
-      <c r="I659" s="12" t="inlineStr">
-        <is>
-          <t>Pitch 2 - Midi B</t>
-        </is>
-      </c>
-      <c r="J659" s="11" t="inlineStr">
+      <c r="I659" s="14" t="inlineStr">
+        <is>
+          <t>Pitch 2 - Midi A</t>
+        </is>
+      </c>
+      <c r="J659" s="13" t="inlineStr">
         <is>
           <t>U07</t>
         </is>
       </c>
-      <c r="K659" s="12" t="inlineStr">
-        <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Red)</t>
-        </is>
-      </c>
-      <c r="L659" s="12" t="inlineStr">
-        <is>
-          <t>East Malvern Junior SC U07 MiniRoos - Joeys Mixed EMJSC U7 Sunday Orange</t>
-        </is>
-      </c>
-      <c r="M659" s="12" t="inlineStr">
+      <c r="K659" s="14" t="inlineStr">
+        <is>
+          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Green)</t>
+        </is>
+      </c>
+      <c r="L659" s="14" t="inlineStr">
+        <is>
+          <t>Doncaster Rovers SC U07 MiniRoos - Joeys Mixed</t>
+        </is>
+      </c>
+      <c r="M659" s="14" t="inlineStr">
         <is>
           <t>Coles MiniRoos Mixed Sunday (U6 - U11)</t>
         </is>
       </c>
-      <c r="N659" s="11" t="inlineStr">
+      <c r="N659" s="13" t="inlineStr">
         <is>
           <t>Coles MiniRoos Mixed Sunday East 7 Joeys Red</t>
         </is>
       </c>
-      <c r="O659" s="11" t="inlineStr">
+      <c r="O659" s="13" t="inlineStr">
         <is>
           <t>R17</t>
         </is>
       </c>
-      <c r="P659" s="11" t="inlineStr"/>
-      <c r="Q659" s="12" t="inlineStr"/>
+      <c r="P659" s="15" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Q659" s="14" t="inlineStr"/>
     </row>
     <row r="660">
-      <c r="A660" s="9" t="inlineStr">
+      <c r="A660" s="13" t="inlineStr">
         <is>
           <t>30 Aug 2026</t>
         </is>
       </c>
-      <c r="B660" s="9" t="inlineStr">
+      <c r="B660" s="13" t="inlineStr">
         <is>
           <t>Sun</t>
         </is>
       </c>
-      <c r="C660" s="9" t="inlineStr">
+      <c r="C660" s="13" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="D660" s="9" t="inlineStr">
+      <c r="D660" s="13" t="inlineStr">
         <is>
           <t>09:40</t>
         </is>
       </c>
-      <c r="E660" s="9" t="n">
+      <c r="E660" s="13" t="n">
         <v>40</v>
       </c>
-      <c r="F660" s="9" t="inlineStr">
+      <c r="F660" s="13" t="inlineStr">
         <is>
           <t>Powerful Owl Park</t>
         </is>
       </c>
-      <c r="G660" s="9" t="inlineStr">
+      <c r="G660" s="13" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="H660" s="9" t="inlineStr">
+      <c r="H660" s="13" t="inlineStr">
         <is>
           <t>Sub</t>
         </is>
       </c>
-      <c r="I660" s="10" t="inlineStr">
-        <is>
-          <t>Pitch 2 - Midi A</t>
-        </is>
-      </c>
-      <c r="J660" s="9" t="inlineStr">
-        <is>
-          <t>U07</t>
-        </is>
-      </c>
-      <c r="K660" s="10" t="inlineStr">
-        <is>
-          <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Green)</t>
-        </is>
-      </c>
-      <c r="L660" s="10" t="inlineStr">
-        <is>
-          <t>Doncaster Rovers SC U07 MiniRoos - Joeys Mixed</t>
-        </is>
-      </c>
-      <c r="M660" s="10" t="inlineStr">
+      <c r="I660" s="14" t="inlineStr">
+        <is>
+          <t>Pitch 2B</t>
+        </is>
+      </c>
+      <c r="J660" s="13" t="inlineStr">
+        <is>
+          <t>U09</t>
+        </is>
+      </c>
+      <c r="K660" s="14" t="inlineStr">
+        <is>
+          <t>Manningham United Blues FC U09 MiniRoos - Kangaroos Mixed (Emerton's)</t>
+        </is>
+      </c>
+      <c r="L660" s="14" t="inlineStr">
+        <is>
+          <t>Monash City Villarreal FC U09 MiniRoos - Kangaroos Mixed Monash City Villarreal FC U8 Yellow</t>
+        </is>
+      </c>
+      <c r="M660" s="14" t="inlineStr">
         <is>
           <t>Coles MiniRoos Mixed Sunday (U6 - U11)</t>
         </is>
       </c>
-      <c r="N660" s="9" t="inlineStr">
-        <is>
-          <t>Coles MiniRoos Mixed Sunday East 7 Joeys Red</t>
-        </is>
-      </c>
-      <c r="O660" s="9" t="inlineStr">
+      <c r="N660" s="13" t="inlineStr">
+        <is>
+          <t>Coles MiniRoos Mixed Sunday East 9 Kangaroos Red</t>
+        </is>
+      </c>
+      <c r="O660" s="13" t="inlineStr">
         <is>
           <t>R17</t>
         </is>
       </c>
-      <c r="P660" s="9" t="inlineStr"/>
-      <c r="Q660" s="10" t="inlineStr"/>
+      <c r="P660" s="15" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Q660" s="14" t="inlineStr"/>
     </row>
     <row r="661">
       <c r="A661" s="11" t="inlineStr">
@@ -53204,7 +53220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -53256,7 +53272,7 @@
     <row r="7">
       <c r="A7" s="17" t="inlineStr">
         <is>
-          <t>A.  Over-capacity moments: 9 found</t>
+          <t>A.  Over-capacity moments: 10 found</t>
         </is>
       </c>
     </row>
@@ -53712,79 +53728,94 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="22" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="B18" s="20" t="inlineStr">
+        <is>
+          <t>30 Aug 2026</t>
+        </is>
+      </c>
+      <c r="C18" s="20" t="inlineStr">
+        <is>
+          <t>Powerful Owl Park</t>
+        </is>
+      </c>
+      <c r="D18" s="20" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E18" s="21" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="F18" s="20" t="inlineStr">
+        <is>
+          <t>09:40</t>
+        </is>
+      </c>
+      <c r="G18" s="21" t="inlineStr">
+        <is>
+          <t>Pitch over capacity</t>
+        </is>
+      </c>
+      <c r="H18" s="20" t="inlineStr">
+        <is>
+          <t>1×U10-13, 1×U8/9, 2×U6/7 = 1.25</t>
+        </is>
+      </c>
+      <c r="I18" s="20" t="inlineStr">
+        <is>
+          <t>09:00 U11 Pitch 2A (Manningham United Blues FC U11 MiniRoos - Kangaroos Mixed v FC Bulleen Lions U11 MiniRoos - Kangaroos Mixed Anthony &amp; Rob)  |  09:00 U07 Pitch 2 - Midi B (Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Red) v East Malvern Junior SC U07 MiniRoos - Joeys Mixed EMJSC U7 Sunday Orange)  |  09:00 U07 Pitch 2 - Midi A (Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Green) v Doncaster Rovers SC U07 MiniRoos - Joeys Mixed)  |  09:00 U09 Pitch 2B (Manningham United Blues FC U09 MiniRoos - Kangaroos Mixed (Emerton's) v Monash City Villarreal FC U09 MiniRoos - Kangaroos Mixed Monash City Villarreal FC U8 Yellow)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="22" t="inlineStr">
         <is>
           <t>B.  Peak simultaneous games per ground (busiest moment)</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>Ground</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>Max at once</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="D22" s="3" t="inlineStr">
         <is>
           <t>From</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="E22" s="3" t="inlineStr">
         <is>
           <t>Until</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="F22" s="3" t="inlineStr">
         <is>
           <t>Pitches in use then</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="21" t="inlineStr">
-        <is>
-          <t>Pettys Reserve</t>
-        </is>
-      </c>
-      <c r="B22" s="20" t="n">
-        <v>7</v>
-      </c>
-      <c r="C22" s="20" t="inlineStr">
-        <is>
-          <t>Sat 16 May 2026</t>
-        </is>
-      </c>
-      <c r="D22" s="20" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="E22" s="20" t="inlineStr">
-        <is>
-          <t>09:10</t>
-        </is>
-      </c>
-      <c r="F22" s="21" t="inlineStr">
-        <is>
-          <t>Pitch 1A (Bottom Field), Pitch 1B (Bottom Field), Pitch 1E (Bottom Field) - Quarter Pitch 4v4, Pitch 1F (Bottom Field) - Quarter Pitch 4v4, Pitch 2A (Top Field), Pitch 2C (Top Field) - Quarter Pitch 7v7, Pitch 2D (Top Field) - Quarter Pitch 7v7</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="19" t="inlineStr">
         <is>
-          <t>Powerful Owl Park</t>
+          <t>Pettys Reserve</t>
         </is>
       </c>
       <c r="B23" s="18" t="n">
@@ -53792,7 +53823,7 @@
       </c>
       <c r="C23" s="18" t="inlineStr">
         <is>
-          <t>Sun 09 Aug 2026</t>
+          <t>Sat 16 May 2026</t>
         </is>
       </c>
       <c r="D23" s="18" t="inlineStr">
@@ -53807,35 +53838,65 @@
       </c>
       <c r="F23" s="19" t="inlineStr">
         <is>
-          <t>Pitch 1 - Midi Field A, Pitch 1 - Midi Field B, Pitch 1B, Pitch 2A, Pitch 2B, Pitch 3A, Pitch 3B</t>
+          <t>Pitch 1A (Bottom Field), Pitch 1B (Bottom Field), Pitch 1E (Bottom Field) - Quarter Pitch 4v4, Pitch 1F (Bottom Field) - Quarter Pitch 4v4, Pitch 2A (Top Field), Pitch 2C (Top Field) - Quarter Pitch 7v7, Pitch 2D (Top Field) - Quarter Pitch 7v7</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="21" t="inlineStr">
         <is>
+          <t>Powerful Owl Park</t>
+        </is>
+      </c>
+      <c r="B24" s="20" t="n">
+        <v>7</v>
+      </c>
+      <c r="C24" s="20" t="inlineStr">
+        <is>
+          <t>Sun 09 Aug 2026</t>
+        </is>
+      </c>
+      <c r="D24" s="20" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="E24" s="20" t="inlineStr">
+        <is>
+          <t>09:10</t>
+        </is>
+      </c>
+      <c r="F24" s="21" t="inlineStr">
+        <is>
+          <t>Pitch 1 - Midi Field A, Pitch 1 - Midi Field B, Pitch 1B, Pitch 2A, Pitch 2B, Pitch 3A, Pitch 3B</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="19" t="inlineStr">
+        <is>
           <t>Timber Ridge Reserve</t>
         </is>
       </c>
-      <c r="B24" s="20" t="n">
+      <c r="B25" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="C24" s="20" t="inlineStr">
+      <c r="C25" s="18" t="inlineStr">
         <is>
           <t>Sat 18 Jul 2026</t>
         </is>
       </c>
-      <c r="D24" s="20" t="inlineStr">
+      <c r="D25" s="18" t="inlineStr">
         <is>
           <t>09:40</t>
         </is>
       </c>
-      <c r="E24" s="20" t="inlineStr">
+      <c r="E25" s="18" t="inlineStr">
         <is>
           <t>10:40</t>
         </is>
       </c>
-      <c r="F24" s="21" t="inlineStr">
+      <c r="F25" s="19" t="inlineStr">
         <is>
           <t>Pitch 1A, Pitch 1B</t>
         </is>

</xml_diff>

<commit_message>
Add 30 Aug Powl override: U09 Emerton's -> Pitch 1D, resolving field-2 over-capacity
Sun 30 Aug 09:00 Powerful Owl field 2 was over capacity (1.25) after the U09
Kangaroos (Emerton's) game landed on Pitch 2B, which also breaches the U8/9
banned-location rule there. Moved to Pitch 1D (field 1, still under capacity
at 1.0 with the other three quarter-pitch games already scheduled 09:00-09:45).
</commit_message>
<xml_diff>
--- a/Manningham_fixtures_and_overlaps.xlsx
+++ b/Manningham_fixtures_and_overlaps.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="All Games" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Overlaps &amp; Peak Load" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Games" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overlaps &amp; Peak Load" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Games'!$A$1:$Q$690</definedName>
@@ -596,7 +596,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Source: fv.dribl.com, 2026 season, generated 27 Aug 2026</t>
+          <t>Source: fv.dribl.com, 2026 season, generated 28 Aug 2026</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
         </is>
       </c>
       <c r="B11" s="8" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -50121,12 +50121,12 @@
       </c>
       <c r="C651" s="11" t="inlineStr">
         <is>
-          <t>10:10</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="D651" s="11" t="inlineStr">
         <is>
-          <t>10:50</t>
+          <t>09:40</t>
         </is>
       </c>
       <c r="E651" s="11" t="n">
@@ -50149,32 +50149,32 @@
       </c>
       <c r="I651" s="12" t="inlineStr">
         <is>
-          <t>Pitch 1 - Midi Field A</t>
+          <t>Pitch 1D</t>
         </is>
       </c>
       <c r="J651" s="11" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>U09</t>
         </is>
       </c>
       <c r="K651" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Joeys Female (Grace)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Kangaroos Mixed (Emerton's)</t>
         </is>
       </c>
       <c r="L651" s="12" t="inlineStr">
         <is>
-          <t>Croydon City SC U11 MiniRoos - Joeys Female U11 - CCSC</t>
+          <t>Monash City Villarreal FC U09 MiniRoos - Kangaroos Mixed Monash City Villarreal FC U8 Yellow</t>
         </is>
       </c>
       <c r="M651" s="12" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Girls' Sunday (U6 - U11)</t>
+          <t>Coles MiniRoos Mixed Sunday (U6 - U11)</t>
         </is>
       </c>
       <c r="N651" s="11" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Girls' East 11 Joeys</t>
+          <t>Coles MiniRoos Mixed Sunday East 9 Kangaroos Red</t>
         </is>
       </c>
       <c r="O651" s="11" t="inlineStr">
@@ -50183,7 +50183,11 @@
         </is>
       </c>
       <c r="P651" s="11" t="inlineStr"/>
-      <c r="Q651" s="12" t="inlineStr"/>
+      <c r="Q651" s="12" t="inlineStr">
+        <is>
+          <t>Powerful Owl Park Pitch 2B</t>
+        </is>
+      </c>
     </row>
     <row r="652">
       <c r="A652" s="9" t="inlineStr">
@@ -50226,32 +50230,32 @@
       </c>
       <c r="I652" s="10" t="inlineStr">
         <is>
-          <t>Pitch 1 - Midi Field B</t>
+          <t>Pitch 1 - Midi Field A</t>
         </is>
       </c>
       <c r="J652" s="9" t="inlineStr">
         <is>
-          <t>U09</t>
+          <t>U11</t>
         </is>
       </c>
       <c r="K652" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Cahill's)</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Joeys Female (Grace)</t>
         </is>
       </c>
       <c r="L652" s="10" t="inlineStr">
         <is>
-          <t>Ashburton United SC U09 MiniRoos - Wallabies Mixed (Leo)</t>
+          <t>Croydon City SC U11 MiniRoos - Joeys Female U11 - CCSC</t>
         </is>
       </c>
       <c r="M652" s="10" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Sunday (U6 - U11)</t>
+          <t>Coles MiniRoos Girls' Sunday (U6 - U11)</t>
         </is>
       </c>
       <c r="N652" s="9" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Mixed Sunday East 9 Wallabies</t>
+          <t>Coles MiniRoos Girls' East 11 Joeys</t>
         </is>
       </c>
       <c r="O652" s="9" t="inlineStr">
@@ -50275,16 +50279,16 @@
       </c>
       <c r="C653" s="11" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>10:10</t>
         </is>
       </c>
       <c r="D653" s="11" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>10:50</t>
         </is>
       </c>
       <c r="E653" s="11" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="F653" s="11" t="inlineStr">
         <is>
@@ -50303,32 +50307,32 @@
       </c>
       <c r="I653" s="12" t="inlineStr">
         <is>
-          <t>Pitch 1B</t>
+          <t>Pitch 1 - Midi Field B</t>
         </is>
       </c>
       <c r="J653" s="11" t="inlineStr">
         <is>
-          <t>U13</t>
+          <t>U09</t>
         </is>
       </c>
       <c r="K653" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U13 Juniors - C Mixed (Martin)</t>
+          <t>Manningham United Blues FC U09 MiniRoos - Wallabies Mixed (Cahill's)</t>
         </is>
       </c>
       <c r="L653" s="12" t="inlineStr">
         <is>
-          <t>Whitehorse United SC U13 Juniors - C Mixed Shane</t>
+          <t>Ashburton United SC U09 MiniRoos - Wallabies Mixed (Leo)</t>
         </is>
       </c>
       <c r="M653" s="12" t="inlineStr">
         <is>
-          <t>Junior Mixed Sunday (U12 - U16)</t>
+          <t>Coles MiniRoos Mixed Sunday (U6 - U11)</t>
         </is>
       </c>
       <c r="N653" s="11" t="inlineStr">
         <is>
-          <t>Mixed Sunday East 13C Red</t>
+          <t>Coles MiniRoos Mixed Sunday East 9 Wallabies</t>
         </is>
       </c>
       <c r="O653" s="11" t="inlineStr">
@@ -50357,11 +50361,11 @@
       </c>
       <c r="D654" s="9" t="inlineStr">
         <is>
-          <t>12:10</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="E654" s="9" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="F654" s="9" t="inlineStr">
         <is>
@@ -50380,32 +50384,32 @@
       </c>
       <c r="I654" s="10" t="inlineStr">
         <is>
-          <t>Pitch 1 - Midi Field B</t>
+          <t>Pitch 1B</t>
         </is>
       </c>
       <c r="J654" s="9" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>U13</t>
         </is>
       </c>
       <c r="K654" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Female Miniroos Girls U11W (Holly &amp; Marina)</t>
+          <t>Manningham United Blues FC U13 Juniors - C Mixed (Martin)</t>
         </is>
       </c>
       <c r="L654" s="10" t="inlineStr">
         <is>
-          <t>Malvern City FC U11 MiniRoos - Wallabies Female U11 MCFC Girls</t>
+          <t>Whitehorse United SC U13 Juniors - C Mixed Shane</t>
         </is>
       </c>
       <c r="M654" s="10" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Girls' Sunday (U6 - U11)</t>
+          <t>Junior Mixed Sunday (U12 - U16)</t>
         </is>
       </c>
       <c r="N654" s="9" t="inlineStr">
         <is>
-          <t>Coles MiniRoos Girls' East 11 Wallabies</t>
+          <t>Mixed Sunday East 13C Red</t>
         </is>
       </c>
       <c r="O654" s="9" t="inlineStr">
@@ -50429,16 +50433,16 @@
       </c>
       <c r="C655" s="11" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="D655" s="11" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>12:10</t>
         </is>
       </c>
       <c r="E655" s="11" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="F655" s="11" t="inlineStr">
         <is>
@@ -50452,37 +50456,37 @@
       </c>
       <c r="H655" s="11" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Sub</t>
         </is>
       </c>
       <c r="I655" s="12" t="inlineStr">
         <is>
-          <t>Pitch 1</t>
+          <t>Pitch 1 - Midi Field B</t>
         </is>
       </c>
       <c r="J655" s="11" t="inlineStr">
         <is>
-          <t>U14</t>
+          <t>U11</t>
         </is>
       </c>
       <c r="K655" s="12" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U14 Juniors - A Female (Chloe)</t>
+          <t>Manningham United Blues FC U11 MiniRoos - Wallabies Female Miniroos Girls U11W (Holly &amp; Marina)</t>
         </is>
       </c>
       <c r="L655" s="12" t="inlineStr">
         <is>
-          <t>Alamein FC U14 Juniors - A Female</t>
+          <t>Malvern City FC U11 MiniRoos - Wallabies Female U11 MCFC Girls</t>
         </is>
       </c>
       <c r="M655" s="12" t="inlineStr">
         <is>
-          <t>Junior Girls Sunday (U12 - U18)</t>
+          <t>Coles MiniRoos Girls' Sunday (U6 - U11)</t>
         </is>
       </c>
       <c r="N655" s="11" t="inlineStr">
         <is>
-          <t>Girls' South-East 14A</t>
+          <t>Coles MiniRoos Girls' East 11 Wallabies</t>
         </is>
       </c>
       <c r="O655" s="11" t="inlineStr">
@@ -50506,16 +50510,16 @@
       </c>
       <c r="C656" s="9" t="inlineStr">
         <is>
-          <t>14:45</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="D656" s="9" t="inlineStr">
         <is>
-          <t>15:55</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="E656" s="9" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="F656" s="9" t="inlineStr">
         <is>
@@ -50539,17 +50543,17 @@
       </c>
       <c r="J656" s="9" t="inlineStr">
         <is>
-          <t>U17/18</t>
+          <t>U14</t>
         </is>
       </c>
       <c r="K656" s="10" t="inlineStr">
         <is>
-          <t>Manningham United Blues FC U17/18 Juniors - B Female (Marilyn)</t>
+          <t>Manningham United Blues FC U14 Juniors - A Female (Chloe)</t>
         </is>
       </c>
       <c r="L656" s="10" t="inlineStr">
         <is>
-          <t>Mount Eliza SC U17/18 Juniors - B Female Red</t>
+          <t>Alamein FC U14 Juniors - A Female</t>
         </is>
       </c>
       <c r="M656" s="10" t="inlineStr">
@@ -50559,7 +50563,7 @@
       </c>
       <c r="N656" s="9" t="inlineStr">
         <is>
-          <t>Girls' South-East 17/18B</t>
+          <t>Girls' South-East 14A</t>
         </is>
       </c>
       <c r="O656" s="9" t="inlineStr">
@@ -50571,328 +50575,312 @@
       <c r="Q656" s="10" t="inlineStr"/>
     </row>
     <row r="657">
-      <c r="A657" s="13" t="inlineStr">
+      <c r="A657" s="11" t="inlineStr">
         <is>
           <t>30 Aug 2026</t>
         </is>
       </c>
-      <c r="B657" s="13" t="inlineStr">
+      <c r="B657" s="11" t="inlineStr">
         <is>
           <t>Sun</t>
         </is>
       </c>
-      <c r="C657" s="13" t="inlineStr">
+      <c r="C657" s="11" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="D657" s="11" t="inlineStr">
+        <is>
+          <t>15:55</t>
+        </is>
+      </c>
+      <c r="E657" s="11" t="n">
+        <v>70</v>
+      </c>
+      <c r="F657" s="11" t="inlineStr">
+        <is>
+          <t>Powerful Owl Park</t>
+        </is>
+      </c>
+      <c r="G657" s="11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H657" s="11" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="I657" s="12" t="inlineStr">
+        <is>
+          <t>Pitch 1</t>
+        </is>
+      </c>
+      <c r="J657" s="11" t="inlineStr">
+        <is>
+          <t>U17/18</t>
+        </is>
+      </c>
+      <c r="K657" s="12" t="inlineStr">
+        <is>
+          <t>Manningham United Blues FC U17/18 Juniors - B Female (Marilyn)</t>
+        </is>
+      </c>
+      <c r="L657" s="12" t="inlineStr">
+        <is>
+          <t>Mount Eliza SC U17/18 Juniors - B Female Red</t>
+        </is>
+      </c>
+      <c r="M657" s="12" t="inlineStr">
+        <is>
+          <t>Junior Girls Sunday (U12 - U18)</t>
+        </is>
+      </c>
+      <c r="N657" s="11" t="inlineStr">
+        <is>
+          <t>Girls' South-East 17/18B</t>
+        </is>
+      </c>
+      <c r="O657" s="11" t="inlineStr">
+        <is>
+          <t>R17</t>
+        </is>
+      </c>
+      <c r="P657" s="11" t="inlineStr"/>
+      <c r="Q657" s="12" t="inlineStr"/>
+    </row>
+    <row r="658">
+      <c r="A658" s="9" t="inlineStr">
+        <is>
+          <t>30 Aug 2026</t>
+        </is>
+      </c>
+      <c r="B658" s="9" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
+      <c r="C658" s="9" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="D657" s="13" t="inlineStr">
+      <c r="D658" s="9" t="inlineStr">
         <is>
           <t>09:40</t>
         </is>
       </c>
-      <c r="E657" s="13" t="n">
+      <c r="E658" s="9" t="n">
         <v>40</v>
       </c>
-      <c r="F657" s="13" t="inlineStr">
+      <c r="F658" s="9" t="inlineStr">
         <is>
           <t>Powerful Owl Park</t>
         </is>
       </c>
-      <c r="G657" s="13" t="inlineStr">
+      <c r="G658" s="9" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="H657" s="13" t="inlineStr">
+      <c r="H658" s="9" t="inlineStr">
         <is>
           <t>Sub</t>
         </is>
       </c>
-      <c r="I657" s="14" t="inlineStr">
+      <c r="I658" s="10" t="inlineStr">
         <is>
           <t>Pitch 2A</t>
         </is>
       </c>
-      <c r="J657" s="13" t="inlineStr">
+      <c r="J658" s="9" t="inlineStr">
         <is>
           <t>U11</t>
         </is>
       </c>
-      <c r="K657" s="14" t="inlineStr">
+      <c r="K658" s="10" t="inlineStr">
         <is>
           <t>Manningham United Blues FC U11 MiniRoos - Kangaroos Mixed</t>
         </is>
       </c>
-      <c r="L657" s="14" t="inlineStr">
+      <c r="L658" s="10" t="inlineStr">
         <is>
           <t>FC Bulleen Lions U11 MiniRoos - Kangaroos Mixed Anthony &amp; Rob</t>
         </is>
       </c>
-      <c r="M657" s="14" t="inlineStr">
+      <c r="M658" s="10" t="inlineStr">
         <is>
           <t>Coles MiniRoos Mixed Sunday (U6 - U11)</t>
         </is>
       </c>
-      <c r="N657" s="13" t="inlineStr">
+      <c r="N658" s="9" t="inlineStr">
         <is>
           <t>Coles MiniRoos Mixed Sunday East 11 Kangaroos Red</t>
         </is>
       </c>
-      <c r="O657" s="13" t="inlineStr">
+      <c r="O658" s="9" t="inlineStr">
         <is>
           <t>R17</t>
         </is>
       </c>
-      <c r="P657" s="15" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="Q657" s="14" t="inlineStr"/>
-    </row>
-    <row r="658">
-      <c r="A658" s="13" t="inlineStr">
+      <c r="P658" s="9" t="inlineStr"/>
+      <c r="Q658" s="10" t="inlineStr"/>
+    </row>
+    <row r="659">
+      <c r="A659" s="11" t="inlineStr">
         <is>
           <t>30 Aug 2026</t>
         </is>
       </c>
-      <c r="B658" s="13" t="inlineStr">
+      <c r="B659" s="11" t="inlineStr">
         <is>
           <t>Sun</t>
         </is>
       </c>
-      <c r="C658" s="13" t="inlineStr">
+      <c r="C659" s="11" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="D658" s="13" t="inlineStr">
+      <c r="D659" s="11" t="inlineStr">
         <is>
           <t>09:40</t>
         </is>
       </c>
-      <c r="E658" s="13" t="n">
+      <c r="E659" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="F658" s="13" t="inlineStr">
+      <c r="F659" s="11" t="inlineStr">
         <is>
           <t>Powerful Owl Park</t>
         </is>
       </c>
-      <c r="G658" s="13" t="inlineStr">
+      <c r="G659" s="11" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="H658" s="13" t="inlineStr">
+      <c r="H659" s="11" t="inlineStr">
         <is>
           <t>Sub</t>
         </is>
       </c>
-      <c r="I658" s="14" t="inlineStr">
+      <c r="I659" s="12" t="inlineStr">
         <is>
           <t>Pitch 2 - Midi B</t>
         </is>
       </c>
-      <c r="J658" s="13" t="inlineStr">
+      <c r="J659" s="11" t="inlineStr">
         <is>
           <t>U07</t>
         </is>
       </c>
-      <c r="K658" s="14" t="inlineStr">
+      <c r="K659" s="12" t="inlineStr">
         <is>
           <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Red)</t>
         </is>
       </c>
-      <c r="L658" s="14" t="inlineStr">
+      <c r="L659" s="12" t="inlineStr">
         <is>
           <t>East Malvern Junior SC U07 MiniRoos - Joeys Mixed EMJSC U7 Sunday Orange</t>
         </is>
       </c>
-      <c r="M658" s="14" t="inlineStr">
+      <c r="M659" s="12" t="inlineStr">
         <is>
           <t>Coles MiniRoos Mixed Sunday (U6 - U11)</t>
         </is>
       </c>
-      <c r="N658" s="13" t="inlineStr">
+      <c r="N659" s="11" t="inlineStr">
         <is>
           <t>Coles MiniRoos Mixed Sunday East 7 Joeys Red</t>
         </is>
       </c>
-      <c r="O658" s="13" t="inlineStr">
+      <c r="O659" s="11" t="inlineStr">
         <is>
           <t>R17</t>
         </is>
       </c>
-      <c r="P658" s="15" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="Q658" s="14" t="inlineStr"/>
-    </row>
-    <row r="659">
-      <c r="A659" s="13" t="inlineStr">
+      <c r="P659" s="11" t="inlineStr"/>
+      <c r="Q659" s="12" t="inlineStr"/>
+    </row>
+    <row r="660">
+      <c r="A660" s="9" t="inlineStr">
         <is>
           <t>30 Aug 2026</t>
         </is>
       </c>
-      <c r="B659" s="13" t="inlineStr">
+      <c r="B660" s="9" t="inlineStr">
         <is>
           <t>Sun</t>
         </is>
       </c>
-      <c r="C659" s="13" t="inlineStr">
+      <c r="C660" s="9" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="D659" s="13" t="inlineStr">
+      <c r="D660" s="9" t="inlineStr">
         <is>
           <t>09:40</t>
         </is>
       </c>
-      <c r="E659" s="13" t="n">
+      <c r="E660" s="9" t="n">
         <v>40</v>
       </c>
-      <c r="F659" s="13" t="inlineStr">
+      <c r="F660" s="9" t="inlineStr">
         <is>
           <t>Powerful Owl Park</t>
         </is>
       </c>
-      <c r="G659" s="13" t="inlineStr">
+      <c r="G660" s="9" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="H659" s="13" t="inlineStr">
+      <c r="H660" s="9" t="inlineStr">
         <is>
           <t>Sub</t>
         </is>
       </c>
-      <c r="I659" s="14" t="inlineStr">
+      <c r="I660" s="10" t="inlineStr">
         <is>
           <t>Pitch 2 - Midi A</t>
         </is>
       </c>
-      <c r="J659" s="13" t="inlineStr">
+      <c r="J660" s="9" t="inlineStr">
         <is>
           <t>U07</t>
         </is>
       </c>
-      <c r="K659" s="14" t="inlineStr">
+      <c r="K660" s="10" t="inlineStr">
         <is>
           <t>Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Green)</t>
         </is>
       </c>
-      <c r="L659" s="14" t="inlineStr">
+      <c r="L660" s="10" t="inlineStr">
         <is>
           <t>Doncaster Rovers SC U07 MiniRoos - Joeys Mixed</t>
         </is>
       </c>
-      <c r="M659" s="14" t="inlineStr">
+      <c r="M660" s="10" t="inlineStr">
         <is>
           <t>Coles MiniRoos Mixed Sunday (U6 - U11)</t>
         </is>
       </c>
-      <c r="N659" s="13" t="inlineStr">
+      <c r="N660" s="9" t="inlineStr">
         <is>
           <t>Coles MiniRoos Mixed Sunday East 7 Joeys Red</t>
         </is>
       </c>
-      <c r="O659" s="13" t="inlineStr">
+      <c r="O660" s="9" t="inlineStr">
         <is>
           <t>R17</t>
         </is>
       </c>
-      <c r="P659" s="15" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="Q659" s="14" t="inlineStr"/>
-    </row>
-    <row r="660">
-      <c r="A660" s="13" t="inlineStr">
-        <is>
-          <t>30 Aug 2026</t>
-        </is>
-      </c>
-      <c r="B660" s="13" t="inlineStr">
-        <is>
-          <t>Sun</t>
-        </is>
-      </c>
-      <c r="C660" s="13" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="D660" s="13" t="inlineStr">
-        <is>
-          <t>09:40</t>
-        </is>
-      </c>
-      <c r="E660" s="13" t="n">
-        <v>40</v>
-      </c>
-      <c r="F660" s="13" t="inlineStr">
-        <is>
-          <t>Powerful Owl Park</t>
-        </is>
-      </c>
-      <c r="G660" s="13" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="H660" s="13" t="inlineStr">
-        <is>
-          <t>Sub</t>
-        </is>
-      </c>
-      <c r="I660" s="14" t="inlineStr">
-        <is>
-          <t>Pitch 2B</t>
-        </is>
-      </c>
-      <c r="J660" s="13" t="inlineStr">
-        <is>
-          <t>U09</t>
-        </is>
-      </c>
-      <c r="K660" s="14" t="inlineStr">
-        <is>
-          <t>Manningham United Blues FC U09 MiniRoos - Kangaroos Mixed (Emerton's)</t>
-        </is>
-      </c>
-      <c r="L660" s="14" t="inlineStr">
-        <is>
-          <t>Monash City Villarreal FC U09 MiniRoos - Kangaroos Mixed Monash City Villarreal FC U8 Yellow</t>
-        </is>
-      </c>
-      <c r="M660" s="14" t="inlineStr">
-        <is>
-          <t>Coles MiniRoos Mixed Sunday (U6 - U11)</t>
-        </is>
-      </c>
-      <c r="N660" s="13" t="inlineStr">
-        <is>
-          <t>Coles MiniRoos Mixed Sunday East 9 Kangaroos Red</t>
-        </is>
-      </c>
-      <c r="O660" s="13" t="inlineStr">
-        <is>
-          <t>R17</t>
-        </is>
-      </c>
-      <c r="P660" s="15" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="Q660" s="14" t="inlineStr"/>
+      <c r="P660" s="9" t="inlineStr"/>
+      <c r="Q660" s="10" t="inlineStr"/>
     </row>
     <row r="661">
       <c r="A661" s="11" t="inlineStr">
@@ -53220,7 +53208,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -53272,7 +53260,7 @@
     <row r="7">
       <c r="A7" s="17" t="inlineStr">
         <is>
-          <t>A.  Over-capacity moments: 10 found</t>
+          <t>A.  Over-capacity moments: 9 found</t>
         </is>
       </c>
     </row>
@@ -53728,94 +53716,79 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="20" t="n">
-        <v>10</v>
-      </c>
-      <c r="B18" s="20" t="inlineStr">
-        <is>
-          <t>30 Aug 2026</t>
-        </is>
-      </c>
-      <c r="C18" s="20" t="inlineStr">
-        <is>
-          <t>Powerful Owl Park</t>
-        </is>
-      </c>
-      <c r="D18" s="20" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E18" s="21" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="22" t="inlineStr">
+        <is>
+          <t>B.  Peak simultaneous games per ground (busiest moment)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Ground</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Max at once</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>From</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Until</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Pitches in use then</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="21" t="inlineStr">
+        <is>
+          <t>Pettys Reserve</t>
+        </is>
+      </c>
+      <c r="B22" s="20" t="n">
+        <v>7</v>
+      </c>
+      <c r="C22" s="20" t="inlineStr">
+        <is>
+          <t>Sat 16 May 2026</t>
+        </is>
+      </c>
+      <c r="D22" s="20" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="F18" s="20" t="inlineStr">
-        <is>
-          <t>09:40</t>
-        </is>
-      </c>
-      <c r="G18" s="21" t="inlineStr">
-        <is>
-          <t>Pitch over capacity</t>
-        </is>
-      </c>
-      <c r="H18" s="20" t="inlineStr">
-        <is>
-          <t>1×U10-13, 1×U8/9, 2×U6/7 = 1.25</t>
-        </is>
-      </c>
-      <c r="I18" s="20" t="inlineStr">
-        <is>
-          <t>09:00 U11 Pitch 2A (Manningham United Blues FC U11 MiniRoos - Kangaroos Mixed v FC Bulleen Lions U11 MiniRoos - Kangaroos Mixed Anthony &amp; Rob)  |  09:00 U07 Pitch 2 - Midi B (Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Red) v East Malvern Junior SC U07 MiniRoos - Joeys Mixed EMJSC U7 Sunday Orange)  |  09:00 U07 Pitch 2 - Midi A (Manningham United Blues FC U07 MiniRoos - Joeys Mixed (Green) v Doncaster Rovers SC U07 MiniRoos - Joeys Mixed)  |  09:00 U09 Pitch 2B (Manningham United Blues FC U09 MiniRoos - Kangaroos Mixed (Emerton's) v Monash City Villarreal FC U09 MiniRoos - Kangaroos Mixed Monash City Villarreal FC U8 Yellow)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="22" t="inlineStr">
-        <is>
-          <t>B.  Peak simultaneous games per ground (busiest moment)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>Ground</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>Max at once</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>From</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>Until</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>Pitches in use then</t>
+      <c r="E22" s="20" t="inlineStr">
+        <is>
+          <t>09:10</t>
+        </is>
+      </c>
+      <c r="F22" s="21" t="inlineStr">
+        <is>
+          <t>Pitch 1A (Bottom Field), Pitch 1B (Bottom Field), Pitch 1E (Bottom Field) - Quarter Pitch 4v4, Pitch 1F (Bottom Field) - Quarter Pitch 4v4, Pitch 2A (Top Field), Pitch 2C (Top Field) - Quarter Pitch 7v7, Pitch 2D (Top Field) - Quarter Pitch 7v7</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="19" t="inlineStr">
         <is>
-          <t>Pettys Reserve</t>
+          <t>Powerful Owl Park</t>
         </is>
       </c>
       <c r="B23" s="18" t="n">
@@ -53823,7 +53796,7 @@
       </c>
       <c r="C23" s="18" t="inlineStr">
         <is>
-          <t>Sat 16 May 2026</t>
+          <t>Sun 09 Aug 2026</t>
         </is>
       </c>
       <c r="D23" s="18" t="inlineStr">
@@ -53838,65 +53811,35 @@
       </c>
       <c r="F23" s="19" t="inlineStr">
         <is>
-          <t>Pitch 1A (Bottom Field), Pitch 1B (Bottom Field), Pitch 1E (Bottom Field) - Quarter Pitch 4v4, Pitch 1F (Bottom Field) - Quarter Pitch 4v4, Pitch 2A (Top Field), Pitch 2C (Top Field) - Quarter Pitch 7v7, Pitch 2D (Top Field) - Quarter Pitch 7v7</t>
+          <t>Pitch 1 - Midi Field A, Pitch 1 - Midi Field B, Pitch 1B, Pitch 2A, Pitch 2B, Pitch 3A, Pitch 3B</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="21" t="inlineStr">
         <is>
-          <t>Powerful Owl Park</t>
+          <t>Timber Ridge Reserve</t>
         </is>
       </c>
       <c r="B24" s="20" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C24" s="20" t="inlineStr">
         <is>
-          <t>Sun 09 Aug 2026</t>
+          <t>Sat 18 Jul 2026</t>
         </is>
       </c>
       <c r="D24" s="20" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>09:40</t>
         </is>
       </c>
       <c r="E24" s="20" t="inlineStr">
         <is>
-          <t>09:10</t>
+          <t>10:40</t>
         </is>
       </c>
       <c r="F24" s="21" t="inlineStr">
-        <is>
-          <t>Pitch 1 - Midi Field A, Pitch 1 - Midi Field B, Pitch 1B, Pitch 2A, Pitch 2B, Pitch 3A, Pitch 3B</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="19" t="inlineStr">
-        <is>
-          <t>Timber Ridge Reserve</t>
-        </is>
-      </c>
-      <c r="B25" s="18" t="n">
-        <v>2</v>
-      </c>
-      <c r="C25" s="18" t="inlineStr">
-        <is>
-          <t>Sat 18 Jul 2026</t>
-        </is>
-      </c>
-      <c r="D25" s="18" t="inlineStr">
-        <is>
-          <t>09:40</t>
-        </is>
-      </c>
-      <c r="E25" s="18" t="inlineStr">
-        <is>
-          <t>10:40</t>
-        </is>
-      </c>
-      <c r="F25" s="19" t="inlineStr">
         <is>
           <t>Pitch 1A, Pitch 1B</t>
         </is>

</xml_diff>

<commit_message>
Auto-refresh fixtures from Dribl (2026-08-28)
</commit_message>
<xml_diff>
--- a/Manningham_fixtures_and_overlaps.xlsx
+++ b/Manningham_fixtures_and_overlaps.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Games" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overlaps &amp; Peak Load" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="All Games" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Overlaps &amp; Peak Load" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Games'!$A$1:$Q$690</definedName>

</xml_diff>